<commit_message>
chore: spreadsheet rebuild (2026-09-06)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/5/26)</t>
+          <t>Hiring AEs? (9/6/26)</t>
         </is>
       </c>
     </row>
@@ -2498,7 +2498,7 @@
       </c>
       <c r="F53" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://www.365labs.com/car</t>
+          <t>Unknown - HTTP 403 for https://www.365labs.com/car</t>
         </is>
       </c>
     </row>
@@ -9826,9 +9826,9 @@
           <t>Digital dashboards and signage for public safety - exhibited at IACP 2026</t>
         </is>
       </c>
-      <c r="F304" s="4" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F304" s="8" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -11134,7 +11134,7 @@
       </c>
       <c r="F1" s="59" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/5/26)</t>
+          <t>Hiring AEs? (9/6/26)</t>
         </is>
       </c>
     </row>
@@ -14442,7 +14442,7 @@
       </c>
       <c r="F1" s="65" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/5/26)</t>
+          <t>Hiring AEs? (9/6/26)</t>
         </is>
       </c>
     </row>
@@ -17048,7 +17048,7 @@
       </c>
       <c r="F1" s="71" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/5/26)</t>
+          <t>Hiring AEs? (9/6/26)</t>
         </is>
       </c>
     </row>
@@ -17290,7 +17290,7 @@
       </c>
       <c r="F10" s="74" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.affordablehousi</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -17516,7 +17516,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/5/26)</t>
+          <t>Hiring AEs? (9/6/26)</t>
         </is>
       </c>
     </row>
@@ -24646,7 +24646,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/5/26)</t>
+          <t>Hiring AEs? (9/6/26)</t>
         </is>
       </c>
     </row>
@@ -24916,7 +24916,7 @@
       </c>
       <c r="F10" s="21" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://zencity.io/careers</t>
+          <t>Unknown - HTTP 403 for https://zencity.io/careers</t>
         </is>
       </c>
     </row>
@@ -29774,7 +29774,7 @@
       </c>
       <c r="F175" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 500 for https://lcptracker.com/care</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -31728,7 +31728,7 @@
       </c>
       <c r="F241" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://passportworkforce.c</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -31872,7 +31872,7 @@
       </c>
       <c r="F246" s="21" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 403 for https://www.geographicsolut</t>
         </is>
       </c>
     </row>
@@ -38524,7 +38524,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/5/26)</t>
+          <t>Hiring AEs? (9/6/26)</t>
         </is>
       </c>
     </row>
@@ -43034,7 +43034,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/5/26)</t>
+          <t>Hiring AEs? (9/6/26)</t>
         </is>
       </c>
     </row>
@@ -47130,7 +47130,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/5/26)</t>
+          <t>Hiring AEs? (9/6/26)</t>
         </is>
       </c>
     </row>
@@ -47430,7 +47430,7 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://www.modeshift.com/c</t>
+          <t>Unknown - HTTP 403 for https://www.modeshift.com/c</t>
         </is>
       </c>
     </row>
@@ -48056,7 +48056,7 @@
       </c>
       <c r="F32" s="40" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://www.enghouse.com/ca</t>
+          <t>Unknown - HTTP 403 for https://www.enghouse.com/ca</t>
         </is>
       </c>
     </row>
@@ -50140,7 +50140,7 @@
       </c>
       <c r="F102" s="40" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://www.hanoverdisplays</t>
+          <t>Unknown - HTTP 403 for https://www.hanoverdisplays</t>
         </is>
       </c>
     </row>
@@ -50558,7 +50558,7 @@
       </c>
       <c r="F116" s="40" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://qryde.com/employmen</t>
+          <t>Unknown - HTTP 403 for https://qryde.com/employmen</t>
         </is>
       </c>
     </row>
@@ -50936,9 +50936,9 @@
           <t>On-demand transit software converting fixed routes to demand-response for agencies</t>
         </is>
       </c>
-      <c r="F129" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F129" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - HTTP 403 for https://pantonium.com/caree</t>
         </is>
       </c>
     </row>
@@ -53002,7 +53002,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/5/26)</t>
+          <t>Hiring AEs? (9/6/26)</t>
         </is>
       </c>
     </row>
@@ -53720,9 +53720,9 @@
           <t>Adaptive smart street lighting sensors and CMS for municipalities</t>
         </is>
       </c>
-      <c r="F25" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -56532,7 +56532,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/5/26)</t>
+          <t>Hiring AEs? (9/6/26)</t>
         </is>
       </c>
     </row>
@@ -58168,7 +58168,7 @@
       </c>
       <c r="F56" s="51" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -58378,7 +58378,7 @@
       </c>
       <c r="F63" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.grab.careers/en</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -60056,7 +60056,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/5/26)</t>
+          <t>Hiring AEs? (9/6/26)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-09-07)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/6/26)</t>
+          <t>Hiring AEs? (9/7/26)</t>
         </is>
       </c>
     </row>
@@ -11134,7 +11134,7 @@
       </c>
       <c r="F1" s="59" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/6/26)</t>
+          <t>Hiring AEs? (9/7/26)</t>
         </is>
       </c>
     </row>
@@ -14442,7 +14442,7 @@
       </c>
       <c r="F1" s="65" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/6/26)</t>
+          <t>Hiring AEs? (9/7/26)</t>
         </is>
       </c>
     </row>
@@ -17048,7 +17048,7 @@
       </c>
       <c r="F1" s="71" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/6/26)</t>
+          <t>Hiring AEs? (9/7/26)</t>
         </is>
       </c>
     </row>
@@ -17516,7 +17516,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/6/26)</t>
+          <t>Hiring AEs? (9/7/26)</t>
         </is>
       </c>
     </row>
@@ -24646,7 +24646,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/6/26)</t>
+          <t>Hiring AEs? (9/7/26)</t>
         </is>
       </c>
     </row>
@@ -28024,7 +28024,7 @@
       </c>
       <c r="F116" s="23" t="inlineStr">
         <is>
-          <t>Yes - Business Development Manager (Winnipeg)</t>
+          <t>Yes - Account Executive - CES (London)</t>
         </is>
       </c>
     </row>
@@ -30716,7 +30716,7 @@
       </c>
       <c r="F207" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (London)</t>
+          <t>Yes - Account Executive (Singapore, Singapo)</t>
         </is>
       </c>
     </row>
@@ -31728,7 +31728,7 @@
       </c>
       <c r="F241" s="7" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - HTTP 403 for https://passportworkforce.c</t>
         </is>
       </c>
     </row>
@@ -31872,7 +31872,7 @@
       </c>
       <c r="F246" s="21" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.geographicsolut</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -38524,7 +38524,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/6/26)</t>
+          <t>Hiring AEs? (9/7/26)</t>
         </is>
       </c>
     </row>
@@ -42170,7 +42170,7 @@
       </c>
       <c r="F123" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Manager (Barcelona)</t>
+          <t>Yes - Account Executive (Barcelona)</t>
         </is>
       </c>
     </row>
@@ -43034,7 +43034,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/6/26)</t>
+          <t>Hiring AEs? (9/7/26)</t>
         </is>
       </c>
     </row>
@@ -46492,7 +46492,7 @@
       </c>
       <c r="F118" s="34" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -47130,7 +47130,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/6/26)</t>
+          <t>Hiring AEs? (9/7/26)</t>
         </is>
       </c>
     </row>
@@ -50936,9 +50936,9 @@
           <t>On-demand transit software converting fixed routes to demand-response for agencies</t>
         </is>
       </c>
-      <c r="F129" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - HTTP 403 for https://pantonium.com/caree</t>
+      <c r="F129" s="10" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -52004,7 +52004,7 @@
       </c>
       <c r="F165" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -53002,7 +53002,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/6/26)</t>
+          <t>Hiring AEs? (9/7/26)</t>
         </is>
       </c>
     </row>
@@ -53720,9 +53720,9 @@
           <t>Adaptive smart street lighting sensors and CMS for municipalities</t>
         </is>
       </c>
-      <c r="F25" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+      <c r="F25" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -54382,7 +54382,7 @@
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Business Development Specialist only</t>
+          <t>Sales (non-AE) - Business Analyst - Customer Succes only</t>
         </is>
       </c>
     </row>
@@ -54500,9 +54500,9 @@
           <t>Grid software, ADMS and transmission equipment for public and investor utilities</t>
         </is>
       </c>
-      <c r="F51" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -56410,7 +56410,7 @@
       </c>
       <c r="F115" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -56532,7 +56532,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/6/26)</t>
+          <t>Hiring AEs? (9/7/26)</t>
         </is>
       </c>
     </row>
@@ -58168,7 +58168,7 @@
       </c>
       <c r="F56" s="51" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -58586,9 +58586,9 @@
           <t>Alcatraz AI Rock: 3D facial authentication and tailgating detection device that replaces or augments badge readers at secure doors, integrating with existing access control systems.</t>
         </is>
       </c>
-      <c r="F70" s="51" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F70" s="52" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -60056,7 +60056,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/6/26)</t>
+          <t>Hiring AEs? (9/7/26)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-09-08)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/7/26)</t>
+          <t>Hiring AEs? (9/8/26)</t>
         </is>
       </c>
     </row>
@@ -2498,7 +2498,7 @@
       </c>
       <c r="F53" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.365labs.com/car</t>
+          <t>Unknown - HTTP 202 for https://www.365labs.com/car</t>
         </is>
       </c>
     </row>
@@ -9062,7 +9062,7 @@
       </c>
       <c r="F274" s="4" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 503 for https://norix.com/about-us/</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -11134,7 +11134,7 @@
       </c>
       <c r="F1" s="59" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/7/26)</t>
+          <t>Hiring AEs? (9/8/26)</t>
         </is>
       </c>
     </row>
@@ -14442,7 +14442,7 @@
       </c>
       <c r="F1" s="65" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/7/26)</t>
+          <t>Hiring AEs? (9/8/26)</t>
         </is>
       </c>
     </row>
@@ -14986,9 +14986,9 @@
           <t>No-code IT service management, asset management, project portfolio, and integration platform for universities, school districts, and government agencies - exhibited at EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F20" s="69" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Associate Customer Success Manager only</t>
+      <c r="F20" s="68" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -17048,7 +17048,7 @@
       </c>
       <c r="F1" s="71" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/7/26)</t>
+          <t>Hiring AEs? (9/8/26)</t>
         </is>
       </c>
     </row>
@@ -17290,7 +17290,7 @@
       </c>
       <c r="F10" s="74" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 403 for https://www.affordablehousi</t>
         </is>
       </c>
     </row>
@@ -17516,7 +17516,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/7/26)</t>
+          <t>Hiring AEs? (9/8/26)</t>
         </is>
       </c>
     </row>
@@ -23064,7 +23064,7 @@
       </c>
       <c r="F188" s="16" t="inlineStr">
         <is>
-          <t>Yes - Account Executive, Enterprise - Ce (United States - Re)</t>
+          <t>Yes - Account Executive, CMRL - MX (Mexico - Remote)</t>
         </is>
       </c>
     </row>
@@ -24646,7 +24646,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/7/26)</t>
+          <t>Hiring AEs? (9/8/26)</t>
         </is>
       </c>
     </row>
@@ -24916,7 +24916,7 @@
       </c>
       <c r="F10" s="21" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://zencity.io/careers</t>
+          <t>Unknown - HTTP 202 for https://zencity.io/careers</t>
         </is>
       </c>
     </row>
@@ -27932,9 +27932,9 @@
           <t>Objective Build planning and building consent software for government regulators</t>
         </is>
       </c>
-      <c r="F113" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Business Development Manager (Reading)</t>
+      <c r="F113" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Account Director only</t>
         </is>
       </c>
     </row>
@@ -30570,7 +30570,7 @@
       </c>
       <c r="F202" s="21" t="inlineStr">
         <is>
-          <t>None found</t>
+          <t>Unknown - no jobs parsed from iCIMS portal</t>
         </is>
       </c>
     </row>
@@ -31728,7 +31728,7 @@
       </c>
       <c r="F241" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://passportworkforce.c</t>
+          <t>Unknown - HTTP 202 for https://passportworkforce.c</t>
         </is>
       </c>
     </row>
@@ -38524,7 +38524,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/7/26)</t>
+          <t>Hiring AEs? (9/8/26)</t>
         </is>
       </c>
     </row>
@@ -42648,9 +42648,9 @@
           <t>Event volunteer scheduling and check-in for festivals and public events</t>
         </is>
       </c>
-      <c r="F139" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Account Executive Level 2 (Remote, US)</t>
+      <c r="F139" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -43034,7 +43034,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/7/26)</t>
+          <t>Hiring AEs? (9/8/26)</t>
         </is>
       </c>
     </row>
@@ -43924,9 +43924,9 @@
           <t>InformaCast mass notification and paging for school districts</t>
         </is>
       </c>
-      <c r="F31" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -44338,7 +44338,7 @@
       </c>
       <c r="F45" s="10" t="inlineStr">
         <is>
-          <t>Yes - Strategic Sales Director - Enterpr</t>
+          <t>Yes - Sales Account Executive – Mid-Mark</t>
         </is>
       </c>
     </row>
@@ -44908,7 +44908,7 @@
       </c>
       <c r="F64" s="35" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Customer Success Manager only</t>
+          <t>Sales (non-AE) - Customer Success Manager (CA) only</t>
         </is>
       </c>
     </row>
@@ -47130,7 +47130,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/7/26)</t>
+          <t>Hiring AEs? (9/8/26)</t>
         </is>
       </c>
     </row>
@@ -47430,7 +47430,7 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.modeshift.com/c</t>
+          <t>Unknown - HTTP 202 for https://www.modeshift.com/c</t>
         </is>
       </c>
     </row>
@@ -48056,7 +48056,7 @@
       </c>
       <c r="F32" s="40" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.enghouse.com/ca</t>
+          <t>Unknown - HTTP 202 for https://www.enghouse.com/ca</t>
         </is>
       </c>
     </row>
@@ -50140,7 +50140,7 @@
       </c>
       <c r="F102" s="40" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.hanoverdisplays</t>
+          <t>Unknown - HTTP 202 for https://www.hanoverdisplays</t>
         </is>
       </c>
     </row>
@@ -50558,7 +50558,7 @@
       </c>
       <c r="F116" s="40" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://qryde.com/employmen</t>
+          <t>Unknown - HTTP 202 for https://qryde.com/employmen</t>
         </is>
       </c>
     </row>
@@ -52862,7 +52862,7 @@
       </c>
       <c r="F197" s="10" t="inlineStr">
         <is>
-          <t>Yes - Strategic Sales Director - Enterpr</t>
+          <t>Yes - Sales Account Executive – Mid-Mark</t>
         </is>
       </c>
     </row>
@@ -53002,7 +53002,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/7/26)</t>
+          <t>Hiring AEs? (9/8/26)</t>
         </is>
       </c>
     </row>
@@ -56410,7 +56410,7 @@
       </c>
       <c r="F115" s="7" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -56532,7 +56532,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/7/26)</t>
+          <t>Hiring AEs? (9/8/26)</t>
         </is>
       </c>
     </row>
@@ -58016,9 +58016,9 @@
           <t>Baggage handling systems and terminal logistics for airports</t>
         </is>
       </c>
-      <c r="F51" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -58378,7 +58378,7 @@
       </c>
       <c r="F63" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 403 for https://www.grab.careers/en</t>
         </is>
       </c>
     </row>
@@ -58586,9 +58586,9 @@
           <t>Alcatraz AI Rock: 3D facial authentication and tailgating detection device that replaces or augments badge readers at secure doors, integrating with existing access control systems.</t>
         </is>
       </c>
-      <c r="F70" s="52" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F70" s="51" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -60056,7 +60056,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/7/26)</t>
+          <t>Hiring AEs? (9/8/26)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-09-12)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -267,8 +267,8 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -943,7 +943,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/11/26)</t>
+          <t>Hiring AEs? (9/12/26)</t>
         </is>
       </c>
     </row>
@@ -2523,7 +2523,7 @@
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://www.365labs.com/car</t>
+          <t>Unknown - HTTP 403 for https://www.365labs.com/car</t>
         </is>
       </c>
     </row>
@@ -5893,9 +5893,9 @@
           <t>Incident records and ePCR data platform for EMS and fire agencies - exhibited at IAFC FRI 2026</t>
         </is>
       </c>
-      <c r="F168" s="4" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F168" s="11" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="F179" s="7" t="inlineStr">
         <is>
-          <t>Unknown - board is another company's - not read</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -8639,7 +8639,7 @@
       </c>
       <c r="F260" s="11" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - State Partnerships Manager (Austin only</t>
+          <t>Sales (non-AE) - State Partnerships Manager only</t>
         </is>
       </c>
     </row>
@@ -10304,7 +10304,9 @@
         </is>
       </c>
       <c r="B324" s="2" t="n"/>
-      <c r="C324" s="3" t="n"/>
+      <c r="C324" s="3" t="n">
+        <v>2013</v>
+      </c>
       <c r="D324" s="2" t="inlineStr">
         <is>
           <t>Suppliers &amp; Services</t>
@@ -11135,7 +11137,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/11/26)</t>
+          <t>Hiring AEs? (9/12/26)</t>
         </is>
       </c>
     </row>
@@ -12423,9 +12425,9 @@
           <t>Care coordination and PDMP network software (PMP AWARxE, OpenBeds) for states, counties, and health systems (Appriss lineage)</t>
         </is>
       </c>
-      <c r="F47" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F47" s="10" t="inlineStr">
+        <is>
+          <t>Yes - Bamboo Bridge Strategic Account Ma</t>
         </is>
       </c>
     </row>
@@ -12981,9 +12983,9 @@
           <t>Human services EHR and care coordination software for behavioral health, residential, vocational rehab, and food assistance providers - exhibited at NatCon 2026</t>
         </is>
       </c>
-      <c r="F67" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+      <c r="F67" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Customer Success Manager only</t>
         </is>
       </c>
     </row>
@@ -14419,7 +14421,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/11/26)</t>
+          <t>Hiring AEs? (9/12/26)</t>
         </is>
       </c>
     </row>
@@ -16073,7 +16075,7 @@
       </c>
       <c r="F60" s="69" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -17025,7 +17027,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/11/26)</t>
+          <t>Hiring AEs? (9/12/26)</t>
         </is>
       </c>
     </row>
@@ -17493,7 +17495,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/11/26)</t>
+          <t>Hiring AEs? (9/12/26)</t>
         </is>
       </c>
     </row>
@@ -20759,9 +20761,9 @@
           <t>Permitting, compliance, and workflow software for water utilities - exhibited at AWWA ACE 2026, WEFTEC 2026</t>
         </is>
       </c>
-      <c r="F111" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Strategic Account Executive - USA</t>
+      <c r="F111" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Solutions Engineer only</t>
         </is>
       </c>
     </row>
@@ -20936,7 +20938,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t>Floodplain management software: NFIP/CRS compliance, elevation certificates; $26.3M Series B</t>
+          <t>Floodplain management software: NFIP/CRS compliance, elevation certificates; $26.3M Series B - exhibited at StormCon 2026</t>
         </is>
       </c>
       <c r="F117" s="7" t="inlineStr">
@@ -21326,7 +21328,7 @@
       </c>
       <c r="E130" s="13" t="inlineStr">
         <is>
-          <t>Water quality and level monitoring instruments for agencies and utilities - exhibited at AWWA ACE 2026, WEFTEC 2026</t>
+          <t>Water quality and level monitoring instruments for agencies and utilities - exhibited at AWWA ACE 2026, WEFTEC 2026, StormCon 2026</t>
         </is>
       </c>
       <c r="F130" s="16" t="inlineStr">
@@ -21716,7 +21718,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t>Sewer flow monitoring and I&amp;I analytics for municipal wastewater utilities - exhibited at WEFTEC 2026</t>
+          <t>Sewer flow monitoring and I&amp;I analytics for municipal wastewater utilities - exhibited at WEFTEC 2026, StormCon 2026</t>
         </is>
       </c>
       <c r="F143" s="7" t="inlineStr">
@@ -24623,7 +24625,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/11/26)</t>
+          <t>Hiring AEs? (9/12/26)</t>
         </is>
       </c>
     </row>
@@ -24708,12 +24710,12 @@
       </c>
       <c r="E4" s="19" t="inlineStr">
         <is>
-          <t>Municipal websites, 311/CRM, mass notification, and agenda software - exhibited at NLC City Summit 2026, AWWA ACE 2026, 3CMA 2026, WEFTEC 2026</t>
+          <t>Municipal websites, 311/CRM, mass notification, and agenda software - exhibited at NLC City Summit 2026, AWWA ACE 2026, 3CMA 2026, WEFTEC 2026, StormCon 2026</t>
         </is>
       </c>
       <c r="F4" s="22" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -24771,7 +24773,7 @@
           <t>Community surveys, benchmarking, and budget simulation (owns National Research Center)</t>
         </is>
       </c>
-      <c r="F6" s="23" t="inlineStr">
+      <c r="F6" s="22" t="inlineStr">
         <is>
           <t>Yes - Account Executive (Madison, WI)</t>
         </is>
@@ -24893,7 +24895,7 @@
       </c>
       <c r="F10" s="21" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://zencity.io/careers</t>
+          <t>Unknown - HTTP 403 for https://zencity.io/careers</t>
         </is>
       </c>
     </row>
@@ -25011,7 +25013,7 @@
           <t>Community participation platform: surveys, ideation, participatory budgeting (ex-CitizenLab) - exhibited at 3CMA 2026</t>
         </is>
       </c>
-      <c r="F14" s="23" t="inlineStr">
+      <c r="F14" s="22" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -25551,7 +25553,7 @@
           <t>Citizen identity and digital service portals (CitizenOne) plus digital trust/signatures (Notarius)</t>
         </is>
       </c>
-      <c r="F32" s="22" t="inlineStr">
+      <c r="F32" s="23" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Représentant du développement des  only</t>
         </is>
@@ -26019,7 +26021,7 @@
           <t>Workflow automation, online forms and eSignature for state/local agencies - exhibited at Healthcare IT Connect 2026</t>
         </is>
       </c>
-      <c r="F48" s="22" t="inlineStr">
+      <c r="F48" s="23" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Customer Success Manager only</t>
         </is>
@@ -26197,7 +26199,7 @@
           <t>Digital experience platform and forms for government; UK vendor with US clients</t>
         </is>
       </c>
-      <c r="F54" s="23" t="inlineStr">
+      <c r="F54" s="22" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -26377,7 +26379,7 @@
           <t>Cloud apps for permits, code enforcement and citizen requests in small cities</t>
         </is>
       </c>
-      <c r="F60" s="23" t="inlineStr">
+      <c r="F60" s="22" t="inlineStr">
         <is>
           <t>Yes - Sales Account Executive - Smart XE</t>
         </is>
@@ -26435,7 +26437,7 @@
           <t>GIS, asset and citizen-facing software for small and rural local governments</t>
         </is>
       </c>
-      <c r="F62" s="22" t="inlineStr">
+      <c r="F62" s="23" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -26887,7 +26889,7 @@
           <t>Permitting, budgeting, procurement, and asset management cloud suite (Cox-owned) - exhibited at GFOA 2026, NLC City Summit 2026, NACE 2026, AWWA ACE 2026, GMIS International 2026, Maryland Municipal League 2026, WEFTEC 2026</t>
         </is>
       </c>
-      <c r="F78" s="23" t="inlineStr">
+      <c r="F78" s="22" t="inlineStr">
         <is>
           <t>Yes - Enterprise Account Executive (US | Illinois | Ch)</t>
         </is>
@@ -26947,7 +26949,7 @@
           <t>AI permitting and licensing platform: 24/7 resident assistant, AI code-compliance review - exhibited at NLC City Summit 2026, Maryland Municipal League 2026</t>
         </is>
       </c>
-      <c r="F80" s="23" t="inlineStr">
+      <c r="F80" s="22" t="inlineStr">
         <is>
           <t>Yes - Business Development Manager (New York, NY)</t>
         </is>
@@ -27007,7 +27009,7 @@
           <t>Special event, film, and complex permit approval workflow SaaS for cities</t>
         </is>
       </c>
-      <c r="F82" s="23" t="inlineStr">
+      <c r="F82" s="22" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -27367,7 +27369,7 @@
           <t>ProjectDox electronic plan review for building, fire, planning, and public works agencies</t>
         </is>
       </c>
-      <c r="F94" s="23" t="inlineStr">
+      <c r="F94" s="22" t="inlineStr">
         <is>
           <t>Yes - Account Executive (GovTech SaaS)</t>
         </is>
@@ -27887,7 +27889,7 @@
           <t>Electronic plan review software for building and public works departments</t>
         </is>
       </c>
-      <c r="F112" s="23" t="inlineStr">
+      <c r="F112" s="22" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -28059,7 +28061,7 @@
           <t>Objective Build planning and building consent software for government regulators</t>
         </is>
       </c>
-      <c r="F118" s="22" t="inlineStr">
+      <c r="F118" s="23" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Account Director only</t>
         </is>
@@ -28233,7 +28235,7 @@
           <t>The govtech giant: ERP, courts, public safety, permitting, and payments - exhibited at GFOA 2026, NLC City Summit 2026, PSHRA 2026, AWWA ACE 2026, IAAO 2026, NASCIO 2026, GMIS International 2026, NACM 2026, APPA Probation 2026, Iowa State Association of Counties 2026, Maryland Municipal League 2026, IAFC FRI 2026, APCO 2026, NAPT Summit 2026</t>
         </is>
       </c>
-      <c r="F124" s="23" t="inlineStr">
+      <c r="F124" s="22" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -28353,7 +28355,7 @@
           <t>Local government ERP: financials, property tax, assessing, utility billing - Michigan standard going national - exhibited at GFOA 2026</t>
         </is>
       </c>
-      <c r="F128" s="23" t="inlineStr">
+      <c r="F128" s="22" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -28473,7 +28475,7 @@
           <t>AI workflow for county assessors: deed processing, exemptions, taxpayer communication (YC S17) - exhibited at NLC City Summit 2026, IAAO 2026</t>
         </is>
       </c>
-      <c r="F132" s="22" t="inlineStr">
+      <c r="F132" s="23" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Customer Success Manager (West Coa only</t>
         </is>
@@ -28533,7 +28535,7 @@
           <t>VIP public-sector ERP for Ohio-area local governments; 100% employee-owned - exhibited at GFOA 2026</t>
         </is>
       </c>
-      <c r="F134" s="22" t="inlineStr">
+      <c r="F134" s="23" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -28745,7 +28747,7 @@
       </c>
       <c r="F141" s="9" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Business Development Officer only</t>
+          <t>Sales (non-AE) - Senior Business Development Office only</t>
         </is>
       </c>
     </row>
@@ -29301,7 +29303,7 @@
           <t>Cloud ERP for cities and counties covering finance, budgeting, utility billing, payroll, permitting, licensing and code enforcement, built on Oracle NetSuite - exhibited at GFOA 2026</t>
         </is>
       </c>
-      <c r="F160" s="23" t="inlineStr">
+      <c r="F160" s="22" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -29599,7 +29601,7 @@
           <t>Bill presentment and payments for governments and utilities (public co) - exhibited at GFOA 2026, NAHRO 2026, EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F170" s="23" t="inlineStr">
+      <c r="F170" s="22" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -29779,7 +29781,7 @@
           <t>Source-to-contract procurement ecosystem (BidNet Direct, Periscope S2G; ex-mdf commerce)</t>
         </is>
       </c>
-      <c r="F176" s="23" t="inlineStr">
+      <c r="F176" s="22" t="inlineStr">
         <is>
           <t>Yes - Account Executive (United States)</t>
         </is>
@@ -30079,7 +30081,7 @@
           <t>Supplier onboarding and payee identity verification preventing payments fraud for gov and higher-ed - exhibited at GFOA 2026</t>
         </is>
       </c>
-      <c r="F186" s="23" t="inlineStr">
+      <c r="F186" s="22" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -30109,9 +30111,9 @@
           <t>Supplier ratings and performance reviews platform for public-sector buyers</t>
         </is>
       </c>
-      <c r="F187" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F187" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -30493,7 +30495,7 @@
           <t>Expense management and payment software - exhibited at NIGP 2026, NACUBO 2026</t>
         </is>
       </c>
-      <c r="F200" s="23" t="inlineStr">
+      <c r="F200" s="22" t="inlineStr">
         <is>
           <t>Yes - Account Executive - Midmarket (rem (Atlanta, GA)</t>
         </is>
@@ -30841,7 +30843,7 @@
           <t>Source-to-pay suite with public sector practice serving states and agencies</t>
         </is>
       </c>
-      <c r="F212" s="23" t="inlineStr">
+      <c r="F212" s="22" t="inlineStr">
         <is>
           <t>Yes - Account Executive (Singapore, Singapo)</t>
         </is>
@@ -30933,7 +30935,7 @@
       </c>
       <c r="F215" s="10" t="inlineStr">
         <is>
-          <t>Yes - Enterprise Account Executive – Hea (United States)</t>
+          <t>Yes - Enterprise Account Executive (United States)</t>
         </is>
       </c>
     </row>
@@ -31733,7 +31735,7 @@
           <t>Benefits administration and enrollment built exclusively for public-sector employers - exhibited at SALGBA 2026</t>
         </is>
       </c>
-      <c r="F242" s="22" t="inlineStr">
+      <c r="F242" s="23" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -31855,7 +31857,7 @@
       </c>
       <c r="F246" s="21" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://passportworkforce.c</t>
+          <t>Unknown - HTTP 403 for https://passportworkforce.c</t>
         </is>
       </c>
     </row>
@@ -31913,7 +31915,7 @@
           <t>Digital heart health app and monitoring - exhibited at NACo 2026, PSHRA 2026, SALGBA 2026</t>
         </is>
       </c>
-      <c r="F248" s="22" t="inlineStr">
+      <c r="F248" s="23" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Associate Director, Client Success only</t>
         </is>
@@ -31937,9 +31939,9 @@
           <t>EHS compliance software and services - exhibited at ICMA 2025</t>
         </is>
       </c>
-      <c r="F249" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Account Executive - Automotive (Atlanta, GA)</t>
+      <c r="F249" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -32203,7 +32205,7 @@
           <t>Time, attendance and scheduling for government, education and public safety - exhibited at GFOA 2026</t>
         </is>
       </c>
-      <c r="F258" s="23" t="inlineStr">
+      <c r="F258" s="22" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -32501,7 +32503,7 @@
           <t>License verification and workforce compliance for agencies and regulators</t>
         </is>
       </c>
-      <c r="F268" s="23" t="inlineStr">
+      <c r="F268" s="22" t="inlineStr">
         <is>
           <t>Yes - Sales Executive - Central Region ( (Remote - US)</t>
         </is>
@@ -32561,9 +32563,9 @@
           <t>Local government ERP including payroll and personnel modules - exhibited at GFOA 2026, Maryland Municipal League 2026</t>
         </is>
       </c>
-      <c r="F270" s="22" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Client Success Manager only</t>
+      <c r="F270" s="23" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Sales Development Representative only</t>
         </is>
       </c>
     </row>
@@ -32829,7 +32831,7 @@
       </c>
       <c r="F279" s="7" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -33437,7 +33439,7 @@
           <t>Work management and collaboration software - exhibited at NACo 2026</t>
         </is>
       </c>
-      <c r="F300" s="23" t="inlineStr">
+      <c r="F300" s="22" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -33489,7 +33491,7 @@
           <t>Cybersecurity software and network security platforms - exhibited at IACP 2026, NASCIO 2026, CoSN 2026, EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F302" s="23" t="inlineStr">
+      <c r="F302" s="22" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -33549,7 +33551,7 @@
           <t>Claude, sold to state and local agencies through GSA and cooperative vehicles alongside its commercial business</t>
         </is>
       </c>
-      <c r="F304" s="23" t="inlineStr">
+      <c r="F304" s="22" t="inlineStr">
         <is>
           <t>Yes - Account Executive, AI Native (New York City, NY;)</t>
         </is>
@@ -33827,7 +33829,7 @@
           <t>Strategic planning, performance measurement, and public dashboards built for local government</t>
         </is>
       </c>
-      <c r="F314" s="23" t="inlineStr">
+      <c r="F314" s="22" t="inlineStr">
         <is>
           <t>Yes - Senior Account Executive - Public  (Canada)</t>
         </is>
@@ -33887,7 +33889,7 @@
           <t>Policy and rulemaking workflow: draft, route, approve, and track regulations for agencies</t>
         </is>
       </c>
-      <c r="F316" s="23" t="inlineStr">
+      <c r="F316" s="22" t="inlineStr">
         <is>
           <t>Yes - Strategic Account Executive - West (Remote)</t>
         </is>
@@ -34001,7 +34003,7 @@
           <t>Public affairs and legislative tracking software - exhibited at NACo 2026, NLC City Summit 2026</t>
         </is>
       </c>
-      <c r="F320" s="23" t="inlineStr">
+      <c r="F320" s="22" t="inlineStr">
         <is>
           <t>Yes - Account Manager (Washington D.C.)</t>
         </is>
@@ -34173,7 +34175,7 @@
           <t>Governance, performance and risk management platform for public sector organizations</t>
         </is>
       </c>
-      <c r="F326" s="22" t="inlineStr">
+      <c r="F326" s="23" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -34819,7 +34821,7 @@
           <t>Digital ballot scanning, tabulation and audit systems for election offices</t>
         </is>
       </c>
-      <c r="F348" s="22" t="inlineStr">
+      <c r="F348" s="23" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -35239,7 +35241,7 @@
           <t>Ballot tracking, electronic ballot delivery and election tools for jurisdictions</t>
         </is>
       </c>
-      <c r="F362" s="22" t="inlineStr">
+      <c r="F362" s="23" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -35533,7 +35535,7 @@
           <t>Ballot printing and election materials for county boards of elections - exhibited at Maryland Municipal League 2026</t>
         </is>
       </c>
-      <c r="F372" s="23" t="inlineStr">
+      <c r="F372" s="22" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -36259,7 +36261,7 @@
           <t>Web-based mapping, demographic, and consumer data visualization application for university and public library patrons - exhibited at PLA 2026</t>
         </is>
       </c>
-      <c r="F398" s="23" t="inlineStr">
+      <c r="F398" s="22" t="inlineStr">
         <is>
           <t>Yes - Senior Account Executive - B2B Saa</t>
         </is>
@@ -36529,7 +36531,7 @@
           <t>Research databases, ebook collections and discovery software licensed to public libraries, academic libraries, schools and healthcare organizations - exhibited at PLA 2026</t>
         </is>
       </c>
-      <c r="F408" s="23" t="inlineStr">
+      <c r="F408" s="22" t="inlineStr">
         <is>
           <t>Yes - Regional Sales Manager, AMC – Virg</t>
         </is>
@@ -38081,7 +38083,7 @@
           <t>Payment processing platform - exhibited at ICMA 2025</t>
         </is>
       </c>
-      <c r="F466" s="23" t="inlineStr">
+      <c r="F466" s="22" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -38229,7 +38231,7 @@
           <t>Construction project management software - exhibited at ICMA 2025, PWX 2026</t>
         </is>
       </c>
-      <c r="F472" s="22" t="inlineStr">
+      <c r="F472" s="23" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -38707,7 +38709,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/11/26)</t>
+          <t>Hiring AEs? (9/12/26)</t>
         </is>
       </c>
     </row>
@@ -41427,7 +41429,7 @@
       </c>
       <c r="F92" s="29" t="inlineStr">
         <is>
-          <t>Yes - Account Manager (Remote - Canada)</t>
+          <t>Yes - Sr. Account Manager - Pacific West (Remote - Californi)</t>
         </is>
       </c>
     </row>
@@ -42989,7 +42991,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/11/26)</t>
+          <t>Hiring AEs? (9/12/26)</t>
         </is>
       </c>
     </row>
@@ -43049,7 +43051,7 @@
       </c>
       <c r="F3" s="10" t="inlineStr">
         <is>
-          <t>Yes - Sales Executive, Cross-Sell (North (Remote Worker - N/)</t>
+          <t>Yes - Senior Sales Executive (VA/WV/OH) (Remote Worker - N/)</t>
         </is>
       </c>
     </row>
@@ -43553,7 +43555,7 @@
       </c>
       <c r="F20" s="33" t="inlineStr">
         <is>
-          <t>Yes - Account Executive - Canada (Toronto, Ontario)</t>
+          <t>Yes - Commercial Account Executive - Cen (Dallas, Texas)</t>
         </is>
       </c>
     </row>
@@ -46281,7 +46283,7 @@
       </c>
       <c r="F112" s="35" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Inside Sales Account Executive - M only</t>
+          <t>Sales (non-AE) - Senior Salesforce Developer only</t>
         </is>
       </c>
     </row>
@@ -47085,7 +47087,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/11/26)</t>
+          <t>Hiring AEs? (9/12/26)</t>
         </is>
       </c>
     </row>
@@ -47385,7 +47387,7 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://www.modeshift.com/c</t>
+          <t>Unknown - HTTP 403 for https://www.modeshift.com/c</t>
         </is>
       </c>
     </row>
@@ -47981,7 +47983,7 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://www.enghouse.com/ca</t>
+          <t>Unknown - HTTP 403 for https://www.enghouse.com/ca</t>
         </is>
       </c>
     </row>
@@ -48835,7 +48837,7 @@
       </c>
       <c r="F60" s="40" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -50035,7 +50037,7 @@
       </c>
       <c r="F100" s="40" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://www.hanoverdisplays</t>
+          <t>Unknown - HTTP 403 for https://www.hanoverdisplays</t>
         </is>
       </c>
     </row>
@@ -50423,7 +50425,7 @@
       </c>
       <c r="F113" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://qryde.com/employmen</t>
+          <t>Unknown - HTTP 403 for https://qryde.com/employmen</t>
         </is>
       </c>
     </row>
@@ -50771,9 +50773,9 @@
           <t>On-demand transit software converting fixed routes to demand-response for agencies</t>
         </is>
       </c>
-      <c r="F125" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+      <c r="F125" s="10" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -52391,9 +52393,9 @@
           <t>Security and intelligence analytics software - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F181" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F181" s="10" t="inlineStr">
+        <is>
+          <t>Yes - Enterprise Sales Executive – New L (2 Locations)</t>
         </is>
       </c>
     </row>
@@ -52727,7 +52729,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/11/26)</t>
+          <t>Hiring AEs? (9/12/26)</t>
         </is>
       </c>
     </row>
@@ -54285,9 +54287,9 @@
           <t>Metering, CIS, billing and grid analytics for public power utilities</t>
         </is>
       </c>
-      <c r="F53" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - HTTP 301 for https://www.oracle.com/corp</t>
+      <c r="F53" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -54977,7 +54979,7 @@
       </c>
       <c r="F76" s="45" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -56257,7 +56259,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/11/26)</t>
+          <t>Hiring AEs? (9/12/26)</t>
         </is>
       </c>
     </row>
@@ -57741,9 +57743,9 @@
           <t>Baggage handling systems and terminal logistics for airports</t>
         </is>
       </c>
-      <c r="F51" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F51" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -59327,9 +59329,9 @@
           <t>Parking operations, payments and analytics for airports and venues</t>
         </is>
       </c>
-      <c r="F104" s="52" t="inlineStr">
-        <is>
-          <t>Yes - Associate Account Executive (Dallas)</t>
+      <c r="F104" s="53" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Client Success Manager only</t>
         </is>
       </c>
     </row>
@@ -59781,7 +59783,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/11/26)</t>
+          <t>Hiring AEs? (9/12/26)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-09-13)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -230,7 +230,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -357,7 +357,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="25" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="25" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -943,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/12/26)</t>
+          <t>Hiring AEs? (9/13/26)</t>
         </is>
       </c>
     </row>
@@ -2523,7 +2522,7 @@
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.365labs.com/car</t>
+          <t>Unknown - HTTP 202 for https://www.365labs.com/car</t>
         </is>
       </c>
     </row>
@@ -5893,9 +5892,9 @@
           <t>Incident records and ePCR data platform for EMS and fire agencies - exhibited at IAFC FRI 2026</t>
         </is>
       </c>
-      <c r="F168" s="11" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F168" s="4" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -11137,7 +11136,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/12/26)</t>
+          <t>Hiring AEs? (9/13/26)</t>
         </is>
       </c>
     </row>
@@ -11189,7 +11188,7 @@
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -11213,7 +11212,7 @@
       </c>
       <c r="F4" s="63" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -11285,7 +11284,7 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -11309,7 +11308,7 @@
       </c>
       <c r="F8" s="63" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -12137,7 +12136,7 @@
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -12161,7 +12160,7 @@
       </c>
       <c r="F38" s="63" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -14421,7 +14420,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/12/26)</t>
+          <t>Hiring AEs? (9/13/26)</t>
         </is>
       </c>
     </row>
@@ -17027,7 +17026,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/12/26)</t>
+          <t>Hiring AEs? (9/13/26)</t>
         </is>
       </c>
     </row>
@@ -17431,9 +17430,9 @@
           <t>GURU site selection, property data and property tax mapping platform for economic development organizations and assessor offices - exhibited at IEDC 2026</t>
         </is>
       </c>
-      <c r="F16" s="76" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F16" s="75" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -17495,7 +17494,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/12/26)</t>
+          <t>Hiring AEs? (9/13/26)</t>
         </is>
       </c>
     </row>
@@ -22511,9 +22510,9 @@
           <t>Network data analytics software for water utilities covering leakage, infiltration, energy use and capital planning - exhibited at AWWA ACE 2026</t>
         </is>
       </c>
-      <c r="F170" s="16" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F170" s="15" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -24625,7 +24624,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/12/26)</t>
+          <t>Hiring AEs? (9/13/26)</t>
         </is>
       </c>
     </row>
@@ -24895,7 +24894,7 @@
       </c>
       <c r="F10" s="21" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://zencity.io/careers</t>
+          <t>Unknown - HTTP 202 for https://zencity.io/careers</t>
         </is>
       </c>
     </row>
@@ -26199,9 +26198,9 @@
           <t>Digital experience platform and forms for government; UK vendor with US clients</t>
         </is>
       </c>
-      <c r="F54" s="22" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F54" s="21" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -30111,9 +30110,9 @@
           <t>Supplier ratings and performance reviews platform for public-sector buyers</t>
         </is>
       </c>
-      <c r="F187" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F187" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -30845,7 +30844,7 @@
       </c>
       <c r="F212" s="22" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (Singapore, Singapo)</t>
+          <t>Yes - Account Executive (London)</t>
         </is>
       </c>
     </row>
@@ -31857,7 +31856,7 @@
       </c>
       <c r="F246" s="21" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://passportworkforce.c</t>
+          <t>Unknown - HTTP 202 for https://passportworkforce.c</t>
         </is>
       </c>
     </row>
@@ -31967,7 +31966,7 @@
       </c>
       <c r="F250" s="21" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -32175,9 +32174,9 @@
           <t>Employee benefits, enrollment and HR services for public sector employers</t>
         </is>
       </c>
-      <c r="F257" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - no ATS on file</t>
+      <c r="F257" s="10" t="inlineStr">
+        <is>
+          <t>Yes - Account Manager (3 Locations)</t>
         </is>
       </c>
     </row>
@@ -32297,7 +32296,7 @@
       </c>
       <c r="F261" s="7" t="inlineStr">
         <is>
-          <t>Unknown - board is another company's - not read</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -33771,7 +33770,7 @@
       </c>
       <c r="F312" s="21" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -38709,7 +38708,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/12/26)</t>
+          <t>Hiring AEs? (9/13/26)</t>
         </is>
       </c>
     </row>
@@ -42991,7 +42990,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/12/26)</t>
+          <t>Hiring AEs? (9/13/26)</t>
         </is>
       </c>
     </row>
@@ -47087,7 +47086,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/12/26)</t>
+          <t>Hiring AEs? (9/13/26)</t>
         </is>
       </c>
     </row>
@@ -47387,7 +47386,7 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.modeshift.com/c</t>
+          <t>Unknown - HTTP 202 for https://www.modeshift.com/c</t>
         </is>
       </c>
     </row>
@@ -47983,7 +47982,7 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.enghouse.com/ca</t>
+          <t>Unknown - HTTP 202 for https://www.enghouse.com/ca</t>
         </is>
       </c>
     </row>
@@ -49797,7 +49796,7 @@
       </c>
       <c r="F92" s="39" t="inlineStr">
         <is>
-          <t>Yes - Strategic Account Executive (North Carolina_Rem)</t>
+          <t>Yes - Strategic Account Executive (Tennessee_Remote_C)</t>
         </is>
       </c>
     </row>
@@ -50037,7 +50036,7 @@
       </c>
       <c r="F100" s="40" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.hanoverdisplays</t>
+          <t>Unknown - HTTP 202 for https://www.hanoverdisplays</t>
         </is>
       </c>
     </row>
@@ -50773,9 +50772,9 @@
           <t>On-demand transit software converting fixed routes to demand-response for agencies</t>
         </is>
       </c>
-      <c r="F125" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F125" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -52729,7 +52728,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/12/26)</t>
+          <t>Hiring AEs? (9/13/26)</t>
         </is>
       </c>
     </row>
@@ -55543,7 +55542,7 @@
       </c>
       <c r="F95" s="10" t="inlineStr">
         <is>
-          <t>Yes - Senior Account Executive (Portland, ME)</t>
+          <t>Yes - Enterprise Account Executive (Portland, ME)</t>
         </is>
       </c>
     </row>
@@ -56259,7 +56258,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/12/26)</t>
+          <t>Hiring AEs? (9/13/26)</t>
         </is>
       </c>
     </row>
@@ -57357,7 +57356,7 @@
       </c>
       <c r="F38" s="51" t="inlineStr">
         <is>
-          <t>None found</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -58375,7 +58374,7 @@
       </c>
       <c r="F72" s="51" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -59783,7 +59782,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/12/26)</t>
+          <t>Hiring AEs? (9/13/26)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-09-14)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/13/26)</t>
+          <t>Hiring AEs? (9/14/26)</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2522,7 @@
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://www.365labs.com/car</t>
+          <t>Unknown - HTTP 403 for https://www.365labs.com/car</t>
         </is>
       </c>
     </row>
@@ -3272,7 +3272,7 @@
       </c>
       <c r="F79" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 500 for https://www.lenslock.com/ca</t>
         </is>
       </c>
     </row>
@@ -11136,7 +11136,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/13/26)</t>
+          <t>Hiring AEs? (9/14/26)</t>
         </is>
       </c>
     </row>
@@ -14420,7 +14420,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/13/26)</t>
+          <t>Hiring AEs? (9/14/26)</t>
         </is>
       </c>
     </row>
@@ -17026,7 +17026,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/13/26)</t>
+          <t>Hiring AEs? (9/14/26)</t>
         </is>
       </c>
     </row>
@@ -17494,7 +17494,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/13/26)</t>
+          <t>Hiring AEs? (9/14/26)</t>
         </is>
       </c>
     </row>
@@ -22682,7 +22682,7 @@
       </c>
       <c r="F176" s="16" t="inlineStr">
         <is>
-          <t>Yes - Business Development Manager (Remo (Sydney, Australia )</t>
+          <t>Yes - Partner Account Manager (Remote - Canada)</t>
         </is>
       </c>
     </row>
@@ -23998,7 +23998,7 @@
       </c>
       <c r="F220" s="15" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 503 for https://www.sawatchlabs.com</t>
         </is>
       </c>
     </row>
@@ -24624,7 +24624,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/13/26)</t>
+          <t>Hiring AEs? (9/14/26)</t>
         </is>
       </c>
     </row>
@@ -24894,7 +24894,7 @@
       </c>
       <c r="F10" s="21" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://zencity.io/careers</t>
+          <t>Unknown - HTTP 403 for https://zencity.io/careers</t>
         </is>
       </c>
     </row>
@@ -31856,7 +31856,7 @@
       </c>
       <c r="F246" s="21" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://passportworkforce.c</t>
+          <t>Unknown - HTTP 403 for https://passportworkforce.c</t>
         </is>
       </c>
     </row>
@@ -32176,7 +32176,7 @@
       </c>
       <c r="F257" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Manager (3 Locations)</t>
+          <t>Yes - Account Manager (Denver, Colorado)</t>
         </is>
       </c>
     </row>
@@ -34174,9 +34174,9 @@
           <t>Governance, performance and risk management platform for public sector organizations</t>
         </is>
       </c>
-      <c r="F326" s="23" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F326" s="22" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -38708,7 +38708,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/13/26)</t>
+          <t>Hiring AEs? (9/14/26)</t>
         </is>
       </c>
     </row>
@@ -42990,7 +42990,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/13/26)</t>
+          <t>Hiring AEs? (9/14/26)</t>
         </is>
       </c>
     </row>
@@ -47086,7 +47086,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/13/26)</t>
+          <t>Hiring AEs? (9/14/26)</t>
         </is>
       </c>
     </row>
@@ -47386,7 +47386,7 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://www.modeshift.com/c</t>
+          <t>Unknown - HTTP 403 for https://www.modeshift.com/c</t>
         </is>
       </c>
     </row>
@@ -47982,7 +47982,7 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://www.enghouse.com/ca</t>
+          <t>Unknown - HTTP 403 for https://www.enghouse.com/ca</t>
         </is>
       </c>
     </row>
@@ -49796,7 +49796,7 @@
       </c>
       <c r="F92" s="39" t="inlineStr">
         <is>
-          <t>Yes - Strategic Account Executive (Tennessee_Remote_C)</t>
+          <t>Yes - Strategic Account Executive (North Carolina_Rem)</t>
         </is>
       </c>
     </row>
@@ -50036,7 +50036,7 @@
       </c>
       <c r="F100" s="40" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://www.hanoverdisplays</t>
+          <t>Unknown - HTTP 403 for https://www.hanoverdisplays</t>
         </is>
       </c>
     </row>
@@ -52728,7 +52728,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/13/26)</t>
+          <t>Hiring AEs? (9/14/26)</t>
         </is>
       </c>
     </row>
@@ -56258,7 +56258,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/13/26)</t>
+          <t>Hiring AEs? (9/14/26)</t>
         </is>
       </c>
     </row>
@@ -58374,7 +58374,7 @@
       </c>
       <c r="F72" s="51" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -59782,7 +59782,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/13/26)</t>
+          <t>Hiring AEs? (9/14/26)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-09-16)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/14/26)</t>
+          <t>Hiring AEs? (9/16/26)</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
       </c>
       <c r="F78" s="4" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 404 for https://www.ndi-rs.com/care</t>
         </is>
       </c>
     </row>
@@ -3272,7 +3272,7 @@
       </c>
       <c r="F79" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 500 for https://www.lenslock.com/ca</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -3422,7 +3422,7 @@
       </c>
       <c r="F84" s="8" t="inlineStr">
         <is>
-          <t>Yes - Business Development Manager - LAT (São Paulo, Brazil)</t>
+          <t>Yes - Business Development Manager (Rome, Rome, Italy)</t>
         </is>
       </c>
     </row>
@@ -4350,9 +4350,9 @@
           <t>Cyber-over-RF counter-drone detect, track, and mitigate systems for LE, prisons, and infrastructure</t>
         </is>
       </c>
-      <c r="F115" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F115" s="10" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -5232,9 +5232,9 @@
           <t>Video review and analytics software used by police investigators</t>
         </is>
       </c>
-      <c r="F146" s="11" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F146" s="4" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -11136,7 +11136,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/14/26)</t>
+          <t>Hiring AEs? (9/16/26)</t>
         </is>
       </c>
     </row>
@@ -13192,9 +13192,9 @@
           <t>AI clinical documentation and chart auditing platform purpose-built for behavioral health providers including CCBHCs and human services organizations - exhibited at NatCon 2026</t>
         </is>
       </c>
-      <c r="F75" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F75" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - VP of Revenue only</t>
         </is>
       </c>
     </row>
@@ -14420,7 +14420,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/14/26)</t>
+          <t>Hiring AEs? (9/16/26)</t>
         </is>
       </c>
     </row>
@@ -15936,7 +15936,7 @@
       </c>
       <c r="F55" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (US - Remote)</t>
+          <t>Yes - Account Executive, EMEA (UK - Remote)</t>
         </is>
       </c>
     </row>
@@ -16386,7 +16386,7 @@
       </c>
       <c r="F72" s="70" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Vice President, Sales only</t>
+          <t>Sales (non-AE) - Senior Solutions Engineer only</t>
         </is>
       </c>
     </row>
@@ -17026,7 +17026,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/14/26)</t>
+          <t>Hiring AEs? (9/16/26)</t>
         </is>
       </c>
     </row>
@@ -17494,7 +17494,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/14/26)</t>
+          <t>Hiring AEs? (9/16/26)</t>
         </is>
       </c>
     </row>
@@ -17642,9 +17642,9 @@
           <t>AI recycling-sorting robots and real-time bale/line data</t>
         </is>
       </c>
-      <c r="F6" s="16" t="inlineStr">
-        <is>
-          <t>Yes - Account Executive - Climate Tech ( (Remote East Coast )</t>
+      <c r="F6" s="15" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -22682,7 +22682,7 @@
       </c>
       <c r="F176" s="16" t="inlineStr">
         <is>
-          <t>Yes - Partner Account Manager (Remote - Canada)</t>
+          <t>Yes - Partner Account Manager UK&amp;I (London, England - )</t>
         </is>
       </c>
     </row>
@@ -23998,7 +23998,7 @@
       </c>
       <c r="F220" s="15" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 503 for https://www.sawatchlabs.com</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -24624,7 +24624,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/14/26)</t>
+          <t>Hiring AEs? (9/16/26)</t>
         </is>
       </c>
     </row>
@@ -26022,7 +26022,7 @@
       </c>
       <c r="F48" s="23" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Customer Success Manager only</t>
+          <t>Sales (non-AE) - Sales Development Representative only</t>
         </is>
       </c>
     </row>
@@ -26380,7 +26380,7 @@
       </c>
       <c r="F60" s="22" t="inlineStr">
         <is>
-          <t>Yes - Sales Account Executive - Smart XE</t>
+          <t>Yes - Sales Account Executive - GovTech</t>
         </is>
       </c>
     </row>
@@ -33582,7 +33582,7 @@
       </c>
       <c r="F305" s="9" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Account Director - Tokyo only</t>
+          <t>Sales (non-AE) - Account Director, Large Enterprise only</t>
         </is>
       </c>
     </row>
@@ -38708,7 +38708,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/14/26)</t>
+          <t>Hiring AEs? (9/16/26)</t>
         </is>
       </c>
     </row>
@@ -39122,7 +39122,7 @@
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (Howell, MI)</t>
+          <t>Yes - Account Executive (Hillsboro, TX)</t>
         </is>
       </c>
     </row>
@@ -40526,9 +40526,9 @@
           <t>Space and facility booking platform used by municipal and campus facilities</t>
         </is>
       </c>
-      <c r="F62" s="27" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Director, Sales (Hybrid / Boston,  only</t>
+      <c r="F62" s="28" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -42990,7 +42990,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/14/26)</t>
+          <t>Hiring AEs? (9/16/26)</t>
         </is>
       </c>
     </row>
@@ -43050,7 +43050,7 @@
       </c>
       <c r="F3" s="10" t="inlineStr">
         <is>
-          <t>Yes - Senior Sales Executive (VA/WV/OH) (Remote Worker - N/)</t>
+          <t>Yes - Sales Executive - Pacific Northwes (Remote Worker - N/)</t>
         </is>
       </c>
     </row>
@@ -44862,9 +44862,9 @@
           <t>Electric school bus fleet-as-a-service subscriptions for districts</t>
         </is>
       </c>
-      <c r="F64" s="35" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Customer Success Manager (CA) only</t>
+      <c r="F64" s="34" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -45252,9 +45252,9 @@
           <t>Synergy SIS, MTSS and analytics for K-12 school districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F77" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Sales Representative (Mesa)</t>
+      <c r="F77" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -45372,9 +45372,9 @@
           <t>K-12 ERP, nutrition, payments and forms platform for districts</t>
         </is>
       </c>
-      <c r="F81" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Associate Client Success Manager only</t>
+      <c r="F81" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -46136,9 +46136,9 @@
           <t>Digital hall pass, tardy tracking, behavior management, and campus engagement platform for K-12 schools and districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F107" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Chief Revenue Officer (CRO) only</t>
+      <c r="F107" s="10" t="inlineStr">
+        <is>
+          <t>Yes - Account Manager (INTERNAL APPLICAN</t>
         </is>
       </c>
     </row>
@@ -46280,9 +46280,9 @@
           <t>Library, technology asset, and facilities management software for K-12 school districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F112" s="35" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Senior Salesforce Developer only</t>
+      <c r="F112" s="34" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -47086,7 +47086,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/14/26)</t>
+          <t>Hiring AEs? (9/16/26)</t>
         </is>
       </c>
     </row>
@@ -47502,7 +47502,7 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -49344,9 +49344,9 @@
           <t>Digital vehicle inspections and maintenance for municipal fleets</t>
         </is>
       </c>
-      <c r="F77" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F77" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Operations Manager, Customer Succe only</t>
         </is>
       </c>
     </row>
@@ -49796,7 +49796,7 @@
       </c>
       <c r="F92" s="39" t="inlineStr">
         <is>
-          <t>Yes - Strategic Account Executive (North Carolina_Rem)</t>
+          <t>Yes - Strategic Account Executive (Tennessee_Remote_C)</t>
         </is>
       </c>
     </row>
@@ -52728,7 +52728,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/14/26)</t>
+          <t>Hiring AEs? (9/16/26)</t>
         </is>
       </c>
     </row>
@@ -56258,7 +56258,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/14/26)</t>
+          <t>Hiring AEs? (9/16/26)</t>
         </is>
       </c>
     </row>
@@ -57742,9 +57742,9 @@
           <t>Baggage handling systems and terminal logistics for airports</t>
         </is>
       </c>
-      <c r="F51" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -58044,7 +58044,7 @@
       </c>
       <c r="F61" s="10" t="inlineStr">
         <is>
-          <t>Yes - Senior Account Executive</t>
+          <t>Yes - Senior Account Executive - West &amp;</t>
         </is>
       </c>
     </row>
@@ -58554,7 +58554,7 @@
       </c>
       <c r="F78" s="52" t="inlineStr">
         <is>
-          <t>Yes - Technical Sales Representative, So</t>
+          <t>Yes - Account Manager Molecular Diagnost</t>
         </is>
       </c>
     </row>
@@ -59782,7 +59782,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/14/26)</t>
+          <t>Hiring AEs? (9/16/26)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-09-17)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -286,9 +286,9 @@
     <xf numFmtId="1" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/16/26)</t>
+          <t>Hiring AEs? (9/17/26)</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2522,7 @@
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.365labs.com/car</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -11136,7 +11136,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/16/26)</t>
+          <t>Hiring AEs? (9/17/26)</t>
         </is>
       </c>
     </row>
@@ -14420,7 +14420,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/16/26)</t>
+          <t>Hiring AEs? (9/17/26)</t>
         </is>
       </c>
     </row>
@@ -16386,7 +16386,7 @@
       </c>
       <c r="F72" s="70" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Senior Solutions Engineer only</t>
+          <t>Sales (non-AE) - Vice President, Sales only</t>
         </is>
       </c>
     </row>
@@ -17026,7 +17026,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/16/26)</t>
+          <t>Hiring AEs? (9/17/26)</t>
         </is>
       </c>
     </row>
@@ -17494,7 +17494,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/16/26)</t>
+          <t>Hiring AEs? (9/17/26)</t>
         </is>
       </c>
     </row>
@@ -20762,7 +20762,7 @@
       </c>
       <c r="F111" s="9" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Solutions Engineer only</t>
+          <t>Sales (non-AE) - Senior Customer Success Manager only</t>
         </is>
       </c>
     </row>
@@ -24624,7 +24624,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/16/26)</t>
+          <t>Hiring AEs? (9/17/26)</t>
         </is>
       </c>
     </row>
@@ -26380,7 +26380,7 @@
       </c>
       <c r="F60" s="22" t="inlineStr">
         <is>
-          <t>Yes - Sales Account Executive - GovTech</t>
+          <t>Yes - Outbound Sales Representative-iWor</t>
         </is>
       </c>
     </row>
@@ -31856,7 +31856,7 @@
       </c>
       <c r="F246" s="21" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://passportworkforce.c</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -33720,9 +33720,9 @@
           <t>Symmetri AI operations platform for critical infrastructure operators in water, energy, telecom and healthcare - exhibited at AWWA ACE 2026</t>
         </is>
       </c>
-      <c r="F310" s="21" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F310" s="23" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Technical Sales Engineer only</t>
         </is>
       </c>
     </row>
@@ -36530,9 +36530,9 @@
           <t>Research databases, ebook collections and discovery software licensed to public libraries, academic libraries, schools and healthcare organizations - exhibited at PLA 2026</t>
         </is>
       </c>
-      <c r="F408" s="22" t="inlineStr">
-        <is>
-          <t>Yes - Regional Sales Manager, AMC – Virg</t>
+      <c r="F408" s="23" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Customer Account Specialist, FOLIO only</t>
         </is>
       </c>
     </row>
@@ -38708,7 +38708,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/16/26)</t>
+          <t>Hiring AEs? (9/17/26)</t>
         </is>
       </c>
     </row>
@@ -39122,7 +39122,7 @@
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (Hillsboro, TX)</t>
+          <t>Yes - Account Executive (Shreveport, LA)</t>
         </is>
       </c>
     </row>
@@ -42384,9 +42384,9 @@
           <t>ShoWare ticketing and guest experience for municipal arenas and attractions</t>
         </is>
       </c>
-      <c r="F124" s="28" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F124" s="27" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Head of Sales only</t>
         </is>
       </c>
     </row>
@@ -42990,7 +42990,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/16/26)</t>
+          <t>Hiring AEs? (9/17/26)</t>
         </is>
       </c>
     </row>
@@ -43020,7 +43020,7 @@
       </c>
       <c r="F2" s="33" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (Remote - US)</t>
+          <t>Sales (non-AE) - Senior Manager, Global Deal Desk only</t>
         </is>
       </c>
     </row>
@@ -43050,7 +43050,7 @@
       </c>
       <c r="F3" s="10" t="inlineStr">
         <is>
-          <t>Yes - Sales Executive - Pacific Northwes (Remote Worker - N/)</t>
+          <t>Yes - Sales Executive, Cross-Sell (North (Remote Worker - N/)</t>
         </is>
       </c>
     </row>
@@ -43198,7 +43198,7 @@
           <t>Cloud web filtering and student safety monitoring - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F8" s="33" t="inlineStr">
+      <c r="F8" s="35" t="inlineStr">
         <is>
           <t>Yes - Account Executive, Large/Enterpris (United States of A)</t>
         </is>
@@ -43258,7 +43258,7 @@
           <t>Web filtering and student safety monitoring for school districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F10" s="33" t="inlineStr">
+      <c r="F10" s="35" t="inlineStr">
         <is>
           <t>Yes - Account Manager (REMOTE, United Kin)</t>
         </is>
@@ -43378,7 +43378,7 @@
           <t>AI web filtering and student threat detection for K-12 districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F14" s="35" t="inlineStr">
+      <c r="F14" s="33" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -43552,7 +43552,7 @@
           <t>Cloud video security and sensors for schools and public agencies</t>
         </is>
       </c>
-      <c r="F20" s="33" t="inlineStr">
+      <c r="F20" s="35" t="inlineStr">
         <is>
           <t>Yes - Commercial Account Executive - Cen (Dallas, Texas)</t>
         </is>
@@ -43732,7 +43732,7 @@
           <t>AI-based weapons screening gateways for schools, venues and public buildings</t>
         </is>
       </c>
-      <c r="F26" s="33" t="inlineStr">
+      <c r="F26" s="35" t="inlineStr">
         <is>
           <t>Yes - Regional Sales Manager (Boston, Massachuse)</t>
         </is>
@@ -43910,7 +43910,7 @@
           <t>Emergency mass notification hardware and software for schools and agencies - exhibited at EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F32" s="33" t="inlineStr">
+      <c r="F32" s="35" t="inlineStr">
         <is>
           <t>Yes - Regional Account Manager - Educati (Baltimore, MD)</t>
         </is>
@@ -44234,7 +44234,7 @@
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 404 for https://www.ridezum.com/com</t>
         </is>
       </c>
     </row>
@@ -44262,7 +44262,7 @@
           <t>Vetted small-vehicle student rides supplementing district bus fleets - exhibited at NAPT Summit 2026</t>
         </is>
       </c>
-      <c r="F44" s="33" t="inlineStr">
+      <c r="F44" s="35" t="inlineStr">
         <is>
           <t>Yes - Regional Account Manager (Remote USA)</t>
         </is>
@@ -45162,7 +45162,7 @@
           <t>Student information system and school business/ERP suite for K-12 districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F74" s="35" t="inlineStr">
+      <c r="F74" s="33" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Customer Success Technical Special only</t>
         </is>
@@ -45342,7 +45342,7 @@
           <t>Cloud SIS and LMS for K-12 districts and charter networks</t>
         </is>
       </c>
-      <c r="F80" s="33" t="inlineStr">
+      <c r="F80" s="35" t="inlineStr">
         <is>
           <t>Yes - Account Executive</t>
         </is>
@@ -45520,7 +45520,7 @@
           <t>School bus routing, fleet and student transportation software for districts</t>
         </is>
       </c>
-      <c r="F86" s="33" t="inlineStr">
+      <c r="F86" s="35" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -45640,7 +45640,7 @@
           <t>Website, CMS and mass communications platform for school districts</t>
         </is>
       </c>
-      <c r="F90" s="35" t="inlineStr">
+      <c r="F90" s="33" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -45700,7 +45700,7 @@
           <t>Family engagement, attendance and communications platform for districts</t>
         </is>
       </c>
-      <c r="F92" s="33" t="inlineStr">
+      <c r="F92" s="35" t="inlineStr">
         <is>
           <t>Yes - Account Executive (Future Opportun (Remote)</t>
         </is>
@@ -45820,7 +45820,7 @@
           <t>K-12 hiring, applicant tracking and talent matching for districts</t>
         </is>
       </c>
-      <c r="F96" s="35" t="inlineStr">
+      <c r="F96" s="33" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -46388,7 +46388,7 @@
           <t>AI browser extension that generates lesson plans, quizzes, and student feedback inside Google Workspace and LMS tools for teachers and school districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F116" s="33" t="inlineStr">
+      <c r="F116" s="35" t="inlineStr">
         <is>
           <t>Yes - Mid-Market Account Executive (Remote)</t>
         </is>
@@ -46612,7 +46612,7 @@
           <t>AI platform for K-12 districts giving teachers lesson and assessment generation tools and students guided AI, with district-level policy and privacy controls - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F124" s="35" t="inlineStr">
+      <c r="F124" s="33" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Senior Customer Success Manager -  only</t>
         </is>
@@ -46778,7 +46778,7 @@
           <t>Browser-delivered virtual computer labs, classroom AI safety controls and work-based learning software for school districts and colleges - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F130" s="33" t="inlineStr">
+      <c r="F130" s="35" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -47086,7 +47086,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/16/26)</t>
+          <t>Hiring AEs? (9/17/26)</t>
         </is>
       </c>
     </row>
@@ -47502,7 +47502,7 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -49796,7 +49796,7 @@
       </c>
       <c r="F92" s="39" t="inlineStr">
         <is>
-          <t>Yes - Strategic Account Executive (Tennessee_Remote_C)</t>
+          <t>Yes - Strategic Account Executive (North Carolina_Rem)</t>
         </is>
       </c>
     </row>
@@ -52728,7 +52728,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/16/26)</t>
+          <t>Hiring AEs? (9/17/26)</t>
         </is>
       </c>
     </row>
@@ -54438,7 +54438,7 @@
       </c>
       <c r="F58" s="45" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -56258,7 +56258,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/16/26)</t>
+          <t>Hiring AEs? (9/17/26)</t>
         </is>
       </c>
     </row>
@@ -57862,9 +57862,9 @@
           <t>Self-service kiosks, bag drop and passenger processing for airports</t>
         </is>
       </c>
-      <c r="F55" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F55" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - HTTP 404 for https://www.embross.com/car</t>
         </is>
       </c>
     </row>
@@ -58554,7 +58554,7 @@
       </c>
       <c r="F78" s="52" t="inlineStr">
         <is>
-          <t>Yes - Account Manager Molecular Diagnost</t>
+          <t>Yes - Sales Account Manager</t>
         </is>
       </c>
     </row>
@@ -59782,7 +59782,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/16/26)</t>
+          <t>Hiring AEs? (9/17/26)</t>
         </is>
       </c>
     </row>
@@ -60298,7 +60298,7 @@
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>Yes - Enterprise Account Executive (Stat (United States)</t>
+          <t>Yes - Enterprise Account Executive (Stat (New York, New York)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-09-18)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/17/26)</t>
+          <t>Hiring AEs? (9/18/26)</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2522,7 @@
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - HTTP 403 for https://www.365labs.com/car</t>
         </is>
       </c>
     </row>
@@ -3870,9 +3870,9 @@
           <t>OfficerTRAK off-duty detail management: scheduling, billing, insurance - exhibited at NLC City Summit 2026</t>
         </is>
       </c>
-      <c r="F99" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F99" s="10" t="inlineStr">
+        <is>
+          <t>Yes - Business Development Manager - Mid (Charlotte, North C)</t>
         </is>
       </c>
     </row>
@@ -5982,9 +5982,9 @@
           <t>Assistive AI for 911 centers: transcription, translation, text-to-911, and video</t>
         </is>
       </c>
-      <c r="F171" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F171" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -11136,7 +11136,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/17/26)</t>
+          <t>Hiring AEs? (9/18/26)</t>
         </is>
       </c>
     </row>
@@ -14420,7 +14420,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/17/26)</t>
+          <t>Hiring AEs? (9/18/26)</t>
         </is>
       </c>
     </row>
@@ -17026,7 +17026,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/17/26)</t>
+          <t>Hiring AEs? (9/18/26)</t>
         </is>
       </c>
     </row>
@@ -17494,7 +17494,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/17/26)</t>
+          <t>Hiring AEs? (9/18/26)</t>
         </is>
       </c>
     </row>
@@ -18878,9 +18878,9 @@
           <t>Traffic data collection and smart intersection technology</t>
         </is>
       </c>
-      <c r="F48" s="16" t="inlineStr">
-        <is>
-          <t>Yes - Enterprise Account Executive, Opti (Southeastern USA)</t>
+      <c r="F48" s="17" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Technical Customer Success Manager only</t>
         </is>
       </c>
     </row>
@@ -20642,7 +20642,7 @@
       </c>
       <c r="F107" s="10" t="inlineStr">
         <is>
-          <t>Yes - Key Account Manager (Budapest, Hungary)</t>
+          <t>Yes - Executive Sales Representative - N (12 Locations)</t>
         </is>
       </c>
     </row>
@@ -22650,9 +22650,9 @@
           <t>IoT telematics and video safety for government fleets (public co) - exhibited at NLC City Summit 2026, PRIMA 2026, NAFA I&amp;E 2026, NAPT Summit 2026, SWANA WASTECON 2025</t>
         </is>
       </c>
-      <c r="F175" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F175" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -24624,7 +24624,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/17/26)</t>
+          <t>Hiring AEs? (9/18/26)</t>
         </is>
       </c>
     </row>
@@ -31112,9 +31112,9 @@
           <t>Tax collection, auctions and payment processing software for governments - exhibited at GFOA 2026</t>
         </is>
       </c>
-      <c r="F221" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Account Executive (United States (Rem)</t>
+      <c r="F221" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -31856,7 +31856,7 @@
       </c>
       <c r="F246" s="21" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - HTTP 403 for https://passportworkforce.c</t>
         </is>
       </c>
     </row>
@@ -38708,7 +38708,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/17/26)</t>
+          <t>Hiring AEs? (9/18/26)</t>
         </is>
       </c>
     </row>
@@ -39902,7 +39902,7 @@
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -42054,9 +42054,9 @@
           <t>Short-term rental market data for tourism offices and city agencies</t>
         </is>
       </c>
-      <c r="F113" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Account Executive (Barcelona)</t>
+      <c r="F113" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Sales Manager - Uplisting only</t>
         </is>
       </c>
     </row>
@@ -42990,7 +42990,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/17/26)</t>
+          <t>Hiring AEs? (9/18/26)</t>
         </is>
       </c>
     </row>
@@ -43020,7 +43020,7 @@
       </c>
       <c r="F2" s="33" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Senior Manager, Global Deal Desk only</t>
+          <t>Sales (non-AE) - Director, GTM Finance only</t>
         </is>
       </c>
     </row>
@@ -43050,7 +43050,7 @@
       </c>
       <c r="F3" s="10" t="inlineStr">
         <is>
-          <t>Yes - Sales Executive, Cross-Sell (North (Remote Worker - N/)</t>
+          <t>Yes - Senior Sales Executive (VA/WV/OH) (Remote Worker - N/)</t>
         </is>
       </c>
     </row>
@@ -43880,9 +43880,9 @@
           <t>InformaCast mass notification and paging for school districts</t>
         </is>
       </c>
-      <c r="F31" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -44234,7 +44234,7 @@
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 404 for https://www.ridezum.com/com</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -47086,7 +47086,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/17/26)</t>
+          <t>Hiring AEs? (9/18/26)</t>
         </is>
       </c>
     </row>
@@ -52728,7 +52728,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/17/26)</t>
+          <t>Hiring AEs? (9/18/26)</t>
         </is>
       </c>
     </row>
@@ -54438,7 +54438,7 @@
       </c>
       <c r="F58" s="45" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - HTTP 504 for https://www.sedata.com/care</t>
         </is>
       </c>
     </row>
@@ -56258,7 +56258,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/17/26)</t>
+          <t>Hiring AEs? (9/18/26)</t>
         </is>
       </c>
     </row>
@@ -57742,9 +57742,9 @@
           <t>Baggage handling systems and terminal logistics for airports</t>
         </is>
       </c>
-      <c r="F51" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F51" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -57862,9 +57862,9 @@
           <t>Self-service kiosks, bag drop and passenger processing for airports</t>
         </is>
       </c>
-      <c r="F55" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - HTTP 404 for https://www.embross.com/car</t>
+      <c r="F55" s="10" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -57894,7 +57894,7 @@
       </c>
       <c r="F56" s="51" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -58044,7 +58044,7 @@
       </c>
       <c r="F61" s="10" t="inlineStr">
         <is>
-          <t>Yes - Senior Account Executive - West &amp;</t>
+          <t>Yes - Senior Account Executive</t>
         </is>
       </c>
     </row>
@@ -59782,7 +59782,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/17/26)</t>
+          <t>Hiring AEs? (9/18/26)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-09-19)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/18/26)</t>
+          <t>Hiring AEs? (9/19/26)</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2522,7 @@
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.365labs.com/car</t>
+          <t>Unknown - HTTP 202 for https://www.365labs.com/car</t>
         </is>
       </c>
     </row>
@@ -3750,9 +3750,9 @@
           <t>Officer performance management and research-based early intervention (First Sign)</t>
         </is>
       </c>
-      <c r="F95" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F95" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -8018,9 +8018,9 @@
           <t>Intercept and Defender full-body transmission X-ray scanners for jails, courthouses, and borders - exhibited at Michigan Sheriffs Association 2026</t>
         </is>
       </c>
-      <c r="F239" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F239" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -11136,7 +11136,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/18/26)</t>
+          <t>Hiring AEs? (9/19/26)</t>
         </is>
       </c>
     </row>
@@ -14420,7 +14420,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/18/26)</t>
+          <t>Hiring AEs? (9/19/26)</t>
         </is>
       </c>
     </row>
@@ -16252,7 +16252,7 @@
       </c>
       <c r="F67" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 404 for https://www.kuali.co/about-</t>
         </is>
       </c>
     </row>
@@ -17026,7 +17026,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/18/26)</t>
+          <t>Hiring AEs? (9/19/26)</t>
         </is>
       </c>
     </row>
@@ -17494,7 +17494,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/18/26)</t>
+          <t>Hiring AEs? (9/19/26)</t>
         </is>
       </c>
     </row>
@@ -17672,9 +17672,9 @@
           <t>AI waste-recognition cameras and analytics for sorting plants</t>
         </is>
       </c>
-      <c r="F7" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Director of Sales only</t>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -22650,9 +22650,9 @@
           <t>IoT telematics and video safety for government fleets (public co) - exhibited at NLC City Summit 2026, PRIMA 2026, NAFA I&amp;E 2026, NAPT Summit 2026, SWANA WASTECON 2025</t>
         </is>
       </c>
-      <c r="F175" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F175" s="10" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -22682,7 +22682,7 @@
       </c>
       <c r="F176" s="16" t="inlineStr">
         <is>
-          <t>Yes - Partner Account Manager UK&amp;I (London, England - )</t>
+          <t>Yes - Business Development Manager - Mob (Denver, Colorado -)</t>
         </is>
       </c>
     </row>
@@ -24624,7 +24624,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/18/26)</t>
+          <t>Hiring AEs? (9/19/26)</t>
         </is>
       </c>
     </row>
@@ -24894,7 +24894,7 @@
       </c>
       <c r="F10" s="21" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://zencity.io/careers</t>
+          <t>Unknown - HTTP 202 for https://zencity.io/careers</t>
         </is>
       </c>
     </row>
@@ -26918,9 +26918,9 @@
           <t>Community development permitting and licensing software (founded as BasicGov)</t>
         </is>
       </c>
-      <c r="F79" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F79" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Business Development Representativ only</t>
         </is>
       </c>
     </row>
@@ -29962,7 +29962,7 @@
       </c>
       <c r="F182" s="21" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 404 for https://www.governmentwindo</t>
+          <t>Unknown - HTTP 403 for https://www.governmentwindo</t>
         </is>
       </c>
     </row>
@@ -31856,7 +31856,7 @@
       </c>
       <c r="F246" s="21" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://passportworkforce.c</t>
+          <t>Unknown - HTTP 202 for https://passportworkforce.c</t>
         </is>
       </c>
     </row>
@@ -32564,7 +32564,7 @@
       </c>
       <c r="F270" s="23" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Sales Development Representative only</t>
+          <t>Sales (non-AE) - Client Success Manager only</t>
         </is>
       </c>
     </row>
@@ -38708,7 +38708,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/18/26)</t>
+          <t>Hiring AEs? (9/19/26)</t>
         </is>
       </c>
     </row>
@@ -39542,7 +39542,7 @@
       </c>
       <c r="F29" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Manager (GameChanger Remote)</t>
+          <t>Yes - Account Executive (GameChanger Remote)</t>
         </is>
       </c>
     </row>
@@ -39902,7 +39902,7 @@
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -40080,9 +40080,9 @@
           <t>Camp management and registration software for camps including municipal programs</t>
         </is>
       </c>
-      <c r="F47" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Customer Success Manager - Mid Mar only</t>
+      <c r="F47" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -40260,9 +40260,9 @@
           <t>Campground reservation and management software for public and private campgrounds</t>
         </is>
       </c>
-      <c r="F53" s="10" t="inlineStr">
-        <is>
-          <t>Yes - National Outbound Sales Account Ex</t>
+      <c r="F53" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Manager, Account Management only</t>
         </is>
       </c>
     </row>
@@ -42990,7 +42990,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/18/26)</t>
+          <t>Hiring AEs? (9/19/26)</t>
         </is>
       </c>
     </row>
@@ -43168,9 +43168,9 @@
           <t>Device filtering, classroom management, and student wellness (Beacon)</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - New Business Executive - Strategic only</t>
         </is>
       </c>
     </row>
@@ -43260,7 +43260,7 @@
       </c>
       <c r="F10" s="35" t="inlineStr">
         <is>
-          <t>Yes - Account Manager (REMOTE, United Kin)</t>
+          <t>Yes - Account Executive (Austin, Texas, Uni)</t>
         </is>
       </c>
     </row>
@@ -43880,9 +43880,9 @@
           <t>InformaCast mass notification and paging for school districts</t>
         </is>
       </c>
-      <c r="F31" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F31" s="10" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -47086,7 +47086,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/18/26)</t>
+          <t>Hiring AEs? (9/19/26)</t>
         </is>
       </c>
     </row>
@@ -47386,7 +47386,7 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.modeshift.com/c</t>
+          <t>Unknown - HTTP 202 for https://www.modeshift.com/c</t>
         </is>
       </c>
     </row>
@@ -47982,7 +47982,7 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.enghouse.com/ca</t>
+          <t>Unknown - HTTP 202 for https://www.enghouse.com/ca</t>
         </is>
       </c>
     </row>
@@ -49796,7 +49796,7 @@
       </c>
       <c r="F92" s="39" t="inlineStr">
         <is>
-          <t>Yes - Strategic Account Executive (North Carolina_Rem)</t>
+          <t>Yes - Strategic Account Executive (Tennessee_Remote_C)</t>
         </is>
       </c>
     </row>
@@ -50036,7 +50036,7 @@
       </c>
       <c r="F100" s="40" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.hanoverdisplays</t>
+          <t>Unknown - HTTP 202 for https://www.hanoverdisplays</t>
         </is>
       </c>
     </row>
@@ -50424,7 +50424,7 @@
       </c>
       <c r="F113" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://qryde.com/employmen</t>
+          <t>Unknown - HTTP 202 for https://qryde.com/employmen</t>
         </is>
       </c>
     </row>
@@ -52728,7 +52728,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/18/26)</t>
+          <t>Hiring AEs? (9/19/26)</t>
         </is>
       </c>
     </row>
@@ -54438,7 +54438,7 @@
       </c>
       <c r="F58" s="45" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 504 for https://www.sedata.com/care</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -56258,7 +56258,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/18/26)</t>
+          <t>Hiring AEs? (9/19/26)</t>
         </is>
       </c>
     </row>
@@ -56728,9 +56728,9 @@
           <t>Aviation design and simulation software (AviPLAN, AeroTURN, GuideSIGN) used by airport planners for aircraft movement, apron layout and airside safety analysis.</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Customer Success Representative only</t>
         </is>
       </c>
     </row>
@@ -57742,9 +57742,9 @@
           <t>Baggage handling systems and terminal logistics for airports</t>
         </is>
       </c>
-      <c r="F51" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -57894,7 +57894,7 @@
       </c>
       <c r="F56" s="51" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -59782,7 +59782,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/18/26)</t>
+          <t>Hiring AEs? (9/19/26)</t>
         </is>
       </c>
     </row>
@@ -60298,7 +60298,7 @@
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>Yes - Enterprise Account Executive (Stat (New York, New York)</t>
+          <t>Yes - Enterprise Account Executive (Stat (United States)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-09-20)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/19/26)</t>
+          <t>Hiring AEs? (9/20/26)</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2522,7 @@
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://www.365labs.com/car</t>
+          <t>Unknown - HTTP 403 for https://www.365labs.com/car</t>
         </is>
       </c>
     </row>
@@ -11136,7 +11136,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/19/26)</t>
+          <t>Hiring AEs? (9/20/26)</t>
         </is>
       </c>
     </row>
@@ -14420,7 +14420,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/19/26)</t>
+          <t>Hiring AEs? (9/20/26)</t>
         </is>
       </c>
     </row>
@@ -17026,7 +17026,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/19/26)</t>
+          <t>Hiring AEs? (9/20/26)</t>
         </is>
       </c>
     </row>
@@ -17494,7 +17494,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/19/26)</t>
+          <t>Hiring AEs? (9/20/26)</t>
         </is>
       </c>
     </row>
@@ -24624,7 +24624,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/19/26)</t>
+          <t>Hiring AEs? (9/20/26)</t>
         </is>
       </c>
     </row>
@@ -24894,7 +24894,7 @@
       </c>
       <c r="F10" s="21" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://zencity.io/careers</t>
+          <t>Unknown - HTTP 403 for https://zencity.io/careers</t>
         </is>
       </c>
     </row>
@@ -31856,7 +31856,7 @@
       </c>
       <c r="F246" s="21" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://passportworkforce.c</t>
+          <t>Unknown - HTTP 403 for https://passportworkforce.c</t>
         </is>
       </c>
     </row>
@@ -34354,7 +34354,7 @@
       </c>
       <c r="F332" s="21" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -38708,7 +38708,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/19/26)</t>
+          <t>Hiring AEs? (9/20/26)</t>
         </is>
       </c>
     </row>
@@ -42990,7 +42990,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/19/26)</t>
+          <t>Hiring AEs? (9/20/26)</t>
         </is>
       </c>
     </row>
@@ -47086,7 +47086,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/19/26)</t>
+          <t>Hiring AEs? (9/20/26)</t>
         </is>
       </c>
     </row>
@@ -47386,7 +47386,7 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://www.modeshift.com/c</t>
+          <t>Unknown - HTTP 403 for https://www.modeshift.com/c</t>
         </is>
       </c>
     </row>
@@ -47982,7 +47982,7 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://www.enghouse.com/ca</t>
+          <t>Unknown - HTTP 403 for https://www.enghouse.com/ca</t>
         </is>
       </c>
     </row>
@@ -50036,7 +50036,7 @@
       </c>
       <c r="F100" s="40" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://www.hanoverdisplays</t>
+          <t>Unknown - HTTP 403 for https://www.hanoverdisplays</t>
         </is>
       </c>
     </row>
@@ -50424,7 +50424,7 @@
       </c>
       <c r="F113" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://qryde.com/employmen</t>
+          <t>Unknown - HTTP 403 for https://qryde.com/employmen</t>
         </is>
       </c>
     </row>
@@ -52728,7 +52728,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/19/26)</t>
+          <t>Hiring AEs? (9/20/26)</t>
         </is>
       </c>
     </row>
@@ -56258,7 +56258,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/19/26)</t>
+          <t>Hiring AEs? (9/20/26)</t>
         </is>
       </c>
     </row>
@@ -59782,7 +59782,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/19/26)</t>
+          <t>Hiring AEs? (9/20/26)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-09-21)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -27,7 +27,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Parks &amp; Rec'!$A$1:$F$143</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'K-12 Schools'!$A$1:$F$139</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Transit &amp; Parking'!$A$1:$F$192</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Utilities &amp; Energy'!$A$1:$F$117</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Utilities &amp; Energy'!$A$1:$F$118</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Airports &amp; Aviation'!$A$1:$F$117</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Courts &amp; Justice'!$A$1:$F$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Health &amp; Human Services'!$A$1:$F$117</definedName>
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/20/26)</t>
+          <t>Hiring AEs? (9/21/26)</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2522,7 @@
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.365labs.com/car</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -5774,7 +5774,7 @@
       </c>
       <c r="F164" s="4" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -7930,7 +7930,7 @@
       </c>
       <c r="F236" s="4" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 504 for https://leotechnologies.com</t>
         </is>
       </c>
     </row>
@@ -11136,7 +11136,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/20/26)</t>
+          <t>Hiring AEs? (9/21/26)</t>
         </is>
       </c>
     </row>
@@ -14420,7 +14420,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/20/26)</t>
+          <t>Hiring AEs? (9/21/26)</t>
         </is>
       </c>
     </row>
@@ -16252,7 +16252,7 @@
       </c>
       <c r="F67" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 404 for https://www.kuali.co/about-</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -17026,7 +17026,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/20/26)</t>
+          <t>Hiring AEs? (9/21/26)</t>
         </is>
       </c>
     </row>
@@ -17494,7 +17494,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/20/26)</t>
+          <t>Hiring AEs? (9/21/26)</t>
         </is>
       </c>
     </row>
@@ -19628,9 +19628,9 @@
           <t>AI cameras detecting phone use, seatbelt, and speed violations for road authorities</t>
         </is>
       </c>
-      <c r="F73" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Sales Executive - Automated Speed</t>
+      <c r="F73" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -24624,7 +24624,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/20/26)</t>
+          <t>Hiring AEs? (9/21/26)</t>
         </is>
       </c>
     </row>
@@ -28264,9 +28264,9 @@
           <t>Procurement, budgeting, and grants suite - Bonfire, Questica, eCivis (formerly GTY) - exhibited at NACUBO 2026, GFOA 2026</t>
         </is>
       </c>
-      <c r="F125" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Solutions Consultant only</t>
+      <c r="F125" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -29962,7 +29962,7 @@
       </c>
       <c r="F182" s="21" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.governmentwindo</t>
+          <t>Unknown - HTTP 404 for https://www.governmentwindo</t>
         </is>
       </c>
     </row>
@@ -34354,7 +34354,7 @@
       </c>
       <c r="F332" s="21" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -38708,7 +38708,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/20/26)</t>
+          <t>Hiring AEs? (9/21/26)</t>
         </is>
       </c>
     </row>
@@ -42990,7 +42990,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/20/26)</t>
+          <t>Hiring AEs? (9/21/26)</t>
         </is>
       </c>
     </row>
@@ -47086,7 +47086,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/20/26)</t>
+          <t>Hiring AEs? (9/21/26)</t>
         </is>
       </c>
     </row>
@@ -49796,7 +49796,7 @@
       </c>
       <c r="F92" s="39" t="inlineStr">
         <is>
-          <t>Yes - Strategic Account Executive (Tennessee_Remote_C)</t>
+          <t>Yes - Strategic Account Executive (North Carolina_Rem)</t>
         </is>
       </c>
     </row>
@@ -51726,7 +51726,7 @@
       </c>
       <c r="F157" s="10" t="inlineStr">
         <is>
-          <t>Yes - Junior B2B Account Executive (Prague)</t>
+          <t>Yes - Account Manager (Helsinki)</t>
         </is>
       </c>
     </row>
@@ -52689,7 +52689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F117"/>
+  <dimension ref="A1:F118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -52728,7 +52728,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/20/26)</t>
+          <t>Hiring AEs? (9/21/26)</t>
         </is>
       </c>
     </row>
@@ -55369,46 +55369,44 @@
     <row r="90">
       <c r="A90" s="43" t="inlineStr">
         <is>
-          <t>Cayenta</t>
+          <t>Heron Power</t>
         </is>
       </c>
       <c r="B90" s="43" t="inlineStr">
         <is>
-          <t>Burnaby, Canada</t>
-        </is>
-      </c>
-      <c r="C90" s="44" t="n">
-        <v>1983</v>
-      </c>
+          <t>Scotts Valley, CA</t>
+        </is>
+      </c>
+      <c r="C90" s="44" t="n"/>
       <c r="D90" s="43" t="inlineStr">
         <is>
-          <t>Billing &amp; Customer Systems</t>
+          <t>Grid &amp; Energy</t>
         </is>
       </c>
       <c r="E90" s="43" t="inlineStr">
         <is>
-          <t>Customer information, billing, financials, and work management software for municipal, cooperative, and investor-owned electric, water, gas, and fiber utilities - exhibited at AWWA ACE 2026</t>
-        </is>
-      </c>
-      <c r="F90" s="45" t="inlineStr">
-        <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Solid-state transformers and grid power electronics, sold to data centre and solar-plus-storage developers</t>
+        </is>
+      </c>
+      <c r="F90" s="47" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Head of Sales only</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>Silverblaze</t>
+          <t>Cayenta</t>
         </is>
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>Richmond Hill, Canada</t>
+          <t>Burnaby, Canada</t>
         </is>
       </c>
       <c r="C91" s="6" t="n">
-        <v>1999</v>
+        <v>1983</v>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
@@ -55417,7 +55415,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t>Customer self-service portals, mobile apps, and smart meter analytics for electric, water, gas, and multi-service utilities - exhibited at AWWA ACE 2026</t>
+          <t>Customer information, billing, financials, and work management software for municipal, cooperative, and investor-owned electric, water, gas, and fiber utilities - exhibited at AWWA ACE 2026</t>
         </is>
       </c>
       <c r="F91" s="7" t="inlineStr">
@@ -55429,46 +55427,46 @@
     <row r="92">
       <c r="A92" s="43" t="inlineStr">
         <is>
-          <t>Sitetracker</t>
+          <t>Silverblaze</t>
         </is>
       </c>
       <c r="B92" s="43" t="inlineStr">
         <is>
-          <t>Montclair, NJ</t>
+          <t>Richmond Hill, Canada</t>
         </is>
       </c>
       <c r="C92" s="44" t="n">
-        <v>2013</v>
+        <v>1999</v>
       </c>
       <c r="D92" s="43" t="inlineStr">
         <is>
-          <t>Broadband &amp; Connectivity</t>
+          <t>Billing &amp; Customer Systems</t>
         </is>
       </c>
       <c r="E92" s="43" t="inlineStr">
         <is>
-          <t>SaaS deployment, project, and asset lifecycle management for infrastructure programs; sold to agencies via Carahsoft (SEWP V, NASPO)</t>
+          <t>Customer self-service portals, mobile apps, and smart meter analytics for electric, water, gas, and multi-service utilities - exhibited at AWWA ACE 2026</t>
         </is>
       </c>
       <c r="F92" s="45" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - no ATS on file</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>AirWorks</t>
+          <t>Sitetracker</t>
         </is>
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>Montclair, NJ</t>
         </is>
       </c>
       <c r="C93" s="6" t="n">
-        <v>2017</v>
+        <v>2013</v>
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
@@ -55477,28 +55475,28 @@
       </c>
       <c r="E93" s="5" t="inlineStr">
         <is>
-          <t>AI converting aerial and lidar data into CAD basemaps and site plans; on SEWP V, NCPA, OMNIA contracts</t>
+          <t>SaaS deployment, project, and asset lifecycle management for infrastructure programs; sold to agencies via Carahsoft (SEWP V, NASPO)</t>
         </is>
       </c>
       <c r="F93" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="43" t="inlineStr">
         <is>
-          <t>Calix</t>
+          <t>AirWorks</t>
         </is>
       </c>
       <c r="B94" s="43" t="inlineStr">
         <is>
-          <t>San Jose, CA</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="C94" s="44" t="n">
-        <v>1999</v>
+        <v>2017</v>
       </c>
       <c r="D94" s="43" t="inlineStr">
         <is>
@@ -55507,28 +55505,28 @@
       </c>
       <c r="E94" s="43" t="inlineStr">
         <is>
-          <t>Broadband access platform and cloud software with a dedicated municipal and public-power utility segment</t>
+          <t>AI converting aerial and lidar data into CAD basemaps and site plans; on SEWP V, NCPA, OMNIA contracts</t>
         </is>
       </c>
       <c r="F94" s="45" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - no ATS on file</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
         <is>
-          <t>VETRO</t>
+          <t>Calix</t>
         </is>
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>Portland, Maine</t>
+          <t>San Jose, CA</t>
         </is>
       </c>
       <c r="C95" s="6" t="n">
-        <v>2015</v>
+        <v>1999</v>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
@@ -55537,28 +55535,28 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t>Fiber network mapping and design platform for municipal ISPs and broadband offices</t>
-        </is>
-      </c>
-      <c r="F95" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Enterprise Account Executive (Portland, ME)</t>
+          <t>Broadband access platform and cloud software with a dedicated municipal and public-power utility segment</t>
+        </is>
+      </c>
+      <c r="F95" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="43" t="inlineStr">
         <is>
-          <t>IQGeo</t>
+          <t>VETRO</t>
         </is>
       </c>
       <c r="B96" s="43" t="inlineStr">
         <is>
-          <t>Cambridge, United Kingdom</t>
+          <t>Portland, Maine</t>
         </is>
       </c>
       <c r="C96" s="44" t="n">
-        <v>2002</v>
+        <v>2015</v>
       </c>
       <c r="D96" s="43" t="inlineStr">
         <is>
@@ -55567,28 +55565,28 @@
       </c>
       <c r="E96" s="43" t="inlineStr">
         <is>
-          <t>Geospatial network design and field software for telecom and public utilities</t>
-        </is>
-      </c>
-      <c r="F96" s="47" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Sales Engineer only</t>
+          <t>Fiber network mapping and design platform for municipal ISPs and broadband offices</t>
+        </is>
+      </c>
+      <c r="F96" s="46" t="inlineStr">
+        <is>
+          <t>Yes - Enterprise Account Executive (Portland, ME)</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="5" t="inlineStr">
         <is>
-          <t>Render Networks</t>
+          <t>IQGeo</t>
         </is>
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>Melbourne, Australia</t>
+          <t>Cambridge, United Kingdom</t>
         </is>
       </c>
       <c r="C97" s="6" t="n">
-        <v>2015</v>
+        <v>2002</v>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
@@ -55597,28 +55595,28 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t>Geospatial fiber construction management for network builders and public programs</t>
-        </is>
-      </c>
-      <c r="F97" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Geospatial network design and field software for telecom and public utilities</t>
+        </is>
+      </c>
+      <c r="F97" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Sales Engineer only</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="43" t="inlineStr">
         <is>
-          <t>CostQuest Associates</t>
+          <t>Render Networks</t>
         </is>
       </c>
       <c r="B98" s="43" t="inlineStr">
         <is>
-          <t>Cincinnati, Ohio</t>
+          <t>Melbourne, Australia</t>
         </is>
       </c>
       <c r="C98" s="44" t="n">
-        <v>2002</v>
+        <v>2015</v>
       </c>
       <c r="D98" s="43" t="inlineStr">
         <is>
@@ -55627,7 +55625,7 @@
       </c>
       <c r="E98" s="43" t="inlineStr">
         <is>
-          <t>Broadband serviceable location fabric and cost models for NTIA and states</t>
+          <t>Geospatial fiber construction management for network builders and public programs</t>
         </is>
       </c>
       <c r="F98" s="45" t="inlineStr">
@@ -55639,16 +55637,16 @@
     <row r="99">
       <c r="A99" s="5" t="inlineStr">
         <is>
-          <t>Ookla</t>
+          <t>CostQuest Associates</t>
         </is>
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>Seattle, Washington</t>
+          <t>Cincinnati, Ohio</t>
         </is>
       </c>
       <c r="C99" s="6" t="n">
-        <v>2006</v>
+        <v>2002</v>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
@@ -55657,28 +55655,28 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t>Speed test and broadband coverage data licensed to broadband offices and regulators</t>
-        </is>
-      </c>
-      <c r="F99" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+          <t>Broadband serviceable location fabric and cost models for NTIA and states</t>
+        </is>
+      </c>
+      <c r="F99" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="43" t="inlineStr">
         <is>
-          <t>Ready.net</t>
+          <t>Ookla</t>
         </is>
       </c>
       <c r="B100" s="43" t="inlineStr">
         <is>
-          <t>San Francisco, California</t>
+          <t>Seattle, Washington</t>
         </is>
       </c>
       <c r="C100" s="44" t="n">
-        <v>2020</v>
+        <v>2006</v>
       </c>
       <c r="D100" s="43" t="inlineStr">
         <is>
@@ -55687,28 +55685,28 @@
       </c>
       <c r="E100" s="43" t="inlineStr">
         <is>
-          <t>Broadband grant, challenge process and mapping software for state broadband offices</t>
-        </is>
-      </c>
-      <c r="F100" s="47" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Product Solutions Engineer only</t>
+          <t>Speed test and broadband coverage data licensed to broadband offices and regulators</t>
+        </is>
+      </c>
+      <c r="F100" s="46" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="5" t="inlineStr">
         <is>
-          <t>Adtran</t>
+          <t>Ready.net</t>
         </is>
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
-          <t>Huntsville, Alabama</t>
+          <t>San Francisco, California</t>
         </is>
       </c>
       <c r="C101" s="6" t="n">
-        <v>1985</v>
+        <v>2020</v>
       </c>
       <c r="D101" s="5" t="inlineStr">
         <is>
@@ -55717,28 +55715,28 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t>Fiber access and broadband network equipment for municipal and rural providers</t>
-        </is>
-      </c>
-      <c r="F101" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Sales Director NSP (2 Locations)</t>
+          <t>Broadband grant, challenge process and mapping software for state broadband offices</t>
+        </is>
+      </c>
+      <c r="F101" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Product Solutions Engineer only</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="43" t="inlineStr">
         <is>
-          <t>DZS</t>
+          <t>Adtran</t>
         </is>
       </c>
       <c r="B102" s="43" t="inlineStr">
         <is>
-          <t>Plano, Texas</t>
+          <t>Huntsville, Alabama</t>
         </is>
       </c>
       <c r="C102" s="44" t="n">
-        <v>1999</v>
+        <v>1985</v>
       </c>
       <c r="D102" s="43" t="inlineStr">
         <is>
@@ -55747,27 +55745,29 @@
       </c>
       <c r="E102" s="43" t="inlineStr">
         <is>
-          <t>Broadband access platforms for municipal utilities and public network operators</t>
-        </is>
-      </c>
-      <c r="F102" s="45" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Fiber access and broadband network equipment for municipal and rural providers</t>
+        </is>
+      </c>
+      <c r="F102" s="46" t="inlineStr">
+        <is>
+          <t>Yes - Sales Director NSP (2 Locations)</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="5" t="inlineStr">
         <is>
-          <t>Clearfield</t>
+          <t>DZS</t>
         </is>
       </c>
       <c r="B103" s="5" t="inlineStr">
         <is>
-          <t>Brooklyn Park, Minnesota</t>
-        </is>
-      </c>
-      <c r="C103" s="6" t="n"/>
+          <t>Plano, Texas</t>
+        </is>
+      </c>
+      <c r="C103" s="6" t="n">
+        <v>1999</v>
+      </c>
       <c r="D103" s="5" t="inlineStr">
         <is>
           <t>Broadband &amp; Connectivity</t>
@@ -55775,7 +55775,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t>Fiber management and connectivity products for municipal and community broadband</t>
+          <t>Broadband access platforms for municipal utilities and public network operators</t>
         </is>
       </c>
       <c r="F103" s="7" t="inlineStr">
@@ -55787,17 +55787,15 @@
     <row r="104">
       <c r="A104" s="43" t="inlineStr">
         <is>
-          <t>Cambium Networks</t>
+          <t>Clearfield</t>
         </is>
       </c>
       <c r="B104" s="43" t="inlineStr">
         <is>
-          <t>Rolling Meadows, Illinois</t>
-        </is>
-      </c>
-      <c r="C104" s="44" t="n">
-        <v>2011</v>
-      </c>
+          <t>Brooklyn Park, Minnesota</t>
+        </is>
+      </c>
+      <c r="C104" s="44" t="n"/>
       <c r="D104" s="43" t="inlineStr">
         <is>
           <t>Broadband &amp; Connectivity</t>
@@ -55805,28 +55803,28 @@
       </c>
       <c r="E104" s="43" t="inlineStr">
         <is>
-          <t>Fixed wireless and Wi-Fi networks for cities, schools and public agencies</t>
+          <t>Fiber management and connectivity products for municipal and community broadband</t>
         </is>
       </c>
       <c r="F104" s="45" t="inlineStr">
         <is>
-          <t>None found</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>Tarana Wireless</t>
+          <t>Cambium Networks</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>Milpitas, California</t>
+          <t>Rolling Meadows, Illinois</t>
         </is>
       </c>
       <c r="C105" s="6" t="n">
-        <v>2009</v>
+        <v>2011</v>
       </c>
       <c r="D105" s="5" t="inlineStr">
         <is>
@@ -55835,28 +55833,28 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t>Next-gen fixed wireless access gear for municipal and rural broadband projects</t>
+          <t>Fixed wireless and Wi-Fi networks for cities, schools and public agencies</t>
         </is>
       </c>
       <c r="F105" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="43" t="inlineStr">
         <is>
-          <t>Katapult Engineering</t>
+          <t>Tarana Wireless</t>
         </is>
       </c>
       <c r="B106" s="43" t="inlineStr">
         <is>
-          <t>Harrisburg, Pennsylvania</t>
+          <t>Milpitas, California</t>
         </is>
       </c>
       <c r="C106" s="44" t="n">
-        <v>1991</v>
+        <v>2009</v>
       </c>
       <c r="D106" s="43" t="inlineStr">
         <is>
@@ -55865,27 +55863,29 @@
       </c>
       <c r="E106" s="43" t="inlineStr">
         <is>
-          <t>Pole attachment and make-ready survey software for utilities and broadband builds</t>
+          <t>Next-gen fixed wireless access gear for municipal and rural broadband projects</t>
         </is>
       </c>
       <c r="F106" s="45" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - no ATS on file</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>ikeGPS</t>
+          <t>Katapult Engineering</t>
         </is>
       </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
-          <t>Wellington, New Zealand</t>
-        </is>
-      </c>
-      <c r="C107" s="6" t="n"/>
+          <t>Harrisburg, Pennsylvania</t>
+        </is>
+      </c>
+      <c r="C107" s="6" t="n">
+        <v>1991</v>
+      </c>
       <c r="D107" s="5" t="inlineStr">
         <is>
           <t>Broadband &amp; Connectivity</t>
@@ -55893,29 +55893,27 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t>Pole measurement and joint-use data software for utilities and network builders</t>
+          <t>Pole attachment and make-ready survey software for utilities and broadband builds</t>
         </is>
       </c>
       <c r="F107" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 404 for https://ikegps.com/open-pos</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="43" t="inlineStr">
         <is>
-          <t>Alden Systems</t>
+          <t>ikeGPS</t>
         </is>
       </c>
       <c r="B108" s="43" t="inlineStr">
         <is>
-          <t>Birmingham, Alabama</t>
-        </is>
-      </c>
-      <c r="C108" s="44" t="n">
-        <v>1995</v>
-      </c>
+          <t>Wellington, New Zealand</t>
+        </is>
+      </c>
+      <c r="C108" s="44" t="n"/>
       <c r="D108" s="43" t="inlineStr">
         <is>
           <t>Broadband &amp; Connectivity</t>
@@ -55923,28 +55921,28 @@
       </c>
       <c r="E108" s="43" t="inlineStr">
         <is>
-          <t>Joint use pole asset and attachment management for utilities and municipalities</t>
+          <t>Pole measurement and joint-use data software for utilities and network builders</t>
         </is>
       </c>
       <c r="F108" s="45" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 404 for https://ikegps.com/open-pos</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>3-GIS</t>
+          <t>Alden Systems</t>
         </is>
       </c>
       <c r="B109" s="5" t="inlineStr">
         <is>
-          <t>Decatur, Alabama</t>
+          <t>Birmingham, Alabama</t>
         </is>
       </c>
       <c r="C109" s="6" t="n">
-        <v>2005</v>
+        <v>1995</v>
       </c>
       <c r="D109" s="5" t="inlineStr">
         <is>
@@ -55953,7 +55951,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t>Fiber network design and asset management for public and municipal broadband</t>
+          <t>Joint use pole asset and attachment management for utilities and municipalities</t>
         </is>
       </c>
       <c r="F109" s="7" t="inlineStr">
@@ -55965,16 +55963,16 @@
     <row r="110">
       <c r="A110" s="43" t="inlineStr">
         <is>
-          <t>Biarri Networks</t>
+          <t>3-GIS</t>
         </is>
       </c>
       <c r="B110" s="43" t="inlineStr">
         <is>
-          <t>Melbourne, Australia</t>
+          <t>Decatur, Alabama</t>
         </is>
       </c>
       <c r="C110" s="44" t="n">
-        <v>2009</v>
+        <v>2005</v>
       </c>
       <c r="D110" s="43" t="inlineStr">
         <is>
@@ -55983,7 +55981,7 @@
       </c>
       <c r="E110" s="43" t="inlineStr">
         <is>
-          <t>Automated fiber network design software for broadband programs and operators</t>
+          <t>Fiber network design and asset management for public and municipal broadband</t>
         </is>
       </c>
       <c r="F110" s="45" t="inlineStr">
@@ -55995,15 +55993,17 @@
     <row r="111">
       <c r="A111" s="5" t="inlineStr">
         <is>
-          <t>Comsof</t>
+          <t>Biarri Networks</t>
         </is>
       </c>
       <c r="B111" s="5" t="inlineStr">
         <is>
-          <t>Ghent, Belgium</t>
-        </is>
-      </c>
-      <c r="C111" s="6" t="n"/>
+          <t>Melbourne, Australia</t>
+        </is>
+      </c>
+      <c r="C111" s="6" t="n">
+        <v>2009</v>
+      </c>
       <c r="D111" s="5" t="inlineStr">
         <is>
           <t>Broadband &amp; Connectivity</t>
@@ -56011,29 +56011,27 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t>Fiber and utility network planning software for public broadband deployments</t>
+          <t>Automated fiber network design software for broadband programs and operators</t>
         </is>
       </c>
       <c r="F111" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="43" t="inlineStr">
         <is>
-          <t>Vitruvi Software</t>
+          <t>Comsof</t>
         </is>
       </c>
       <c r="B112" s="43" t="inlineStr">
         <is>
-          <t>Kelowna, Canada</t>
-        </is>
-      </c>
-      <c r="C112" s="44" t="n">
-        <v>2016</v>
-      </c>
+          <t>Ghent, Belgium</t>
+        </is>
+      </c>
+      <c r="C112" s="44" t="n"/>
       <c r="D112" s="43" t="inlineStr">
         <is>
           <t>Broadband &amp; Connectivity</t>
@@ -56041,7 +56039,7 @@
       </c>
       <c r="E112" s="43" t="inlineStr">
         <is>
-          <t>Construction management platform for fiber and municipal infrastructure builds</t>
+          <t>Fiber and utility network planning software for public broadband deployments</t>
         </is>
       </c>
       <c r="F112" s="45" t="inlineStr">
@@ -56053,16 +56051,16 @@
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
-          <t>OSPInsight</t>
+          <t>Vitruvi Software</t>
         </is>
       </c>
       <c r="B113" s="5" t="inlineStr">
         <is>
-          <t>Salt Lake City, Utah</t>
+          <t>Kelowna, Canada</t>
         </is>
       </c>
       <c r="C113" s="6" t="n">
-        <v>1996</v>
+        <v>2016</v>
       </c>
       <c r="D113" s="5" t="inlineStr">
         <is>
@@ -56071,7 +56069,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t>Outside plant fiber management software for municipal utilities and ISPs</t>
+          <t>Construction management platform for fiber and municipal infrastructure builds</t>
         </is>
       </c>
       <c r="F113" s="7" t="inlineStr">
@@ -56083,16 +56081,16 @@
     <row r="114">
       <c r="A114" s="43" t="inlineStr">
         <is>
-          <t>Federated Wireless</t>
+          <t>OSPInsight</t>
         </is>
       </c>
       <c r="B114" s="43" t="inlineStr">
         <is>
-          <t>Arlington, Virginia</t>
+          <t>Salt Lake City, Utah</t>
         </is>
       </c>
       <c r="C114" s="44" t="n">
-        <v>2012</v>
+        <v>1996</v>
       </c>
       <c r="D114" s="43" t="inlineStr">
         <is>
@@ -56101,7 +56099,7 @@
       </c>
       <c r="E114" s="43" t="inlineStr">
         <is>
-          <t>CBRS shared spectrum services for municipal and public agency networks</t>
+          <t>Outside plant fiber management software for municipal utilities and ISPs</t>
         </is>
       </c>
       <c r="F114" s="45" t="inlineStr">
@@ -56113,16 +56111,16 @@
     <row r="115">
       <c r="A115" s="5" t="inlineStr">
         <is>
-          <t>Celona</t>
+          <t>Federated Wireless</t>
         </is>
       </c>
       <c r="B115" s="5" t="inlineStr">
         <is>
-          <t>San Jose, California</t>
+          <t>Arlington, Virginia</t>
         </is>
       </c>
       <c r="C115" s="6" t="n">
-        <v>2019</v>
+        <v>2012</v>
       </c>
       <c r="D115" s="5" t="inlineStr">
         <is>
@@ -56131,28 +56129,28 @@
       </c>
       <c r="E115" s="5" t="inlineStr">
         <is>
-          <t>Private 5G/LTE networks for government agencies, campuses and utilities</t>
+          <t>CBRS shared spectrum services for municipal and public agency networks</t>
         </is>
       </c>
       <c r="F115" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - no ATS on file</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="43" t="inlineStr">
         <is>
-          <t>SiFi Networks</t>
+          <t>Celona</t>
         </is>
       </c>
       <c r="B116" s="43" t="inlineStr">
         <is>
-          <t>Fullerton, California</t>
+          <t>San Jose, California</t>
         </is>
       </c>
       <c r="C116" s="44" t="n">
-        <v>2012</v>
+        <v>2019</v>
       </c>
       <c r="D116" s="43" t="inlineStr">
         <is>
@@ -56161,47 +56159,77 @@
       </c>
       <c r="E116" s="43" t="inlineStr">
         <is>
-          <t>Privately funded citywide open-access fiber built in partnership with municipalities</t>
+          <t>Private 5G/LTE networks for government agencies, campuses and utilities</t>
         </is>
       </c>
       <c r="F116" s="45" t="inlineStr">
         <is>
-          <t>None found</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="5" t="inlineStr">
         <is>
+          <t>SiFi Networks</t>
+        </is>
+      </c>
+      <c r="B117" s="5" t="inlineStr">
+        <is>
+          <t>Fullerton, California</t>
+        </is>
+      </c>
+      <c r="C117" s="6" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D117" s="5" t="inlineStr">
+        <is>
+          <t>Broadband &amp; Connectivity</t>
+        </is>
+      </c>
+      <c r="E117" s="5" t="inlineStr">
+        <is>
+          <t>Privately funded citywide open-access fiber built in partnership with municipalities</t>
+        </is>
+      </c>
+      <c r="F117" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="43" t="inlineStr">
+        <is>
           <t>Boldyn Networks</t>
         </is>
       </c>
-      <c r="B117" s="5" t="inlineStr">
+      <c r="B118" s="43" t="inlineStr">
         <is>
           <t>New York, New York</t>
         </is>
       </c>
-      <c r="C117" s="6" t="n">
+      <c r="C118" s="44" t="n">
         <v>2023</v>
       </c>
-      <c r="D117" s="5" t="inlineStr">
+      <c r="D118" s="43" t="inlineStr">
         <is>
           <t>Broadband &amp; Connectivity</t>
         </is>
       </c>
-      <c r="E117" s="5" t="inlineStr">
+      <c r="E118" s="43" t="inlineStr">
         <is>
           <t>Neutral-host wireless and fiber networks for transit authorities and cities - exhibited at NACUBO 2026, EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F117" s="7" t="inlineStr">
+      <c r="F118" s="45" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F117"/>
+  <autoFilter ref="A1:F118"/>
   <dataValidations count="1">
     <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid category" error="Pick one of: Street Lighting &amp; Poles, Grid &amp; Energy, Suppliers &amp; Services, Billing &amp; Customer Systems, Broadband &amp; Connectivity" type="list">
       <formula1>"Street Lighting &amp; Poles,Grid &amp; Energy,Suppliers &amp; Services,Billing &amp; Customer Systems,Broadband &amp; Connectivity"</formula1>
@@ -56258,7 +56286,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/20/26)</t>
+          <t>Hiring AEs? (9/21/26)</t>
         </is>
       </c>
     </row>
@@ -56728,9 +56756,9 @@
           <t>Aviation design and simulation software (AviPLAN, AeroTURN, GuideSIGN) used by airport planners for aircraft movement, apron layout and airside safety analysis.</t>
         </is>
       </c>
-      <c r="F17" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Customer Success Representative only</t>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>Yes - Account Manager (Sales)</t>
         </is>
       </c>
     </row>
@@ -59782,7 +59810,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/20/26)</t>
+          <t>Hiring AEs? (9/21/26)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-09-22)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -246,9 +246,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/21/26)</t>
+          <t>Hiring AEs? (9/22/26)</t>
         </is>
       </c>
     </row>
@@ -1120,9 +1120,9 @@
           <t>Wildfire spread modeling and risk analytics used by CAL FIRE and major utilities</t>
         </is>
       </c>
-      <c r="F7" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Sr. Manager, FP&amp;A &amp; Sales Operatio only</t>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1180,7 @@
           <t>Exterior retardant/foam systems and app-based wildfire defense for homes and HOAs</t>
         </is>
       </c>
-      <c r="F9" s="10" t="inlineStr">
+      <c r="F9" s="9" t="inlineStr">
         <is>
           <t>Yes - Territory Manager - LA (Los Angeles, CA)</t>
         </is>
@@ -1330,7 +1330,7 @@
           <t>Actively tethered situational awareness drones with unlimited flight time for fire/PS</t>
         </is>
       </c>
-      <c r="F14" s="11" t="inlineStr">
+      <c r="F14" s="10" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Sales Engineer only</t>
         </is>
@@ -1414,7 +1414,7 @@
           <t>Cloud fire and EMS records management for departments of all sizes</t>
         </is>
       </c>
-      <c r="F17" s="10" t="inlineStr">
+      <c r="F17" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -1650,7 +1650,7 @@
           <t>Satellite vegetation intelligence for wildfire risk at utilities and agencies</t>
         </is>
       </c>
-      <c r="F25" s="10" t="inlineStr">
+      <c r="F25" s="9" t="inlineStr">
         <is>
           <t>Yes - Enterprise Account Executive, Cana (Remote, Canada)</t>
         </is>
@@ -2070,7 +2070,7 @@
           <t>License plate readers, gunshot detection, and drone-as-first-responder (Aerodome)</t>
         </is>
       </c>
-      <c r="F39" s="9" t="inlineStr">
+      <c r="F39" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Senior Deal Desk Analyst only</t>
         </is>
@@ -2130,7 +2130,7 @@
           <t>911-response and tactical drones staged on police and fire station rooftops</t>
         </is>
       </c>
-      <c r="F41" s="10" t="inlineStr">
+      <c r="F41" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Executive, DFR (Remote (Select Sta)</t>
         </is>
@@ -2190,7 +2190,7 @@
           <t>Data integration and real-time intelligence platform for police and city agencies - exhibited at IAFC FRI 2026</t>
         </is>
       </c>
-      <c r="F43" s="10" t="inlineStr">
+      <c r="F43" s="9" t="inlineStr">
         <is>
           <t>Yes - Federal Account Executive (Washington, D.C.)</t>
         </is>
@@ -2522,7 +2522,7 @@
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - HTTP 403 for https://www.365labs.com/car</t>
         </is>
       </c>
     </row>
@@ -2550,7 +2550,7 @@
           <t>Incident reporting and case management for law enforcement, campus, and healthcare security</t>
         </is>
       </c>
-      <c r="F55" s="9" t="inlineStr">
+      <c r="F55" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -2670,7 +2670,7 @@
           <t>AI audio/video/document redaction (CaseGuard Studio) for police, courts, and gov</t>
         </is>
       </c>
-      <c r="F59" s="10" t="inlineStr">
+      <c r="F59" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Manager (Arlington, VA)</t>
         </is>
@@ -2940,7 +2940,7 @@
           <t>Digital investigation suite for cleansing and evidencing comms data (UK + US LE)</t>
         </is>
       </c>
-      <c r="F68" s="11" t="inlineStr">
+      <c r="F68" s="10" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -2970,7 +2970,7 @@
           <t>Investigation database: pawn/secondhand transactions plus ballistics ID for agencies - exhibited at Michigan Sheriffs Association 2026</t>
         </is>
       </c>
-      <c r="F69" s="10" t="inlineStr">
+      <c r="F69" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -3090,7 +3090,7 @@
           <t>Cloud cameras, access control, and sensors with a dedicated SLED sales org - exhibited at EDUCAUSE 2026, Maryland Municipal League 2026</t>
         </is>
       </c>
-      <c r="F73" s="10" t="inlineStr">
+      <c r="F73" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Executive, France (London)</t>
         </is>
@@ -3330,7 +3330,7 @@
           <t>Drone-as-first-responder software and hardware auto-launching to 911 calls</t>
         </is>
       </c>
-      <c r="F81" s="10" t="inlineStr">
+      <c r="F81" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Executive</t>
         </is>
@@ -3570,7 +3570,7 @@
           <t>Bird and drone detection radars (ELVIRA, IRIS) for airports, security, and C-UAS</t>
         </is>
       </c>
-      <c r="F89" s="10" t="inlineStr">
+      <c r="F89" s="9" t="inlineStr">
         <is>
           <t>Yes - Regional Account Manager - Nordics (Nordics)</t>
         </is>
@@ -3720,7 +3720,7 @@
           <t>Training LMS, scheduling, and readiness software (TargetSolutions, Guardian Tracking) - exhibited at IAFC FRI 2026, APCO 2026</t>
         </is>
       </c>
-      <c r="F94" s="11" t="inlineStr">
+      <c r="F94" s="10" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -3810,7 +3810,7 @@
           <t>Scheduling and workforce management for police, corrections, and 911</t>
         </is>
       </c>
-      <c r="F97" s="10" t="inlineStr">
+      <c r="F97" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -3870,7 +3870,7 @@
           <t>OfficerTRAK off-duty detail management: scheduling, billing, insurance - exhibited at NLC City Summit 2026</t>
         </is>
       </c>
-      <c r="F99" s="10" t="inlineStr">
+      <c r="F99" s="9" t="inlineStr">
         <is>
           <t>Yes - Business Development Manager - Mid (Charlotte, North C)</t>
         </is>
@@ -3930,7 +3930,7 @@
           <t>Online application and recruiting platform for police and civil service hiring</t>
         </is>
       </c>
-      <c r="F101" s="9" t="inlineStr">
+      <c r="F101" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -4350,7 +4350,7 @@
           <t>Cyber-over-RF counter-drone detect, track, and mitigate systems for LE, prisons, and infrastructure</t>
         </is>
       </c>
-      <c r="F115" s="10" t="inlineStr">
+      <c r="F115" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -4738,7 +4738,7 @@
           <t>Retail crime intelligence and reporting platform - exhibited at IACP 2026</t>
         </is>
       </c>
-      <c r="F129" s="10" t="inlineStr">
+      <c r="F129" s="9" t="inlineStr">
         <is>
           <t>Yes - Enterprise Account Manager (Biling (Remote - United St)</t>
         </is>
@@ -4788,7 +4788,7 @@
           <t>Software for first responder agencies - exhibited at IACP 2026, APCO 2026</t>
         </is>
       </c>
-      <c r="F131" s="10" t="inlineStr">
+      <c r="F131" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Executive (United States)</t>
         </is>
@@ -4842,7 +4842,7 @@
           <t>AI investigations platform for law enforcement - exhibited at IACP 2026</t>
         </is>
       </c>
-      <c r="F133" s="10" t="inlineStr">
+      <c r="F133" s="9" t="inlineStr">
         <is>
           <t>Yes - Enterprise Account Executive</t>
         </is>
@@ -5382,7 +5382,7 @@
           <t>FBI-certified mobile fingerprint scanners for police and government</t>
         </is>
       </c>
-      <c r="F151" s="9" t="inlineStr">
+      <c r="F151" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -5412,7 +5412,7 @@
           <t>Data integration and investigative analytics for police and government</t>
         </is>
       </c>
-      <c r="F152" s="11" t="inlineStr">
+      <c r="F152" s="10" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Forward Deployed Enablement Engine only</t>
         </is>
@@ -5862,7 +5862,7 @@
           <t>ePCR, records, and analytics connecting EMS, fire, and hospitals - exhibited at IAFC FRI 2026</t>
         </is>
       </c>
-      <c r="F167" s="10" t="inlineStr">
+      <c r="F167" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Manager (Remote, US (TN/KY))</t>
         </is>
@@ -5922,7 +5922,7 @@
           <t>Intelligent 911 platform streaming device location and data to dispatch - exhibited at APCO 2026</t>
         </is>
       </c>
-      <c r="F169" s="9" t="inlineStr">
+      <c r="F169" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Director, Customer Solutions Engin only</t>
         </is>
@@ -5982,9 +5982,9 @@
           <t>Assistive AI for 911 centers: transcription, translation, text-to-911, and video</t>
         </is>
       </c>
-      <c r="F171" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F171" s="9" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -6282,7 +6282,7 @@
           <t>Pediatric emergency dosing system and app for EMS agencies</t>
         </is>
       </c>
-      <c r="F181" s="10" t="inlineStr">
+      <c r="F181" s="9" t="inlineStr">
         <is>
           <t>Yes - Enterprise Account Executive</t>
         </is>
@@ -6402,7 +6402,7 @@
           <t>Mobile incident command and response for fire/EMS departments - exhibited at IAFC FRI 2026</t>
         </is>
       </c>
-      <c r="F185" s="10" t="inlineStr">
+      <c r="F185" s="9" t="inlineStr">
         <is>
           <t>Yes - Regional Account Executive</t>
         </is>
@@ -6582,7 +6582,7 @@
           <t>911 call routing, Viper call handling and NG911 for PSAPs</t>
         </is>
       </c>
-      <c r="F191" s="10" t="inlineStr">
+      <c r="F191" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -6702,7 +6702,7 @@
           <t>AI triage and quality assurance for emergency dispatch centers</t>
         </is>
       </c>
-      <c r="F195" s="9" t="inlineStr">
+      <c r="F195" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - GTM Engineer only</t>
         </is>
@@ -6968,7 +6968,7 @@
           <t>SARA situational awareness and mass notification for schools, senior living, and gov facilities</t>
         </is>
       </c>
-      <c r="F204" s="11" t="inlineStr">
+      <c r="F204" s="10" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -7538,7 +7538,7 @@
           <t>CID Net inmate calling (450+ facilities), facility monitoring, and family apps</t>
         </is>
       </c>
-      <c r="F223" s="9" t="inlineStr">
+      <c r="F223" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -7930,7 +7930,7 @@
       </c>
       <c r="F236" s="4" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 504 for https://leotechnologies.com</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -8636,7 +8636,7 @@
           <t>Data and case-management tools for state corrections and supervision agencies</t>
         </is>
       </c>
-      <c r="F260" s="11" t="inlineStr">
+      <c r="F260" s="10" t="inlineStr">
         <is>
           <t>Sales (non-AE) - State Partnerships Manager only</t>
         </is>
@@ -9458,9 +9458,9 @@
           <t>Digital forensics and investigation management software - exhibited at IACP 2026</t>
         </is>
       </c>
-      <c r="F289" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F289" s="11" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Sales Operations &amp; GTM Systems Man only</t>
         </is>
       </c>
     </row>
@@ -9584,7 +9584,7 @@
           <t>AI police report writing and investigation software - exhibited at IACP 2026</t>
         </is>
       </c>
-      <c r="F294" s="11" t="inlineStr">
+      <c r="F294" s="10" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -10660,7 +10660,7 @@
           <t>DigiTICKET electronic citation software - exhibited at IACP 2026</t>
         </is>
       </c>
-      <c r="F338" s="11" t="inlineStr">
+      <c r="F338" s="10" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -11136,7 +11136,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/21/26)</t>
+          <t>Hiring AEs? (9/22/26)</t>
         </is>
       </c>
     </row>
@@ -11488,7 +11488,7 @@
       </c>
       <c r="F14" s="64" t="inlineStr">
         <is>
-          <t>Yes - Strategic Account Executive, Marke (Remote – United St)</t>
+          <t>Yes - Commercial Account Executive (Remote – United St)</t>
         </is>
       </c>
     </row>
@@ -12424,7 +12424,7 @@
           <t>Care coordination and PDMP network software (PMP AWARxE, OpenBeds) for states, counties, and health systems (Appriss lineage)</t>
         </is>
       </c>
-      <c r="F47" s="10" t="inlineStr">
+      <c r="F47" s="9" t="inlineStr">
         <is>
           <t>Yes - Bamboo Bridge Strategic Account Ma</t>
         </is>
@@ -12766,9 +12766,9 @@
           <t>Digital substance use disorder prevention, intervention, and recovery support platform for treatment providers, state and county health agencies, drug courts, and Medicaid plans - exhibited at NatCon 2026, NACCHO 360 2026</t>
         </is>
       </c>
-      <c r="F59" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Sales Director, Public Sector &amp; Pr (US)</t>
+      <c r="F59" s="11" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Senior Customer Success Consultant only</t>
         </is>
       </c>
     </row>
@@ -12982,7 +12982,7 @@
           <t>Human services EHR and care coordination software for behavioral health, residential, vocational rehab, and food assistance providers - exhibited at NatCon 2026</t>
         </is>
       </c>
-      <c r="F67" s="9" t="inlineStr">
+      <c r="F67" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Customer Success Manager only</t>
         </is>
@@ -13192,7 +13192,7 @@
           <t>AI clinical documentation and chart auditing platform purpose-built for behavioral health providers including CCBHCs and human services organizations - exhibited at NatCon 2026</t>
         </is>
       </c>
-      <c r="F75" s="9" t="inlineStr">
+      <c r="F75" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - VP of Revenue only</t>
         </is>
@@ -13246,7 +13246,7 @@
           <t>Accredited continuing-education, AI practice simulation and certification platform for behavioral health clinicians and the organizations that employ them - exhibited at NatCon 2026</t>
         </is>
       </c>
-      <c r="F77" s="10" t="inlineStr">
+      <c r="F77" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -13610,7 +13610,7 @@
           <t>Social care coordination network connecting health and social service referrals for govs and payers - exhibited at MESC 2026</t>
         </is>
       </c>
-      <c r="F91" s="10" t="inlineStr">
+      <c r="F91" s="9" t="inlineStr">
         <is>
           <t>Yes - Strategic Sales Director (United States)</t>
         </is>
@@ -13730,7 +13730,7 @@
           <t>Clarity HMIS and homelessness response systems for counties and CoCs</t>
         </is>
       </c>
-      <c r="F95" s="9" t="inlineStr">
+      <c r="F95" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Solutions Consultant only</t>
         </is>
@@ -14018,7 +14018,7 @@
           <t>EHR and case management software for PACE programs, State Units on Aging, Area Agencies on Aging and community-based aging services organizations - exhibited at USAging 2026</t>
         </is>
       </c>
-      <c r="F105" s="10" t="inlineStr">
+      <c r="F105" s="9" t="inlineStr">
         <is>
           <t>Yes - Sales Director, PACE (Remote Worker - N/)</t>
         </is>
@@ -14420,7 +14420,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/21/26)</t>
+          <t>Hiring AEs? (9/22/26)</t>
         </is>
       </c>
     </row>
@@ -14588,7 +14588,7 @@
           <t>Course evaluation, survey, and AI feedback analysis software - Blue, MLY, and Metrics That Matter - for universities and corporate learning teams - exhibited at EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F7" s="10" t="inlineStr">
+      <c r="F7" s="9" t="inlineStr">
         <is>
           <t>Yes - Junior Account Manager</t>
         </is>
@@ -15024,9 +15024,9 @@
           <t>Digital textbook and courseware delivery platform for colleges, universities, and school districts - exhibited at NACUBO 2026</t>
         </is>
       </c>
-      <c r="F22" s="70" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Sales Support - Keyholder only</t>
+      <c r="F22" s="69" t="inlineStr">
+        <is>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -15054,9 +15054,9 @@
           <t>Canvas learning management system plus assessment and credentialing software for universities, school districts, and government training programs - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F23" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Senior Account Executive - Parchme (United States)</t>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>Yes - Senior Account Executive - BizGov (United States)</t>
         </is>
       </c>
     </row>
@@ -15934,7 +15934,7 @@
           <t>Residence life and student housing management software covering applications, room assignment, billing and community programming for universities and colleges - exhibited at EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F55" s="10" t="inlineStr">
+      <c r="F55" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Executive, EMEA (UK - Remote)</t>
         </is>
@@ -16520,7 +16520,7 @@
           <t>Degree planning, advising, transfer pathway and registration software for public universities, community colleges and private institutions - exhibited at EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F77" s="9" t="inlineStr">
+      <c r="F77" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Solutions Consultant only</t>
         </is>
@@ -17026,7 +17026,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/21/26)</t>
+          <t>Hiring AEs? (9/22/26)</t>
         </is>
       </c>
     </row>
@@ -17296,7 +17296,7 @@
           <t>Grant and program administration software for affordable housing, disaster recovery, vouchers and energy rebate programs run by local and state agencies - exhibited at NAHRO 2026</t>
         </is>
       </c>
-      <c r="F11" s="10" t="inlineStr">
+      <c r="F11" s="9" t="inlineStr">
         <is>
           <t>Yes - Technical Account Manager, Strateg (Atlanta)</t>
         </is>
@@ -17494,7 +17494,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/21/26)</t>
+          <t>Hiring AEs? (9/22/26)</t>
         </is>
       </c>
     </row>
@@ -17552,7 +17552,7 @@
           <t>Routing, in-cab fleet tech, and resident apps for waste operations - exhibited at SWANA WASTECON 2025</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="F3" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Customer Success Manager only</t>
         </is>
@@ -17612,7 +17612,7 @@
           <t>AI robotic sorting systems for recycling facilities (MRFs) - exhibited at SWANA WASTECON 2025</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
+      <c r="F5" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Director, Commercial Origination &amp; only</t>
         </is>
@@ -18266,7 +18266,7 @@
           <t>Waste collection route optimization and sensor platform for municipalities</t>
         </is>
       </c>
-      <c r="F27" s="9" t="inlineStr">
+      <c r="F27" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -18968,7 +18968,7 @@
           <t>School bus stop-arm cameras with violator-funded safety programs</t>
         </is>
       </c>
-      <c r="F51" s="9" t="inlineStr">
+      <c r="F51" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Lead Salesforce Developer only</t>
         </is>
@@ -19328,7 +19328,7 @@
           <t>SmartSensor radar vehicle detection for intersections and highways</t>
         </is>
       </c>
-      <c r="F63" s="9" t="inlineStr">
+      <c r="F63" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Sales Manager (Great Lakes) only</t>
         </is>
@@ -20640,7 +20640,7 @@
           <t>Water infrastructure: pumps, treatment, smart meters (Sensus), and analytics - exhibited at AWWA ACE 2026, WEFTEC 2026</t>
         </is>
       </c>
-      <c r="F107" s="10" t="inlineStr">
+      <c r="F107" s="9" t="inlineStr">
         <is>
           <t>Yes - Executive Sales Representative - N (12 Locations)</t>
         </is>
@@ -20672,7 +20672,7 @@
       </c>
       <c r="F108" s="16" t="inlineStr">
         <is>
-          <t>Yes - Account Manager- Private Water (4 Locations)</t>
+          <t>Yes - Municipal Account Manager- South (3 Locations)</t>
         </is>
       </c>
     </row>
@@ -20700,7 +20700,7 @@
           <t>Hydrants, valves, and acoustic leak detection for water systems - exhibited at AWWA ACE 2026, WEFTEC 2026</t>
         </is>
       </c>
-      <c r="F109" s="10" t="inlineStr">
+      <c r="F109" s="9" t="inlineStr">
         <is>
           <t>Yes - Jr. Sales Representative (Remote - Tennessee)</t>
         </is>
@@ -20760,7 +20760,7 @@
           <t>Permitting, compliance, and workflow software for water utilities - exhibited at AWWA ACE 2026, WEFTEC 2026</t>
         </is>
       </c>
-      <c r="F111" s="9" t="inlineStr">
+      <c r="F111" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Senior Customer Success Manager only</t>
         </is>
@@ -20880,7 +20880,7 @@
           <t>AI defect detection and coding for sewer inspection video - exhibited at AWWA ACE 2026, WEFTEC 2026</t>
         </is>
       </c>
-      <c r="F115" s="10" t="inlineStr">
+      <c r="F115" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Executive, Enterprise (Remote)</t>
         </is>
@@ -21000,7 +21000,7 @@
           <t>AI CCTV sewer and stormwater pipe condition assessment for councils and utilities - exhibited at WEFTEC 2026</t>
         </is>
       </c>
-      <c r="F119" s="10" t="inlineStr">
+      <c r="F119" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -21600,7 +21600,7 @@
           <t>Sewer inspection cameras, trucks and software for municipal collection systems - exhibited at Maryland Municipal League 2026, WEFTEC 2026</t>
         </is>
       </c>
-      <c r="F139" s="10" t="inlineStr">
+      <c r="F139" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -21780,7 +21780,7 @@
           <t>AI operations and forecasting software for water and wastewater utilities - exhibited at AWWA ACE 2026, WEFTEC 2026</t>
         </is>
       </c>
-      <c r="F145" s="10" t="inlineStr">
+      <c r="F145" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -21840,7 +21840,7 @@
           <t>Generative design software for water and wastewater treatment plant projects</t>
         </is>
       </c>
-      <c r="F147" s="9" t="inlineStr">
+      <c r="F147" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -22196,7 +22196,7 @@
           <t>AquaTwin digital twin software for water and sewer hydraulic modeling, surge analysis, and asset management, sold to water utilities and engineering consultants - exhibited at AWWA ACE 2026, WEFTEC 2026</t>
         </is>
       </c>
-      <c r="F159" s="10" t="inlineStr">
+      <c r="F159" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -22650,7 +22650,7 @@
           <t>IoT telematics and video safety for government fleets (public co) - exhibited at NLC City Summit 2026, PRIMA 2026, NAFA I&amp;E 2026, NAPT Summit 2026, SWANA WASTECON 2025</t>
         </is>
       </c>
-      <c r="F175" s="10" t="inlineStr">
+      <c r="F175" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -22710,7 +22710,7 @@
           <t>Asset and work order management for DPWs (part of OpenGov)</t>
         </is>
       </c>
-      <c r="F177" s="10" t="inlineStr">
+      <c r="F177" s="9" t="inlineStr">
         <is>
           <t>Yes - Enterprise Account Executive (US | Illinois | Ch)</t>
         </is>
@@ -23010,7 +23010,7 @@
           <t>Fleet maintenance SaaS: work orders, inspections, fuel for commercial and gov fleets - exhibited at NAFA I&amp;E 2026</t>
         </is>
       </c>
-      <c r="F187" s="10" t="inlineStr">
+      <c r="F187" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Executive, Mid-Market (Remote)</t>
         </is>
@@ -23490,7 +23490,7 @@
           <t>collectiveFleet low-code fleet, equipment, and motor pool management for police and municipal fleets</t>
         </is>
       </c>
-      <c r="F203" s="9" t="inlineStr">
+      <c r="F203" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -23726,7 +23726,7 @@
           <t>Cloud CMMS for municipal facilities, water plants and public works</t>
         </is>
       </c>
-      <c r="F211" s="10" t="inlineStr">
+      <c r="F211" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Executive (United Kingdom)</t>
         </is>
@@ -24026,7 +24026,7 @@
           <t>GIS-based asset and work management for local government and utilities - exhibited at AWWA ACE 2026</t>
         </is>
       </c>
-      <c r="F221" s="10" t="inlineStr">
+      <c r="F221" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Executive, Utilities (Homeoffice)</t>
         </is>
@@ -24086,7 +24086,7 @@
           <t>Combined field service and enterprise asset management cloud for water, gas and electric utilities and municipal public works departments - exhibited at AWWA ACE 2026</t>
         </is>
       </c>
-      <c r="F223" s="9" t="inlineStr">
+      <c r="F223" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -24624,7 +24624,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/21/26)</t>
+          <t>Hiring AEs? (9/22/26)</t>
         </is>
       </c>
     </row>
@@ -24682,7 +24682,7 @@
           <t>Resident communications (govDelivery), meeting and agenda management, digital services; destination marketing as Simpleview, now Granicus Destinations - exhibited at 3CMA 2026, GMIS International 2026, APHSA 2026</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
+      <c r="F3" s="9" t="inlineStr">
         <is>
           <t>Yes - Local Government Account Executive</t>
         </is>
@@ -25102,7 +25102,7 @@
           <t>Social media management and archiving for government and public safety (Graham Media)</t>
         </is>
       </c>
-      <c r="F17" s="10" t="inlineStr">
+      <c r="F17" s="9" t="inlineStr">
         <is>
           <t>Yes - Sales Account Executive (USA (Remote))</t>
         </is>
@@ -25522,7 +25522,7 @@
           <t>311/citizen requests, code enforcement, and notifications for ~600 small and mid-size govs - exhibited at 3CMA 2026</t>
         </is>
       </c>
-      <c r="F31" s="10" t="inlineStr">
+      <c r="F31" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -25582,7 +25582,7 @@
           <t>Telephone and virtual town hall mass-engagement platform for county officials and agencies</t>
         </is>
       </c>
-      <c r="F33" s="10" t="inlineStr">
+      <c r="F33" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -25642,7 +25642,7 @@
           <t>Interpretation management and delivery platform (video/phone) used by courts and agencies</t>
         </is>
       </c>
-      <c r="F35" s="9" t="inlineStr">
+      <c r="F35" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Director of Sales only</t>
         </is>
@@ -26228,7 +26228,7 @@
           <t>Emergency and routine mass notification for cities, counties and schools</t>
         </is>
       </c>
-      <c r="F55" s="9" t="inlineStr">
+      <c r="F55" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Customer Success Manager only</t>
         </is>
@@ -26858,7 +26858,7 @@
           <t>Permitting, licensing, and code enforcement platform for state and local government - exhibited at NLC City Summit 2026</t>
         </is>
       </c>
-      <c r="F77" s="10" t="inlineStr">
+      <c r="F77" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Executive (Remote Based - US)</t>
         </is>
@@ -26918,7 +26918,7 @@
           <t>Community development permitting and licensing software (founded as BasicGov)</t>
         </is>
       </c>
-      <c r="F79" s="9" t="inlineStr">
+      <c r="F79" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Business Development Representativ only</t>
         </is>
@@ -26978,7 +26978,7 @@
           <t>AI cameras on city fleet vehicles detect blight, graffiti, dumping for code enforcement - exhibited at NLC City Summit 2026</t>
         </is>
       </c>
-      <c r="F81" s="10" t="inlineStr">
+      <c r="F81" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Executive (Remote)</t>
         </is>
@@ -27038,7 +27038,7 @@
           <t>Cloud e-permitting and community development software for ~500 local governments (Finnish-born)</t>
         </is>
       </c>
-      <c r="F83" s="10" t="inlineStr">
+      <c r="F83" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -27098,7 +27098,7 @@
           <t>Municipal operations software: permitting, licensing, code enforcement; NJ-rooted, going national - exhibited at NLC City Summit 2026</t>
         </is>
       </c>
-      <c r="F85" s="10" t="inlineStr">
+      <c r="F85" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Executive</t>
         </is>
@@ -27218,7 +27218,7 @@
           <t>Cloud permitting, licensing, code enforcement, and GIS workflows for local governments - exhibited at GFOA 2026</t>
         </is>
       </c>
-      <c r="F89" s="10" t="inlineStr">
+      <c r="F89" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Executive</t>
         </is>
@@ -27278,7 +27278,7 @@
           <t>AI permitting and plan review: automated GIS/code compliance checks (Hernando County cut reviews 30 days to 2)</t>
         </is>
       </c>
-      <c r="F91" s="9" t="inlineStr">
+      <c r="F91" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -27916,7 +27916,7 @@
           <t>Digital plan review automation layered on agency permitting systems</t>
         </is>
       </c>
-      <c r="F113" s="9" t="inlineStr">
+      <c r="F113" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -28150,7 +28150,7 @@
           <t>Regulatory, licensing and planning software for public sector authorities - exhibited at PLA 2026</t>
         </is>
       </c>
-      <c r="F121" s="10" t="inlineStr">
+      <c r="F121" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Executive - CES (London)</t>
         </is>
@@ -28264,9 +28264,9 @@
           <t>Procurement, budgeting, and grants suite - Bonfire, Questica, eCivis (formerly GTY) - exhibited at NACUBO 2026, GFOA 2026</t>
         </is>
       </c>
-      <c r="F125" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+      <c r="F125" s="11" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Solutions Consultant only</t>
         </is>
       </c>
     </row>
@@ -28324,7 +28324,7 @@
           <t>Treasury platform for local government finance teams: AI reconciliation and cash forecasting - exhibited at GFOA 2026</t>
         </is>
       </c>
-      <c r="F127" s="9" t="inlineStr">
+      <c r="F127" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Business Development Representativ only</t>
         </is>
@@ -28444,7 +28444,7 @@
           <t>Cloud treasury: debt management, GASB 87/96 lease accounting, and cash management for gov finance - exhibited at NACUBO 2026, GFOA 2026</t>
         </is>
       </c>
-      <c r="F131" s="10" t="inlineStr">
+      <c r="F131" s="9" t="inlineStr">
         <is>
           <t>Yes - Enterprise Account Executive (Charlotte, NC)</t>
         </is>
@@ -28474,9 +28474,9 @@
           <t>AI workflow for county assessors: deed processing, exemptions, taxpayer communication (YC S17) - exhibited at NLC City Summit 2026, IAAO 2026</t>
         </is>
       </c>
-      <c r="F132" s="23" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Customer Success Manager (West Coa only</t>
+      <c r="F132" s="22" t="inlineStr">
+        <is>
+          <t>Yes - Account Executive</t>
         </is>
       </c>
     </row>
@@ -28684,9 +28684,9 @@
           <t>Aerial imagery and property data analytics for county assessors, GIS, and insurers - exhibited at IAAO 2026</t>
         </is>
       </c>
-      <c r="F139" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F139" s="9" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -28744,7 +28744,7 @@
           <t>cashVest liquidity analytics and treasury intelligence for counties, munis, and schools</t>
         </is>
       </c>
-      <c r="F141" s="9" t="inlineStr">
+      <c r="F141" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Senior Business Development Office only</t>
         </is>
@@ -28804,7 +28804,7 @@
           <t>HR, finance and ERP software - exhibited at APTA 2026, ICMA 2025, NACo 2026, NACUBO 2026, GFOA 2026, PSHRA 2026, NASCIO 2026, EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F143" s="10" t="inlineStr">
+      <c r="F143" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Executive (Japan, Tokyo)</t>
         </is>
@@ -28924,7 +28924,7 @@
           <t>Parcel mapping, GIS and assessment systems for county governments</t>
         </is>
       </c>
-      <c r="F147" s="10" t="inlineStr">
+      <c r="F147" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -29272,7 +29272,7 @@
           <t>Fund accounting and ERP software for cities and local governments, covering financials, payroll, utility billing and municipal court - exhibited at GFOA 2026</t>
         </is>
       </c>
-      <c r="F159" s="10" t="inlineStr">
+      <c r="F159" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -29392,7 +29392,7 @@
           <t>Portfolio of vertical software businesses selling ERP, utility billing and public sector operations systems to local governments and utilities - exhibited at GFOA 2026</t>
         </is>
       </c>
-      <c r="F163" s="10" t="inlineStr">
+      <c r="F163" s="9" t="inlineStr">
         <is>
           <t>Yes - (Remote) Sr Account Executive (26 Locations)</t>
         </is>
@@ -29510,7 +29510,7 @@
           <t>Free search marketplace for cooperative contracts (formerly CoProcure)</t>
         </is>
       </c>
-      <c r="F167" s="9" t="inlineStr">
+      <c r="F167" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -29630,7 +29630,7 @@
           <t>Electronic billing and payments for local government and utilities - exhibited at GFOA 2026</t>
         </is>
       </c>
-      <c r="F171" s="10" t="inlineStr">
+      <c r="F171" s="9" t="inlineStr">
         <is>
           <t>Yes - Mid Market Account Executive (Boston, MA)</t>
         </is>
@@ -30050,7 +30050,7 @@
           <t>Source-to-pay eProcurement suite with dedicated public sector and higher-ed verticals - exhibited at NACUBO 2026, GFOA 2026</t>
         </is>
       </c>
-      <c r="F185" s="10" t="inlineStr">
+      <c r="F185" s="9" t="inlineStr">
         <is>
           <t>Yes - Strategic Account Manager (Remote)</t>
         </is>
@@ -30110,7 +30110,7 @@
           <t>Supplier ratings and performance reviews platform for public-sector buyers</t>
         </is>
       </c>
-      <c r="F187" s="9" t="inlineStr">
+      <c r="F187" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -30290,7 +30290,7 @@
           <t>AI-native ConcourseOS: procurement, permitting, courts, and billing across 450+ agencies (Bessemer-backed) - exhibited at NIGP 2026</t>
         </is>
       </c>
-      <c r="F193" s="9" t="inlineStr">
+      <c r="F193" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Founding GTM Engineer only</t>
         </is>
@@ -30468,7 +30468,7 @@
           <t>AI public-sector GTM intelligence: buying signals from gov/school board meetings, budgets, RFPs - sold to vendors selling to gov</t>
         </is>
       </c>
-      <c r="F199" s="10" t="inlineStr">
+      <c r="F199" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Executive - Mid Market (United States)</t>
         </is>
@@ -30578,7 +30578,7 @@
           <t>EProcurement and bid notification platforms for North American public buyers</t>
         </is>
       </c>
-      <c r="F203" s="10" t="inlineStr">
+      <c r="F203" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Executive (United States)</t>
         </is>
@@ -30932,7 +30932,7 @@
           <t>Contract lifecycle management with FedRAMP and state/local government customers</t>
         </is>
       </c>
-      <c r="F215" s="10" t="inlineStr">
+      <c r="F215" s="9" t="inlineStr">
         <is>
           <t>Yes - Enterprise Account Executive (United States)</t>
         </is>
@@ -31352,7 +31352,7 @@
           <t>Cash and digital payments for child support, tolls and government billers</t>
         </is>
       </c>
-      <c r="F229" s="10" t="inlineStr">
+      <c r="F229" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Executive (Credit Unions/B (Remote)</t>
         </is>
@@ -31524,7 +31524,7 @@
           <t>Bill payment kiosks, portals, mobile apps and IVR for municipal agencies and utilities collecting resident payments - exhibited at GFOA 2026</t>
         </is>
       </c>
-      <c r="F235" s="10" t="inlineStr">
+      <c r="F235" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -31674,9 +31674,9 @@
           <t>Pension, OPEB, and labor cost analytics for governments</t>
         </is>
       </c>
-      <c r="F240" s="21" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F240" s="22" t="inlineStr">
+        <is>
+          <t>Yes - Account Executive</t>
         </is>
       </c>
     </row>
@@ -31884,7 +31884,7 @@
           <t>Earned wage access platform for employers - exhibited at NACo 2026</t>
         </is>
       </c>
-      <c r="F247" s="10" t="inlineStr">
+      <c r="F247" s="9" t="inlineStr">
         <is>
           <t>Yes - Business Development Manager (NYC Headquarters)</t>
         </is>
@@ -31994,7 +31994,7 @@
           <t>Payroll and HR software - exhibited at AB Show 2026</t>
         </is>
       </c>
-      <c r="F251" s="10" t="inlineStr">
+      <c r="F251" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -32114,7 +32114,7 @@
           <t>Pension, unemployment insurance and workforce systems for state agencies - exhibited at SNA ANC 2027</t>
         </is>
       </c>
-      <c r="F255" s="10" t="inlineStr">
+      <c r="F255" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -32174,7 +32174,7 @@
           <t>Employee benefits, enrollment and HR services for public sector employers</t>
         </is>
       </c>
-      <c r="F257" s="10" t="inlineStr">
+      <c r="F257" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Manager (Denver, Colorado)</t>
         </is>
@@ -32472,7 +32472,7 @@
           <t>Document-driven workflow for government procurement, budget and HR processes</t>
         </is>
       </c>
-      <c r="F267" s="9" t="inlineStr">
+      <c r="F267" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Customer Success Manager only</t>
         </is>
@@ -33178,7 +33178,7 @@
           <t>Deathcare technology suite including cemetery and memorial management software</t>
         </is>
       </c>
-      <c r="F291" s="9" t="inlineStr">
+      <c r="F291" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -33520,7 +33520,7 @@
           <t>Endpoint management and security platform - exhibited at NACo 2026, NASCIO 2026, EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F303" s="9" t="inlineStr">
+      <c r="F303" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Business Analyst - Salesforce only</t>
         </is>
@@ -33580,7 +33580,7 @@
           <t>ChatGPT and the API, sold to public sector including named state and local government roles</t>
         </is>
       </c>
-      <c r="F305" s="9" t="inlineStr">
+      <c r="F305" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Account Director, Large Enterprise only</t>
         </is>
@@ -33858,7 +33858,7 @@
           <t>Strategic plan and KPI reporting (balanced scorecard) for local governments and enterprises</t>
         </is>
       </c>
-      <c r="F315" s="10" t="inlineStr">
+      <c r="F315" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -34174,9 +34174,9 @@
           <t>Governance, performance and risk management platform for public sector organizations</t>
         </is>
       </c>
-      <c r="F326" s="22" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F326" s="23" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -34910,7 +34910,7 @@
           <t>Open-source voting systems and risk-limiting audit tools for election offices</t>
         </is>
       </c>
-      <c r="F351" s="10" t="inlineStr">
+      <c r="F351" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Executive, Field Sales (United States)</t>
         </is>
@@ -37450,7 +37450,7 @@
           <t>Planning, budgeting and forecasting software - exhibited at ICMA 2025, NACUBO 2026, GFOA 2026</t>
         </is>
       </c>
-      <c r="F441" s="9" t="inlineStr">
+      <c r="F441" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -37558,7 +37558,7 @@
           <t>Purchasing card audit and compliance monitoring - exhibited at NIGP 2026</t>
         </is>
       </c>
-      <c r="F445" s="10" t="inlineStr">
+      <c r="F445" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -38356,7 +38356,7 @@
           <t>CRM and case management cloud software - exhibited at NACo 2026, NIGP 2026, NASWA 2025, NASCIO 2026, APHSA 2026, NatCon 2026, EDUCAUSE 2026, Healthcare IT Connect 2026, MESC 2026</t>
         </is>
       </c>
-      <c r="F477" s="10" t="inlineStr">
+      <c r="F477" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -38708,7 +38708,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/21/26)</t>
+          <t>Hiring AEs? (9/22/26)</t>
         </is>
       </c>
     </row>
@@ -38766,7 +38766,7 @@
           <t>Parks &amp; rec program management and booking platform founded by early Uber employees</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
+      <c r="F3" s="9" t="inlineStr">
         <is>
           <t>Yes - Enterprise Account Executive (San Francisco, CA)</t>
         </is>
@@ -39120,7 +39120,7 @@
           <t>Parks and recreation management software; brands NextRec (formerly PerfectMind), Vermont Systems, RecDesk and ePACT - exhibited at AB Show 2026, NRPA 2026</t>
         </is>
       </c>
-      <c r="F15" s="10" t="inlineStr">
+      <c r="F15" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Executive (Shreveport, LA)</t>
         </is>
@@ -39540,9 +39540,9 @@
           <t>Youth sports scorekeeping and streaming app - exhibited at NRPA 2026</t>
         </is>
       </c>
-      <c r="F29" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Account Executive (GameChanger Remote)</t>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -39840,7 +39840,7 @@
           <t>Club and league management platform for youth soccer organizations</t>
         </is>
       </c>
-      <c r="F39" s="10" t="inlineStr">
+      <c r="F39" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -40200,7 +40200,7 @@
           <t>Campground, park and license reservation systems for state park agencies</t>
         </is>
       </c>
-      <c r="F51" s="9" t="inlineStr">
+      <c r="F51" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Platform Solutions Engineer only</t>
         </is>
@@ -40260,7 +40260,7 @@
           <t>Campground reservation and management software for public and private campgrounds</t>
         </is>
       </c>
-      <c r="F53" s="9" t="inlineStr">
+      <c r="F53" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Manager, Account Management only</t>
         </is>
@@ -40556,7 +40556,7 @@
           <t>Sports facility and program management for municipal and community facilities</t>
         </is>
       </c>
-      <c r="F63" s="9" t="inlineStr">
+      <c r="F63" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -40676,7 +40676,7 @@
           <t>AI drowning-detection and lifeguard assist for public aquatic centers</t>
         </is>
       </c>
-      <c r="F67" s="9" t="inlineStr">
+      <c r="F67" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -40856,7 +40856,7 @@
           <t>Central irrigation control and smart controllers for municipal parks</t>
         </is>
       </c>
-      <c r="F73" s="10" t="inlineStr">
+      <c r="F73" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -41396,7 +41396,7 @@
           <t>Weather safety platform: WBGT heat monitoring, lightning alerts, stations and sirens for parks and athletics</t>
         </is>
       </c>
-      <c r="F91" s="10" t="inlineStr">
+      <c r="F91" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Executive, SLED (Perry Weather Offi)</t>
         </is>
@@ -42056,7 +42056,7 @@
       </c>
       <c r="F113" s="9" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Sales Manager - Uplisting only</t>
+          <t>Yes - Account Manager (Barcelona)</t>
         </is>
       </c>
     </row>
@@ -42294,7 +42294,7 @@
           <t>Event management SaaS: vendor applications, ticketing, maps, and sponsors for festivals and city events</t>
         </is>
       </c>
-      <c r="F121" s="10" t="inlineStr">
+      <c r="F121" s="9" t="inlineStr">
         <is>
           <t>Yes - Enterprise Account Executive</t>
         </is>
@@ -42354,7 +42354,7 @@
           <t>Venue and event management for convention centers and public authorities</t>
         </is>
       </c>
-      <c r="F123" s="9" t="inlineStr">
+      <c r="F123" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Director of Solutions Engineering only</t>
         </is>
@@ -42534,7 +42534,7 @@
           <t>Venue management, ticketing and POS for aquatic centers and attractions</t>
         </is>
       </c>
-      <c r="F129" s="10" t="inlineStr">
+      <c r="F129" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Executive - Mid-Market and (London, United Kin)</t>
         </is>
@@ -42772,7 +42772,7 @@
           <t>Event volunteer scheduling and check-in for festivals and public events</t>
         </is>
       </c>
-      <c r="F137" s="10" t="inlineStr">
+      <c r="F137" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Executive Level 2 (Remote, US)</t>
         </is>
@@ -42990,7 +42990,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/21/26)</t>
+          <t>Hiring AEs? (9/22/26)</t>
         </is>
       </c>
     </row>
@@ -43048,9 +43048,9 @@
           <t>CrisisAlert wearable panic buttons for school staff; 18M+ people covered</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Senior Sales Executive (VA/WV/OH) (Remote Worker - N/)</t>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>Yes - Sales Executive - Pacific Northwes (Remote Worker - N/)</t>
         </is>
       </c>
     </row>
@@ -43168,7 +43168,7 @@
           <t>Device filtering, classroom management, and student wellness (Beacon)</t>
         </is>
       </c>
-      <c r="F7" s="9" t="inlineStr">
+      <c r="F7" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - New Business Executive - Strategic only</t>
         </is>
@@ -43702,7 +43702,7 @@
           <t>AI weapons detection and screening for schools and public buildings</t>
         </is>
       </c>
-      <c r="F25" s="10" t="inlineStr">
+      <c r="F25" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -43880,7 +43880,7 @@
           <t>InformaCast mass notification and paging for school districts</t>
         </is>
       </c>
-      <c r="F31" s="10" t="inlineStr">
+      <c r="F31" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -44292,7 +44292,7 @@
           <t>School bus telematics, electronic inspections, and ridership tracking</t>
         </is>
       </c>
-      <c r="F45" s="10" t="inlineStr">
+      <c r="F45" s="9" t="inlineStr">
         <is>
           <t>Yes - Sales Account Executive – Mid-Mark</t>
         </is>
@@ -44324,7 +44324,7 @@
       </c>
       <c r="F46" s="34" t="inlineStr">
         <is>
-          <t>None found</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -45012,7 +45012,7 @@
           <t>Unified school-home communication platform - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F69" s="9" t="inlineStr">
+      <c r="F69" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -45132,7 +45132,7 @@
           <t>Capital program management and purchasing/AP compliance for 140+ California districts</t>
         </is>
       </c>
-      <c r="F73" s="10" t="inlineStr">
+      <c r="F73" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -45550,7 +45550,7 @@
           <t>Alternative student transportation for school districts (formerly ALC Schools): contracted vehicles and drivers for students a yellow bus cannot serve, with dispatch and tracking for the district - exhibited at NAPT Summit 2026</t>
         </is>
       </c>
-      <c r="F87" s="10" t="inlineStr">
+      <c r="F87" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Executive, Southern Califo (Remote Southern Ca)</t>
         </is>
@@ -45670,7 +45670,7 @@
           <t>School and district websites, apps and communications for public schools</t>
         </is>
       </c>
-      <c r="F91" s="10" t="inlineStr">
+      <c r="F91" s="9" t="inlineStr">
         <is>
           <t>Yes - Sales Executive (Remote Worker - N/)</t>
         </is>
@@ -45760,9 +45760,9 @@
           <t>Absence, substitute placement and time tracking for school districts</t>
         </is>
       </c>
-      <c r="F94" s="34" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F94" s="35" t="inlineStr">
+        <is>
+          <t>Yes - Account Executive (Remote Worker - N/)</t>
         </is>
       </c>
     </row>
@@ -45910,7 +45910,7 @@
           <t>Dismissal, attendance and school safety workflow platform for districts</t>
         </is>
       </c>
-      <c r="F99" s="10" t="inlineStr">
+      <c r="F99" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -45970,7 +45970,7 @@
           <t>Single sign-on, rostering and usage analytics for public school districts - exhibited at CoSN 2026, EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F101" s="10" t="inlineStr">
+      <c r="F101" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -46136,7 +46136,7 @@
           <t>Digital hall pass, tardy tracking, behavior management, and campus engagement platform for K-12 schools and districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F107" s="10" t="inlineStr">
+      <c r="F107" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Manager (INTERNAL APPLICAN</t>
         </is>
@@ -46198,7 +46198,7 @@
       </c>
       <c r="F109" s="7" t="inlineStr">
         <is>
-          <t>None found</t>
+          <t>Unknown - HTTP 404 for https://boards-api.greenhou</t>
         </is>
       </c>
     </row>
@@ -46280,9 +46280,9 @@
           <t>Library, technology asset, and facilities management software for K-12 school districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F112" s="34" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F112" s="33" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Inside Sales Account Executive only</t>
         </is>
       </c>
     </row>
@@ -46528,7 +46528,7 @@
           <t>Classroom browser monitoring, web filtering and student wellbeing alerting software for K-12 schools and districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F121" s="10" t="inlineStr">
+      <c r="F121" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -46642,7 +46642,7 @@
           <t>Student survey, MTSS, behavior analytics and early-warning software for K-12 school districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F125" s="10" t="inlineStr">
+      <c r="F125" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -46806,7 +46806,7 @@
           <t>Phone-free school software that blocks distracting apps during class and records attendance for K-12 districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F131" s="10" t="inlineStr">
+      <c r="F131" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -46972,7 +46972,7 @@
           <t>AI service desk and service operations platform unifying IT, facilities, HR and transportation requests for K-12 districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F137" s="10" t="inlineStr">
+      <c r="F137" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -47086,7 +47086,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/21/26)</t>
+          <t>Hiring AEs? (9/22/26)</t>
         </is>
       </c>
     </row>
@@ -47144,7 +47144,7 @@
           <t>Justride fare payments SaaS used by hundreds of agencies</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="F3" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Customer Success Manager - UK only</t>
         </is>
@@ -47620,7 +47620,7 @@
           <t>Check-in/be-out mobile fare payment for public transport authorities</t>
         </is>
       </c>
-      <c r="F19" s="10" t="inlineStr">
+      <c r="F19" s="9" t="inlineStr">
         <is>
           <t>Yes - Sales &amp; Business Development Manag</t>
         </is>
@@ -47860,7 +47860,7 @@
           <t>HASTUS scheduling, run-cutting, and rostering for transit agencies and postal operators</t>
         </is>
       </c>
-      <c r="F27" s="9" t="inlineStr">
+      <c r="F27" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Director, Strategic Business Devel only</t>
         </is>
@@ -47920,7 +47920,7 @@
           <t>Holding group of ~34 transit software brands under Constellation (Trapeze, Vontas, TransTrack, TripSpark, TransLoc)</t>
         </is>
       </c>
-      <c r="F29" s="9" t="inlineStr">
+      <c r="F29" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Sales &amp; Marketing Director only</t>
         </is>
@@ -48154,7 +48154,7 @@
           <t>iMarq mobile asset maintenance and MRO platform for transit, rail, and fleets</t>
         </is>
       </c>
-      <c r="F37" s="10" t="inlineStr">
+      <c r="F37" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -48334,7 +48334,7 @@
           <t>SCADA systems and the SentientQ automation platform for rail transit, LRT, and utilities</t>
         </is>
       </c>
-      <c r="F43" s="10" t="inlineStr">
+      <c r="F43" s="9" t="inlineStr">
         <is>
           <t>Yes - Business Development Manager</t>
         </is>
@@ -49104,7 +49104,7 @@
           <t>AI dashcam and driver coaching for public fleets</t>
         </is>
       </c>
-      <c r="F69" s="10" t="inlineStr">
+      <c r="F69" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Executive, Mid-Market (USA)</t>
         </is>
@@ -49164,7 +49164,7 @@
           <t>Fleet maintenance software for cities, counties and transit agencies</t>
         </is>
       </c>
-      <c r="F71" s="10" t="inlineStr">
+      <c r="F71" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Executive (Remote Worker)</t>
         </is>
@@ -49224,7 +49224,7 @@
           <t>Fleet maintenance management software for transit and government fleets</t>
         </is>
       </c>
-      <c r="F73" s="10" t="inlineStr">
+      <c r="F73" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -49344,7 +49344,7 @@
           <t>Digital vehicle inspections and maintenance for municipal fleets</t>
         </is>
       </c>
-      <c r="F77" s="9" t="inlineStr">
+      <c r="F77" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Operations Manager, Customer Succe only</t>
         </is>
@@ -49796,7 +49796,7 @@
       </c>
       <c r="F92" s="39" t="inlineStr">
         <is>
-          <t>Yes - Strategic Account Executive (North Carolina_Rem)</t>
+          <t>Yes - Mass Market Account Executive (Arizona_Remote)</t>
         </is>
       </c>
     </row>
@@ -49884,7 +49884,7 @@
           <t>Solar e-paper real-time passenger information displays and cloud CMS for bus stops and stations</t>
         </is>
       </c>
-      <c r="F95" s="10" t="inlineStr">
+      <c r="F95" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -50242,7 +50242,7 @@
           <t>On-demand transit, paratransit, and network planning software for agencies - exhibited at CTAA EXPO 2026</t>
         </is>
       </c>
-      <c r="F107" s="10" t="inlineStr">
+      <c r="F107" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Executive, Western Europe (Paris)</t>
         </is>
@@ -50542,7 +50542,7 @@
           <t>Turnkey autonomous shuttle operations for transit agencies, airports, and communities</t>
         </is>
       </c>
-      <c r="F117" s="9" t="inlineStr">
+      <c r="F117" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -51484,7 +51484,7 @@
           <t>Smart single-space parking meters and enforcement systems</t>
         </is>
       </c>
-      <c r="F149" s="9" t="inlineStr">
+      <c r="F149" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Sr. Client Success Manager only</t>
         </is>
@@ -51664,7 +51664,7 @@
           <t>Parking permits, enforcement, PARCS, and pay stations for universities and cities (Verra Mobility)</t>
         </is>
       </c>
-      <c r="F155" s="10" t="inlineStr">
+      <c r="F155" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -51724,9 +51724,9 @@
           <t>Mobility and curb/parking technology platform - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F157" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Account Manager (Helsinki)</t>
+      <c r="F157" s="9" t="inlineStr">
+        <is>
+          <t>Yes - Junior B2B Account Executive (Prague)</t>
         </is>
       </c>
     </row>
@@ -52392,7 +52392,7 @@
           <t>Security and intelligence analytics software - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F181" s="10" t="inlineStr">
+      <c r="F181" s="9" t="inlineStr">
         <is>
           <t>Yes - Enterprise Sales Executive – New L (2 Locations)</t>
         </is>
@@ -52586,7 +52586,7 @@
           <t>GPS fleet tracking and telematics software - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F189" s="10" t="inlineStr">
+      <c r="F189" s="9" t="inlineStr">
         <is>
           <t>Yes - Sales Account Executive – Mid-Mark</t>
         </is>
@@ -52728,7 +52728,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/21/26)</t>
+          <t>Hiring AEs? (9/22/26)</t>
         </is>
       </c>
     </row>
@@ -52846,7 +52846,7 @@
           <t>Autonomous off-grid solar streetlights with remote monitoring; 1,000+ municipalities, 43 states (French parent)</t>
         </is>
       </c>
-      <c r="F5" s="10" t="inlineStr">
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -53386,7 +53386,7 @@
           <t>Aluminum and steel lighting poles for municipal and DOT projects</t>
         </is>
       </c>
-      <c r="F23" s="10" t="inlineStr">
+      <c r="F23" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -53446,7 +53446,7 @@
           <t>Adaptive smart street lighting sensors and CMS for municipalities</t>
         </is>
       </c>
-      <c r="F25" s="9" t="inlineStr">
+      <c r="F25" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -53506,7 +53506,7 @@
           <t>Street lighting luminaires and connected controls for public authorities</t>
         </is>
       </c>
-      <c r="F27" s="10" t="inlineStr">
+      <c r="F27" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -53986,7 +53986,7 @@
           <t>Exterior LED site and streetscape lighting for public projects</t>
         </is>
       </c>
-      <c r="F43" s="10" t="inlineStr">
+      <c r="F43" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -54046,7 +54046,7 @@
           <t>Pole-mounted sensors + AI (Gridscope) detecting grid faults, vegetation strikes, and wildfire-risk events</t>
         </is>
       </c>
-      <c r="F45" s="9" t="inlineStr">
+      <c r="F45" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Customer Success Manager only</t>
         </is>
@@ -54106,7 +54106,7 @@
           <t>Satellite + AI vegetation management (IVMS) and climate/asset risk SaaS for utilities</t>
         </is>
       </c>
-      <c r="F47" s="9" t="inlineStr">
+      <c r="F47" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Business Analyst - Customer Succes only</t>
         </is>
@@ -54166,7 +54166,7 @@
           <t>EV ARC transportable solar EV charging and storage for government fleets (Nasdaq: BEEM; ex-Envision Solar)</t>
         </is>
       </c>
-      <c r="F49" s="10" t="inlineStr">
+      <c r="F49" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -54286,7 +54286,7 @@
           <t>Metering, CIS, billing and grid analytics for public power utilities</t>
         </is>
       </c>
-      <c r="F53" s="9" t="inlineStr">
+      <c r="F53" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -54466,7 +54466,7 @@
           <t>Smart grid AMI and grid analytics for public power utilities and co-ops</t>
         </is>
       </c>
-      <c r="F59" s="9" t="inlineStr">
+      <c r="F59" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Office &amp; Sales Support Coordinator only</t>
         </is>
@@ -54706,7 +54706,7 @@
           <t>DERMS and virtual power plant programs for utilities including public power</t>
         </is>
       </c>
-      <c r="F67" s="9" t="inlineStr">
+      <c r="F67" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Sales Engineer only</t>
         </is>
@@ -54946,7 +54946,7 @@
           <t>Utility bill management and energy analytics for cities, counties and schools</t>
         </is>
       </c>
-      <c r="F75" s="10" t="inlineStr">
+      <c r="F75" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Executive</t>
         </is>
@@ -55184,7 +55184,7 @@
           <t>Outage notification, billing, and omnichannel customer communication platform for investor-owned, municipal, and cooperative utilities - exhibited at APPA Public Power 2026</t>
         </is>
       </c>
-      <c r="F83" s="10" t="inlineStr">
+      <c r="F83" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Executive (US - Remote)</t>
         </is>
@@ -55598,7 +55598,7 @@
           <t>Geospatial network design and field software for telecom and public utilities</t>
         </is>
       </c>
-      <c r="F97" s="9" t="inlineStr">
+      <c r="F97" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Sales Engineer only</t>
         </is>
@@ -55718,7 +55718,7 @@
           <t>Broadband grant, challenge process and mapping software for state broadband offices</t>
         </is>
       </c>
-      <c r="F101" s="9" t="inlineStr">
+      <c r="F101" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Product Solutions Engineer only</t>
         </is>
@@ -56286,7 +56286,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/21/26)</t>
+          <t>Hiring AEs? (9/22/26)</t>
         </is>
       </c>
     </row>
@@ -56756,7 +56756,7 @@
           <t>Aviation design and simulation software (AviPLAN, AeroTURN, GuideSIGN) used by airport planners for aircraft movement, apron layout and airside safety analysis.</t>
         </is>
       </c>
-      <c r="F17" s="10" t="inlineStr">
+      <c r="F17" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Manager (Sales)</t>
         </is>
@@ -57172,7 +57172,7 @@
           <t>Airport weather observation systems and runway condition sensors for airports - exhibited at NACE 2026</t>
         </is>
       </c>
-      <c r="F31" s="10" t="inlineStr">
+      <c r="F31" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -57232,7 +57232,7 @@
           <t>Bird-strike avoidance radar and wildlife management systems for airports</t>
         </is>
       </c>
-      <c r="F33" s="9" t="inlineStr">
+      <c r="F33" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -57352,7 +57352,7 @@
           <t>ARINC airport systems portfolio: vMUSE common-use passenger processing, SelfPass biometrics, self bag drop, AODB/resource management, FIDS and airport communications sold to airport authorities.</t>
         </is>
       </c>
-      <c r="F37" s="9" t="inlineStr">
+      <c r="F37" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -57590,7 +57590,7 @@
           <t>Passenger flow, queue measurement and airport revenue software for airport operators</t>
         </is>
       </c>
-      <c r="F45" s="10" t="inlineStr">
+      <c r="F45" s="9" t="inlineStr">
         <is>
           <t>Yes - Sales Director Americas (US-based within th)</t>
         </is>
@@ -57710,7 +57710,7 @@
           <t>Gate, docking guidance and apron systems for airport operators</t>
         </is>
       </c>
-      <c r="F49" s="10" t="inlineStr">
+      <c r="F49" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -57890,7 +57890,7 @@
           <t>Self-service kiosks, bag drop and passenger processing for airports</t>
         </is>
       </c>
-      <c r="F55" s="10" t="inlineStr">
+      <c r="F55" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -58070,7 +58070,7 @@
           <t>Airport IQ operations, property and lease management software for airports</t>
         </is>
       </c>
-      <c r="F61" s="10" t="inlineStr">
+      <c r="F61" s="9" t="inlineStr">
         <is>
           <t>Yes - Senior Account Executive</t>
         </is>
@@ -58610,7 +58610,7 @@
           <t>Biometric identity, TSA PreCheck enrollment and airport boarding systems</t>
         </is>
       </c>
-      <c r="F79" s="10" t="inlineStr">
+      <c r="F79" s="9" t="inlineStr">
         <is>
           <t>Yes - Key Account Manager - Smart Biomet</t>
         </is>
@@ -58670,7 +58670,7 @@
           <t>Biometric identity lanes operated under airport and TSA agreements</t>
         </is>
       </c>
-      <c r="F81" s="10" t="inlineStr">
+      <c r="F81" s="9" t="inlineStr">
         <is>
           <t>Yes - Enterprise Account Executive (C1 - (New York, New York)</t>
         </is>
@@ -58790,7 +58790,7 @@
           <t>Perimeter intrusion detection and fence sensors for airports and utilities</t>
         </is>
       </c>
-      <c r="F85" s="10" t="inlineStr">
+      <c r="F85" s="9" t="inlineStr">
         <is>
           <t>Yes - Business Development Manager (Ottawa, Ontario, C)</t>
         </is>
@@ -59028,7 +59028,7 @@
           <t>Automated vehicle inspection portals for airports, borders and government</t>
         </is>
       </c>
-      <c r="F93" s="10" t="inlineStr">
+      <c r="F93" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -59148,7 +59148,7 @@
           <t>Computer-vision checkout-free parking payment platform (drive-in/drive-out billing) plus parking operations and revenue management for airports; owner of SP+.</t>
         </is>
       </c>
-      <c r="F97" s="10" t="inlineStr">
+      <c r="F97" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Manager (Remote USA)</t>
         </is>
@@ -59326,7 +59326,7 @@
           <t>Airport parking reservations and demand channel for airport operators</t>
         </is>
       </c>
-      <c r="F103" s="10" t="inlineStr">
+      <c r="F103" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -59386,7 +59386,7 @@
           <t>Full-service automated parking operations for cities and airports</t>
         </is>
       </c>
-      <c r="F105" s="9" t="inlineStr">
+      <c r="F105" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Sales Development Representative only</t>
         </is>
@@ -59506,7 +59506,7 @@
           <t>AVI readers and ground transportation management systems for airports</t>
         </is>
       </c>
-      <c r="F109" s="10" t="inlineStr">
+      <c r="F109" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -59746,7 +59746,7 @@
           <t>Web-based capital program and construction project management software (cost, contracts, documents, scheduling) used by airport owner-operators and public agencies.</t>
         </is>
       </c>
-      <c r="F117" s="10" t="inlineStr">
+      <c r="F117" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -59810,7 +59810,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/21/26)</t>
+          <t>Hiring AEs? (9/22/26)</t>
         </is>
       </c>
     </row>
@@ -60146,7 +60146,7 @@
           <t>Digital courtroom recording and speech recognition systems for courts</t>
         </is>
       </c>
-      <c r="F13" s="10" t="inlineStr">
+      <c r="F13" s="9" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -60264,7 +60264,7 @@
           <t>Criminal justice data collection and public dashboards for counties and states</t>
         </is>
       </c>
-      <c r="F17" s="9" t="inlineStr">
+      <c r="F17" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -60324,7 +60324,7 @@
           <t>Cloud ediscovery and litigation platform for law firms, corporations, county DAs, and state AGs - exhibited at IMLA 2026, NASCIO 2026</t>
         </is>
       </c>
-      <c r="F19" s="10" t="inlineStr">
+      <c r="F19" s="9" t="inlineStr">
         <is>
           <t>Yes - Enterprise Account Executive (Stat (United States)</t>
         </is>
@@ -60384,7 +60384,7 @@
           <t>PROSECUTORbyKarpel case management software for prosecutor offices - exhibited at IMLA 2026</t>
         </is>
       </c>
-      <c r="F21" s="10" t="inlineStr">
+      <c r="F21" s="9" t="inlineStr">
         <is>
           <t>Yes - Account Manager (Remote Worker - N/)</t>
         </is>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-09-23)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -246,9 +246,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -296,8 +296,8 @@
     <xf numFmtId="1" fontId="2" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/22/26)</t>
+          <t>Hiring AEs? (9/23/26)</t>
         </is>
       </c>
     </row>
@@ -1120,9 +1120,9 @@
           <t>Wildfire spread modeling and risk analytics used by CAL FIRE and major utilities</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Sr. Manager, FP&amp;A &amp; Sales Operatio only</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1180,7 @@
           <t>Exterior retardant/foam systems and app-based wildfire defense for homes and HOAs</t>
         </is>
       </c>
-      <c r="F9" s="9" t="inlineStr">
+      <c r="F9" s="10" t="inlineStr">
         <is>
           <t>Yes - Territory Manager - LA (Los Angeles, CA)</t>
         </is>
@@ -1330,7 +1330,7 @@
           <t>Actively tethered situational awareness drones with unlimited flight time for fire/PS</t>
         </is>
       </c>
-      <c r="F14" s="10" t="inlineStr">
+      <c r="F14" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Sales Engineer only</t>
         </is>
@@ -1414,7 +1414,7 @@
           <t>Cloud fire and EMS records management for departments of all sizes</t>
         </is>
       </c>
-      <c r="F17" s="9" t="inlineStr">
+      <c r="F17" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -1650,7 +1650,7 @@
           <t>Satellite vegetation intelligence for wildfire risk at utilities and agencies</t>
         </is>
       </c>
-      <c r="F25" s="9" t="inlineStr">
+      <c r="F25" s="10" t="inlineStr">
         <is>
           <t>Yes - Enterprise Account Executive, Cana (Remote, Canada)</t>
         </is>
@@ -2070,7 +2070,7 @@
           <t>License plate readers, gunshot detection, and drone-as-first-responder (Aerodome)</t>
         </is>
       </c>
-      <c r="F39" s="11" t="inlineStr">
+      <c r="F39" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Senior Deal Desk Analyst only</t>
         </is>
@@ -2130,7 +2130,7 @@
           <t>911-response and tactical drones staged on police and fire station rooftops</t>
         </is>
       </c>
-      <c r="F41" s="9" t="inlineStr">
+      <c r="F41" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Executive, DFR (Remote (Select Sta)</t>
         </is>
@@ -2190,7 +2190,7 @@
           <t>Data integration and real-time intelligence platform for police and city agencies - exhibited at IAFC FRI 2026</t>
         </is>
       </c>
-      <c r="F43" s="9" t="inlineStr">
+      <c r="F43" s="10" t="inlineStr">
         <is>
           <t>Yes - Federal Account Executive (Washington, D.C.)</t>
         </is>
@@ -2402,7 +2402,7 @@
       </c>
       <c r="F50" s="8" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (U.S. (Remote))</t>
+          <t>Yes - Account Executive - ECC (U.S. (Remote))</t>
         </is>
       </c>
     </row>
@@ -2550,7 +2550,7 @@
           <t>Incident reporting and case management for law enforcement, campus, and healthcare security</t>
         </is>
       </c>
-      <c r="F55" s="11" t="inlineStr">
+      <c r="F55" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -2670,7 +2670,7 @@
           <t>AI audio/video/document redaction (CaseGuard Studio) for police, courts, and gov</t>
         </is>
       </c>
-      <c r="F59" s="9" t="inlineStr">
+      <c r="F59" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Manager (Arlington, VA)</t>
         </is>
@@ -2940,7 +2940,7 @@
           <t>Digital investigation suite for cleansing and evidencing comms data (UK + US LE)</t>
         </is>
       </c>
-      <c r="F68" s="10" t="inlineStr">
+      <c r="F68" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -2970,7 +2970,7 @@
           <t>Investigation database: pawn/secondhand transactions plus ballistics ID for agencies - exhibited at Michigan Sheriffs Association 2026</t>
         </is>
       </c>
-      <c r="F69" s="9" t="inlineStr">
+      <c r="F69" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -3090,7 +3090,7 @@
           <t>Cloud cameras, access control, and sensors with a dedicated SLED sales org - exhibited at EDUCAUSE 2026, Maryland Municipal League 2026</t>
         </is>
       </c>
-      <c r="F73" s="9" t="inlineStr">
+      <c r="F73" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Executive, France (London)</t>
         </is>
@@ -3330,7 +3330,7 @@
           <t>Drone-as-first-responder software and hardware auto-launching to 911 calls</t>
         </is>
       </c>
-      <c r="F81" s="9" t="inlineStr">
+      <c r="F81" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Executive</t>
         </is>
@@ -3570,7 +3570,7 @@
           <t>Bird and drone detection radars (ELVIRA, IRIS) for airports, security, and C-UAS</t>
         </is>
       </c>
-      <c r="F89" s="9" t="inlineStr">
+      <c r="F89" s="10" t="inlineStr">
         <is>
           <t>Yes - Regional Account Manager - Nordics (Nordics)</t>
         </is>
@@ -3720,7 +3720,7 @@
           <t>Training LMS, scheduling, and readiness software (TargetSolutions, Guardian Tracking) - exhibited at IAFC FRI 2026, APCO 2026</t>
         </is>
       </c>
-      <c r="F94" s="10" t="inlineStr">
+      <c r="F94" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -3810,7 +3810,7 @@
           <t>Scheduling and workforce management for police, corrections, and 911</t>
         </is>
       </c>
-      <c r="F97" s="9" t="inlineStr">
+      <c r="F97" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -3870,7 +3870,7 @@
           <t>OfficerTRAK off-duty detail management: scheduling, billing, insurance - exhibited at NLC City Summit 2026</t>
         </is>
       </c>
-      <c r="F99" s="9" t="inlineStr">
+      <c r="F99" s="10" t="inlineStr">
         <is>
           <t>Yes - Business Development Manager - Mid (Charlotte, North C)</t>
         </is>
@@ -3930,7 +3930,7 @@
           <t>Online application and recruiting platform for police and civil service hiring</t>
         </is>
       </c>
-      <c r="F101" s="11" t="inlineStr">
+      <c r="F101" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -4350,7 +4350,7 @@
           <t>Cyber-over-RF counter-drone detect, track, and mitigate systems for LE, prisons, and infrastructure</t>
         </is>
       </c>
-      <c r="F115" s="9" t="inlineStr">
+      <c r="F115" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -4738,7 +4738,7 @@
           <t>Retail crime intelligence and reporting platform - exhibited at IACP 2026</t>
         </is>
       </c>
-      <c r="F129" s="9" t="inlineStr">
+      <c r="F129" s="10" t="inlineStr">
         <is>
           <t>Yes - Enterprise Account Manager (Biling (Remote - United St)</t>
         </is>
@@ -4788,7 +4788,7 @@
           <t>Software for first responder agencies - exhibited at IACP 2026, APCO 2026</t>
         </is>
       </c>
-      <c r="F131" s="9" t="inlineStr">
+      <c r="F131" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Executive (United States)</t>
         </is>
@@ -4842,7 +4842,7 @@
           <t>AI investigations platform for law enforcement - exhibited at IACP 2026</t>
         </is>
       </c>
-      <c r="F133" s="9" t="inlineStr">
+      <c r="F133" s="10" t="inlineStr">
         <is>
           <t>Yes - Enterprise Account Executive</t>
         </is>
@@ -5382,7 +5382,7 @@
           <t>FBI-certified mobile fingerprint scanners for police and government</t>
         </is>
       </c>
-      <c r="F151" s="11" t="inlineStr">
+      <c r="F151" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -5412,7 +5412,7 @@
           <t>Data integration and investigative analytics for police and government</t>
         </is>
       </c>
-      <c r="F152" s="10" t="inlineStr">
+      <c r="F152" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Forward Deployed Enablement Engine only</t>
         </is>
@@ -5862,7 +5862,7 @@
           <t>ePCR, records, and analytics connecting EMS, fire, and hospitals - exhibited at IAFC FRI 2026</t>
         </is>
       </c>
-      <c r="F167" s="9" t="inlineStr">
+      <c r="F167" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Manager (Remote, US (TN/KY))</t>
         </is>
@@ -5922,7 +5922,7 @@
           <t>Intelligent 911 platform streaming device location and data to dispatch - exhibited at APCO 2026</t>
         </is>
       </c>
-      <c r="F169" s="11" t="inlineStr">
+      <c r="F169" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Director, Customer Solutions Engin only</t>
         </is>
@@ -5982,7 +5982,7 @@
           <t>Assistive AI for 911 centers: transcription, translation, text-to-911, and video</t>
         </is>
       </c>
-      <c r="F171" s="9" t="inlineStr">
+      <c r="F171" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -6282,7 +6282,7 @@
           <t>Pediatric emergency dosing system and app for EMS agencies</t>
         </is>
       </c>
-      <c r="F181" s="9" t="inlineStr">
+      <c r="F181" s="10" t="inlineStr">
         <is>
           <t>Yes - Enterprise Account Executive</t>
         </is>
@@ -6402,7 +6402,7 @@
           <t>Mobile incident command and response for fire/EMS departments - exhibited at IAFC FRI 2026</t>
         </is>
       </c>
-      <c r="F185" s="9" t="inlineStr">
+      <c r="F185" s="10" t="inlineStr">
         <is>
           <t>Yes - Regional Account Executive</t>
         </is>
@@ -6582,7 +6582,7 @@
           <t>911 call routing, Viper call handling and NG911 for PSAPs</t>
         </is>
       </c>
-      <c r="F191" s="9" t="inlineStr">
+      <c r="F191" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -6702,7 +6702,7 @@
           <t>AI triage and quality assurance for emergency dispatch centers</t>
         </is>
       </c>
-      <c r="F195" s="11" t="inlineStr">
+      <c r="F195" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - GTM Engineer only</t>
         </is>
@@ -6968,7 +6968,7 @@
           <t>SARA situational awareness and mass notification for schools, senior living, and gov facilities</t>
         </is>
       </c>
-      <c r="F204" s="10" t="inlineStr">
+      <c r="F204" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -7538,7 +7538,7 @@
           <t>CID Net inmate calling (450+ facilities), facility monitoring, and family apps</t>
         </is>
       </c>
-      <c r="F223" s="11" t="inlineStr">
+      <c r="F223" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -8636,7 +8636,7 @@
           <t>Data and case-management tools for state corrections and supervision agencies</t>
         </is>
       </c>
-      <c r="F260" s="10" t="inlineStr">
+      <c r="F260" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - State Partnerships Manager only</t>
         </is>
@@ -9458,7 +9458,7 @@
           <t>Digital forensics and investigation management software - exhibited at IACP 2026</t>
         </is>
       </c>
-      <c r="F289" s="11" t="inlineStr">
+      <c r="F289" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Sales Operations &amp; GTM Systems Man only</t>
         </is>
@@ -9584,7 +9584,7 @@
           <t>AI police report writing and investigation software - exhibited at IACP 2026</t>
         </is>
       </c>
-      <c r="F294" s="10" t="inlineStr">
+      <c r="F294" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -10660,7 +10660,7 @@
           <t>DigiTICKET electronic citation software - exhibited at IACP 2026</t>
         </is>
       </c>
-      <c r="F338" s="10" t="inlineStr">
+      <c r="F338" s="11" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -11136,7 +11136,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/22/26)</t>
+          <t>Hiring AEs? (9/23/26)</t>
         </is>
       </c>
     </row>
@@ -11488,7 +11488,7 @@
       </c>
       <c r="F14" s="64" t="inlineStr">
         <is>
-          <t>Yes - Commercial Account Executive (Remote – United St)</t>
+          <t>Yes - Strategic Account Executive, Marke (Remote – United St)</t>
         </is>
       </c>
     </row>
@@ -12424,7 +12424,7 @@
           <t>Care coordination and PDMP network software (PMP AWARxE, OpenBeds) for states, counties, and health systems (Appriss lineage)</t>
         </is>
       </c>
-      <c r="F47" s="9" t="inlineStr">
+      <c r="F47" s="10" t="inlineStr">
         <is>
           <t>Yes - Bamboo Bridge Strategic Account Ma</t>
         </is>
@@ -12766,7 +12766,7 @@
           <t>Digital substance use disorder prevention, intervention, and recovery support platform for treatment providers, state and county health agencies, drug courts, and Medicaid plans - exhibited at NatCon 2026, NACCHO 360 2026</t>
         </is>
       </c>
-      <c r="F59" s="11" t="inlineStr">
+      <c r="F59" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Senior Customer Success Consultant only</t>
         </is>
@@ -12982,7 +12982,7 @@
           <t>Human services EHR and care coordination software for behavioral health, residential, vocational rehab, and food assistance providers - exhibited at NatCon 2026</t>
         </is>
       </c>
-      <c r="F67" s="11" t="inlineStr">
+      <c r="F67" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Customer Success Manager only</t>
         </is>
@@ -13192,7 +13192,7 @@
           <t>AI clinical documentation and chart auditing platform purpose-built for behavioral health providers including CCBHCs and human services organizations - exhibited at NatCon 2026</t>
         </is>
       </c>
-      <c r="F75" s="11" t="inlineStr">
+      <c r="F75" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - VP of Revenue only</t>
         </is>
@@ -13246,7 +13246,7 @@
           <t>Accredited continuing-education, AI practice simulation and certification platform for behavioral health clinicians and the organizations that employ them - exhibited at NatCon 2026</t>
         </is>
       </c>
-      <c r="F77" s="9" t="inlineStr">
+      <c r="F77" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -13610,7 +13610,7 @@
           <t>Social care coordination network connecting health and social service referrals for govs and payers - exhibited at MESC 2026</t>
         </is>
       </c>
-      <c r="F91" s="9" t="inlineStr">
+      <c r="F91" s="10" t="inlineStr">
         <is>
           <t>Yes - Strategic Sales Director (United States)</t>
         </is>
@@ -13730,7 +13730,7 @@
           <t>Clarity HMIS and homelessness response systems for counties and CoCs</t>
         </is>
       </c>
-      <c r="F95" s="11" t="inlineStr">
+      <c r="F95" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Solutions Consultant only</t>
         </is>
@@ -14018,7 +14018,7 @@
           <t>EHR and case management software for PACE programs, State Units on Aging, Area Agencies on Aging and community-based aging services organizations - exhibited at USAging 2026</t>
         </is>
       </c>
-      <c r="F105" s="9" t="inlineStr">
+      <c r="F105" s="10" t="inlineStr">
         <is>
           <t>Yes - Sales Director, PACE (Remote Worker - N/)</t>
         </is>
@@ -14420,7 +14420,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/22/26)</t>
+          <t>Hiring AEs? (9/23/26)</t>
         </is>
       </c>
     </row>
@@ -14588,7 +14588,7 @@
           <t>Course evaluation, survey, and AI feedback analysis software - Blue, MLY, and Metrics That Matter - for universities and corporate learning teams - exhibited at EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F7" s="9" t="inlineStr">
+      <c r="F7" s="10" t="inlineStr">
         <is>
           <t>Yes - Junior Account Manager</t>
         </is>
@@ -15024,9 +15024,9 @@
           <t>Digital textbook and courseware delivery platform for colleges, universities, and school districts - exhibited at NACUBO 2026</t>
         </is>
       </c>
-      <c r="F22" s="69" t="inlineStr">
-        <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+      <c r="F22" s="70" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Sales Support - Keyholder only</t>
         </is>
       </c>
     </row>
@@ -15054,9 +15054,9 @@
           <t>Canvas learning management system plus assessment and credentialing software for universities, school districts, and government training programs - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F23" s="9" t="inlineStr">
-        <is>
-          <t>Yes - Senior Account Executive - BizGov (United States)</t>
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>Yes - Senior Account Executive - Canvas  (United States)</t>
         </is>
       </c>
     </row>
@@ -15934,7 +15934,7 @@
           <t>Residence life and student housing management software covering applications, room assignment, billing and community programming for universities and colleges - exhibited at EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F55" s="9" t="inlineStr">
+      <c r="F55" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Executive, EMEA (UK - Remote)</t>
         </is>
@@ -16520,7 +16520,7 @@
           <t>Degree planning, advising, transfer pathway and registration software for public universities, community colleges and private institutions - exhibited at EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F77" s="11" t="inlineStr">
+      <c r="F77" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Solutions Consultant only</t>
         </is>
@@ -17026,7 +17026,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/22/26)</t>
+          <t>Hiring AEs? (9/23/26)</t>
         </is>
       </c>
     </row>
@@ -17296,7 +17296,7 @@
           <t>Grant and program administration software for affordable housing, disaster recovery, vouchers and energy rebate programs run by local and state agencies - exhibited at NAHRO 2026</t>
         </is>
       </c>
-      <c r="F11" s="9" t="inlineStr">
+      <c r="F11" s="10" t="inlineStr">
         <is>
           <t>Yes - Technical Account Manager, Strateg (Atlanta)</t>
         </is>
@@ -17494,7 +17494,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/22/26)</t>
+          <t>Hiring AEs? (9/23/26)</t>
         </is>
       </c>
     </row>
@@ -17552,7 +17552,7 @@
           <t>Routing, in-cab fleet tech, and resident apps for waste operations - exhibited at SWANA WASTECON 2025</t>
         </is>
       </c>
-      <c r="F3" s="11" t="inlineStr">
+      <c r="F3" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Customer Success Manager only</t>
         </is>
@@ -17612,7 +17612,7 @@
           <t>AI robotic sorting systems for recycling facilities (MRFs) - exhibited at SWANA WASTECON 2025</t>
         </is>
       </c>
-      <c r="F5" s="11" t="inlineStr">
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Director, Commercial Origination &amp; only</t>
         </is>
@@ -18266,7 +18266,7 @@
           <t>Waste collection route optimization and sensor platform for municipalities</t>
         </is>
       </c>
-      <c r="F27" s="11" t="inlineStr">
+      <c r="F27" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -18648,7 +18648,7 @@
       </c>
       <c r="F40" s="16" t="inlineStr">
         <is>
-          <t>Yes - Regional Sales Manager (2 Locations)</t>
+          <t>Yes - Outside Sales Representative (4 Locations)</t>
         </is>
       </c>
     </row>
@@ -18968,7 +18968,7 @@
           <t>School bus stop-arm cameras with violator-funded safety programs</t>
         </is>
       </c>
-      <c r="F51" s="11" t="inlineStr">
+      <c r="F51" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Lead Salesforce Developer only</t>
         </is>
@@ -19328,7 +19328,7 @@
           <t>SmartSensor radar vehicle detection for intersections and highways</t>
         </is>
       </c>
-      <c r="F63" s="11" t="inlineStr">
+      <c r="F63" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Sales Manager (Great Lakes) only</t>
         </is>
@@ -20640,7 +20640,7 @@
           <t>Water infrastructure: pumps, treatment, smart meters (Sensus), and analytics - exhibited at AWWA ACE 2026, WEFTEC 2026</t>
         </is>
       </c>
-      <c r="F107" s="9" t="inlineStr">
+      <c r="F107" s="10" t="inlineStr">
         <is>
           <t>Yes - Executive Sales Representative - N (12 Locations)</t>
         </is>
@@ -20700,7 +20700,7 @@
           <t>Hydrants, valves, and acoustic leak detection for water systems - exhibited at AWWA ACE 2026, WEFTEC 2026</t>
         </is>
       </c>
-      <c r="F109" s="9" t="inlineStr">
+      <c r="F109" s="10" t="inlineStr">
         <is>
           <t>Yes - Jr. Sales Representative (Remote - Tennessee)</t>
         </is>
@@ -20760,7 +20760,7 @@
           <t>Permitting, compliance, and workflow software for water utilities - exhibited at AWWA ACE 2026, WEFTEC 2026</t>
         </is>
       </c>
-      <c r="F111" s="11" t="inlineStr">
+      <c r="F111" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Senior Customer Success Manager only</t>
         </is>
@@ -20880,7 +20880,7 @@
           <t>AI defect detection and coding for sewer inspection video - exhibited at AWWA ACE 2026, WEFTEC 2026</t>
         </is>
       </c>
-      <c r="F115" s="9" t="inlineStr">
+      <c r="F115" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Executive, Enterprise (Remote)</t>
         </is>
@@ -21000,7 +21000,7 @@
           <t>AI CCTV sewer and stormwater pipe condition assessment for councils and utilities - exhibited at WEFTEC 2026</t>
         </is>
       </c>
-      <c r="F119" s="9" t="inlineStr">
+      <c r="F119" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -21600,7 +21600,7 @@
           <t>Sewer inspection cameras, trucks and software for municipal collection systems - exhibited at Maryland Municipal League 2026, WEFTEC 2026</t>
         </is>
       </c>
-      <c r="F139" s="9" t="inlineStr">
+      <c r="F139" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -21780,7 +21780,7 @@
           <t>AI operations and forecasting software for water and wastewater utilities - exhibited at AWWA ACE 2026, WEFTEC 2026</t>
         </is>
       </c>
-      <c r="F145" s="9" t="inlineStr">
+      <c r="F145" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -21840,7 +21840,7 @@
           <t>Generative design software for water and wastewater treatment plant projects</t>
         </is>
       </c>
-      <c r="F147" s="11" t="inlineStr">
+      <c r="F147" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -22196,7 +22196,7 @@
           <t>AquaTwin digital twin software for water and sewer hydraulic modeling, surge analysis, and asset management, sold to water utilities and engineering consultants - exhibited at AWWA ACE 2026, WEFTEC 2026</t>
         </is>
       </c>
-      <c r="F159" s="9" t="inlineStr">
+      <c r="F159" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -22650,7 +22650,7 @@
           <t>IoT telematics and video safety for government fleets (public co) - exhibited at NLC City Summit 2026, PRIMA 2026, NAFA I&amp;E 2026, NAPT Summit 2026, SWANA WASTECON 2025</t>
         </is>
       </c>
-      <c r="F175" s="9" t="inlineStr">
+      <c r="F175" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -22710,7 +22710,7 @@
           <t>Asset and work order management for DPWs (part of OpenGov)</t>
         </is>
       </c>
-      <c r="F177" s="9" t="inlineStr">
+      <c r="F177" s="10" t="inlineStr">
         <is>
           <t>Yes - Enterprise Account Executive (US | Illinois | Ch)</t>
         </is>
@@ -23010,7 +23010,7 @@
           <t>Fleet maintenance SaaS: work orders, inspections, fuel for commercial and gov fleets - exhibited at NAFA I&amp;E 2026</t>
         </is>
       </c>
-      <c r="F187" s="9" t="inlineStr">
+      <c r="F187" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Executive, Mid-Market (Remote)</t>
         </is>
@@ -23490,7 +23490,7 @@
           <t>collectiveFleet low-code fleet, equipment, and motor pool management for police and municipal fleets</t>
         </is>
       </c>
-      <c r="F203" s="11" t="inlineStr">
+      <c r="F203" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -23726,7 +23726,7 @@
           <t>Cloud CMMS for municipal facilities, water plants and public works</t>
         </is>
       </c>
-      <c r="F211" s="9" t="inlineStr">
+      <c r="F211" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Executive (United Kingdom)</t>
         </is>
@@ -24026,7 +24026,7 @@
           <t>GIS-based asset and work management for local government and utilities - exhibited at AWWA ACE 2026</t>
         </is>
       </c>
-      <c r="F221" s="9" t="inlineStr">
+      <c r="F221" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Executive, Utilities (Homeoffice)</t>
         </is>
@@ -24086,7 +24086,7 @@
           <t>Combined field service and enterprise asset management cloud for water, gas and electric utilities and municipal public works departments - exhibited at AWWA ACE 2026</t>
         </is>
       </c>
-      <c r="F223" s="11" t="inlineStr">
+      <c r="F223" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -24624,7 +24624,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/22/26)</t>
+          <t>Hiring AEs? (9/23/26)</t>
         </is>
       </c>
     </row>
@@ -24682,7 +24682,7 @@
           <t>Resident communications (govDelivery), meeting and agenda management, digital services; destination marketing as Simpleview, now Granicus Destinations - exhibited at 3CMA 2026, GMIS International 2026, APHSA 2026</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="F3" s="10" t="inlineStr">
         <is>
           <t>Yes - Local Government Account Executive</t>
         </is>
@@ -25102,7 +25102,7 @@
           <t>Social media management and archiving for government and public safety (Graham Media)</t>
         </is>
       </c>
-      <c r="F17" s="9" t="inlineStr">
+      <c r="F17" s="10" t="inlineStr">
         <is>
           <t>Yes - Sales Account Executive (USA (Remote))</t>
         </is>
@@ -25522,7 +25522,7 @@
           <t>311/citizen requests, code enforcement, and notifications for ~600 small and mid-size govs - exhibited at 3CMA 2026</t>
         </is>
       </c>
-      <c r="F31" s="9" t="inlineStr">
+      <c r="F31" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -25582,7 +25582,7 @@
           <t>Telephone and virtual town hall mass-engagement platform for county officials and agencies</t>
         </is>
       </c>
-      <c r="F33" s="9" t="inlineStr">
+      <c r="F33" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -25642,7 +25642,7 @@
           <t>Interpretation management and delivery platform (video/phone) used by courts and agencies</t>
         </is>
       </c>
-      <c r="F35" s="11" t="inlineStr">
+      <c r="F35" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Director of Sales only</t>
         </is>
@@ -26228,7 +26228,7 @@
           <t>Emergency and routine mass notification for cities, counties and schools</t>
         </is>
       </c>
-      <c r="F55" s="11" t="inlineStr">
+      <c r="F55" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Customer Success Manager only</t>
         </is>
@@ -26858,7 +26858,7 @@
           <t>Permitting, licensing, and code enforcement platform for state and local government - exhibited at NLC City Summit 2026</t>
         </is>
       </c>
-      <c r="F77" s="9" t="inlineStr">
+      <c r="F77" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Executive (Remote Based - US)</t>
         </is>
@@ -26918,7 +26918,7 @@
           <t>Community development permitting and licensing software (founded as BasicGov)</t>
         </is>
       </c>
-      <c r="F79" s="11" t="inlineStr">
+      <c r="F79" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Business Development Representativ only</t>
         </is>
@@ -26978,7 +26978,7 @@
           <t>AI cameras on city fleet vehicles detect blight, graffiti, dumping for code enforcement - exhibited at NLC City Summit 2026</t>
         </is>
       </c>
-      <c r="F81" s="9" t="inlineStr">
+      <c r="F81" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Executive (Remote)</t>
         </is>
@@ -27038,7 +27038,7 @@
           <t>Cloud e-permitting and community development software for ~500 local governments (Finnish-born)</t>
         </is>
       </c>
-      <c r="F83" s="9" t="inlineStr">
+      <c r="F83" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -27098,7 +27098,7 @@
           <t>Municipal operations software: permitting, licensing, code enforcement; NJ-rooted, going national - exhibited at NLC City Summit 2026</t>
         </is>
       </c>
-      <c r="F85" s="9" t="inlineStr">
+      <c r="F85" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Executive</t>
         </is>
@@ -27218,7 +27218,7 @@
           <t>Cloud permitting, licensing, code enforcement, and GIS workflows for local governments - exhibited at GFOA 2026</t>
         </is>
       </c>
-      <c r="F89" s="9" t="inlineStr">
+      <c r="F89" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Executive</t>
         </is>
@@ -27278,7 +27278,7 @@
           <t>AI permitting and plan review: automated GIS/code compliance checks (Hernando County cut reviews 30 days to 2)</t>
         </is>
       </c>
-      <c r="F91" s="11" t="inlineStr">
+      <c r="F91" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -27916,7 +27916,7 @@
           <t>Digital plan review automation layered on agency permitting systems</t>
         </is>
       </c>
-      <c r="F113" s="11" t="inlineStr">
+      <c r="F113" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -28150,7 +28150,7 @@
           <t>Regulatory, licensing and planning software for public sector authorities - exhibited at PLA 2026</t>
         </is>
       </c>
-      <c r="F121" s="9" t="inlineStr">
+      <c r="F121" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Executive - CES (London)</t>
         </is>
@@ -28264,7 +28264,7 @@
           <t>Procurement, budgeting, and grants suite - Bonfire, Questica, eCivis (formerly GTY) - exhibited at NACUBO 2026, GFOA 2026</t>
         </is>
       </c>
-      <c r="F125" s="11" t="inlineStr">
+      <c r="F125" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Solutions Consultant only</t>
         </is>
@@ -28324,7 +28324,7 @@
           <t>Treasury platform for local government finance teams: AI reconciliation and cash forecasting - exhibited at GFOA 2026</t>
         </is>
       </c>
-      <c r="F127" s="11" t="inlineStr">
+      <c r="F127" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Business Development Representativ only</t>
         </is>
@@ -28444,7 +28444,7 @@
           <t>Cloud treasury: debt management, GASB 87/96 lease accounting, and cash management for gov finance - exhibited at NACUBO 2026, GFOA 2026</t>
         </is>
       </c>
-      <c r="F131" s="9" t="inlineStr">
+      <c r="F131" s="10" t="inlineStr">
         <is>
           <t>Yes - Enterprise Account Executive (Charlotte, NC)</t>
         </is>
@@ -28684,7 +28684,7 @@
           <t>Aerial imagery and property data analytics for county assessors, GIS, and insurers - exhibited at IAAO 2026</t>
         </is>
       </c>
-      <c r="F139" s="9" t="inlineStr">
+      <c r="F139" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -28744,7 +28744,7 @@
           <t>cashVest liquidity analytics and treasury intelligence for counties, munis, and schools</t>
         </is>
       </c>
-      <c r="F141" s="11" t="inlineStr">
+      <c r="F141" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Senior Business Development Office only</t>
         </is>
@@ -28804,7 +28804,7 @@
           <t>HR, finance and ERP software - exhibited at APTA 2026, ICMA 2025, NACo 2026, NACUBO 2026, GFOA 2026, PSHRA 2026, NASCIO 2026, EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F143" s="9" t="inlineStr">
+      <c r="F143" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Executive (Japan, Tokyo)</t>
         </is>
@@ -28924,7 +28924,7 @@
           <t>Parcel mapping, GIS and assessment systems for county governments</t>
         </is>
       </c>
-      <c r="F147" s="9" t="inlineStr">
+      <c r="F147" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -29272,7 +29272,7 @@
           <t>Fund accounting and ERP software for cities and local governments, covering financials, payroll, utility billing and municipal court - exhibited at GFOA 2026</t>
         </is>
       </c>
-      <c r="F159" s="9" t="inlineStr">
+      <c r="F159" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -29392,7 +29392,7 @@
           <t>Portfolio of vertical software businesses selling ERP, utility billing and public sector operations systems to local governments and utilities - exhibited at GFOA 2026</t>
         </is>
       </c>
-      <c r="F163" s="9" t="inlineStr">
+      <c r="F163" s="10" t="inlineStr">
         <is>
           <t>Yes - (Remote) Sr Account Executive (26 Locations)</t>
         </is>
@@ -29510,7 +29510,7 @@
           <t>Free search marketplace for cooperative contracts (formerly CoProcure)</t>
         </is>
       </c>
-      <c r="F167" s="11" t="inlineStr">
+      <c r="F167" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -29630,7 +29630,7 @@
           <t>Electronic billing and payments for local government and utilities - exhibited at GFOA 2026</t>
         </is>
       </c>
-      <c r="F171" s="9" t="inlineStr">
+      <c r="F171" s="10" t="inlineStr">
         <is>
           <t>Yes - Mid Market Account Executive (Boston, MA)</t>
         </is>
@@ -30050,9 +30050,9 @@
           <t>Source-to-pay eProcurement suite with dedicated public sector and higher-ed verticals - exhibited at NACUBO 2026, GFOA 2026</t>
         </is>
       </c>
-      <c r="F185" s="9" t="inlineStr">
-        <is>
-          <t>Yes - Strategic Account Manager (Remote)</t>
+      <c r="F185" s="10" t="inlineStr">
+        <is>
+          <t>Yes - Account Executive/Enterprise Accou</t>
         </is>
       </c>
     </row>
@@ -30110,7 +30110,7 @@
           <t>Supplier ratings and performance reviews platform for public-sector buyers</t>
         </is>
       </c>
-      <c r="F187" s="11" t="inlineStr">
+      <c r="F187" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -30290,7 +30290,7 @@
           <t>AI-native ConcourseOS: procurement, permitting, courts, and billing across 450+ agencies (Bessemer-backed) - exhibited at NIGP 2026</t>
         </is>
       </c>
-      <c r="F193" s="11" t="inlineStr">
+      <c r="F193" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Founding GTM Engineer only</t>
         </is>
@@ -30468,7 +30468,7 @@
           <t>AI public-sector GTM intelligence: buying signals from gov/school board meetings, budgets, RFPs - sold to vendors selling to gov</t>
         </is>
       </c>
-      <c r="F199" s="9" t="inlineStr">
+      <c r="F199" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Executive - Mid Market (United States)</t>
         </is>
@@ -30578,7 +30578,7 @@
           <t>EProcurement and bid notification platforms for North American public buyers</t>
         </is>
       </c>
-      <c r="F203" s="9" t="inlineStr">
+      <c r="F203" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Executive (United States)</t>
         </is>
@@ -30844,7 +30844,7 @@
       </c>
       <c r="F212" s="22" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (London)</t>
+          <t>Yes - Account Executive (Singapore, Singapo)</t>
         </is>
       </c>
     </row>
@@ -30932,7 +30932,7 @@
           <t>Contract lifecycle management with FedRAMP and state/local government customers</t>
         </is>
       </c>
-      <c r="F215" s="9" t="inlineStr">
+      <c r="F215" s="10" t="inlineStr">
         <is>
           <t>Yes - Enterprise Account Executive (United States)</t>
         </is>
@@ -31352,7 +31352,7 @@
           <t>Cash and digital payments for child support, tolls and government billers</t>
         </is>
       </c>
-      <c r="F229" s="9" t="inlineStr">
+      <c r="F229" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Executive (Credit Unions/B (Remote)</t>
         </is>
@@ -31524,7 +31524,7 @@
           <t>Bill payment kiosks, portals, mobile apps and IVR for municipal agencies and utilities collecting resident payments - exhibited at GFOA 2026</t>
         </is>
       </c>
-      <c r="F235" s="9" t="inlineStr">
+      <c r="F235" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -31884,7 +31884,7 @@
           <t>Earned wage access platform for employers - exhibited at NACo 2026</t>
         </is>
       </c>
-      <c r="F247" s="9" t="inlineStr">
+      <c r="F247" s="10" t="inlineStr">
         <is>
           <t>Yes - Business Development Manager (NYC Headquarters)</t>
         </is>
@@ -31994,7 +31994,7 @@
           <t>Payroll and HR software - exhibited at AB Show 2026</t>
         </is>
       </c>
-      <c r="F251" s="9" t="inlineStr">
+      <c r="F251" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -32114,7 +32114,7 @@
           <t>Pension, unemployment insurance and workforce systems for state agencies - exhibited at SNA ANC 2027</t>
         </is>
       </c>
-      <c r="F255" s="9" t="inlineStr">
+      <c r="F255" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -32174,7 +32174,7 @@
           <t>Employee benefits, enrollment and HR services for public sector employers</t>
         </is>
       </c>
-      <c r="F257" s="9" t="inlineStr">
+      <c r="F257" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Manager (Denver, Colorado)</t>
         </is>
@@ -32472,7 +32472,7 @@
           <t>Document-driven workflow for government procurement, budget and HR processes</t>
         </is>
       </c>
-      <c r="F267" s="11" t="inlineStr">
+      <c r="F267" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Customer Success Manager only</t>
         </is>
@@ -33178,7 +33178,7 @@
           <t>Deathcare technology suite including cemetery and memorial management software</t>
         </is>
       </c>
-      <c r="F291" s="11" t="inlineStr">
+      <c r="F291" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -33520,7 +33520,7 @@
           <t>Endpoint management and security platform - exhibited at NACo 2026, NASCIO 2026, EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F303" s="11" t="inlineStr">
+      <c r="F303" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Business Analyst - Salesforce only</t>
         </is>
@@ -33580,7 +33580,7 @@
           <t>ChatGPT and the API, sold to public sector including named state and local government roles</t>
         </is>
       </c>
-      <c r="F305" s="11" t="inlineStr">
+      <c r="F305" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Account Director, Large Enterprise only</t>
         </is>
@@ -33858,7 +33858,7 @@
           <t>Strategic plan and KPI reporting (balanced scorecard) for local governments and enterprises</t>
         </is>
       </c>
-      <c r="F315" s="9" t="inlineStr">
+      <c r="F315" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -34910,7 +34910,7 @@
           <t>Open-source voting systems and risk-limiting audit tools for election offices</t>
         </is>
       </c>
-      <c r="F351" s="9" t="inlineStr">
+      <c r="F351" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Executive, Field Sales (United States)</t>
         </is>
@@ -37450,7 +37450,7 @@
           <t>Planning, budgeting and forecasting software - exhibited at ICMA 2025, NACUBO 2026, GFOA 2026</t>
         </is>
       </c>
-      <c r="F441" s="11" t="inlineStr">
+      <c r="F441" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -37558,7 +37558,7 @@
           <t>Purchasing card audit and compliance monitoring - exhibited at NIGP 2026</t>
         </is>
       </c>
-      <c r="F445" s="9" t="inlineStr">
+      <c r="F445" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -38356,7 +38356,7 @@
           <t>CRM and case management cloud software - exhibited at NACo 2026, NIGP 2026, NASWA 2025, NASCIO 2026, APHSA 2026, NatCon 2026, EDUCAUSE 2026, Healthcare IT Connect 2026, MESC 2026</t>
         </is>
       </c>
-      <c r="F477" s="9" t="inlineStr">
+      <c r="F477" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -38708,7 +38708,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/22/26)</t>
+          <t>Hiring AEs? (9/23/26)</t>
         </is>
       </c>
     </row>
@@ -38766,7 +38766,7 @@
           <t>Parks &amp; rec program management and booking platform founded by early Uber employees</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="F3" s="10" t="inlineStr">
         <is>
           <t>Yes - Enterprise Account Executive (San Francisco, CA)</t>
         </is>
@@ -39120,7 +39120,7 @@
           <t>Parks and recreation management software; brands NextRec (formerly PerfectMind), Vermont Systems, RecDesk and ePACT - exhibited at AB Show 2026, NRPA 2026</t>
         </is>
       </c>
-      <c r="F15" s="9" t="inlineStr">
+      <c r="F15" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Executive (Shreveport, LA)</t>
         </is>
@@ -39360,9 +39360,9 @@
           <t>Team and league management apps for youth sports, with a business tier for rec orgs</t>
         </is>
       </c>
-      <c r="F23" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>Yes - Account Manager, Large Market (Remote)</t>
         </is>
       </c>
     </row>
@@ -39840,7 +39840,7 @@
           <t>Club and league management platform for youth soccer organizations</t>
         </is>
       </c>
-      <c r="F39" s="9" t="inlineStr">
+      <c r="F39" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -40200,7 +40200,7 @@
           <t>Campground, park and license reservation systems for state park agencies</t>
         </is>
       </c>
-      <c r="F51" s="11" t="inlineStr">
+      <c r="F51" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Platform Solutions Engineer only</t>
         </is>
@@ -40260,7 +40260,7 @@
           <t>Campground reservation and management software for public and private campgrounds</t>
         </is>
       </c>
-      <c r="F53" s="11" t="inlineStr">
+      <c r="F53" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Manager, Account Management only</t>
         </is>
@@ -40556,7 +40556,7 @@
           <t>Sports facility and program management for municipal and community facilities</t>
         </is>
       </c>
-      <c r="F63" s="11" t="inlineStr">
+      <c r="F63" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -40676,7 +40676,7 @@
           <t>AI drowning-detection and lifeguard assist for public aquatic centers</t>
         </is>
       </c>
-      <c r="F67" s="11" t="inlineStr">
+      <c r="F67" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -40856,7 +40856,7 @@
           <t>Central irrigation control and smart controllers for municipal parks</t>
         </is>
       </c>
-      <c r="F73" s="9" t="inlineStr">
+      <c r="F73" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -41396,7 +41396,7 @@
           <t>Weather safety platform: WBGT heat monitoring, lightning alerts, stations and sirens for parks and athletics</t>
         </is>
       </c>
-      <c r="F91" s="9" t="inlineStr">
+      <c r="F91" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Executive, SLED (Perry Weather Offi)</t>
         </is>
@@ -42054,7 +42054,7 @@
           <t>Short-term rental market data for tourism offices and city agencies</t>
         </is>
       </c>
-      <c r="F113" s="9" t="inlineStr">
+      <c r="F113" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Manager (Barcelona)</t>
         </is>
@@ -42294,7 +42294,7 @@
           <t>Event management SaaS: vendor applications, ticketing, maps, and sponsors for festivals and city events</t>
         </is>
       </c>
-      <c r="F121" s="9" t="inlineStr">
+      <c r="F121" s="10" t="inlineStr">
         <is>
           <t>Yes - Enterprise Account Executive</t>
         </is>
@@ -42354,7 +42354,7 @@
           <t>Venue and event management for convention centers and public authorities</t>
         </is>
       </c>
-      <c r="F123" s="11" t="inlineStr">
+      <c r="F123" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Director of Solutions Engineering only</t>
         </is>
@@ -42534,7 +42534,7 @@
           <t>Venue management, ticketing and POS for aquatic centers and attractions</t>
         </is>
       </c>
-      <c r="F129" s="9" t="inlineStr">
+      <c r="F129" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Executive - Mid-Market and (London, United Kin)</t>
         </is>
@@ -42772,7 +42772,7 @@
           <t>Event volunteer scheduling and check-in for festivals and public events</t>
         </is>
       </c>
-      <c r="F137" s="9" t="inlineStr">
+      <c r="F137" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Executive Level 2 (Remote, US)</t>
         </is>
@@ -42990,7 +42990,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/22/26)</t>
+          <t>Hiring AEs? (9/23/26)</t>
         </is>
       </c>
     </row>
@@ -43048,7 +43048,7 @@
           <t>CrisisAlert wearable panic buttons for school staff; 18M+ people covered</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="F3" s="10" t="inlineStr">
         <is>
           <t>Yes - Sales Executive - Pacific Northwes (Remote Worker - N/)</t>
         </is>
@@ -43168,7 +43168,7 @@
           <t>Device filtering, classroom management, and student wellness (Beacon)</t>
         </is>
       </c>
-      <c r="F7" s="11" t="inlineStr">
+      <c r="F7" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - New Business Executive - Strategic only</t>
         </is>
@@ -43702,7 +43702,7 @@
           <t>AI weapons detection and screening for schools and public buildings</t>
         </is>
       </c>
-      <c r="F25" s="9" t="inlineStr">
+      <c r="F25" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -43880,7 +43880,7 @@
           <t>InformaCast mass notification and paging for school districts</t>
         </is>
       </c>
-      <c r="F31" s="9" t="inlineStr">
+      <c r="F31" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -44292,7 +44292,7 @@
           <t>School bus telematics, electronic inspections, and ridership tracking</t>
         </is>
       </c>
-      <c r="F45" s="9" t="inlineStr">
+      <c r="F45" s="10" t="inlineStr">
         <is>
           <t>Yes - Sales Account Executive – Mid-Mark</t>
         </is>
@@ -45012,7 +45012,7 @@
           <t>Unified school-home communication platform - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F69" s="11" t="inlineStr">
+      <c r="F69" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -45132,7 +45132,7 @@
           <t>Capital program management and purchasing/AP compliance for 140+ California districts</t>
         </is>
       </c>
-      <c r="F73" s="9" t="inlineStr">
+      <c r="F73" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -45550,7 +45550,7 @@
           <t>Alternative student transportation for school districts (formerly ALC Schools): contracted vehicles and drivers for students a yellow bus cannot serve, with dispatch and tracking for the district - exhibited at NAPT Summit 2026</t>
         </is>
       </c>
-      <c r="F87" s="9" t="inlineStr">
+      <c r="F87" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Executive, Southern Califo (Remote Southern Ca)</t>
         </is>
@@ -45670,7 +45670,7 @@
           <t>School and district websites, apps and communications for public schools</t>
         </is>
       </c>
-      <c r="F91" s="9" t="inlineStr">
+      <c r="F91" s="10" t="inlineStr">
         <is>
           <t>Yes - Sales Executive (Remote Worker - N/)</t>
         </is>
@@ -45910,7 +45910,7 @@
           <t>Dismissal, attendance and school safety workflow platform for districts</t>
         </is>
       </c>
-      <c r="F99" s="9" t="inlineStr">
+      <c r="F99" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -45970,9 +45970,9 @@
           <t>Single sign-on, rostering and usage analytics for public school districts - exhibited at CoSN 2026, EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F101" s="9" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F101" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -46136,7 +46136,7 @@
           <t>Digital hall pass, tardy tracking, behavior management, and campus engagement platform for K-12 schools and districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F107" s="9" t="inlineStr">
+      <c r="F107" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Manager (INTERNAL APPLICAN</t>
         </is>
@@ -46198,7 +46198,7 @@
       </c>
       <c r="F109" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 404 for https://boards-api.greenhou</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -46528,7 +46528,7 @@
           <t>Classroom browser monitoring, web filtering and student wellbeing alerting software for K-12 schools and districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F121" s="9" t="inlineStr">
+      <c r="F121" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -46642,7 +46642,7 @@
           <t>Student survey, MTSS, behavior analytics and early-warning software for K-12 school districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F125" s="9" t="inlineStr">
+      <c r="F125" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -46806,7 +46806,7 @@
           <t>Phone-free school software that blocks distracting apps during class and records attendance for K-12 districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F131" s="9" t="inlineStr">
+      <c r="F131" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -46972,7 +46972,7 @@
           <t>AI service desk and service operations platform unifying IT, facilities, HR and transportation requests for K-12 districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F137" s="9" t="inlineStr">
+      <c r="F137" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -47086,7 +47086,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/22/26)</t>
+          <t>Hiring AEs? (9/23/26)</t>
         </is>
       </c>
     </row>
@@ -47116,7 +47116,7 @@
       </c>
       <c r="F2" s="39" t="inlineStr">
         <is>
-          <t>Yes - Account Manager - East Coast (2 Locations)</t>
+          <t>Unknown - HTTP 520 for https://cubic.wd1.myworkday</t>
         </is>
       </c>
     </row>
@@ -47144,7 +47144,7 @@
           <t>Justride fare payments SaaS used by hundreds of agencies</t>
         </is>
       </c>
-      <c r="F3" s="11" t="inlineStr">
+      <c r="F3" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Customer Success Manager - UK only</t>
         </is>
@@ -47174,7 +47174,7 @@
           <t>Mobile fare payment app covering 200+ North American agencies</t>
         </is>
       </c>
-      <c r="F4" s="40" t="inlineStr">
+      <c r="F4" s="39" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -47234,7 +47234,7 @@
           <t>Automated fare collection plus parking and rail signalling systems (US office Lowell, MA)</t>
         </is>
       </c>
-      <c r="F6" s="40" t="inlineStr">
+      <c r="F6" s="39" t="inlineStr">
         <is>
           <t>Unknown - HTTP 404 for https://www.scheidt-bachman</t>
         </is>
@@ -47294,7 +47294,7 @@
           <t>Account-based ticketing and open-loop EMV fare collection in 150+ cities (BPC Group)</t>
         </is>
       </c>
-      <c r="F8" s="40" t="inlineStr">
+      <c r="F8" s="39" t="inlineStr">
         <is>
           <t>Unknown - board is another company's - not read</t>
         </is>
@@ -47354,7 +47354,7 @@
           <t>KubaPay cloud fare collection and account-based ticketing in 500+ cities (ICM group, not Cubic)</t>
         </is>
       </c>
-      <c r="F10" s="40" t="inlineStr">
+      <c r="F10" s="39" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -47414,7 +47414,7 @@
           <t>Automated fare collection and tolling/ITS for US agencies (LA, Bay Area, DC); Samsung SDS lineage</t>
         </is>
       </c>
-      <c r="F12" s="40" t="inlineStr">
+      <c r="F12" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -47472,7 +47472,7 @@
           <t>Fareboxes, validators, and the Universal Platform for automated fare management</t>
         </is>
       </c>
-      <c r="F14" s="40" t="inlineStr">
+      <c r="F14" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -47530,7 +47530,7 @@
           <t>Transit scheduling, fare and paratransit software for public operators</t>
         </is>
       </c>
-      <c r="F16" s="40" t="inlineStr">
+      <c r="F16" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -47590,7 +47590,7 @@
           <t>Tolling operations and back-office payment services for toll agencies</t>
         </is>
       </c>
-      <c r="F18" s="40" t="inlineStr">
+      <c r="F18" s="39" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -47620,7 +47620,7 @@
           <t>Check-in/be-out mobile fare payment for public transport authorities</t>
         </is>
       </c>
-      <c r="F19" s="9" t="inlineStr">
+      <c r="F19" s="10" t="inlineStr">
         <is>
           <t>Yes - Sales &amp; Business Development Manag</t>
         </is>
@@ -47650,7 +47650,7 @@
           <t>Account-based fare collection and validators for public transit operators</t>
         </is>
       </c>
-      <c r="F20" s="39" t="inlineStr">
+      <c r="F20" s="40" t="inlineStr">
         <is>
           <t>Yes - Senior Enterprise Account Executiv (Spain, Spain)</t>
         </is>
@@ -47710,7 +47710,7 @@
           <t>Bus ITS: CAD/AVL, real-time passenger info, and fleet health</t>
         </is>
       </c>
-      <c r="F22" s="40" t="inlineStr">
+      <c r="F22" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -47770,7 +47770,7 @@
           <t>Real-time transit data: arrival predictions and on-time performance</t>
         </is>
       </c>
-      <c r="F24" s="39" t="inlineStr">
+      <c r="F24" s="40" t="inlineStr">
         <is>
           <t>Yes - Senior Account Manager (United States)</t>
         </is>
@@ -47830,7 +47830,7 @@
           <t>myAvail enterprise transit management ITS and CAD/AVL for mid-size US agencies</t>
         </is>
       </c>
-      <c r="F26" s="40" t="inlineStr">
+      <c r="F26" s="39" t="inlineStr">
         <is>
           <t>Unknown - HTTP 404 for https://availtec.com/career</t>
         </is>
@@ -47860,7 +47860,7 @@
           <t>HASTUS scheduling, run-cutting, and rostering for transit agencies and postal operators</t>
         </is>
       </c>
-      <c r="F27" s="11" t="inlineStr">
+      <c r="F27" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Director, Strategic Business Devel only</t>
         </is>
@@ -47890,7 +47890,7 @@
           <t>IVU.suite planning, scheduling, dispatch, and ticketing for transit and rail operators</t>
         </is>
       </c>
-      <c r="F28" s="40" t="inlineStr">
+      <c r="F28" s="39" t="inlineStr">
         <is>
           <t>Unknown - HTTP 404 for https://www.ivu.com/career</t>
         </is>
@@ -47920,7 +47920,7 @@
           <t>Holding group of ~34 transit software brands under Constellation (Trapeze, Vontas, TransTrack, TripSpark, TransLoc)</t>
         </is>
       </c>
-      <c r="F29" s="11" t="inlineStr">
+      <c r="F29" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Sales &amp; Marketing Director only</t>
         </is>
@@ -47950,7 +47950,7 @@
           <t>Transit dispatch, CAD/AVL, and communications software (Modaxo brand, ex-Trapeze ITS)</t>
         </is>
       </c>
-      <c r="F30" s="40" t="inlineStr">
+      <c r="F30" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -48010,7 +48010,7 @@
           <t>Consat Telematics real-time CAD/AVL, passenger info, and electromobility analytics (NA office Sudbury ON)</t>
         </is>
       </c>
-      <c r="F32" s="40" t="inlineStr">
+      <c r="F32" s="39" t="inlineStr">
         <is>
           <t>Unknown - HTTP 404 for https://www.consat.com/care</t>
         </is>
@@ -48070,7 +48070,7 @@
           <t>Transit performance data warehousing, BI, and automated NTD reporting (Modaxo brand) - exhibited at CTAA EXPO 2026</t>
         </is>
       </c>
-      <c r="F34" s="40" t="inlineStr">
+      <c r="F34" s="39" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -48124,7 +48124,7 @@
           <t>Cloud CAD/AVL and in-vehicle tech for transit agencies and campus systems (SDVOSB)</t>
         </is>
       </c>
-      <c r="F36" s="40" t="inlineStr">
+      <c r="F36" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -48154,7 +48154,7 @@
           <t>iMarq mobile asset maintenance and MRO platform for transit, rail, and fleets</t>
         </is>
       </c>
-      <c r="F37" s="9" t="inlineStr">
+      <c r="F37" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -48184,7 +48184,7 @@
           <t>IBM Maximo consulting plus Mobile Informer EAM for transit agencies, airports, and utilities</t>
         </is>
       </c>
-      <c r="F38" s="40" t="inlineStr">
+      <c r="F38" s="39" t="inlineStr">
         <is>
           <t>Unknown - HTTP 404 for https://www.interlocsolutio</t>
         </is>
@@ -48244,7 +48244,7 @@
           <t>Trainwise onboard train control/monitoring and Fleetwise wayside fleet management for transit</t>
         </is>
       </c>
-      <c r="F40" s="40" t="inlineStr">
+      <c r="F40" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -48304,7 +48304,7 @@
           <t>Rail terminal management, track inspection, and crew compliance for short lines and commuter rail</t>
         </is>
       </c>
-      <c r="F42" s="40" t="inlineStr">
+      <c r="F42" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -48334,7 +48334,7 @@
           <t>SCADA systems and the SentientQ automation platform for rail transit, LRT, and utilities</t>
         </is>
       </c>
-      <c r="F43" s="9" t="inlineStr">
+      <c r="F43" s="10" t="inlineStr">
         <is>
           <t>Yes - Business Development Manager</t>
         </is>
@@ -48364,7 +48364,7 @@
           <t>Ultra-wideband train positioning, worker protection, and ATP for transit agencies (NYC MTA)</t>
         </is>
       </c>
-      <c r="F44" s="40" t="inlineStr">
+      <c r="F44" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -48424,7 +48424,7 @@
           <t>CylusOne rail OT cybersecurity: threat detection for signaling, trackside, and onboard networks</t>
         </is>
       </c>
-      <c r="F46" s="40" t="inlineStr">
+      <c r="F46" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -48482,7 +48482,7 @@
           <t>ConnX Maestro unified communications and contact center for transit agencies (SEPTA)</t>
         </is>
       </c>
-      <c r="F48" s="40" t="inlineStr">
+      <c r="F48" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -48540,7 +48540,7 @@
           <t>Non-invasive sensors and cloud analytics for elevator, escalator, and HVAC uptime in transit stations</t>
         </is>
       </c>
-      <c r="F50" s="40" t="inlineStr">
+      <c r="F50" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -48598,7 +48598,7 @@
           <t>Virtual Optical Fiber high-speed data offload between transit vehicles and depots</t>
         </is>
       </c>
-      <c r="F52" s="40" t="inlineStr">
+      <c r="F52" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -48658,7 +48658,7 @@
           <t>AI smart inspection for rail infrastructure: sensor robot plus defect detection and predictive maintenance</t>
         </is>
       </c>
-      <c r="F54" s="40" t="inlineStr">
+      <c r="F54" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -48714,7 +48714,7 @@
           <t>Mobile video surveillance, DVRs, and MotoTrax analytics for transit, school, and municipal fleets - exhibited at CTAA EXPO 2026, NAPT Summit 2026</t>
         </is>
       </c>
-      <c r="F56" s="39" t="inlineStr">
+      <c r="F56" s="40" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -48774,7 +48774,7 @@
           <t>Onboard transit systems: Horizon CCTV, NetSpire passenger info, iConnex real-time (US in Buffalo NY)</t>
         </is>
       </c>
-      <c r="F58" s="40" t="inlineStr">
+      <c r="F58" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -48834,7 +48834,7 @@
           <t>Intelligent video, AI stop-arm analytics, and cloud safety platforms for transit and school districts - exhibited at CTAA EXPO 2026, NAPT Summit 2026</t>
         </is>
       </c>
-      <c r="F60" s="40" t="inlineStr">
+      <c r="F60" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -48894,7 +48894,7 @@
           <t>AI dashcams, MDVRs, and fleet video telematics for transit, school bus, and commercial fleets (US: Houston)</t>
         </is>
       </c>
-      <c r="F62" s="40" t="inlineStr">
+      <c r="F62" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -48954,7 +48954,7 @@
           <t>3D AI people-flow sensors for passenger counting, queue, and dwell in transit hubs and airports</t>
         </is>
       </c>
-      <c r="F64" s="40" t="inlineStr">
+      <c r="F64" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -49014,7 +49014,7 @@
           <t>Automatic passenger counting hardware and analysis software for bus, rail, and paratransit</t>
         </is>
       </c>
-      <c r="F66" s="40" t="inlineStr">
+      <c r="F66" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -49074,7 +49074,7 @@
           <t>Video telematics and driver safety for municipal and transit fleets - exhibited at SWANA WASTECON 2025</t>
         </is>
       </c>
-      <c r="F68" s="40" t="inlineStr">
+      <c r="F68" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -49104,7 +49104,7 @@
           <t>AI dashcam and driver coaching for public fleets</t>
         </is>
       </c>
-      <c r="F69" s="9" t="inlineStr">
+      <c r="F69" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Executive, Mid-Market (USA)</t>
         </is>
@@ -49134,7 +49134,7 @@
           <t>Telematics devices and fleet tracking software for public fleets</t>
         </is>
       </c>
-      <c r="F70" s="40" t="inlineStr">
+      <c r="F70" s="39" t="inlineStr">
         <is>
           <t>Unknown - no jobs parsed from iCIMS portal</t>
         </is>
@@ -49164,7 +49164,7 @@
           <t>Fleet maintenance software for cities, counties and transit agencies</t>
         </is>
       </c>
-      <c r="F71" s="9" t="inlineStr">
+      <c r="F71" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Executive (Remote Worker)</t>
         </is>
@@ -49194,7 +49194,7 @@
           <t>FleetWave fleet asset management for public sector fleets</t>
         </is>
       </c>
-      <c r="F72" s="40" t="inlineStr">
+      <c r="F72" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -49224,7 +49224,7 @@
           <t>Fleet maintenance management software for transit and government fleets</t>
         </is>
       </c>
-      <c r="F73" s="9" t="inlineStr">
+      <c r="F73" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -49254,7 +49254,7 @@
           <t>FleetCommander motor pool and vehicle sharing for agencies</t>
         </is>
       </c>
-      <c r="F74" s="40" t="inlineStr">
+      <c r="F74" s="39" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -49314,7 +49314,7 @@
           <t>Fleet data analytics and benchmarking for public and utility fleets</t>
         </is>
       </c>
-      <c r="F76" s="40" t="inlineStr">
+      <c r="F76" s="39" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -49344,7 +49344,7 @@
           <t>Digital vehicle inspections and maintenance for municipal fleets</t>
         </is>
       </c>
-      <c r="F77" s="11" t="inlineStr">
+      <c r="F77" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Operations Manager, Customer Succe only</t>
         </is>
@@ -49374,7 +49374,7 @@
           <t>Fleet automation and motor pool platform for public agencies</t>
         </is>
       </c>
-      <c r="F78" s="40" t="inlineStr">
+      <c r="F78" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -49434,7 +49434,7 @@
           <t>Onboard surveillance and video management for transit fleets</t>
         </is>
       </c>
-      <c r="F80" s="40" t="inlineStr">
+      <c r="F80" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -49554,7 +49554,7 @@
           <t>On-demand transit and shared mobility software for public agencies</t>
         </is>
       </c>
-      <c r="F84" s="40" t="inlineStr">
+      <c r="F84" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -49614,7 +49614,7 @@
           <t>Parking meters, kiosks and transit fare systems for cities</t>
         </is>
       </c>
-      <c r="F86" s="40" t="inlineStr">
+      <c r="F86" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -49674,7 +49674,7 @@
           <t>Mobile parking payments for city and municipal parking operators</t>
         </is>
       </c>
-      <c r="F88" s="39" t="inlineStr">
+      <c r="F88" s="40" t="inlineStr">
         <is>
           <t>Yes - Corporate Sales Executive</t>
         </is>
@@ -49734,7 +49734,7 @@
           <t>Parking access and revenue control systems for public garages</t>
         </is>
       </c>
-      <c r="F90" s="40" t="inlineStr">
+      <c r="F90" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -49794,7 +49794,7 @@
           <t>Automated enforcement: school-zone speed, red-light, and bus-lane cameras - exhibited at North Carolina Sheriffs' Association 2026</t>
         </is>
       </c>
-      <c r="F92" s="39" t="inlineStr">
+      <c r="F92" s="40" t="inlineStr">
         <is>
           <t>Yes - Mass Market Account Executive (Arizona_Remote)</t>
         </is>
@@ -49854,7 +49854,7 @@
           <t>Multimodal trip planning app plus a paid agency suite (white-label apps, sponsored Royale, rider data) - exhibited at CTAA EXPO 2026, NAPT Summit 2026</t>
         </is>
       </c>
-      <c r="F94" s="40" t="inlineStr">
+      <c r="F94" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -49884,7 +49884,7 @@
           <t>Solar e-paper real-time passenger information displays and cloud CMS for bus stops and stations</t>
         </is>
       </c>
-      <c r="F95" s="9" t="inlineStr">
+      <c r="F95" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -49914,7 +49914,7 @@
           <t>ePaper Digital Bus Stop, SmartStop kiosks, and CPAM content management for transit agencies</t>
         </is>
       </c>
-      <c r="F96" s="40" t="inlineStr">
+      <c r="F96" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -50034,7 +50034,7 @@
           <t>Bus destination displays, controllers, and next-stop passenger information systems</t>
         </is>
       </c>
-      <c r="F100" s="40" t="inlineStr">
+      <c r="F100" s="39" t="inlineStr">
         <is>
           <t>Unknown - HTTP 403 for https://www.hanoverdisplays</t>
         </is>
@@ -50092,7 +50092,7 @@
           <t>TRACC travel-time and accessibility analysis plus transport datasets for government transport agencies</t>
         </is>
       </c>
-      <c r="F102" s="40" t="inlineStr">
+      <c r="F102" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -50152,7 +50152,7 @@
           <t>Solar smart bus stops with edge AI plus the ORA platform: signage, lane enforcement, passenger counting</t>
         </is>
       </c>
-      <c r="F104" s="40" t="inlineStr">
+      <c r="F104" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -50212,7 +50212,7 @@
           <t>Real-time transit display screens and rider information for agencies and cities</t>
         </is>
       </c>
-      <c r="F106" s="40" t="inlineStr">
+      <c r="F106" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -50242,7 +50242,7 @@
           <t>On-demand transit, paratransit, and network planning software for agencies - exhibited at CTAA EXPO 2026</t>
         </is>
       </c>
-      <c r="F107" s="9" t="inlineStr">
+      <c r="F107" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Executive, Western Europe (Paris)</t>
         </is>
@@ -50272,7 +50272,7 @@
           <t>Elevated automated transit pods on prefabricated guideways (ex-skyTran team) for cities and campuses</t>
         </is>
       </c>
-      <c r="F108" s="40" t="inlineStr">
+      <c r="F108" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -50332,7 +50332,7 @@
           <t>On-demand microtransit software with rider/driver apps and AI dispatch for large agencies - exhibited at CTAA EXPO 2026</t>
         </is>
       </c>
-      <c r="F110" s="39" t="inlineStr">
+      <c r="F110" s="40" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -50392,7 +50392,7 @@
           <t>Assisted-mobility platform and driver network delivering ADA paratransit and door-through-door trips - exhibited at CTAA EXPO 2026</t>
         </is>
       </c>
-      <c r="F112" s="40" t="inlineStr">
+      <c r="F112" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -50452,7 +50452,7 @@
           <t>Transit management software for paratransit, demand-response, microtransit, and taxi fleets - exhibited at CTAA EXPO 2026</t>
         </is>
       </c>
-      <c r="F114" s="40" t="inlineStr">
+      <c r="F114" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -50512,7 +50512,7 @@
           <t>Autonomous vehicle technology and driverless shuttle service for transit agencies and cities</t>
         </is>
       </c>
-      <c r="F116" s="40" t="inlineStr">
+      <c r="F116" s="39" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -50542,9 +50542,9 @@
           <t>Turnkey autonomous shuttle operations for transit agencies, airports, and communities</t>
         </is>
       </c>
-      <c r="F117" s="11" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F117" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -50572,7 +50572,7 @@
           <t>flowride.ai SAE Level-4 automated driving software retrofitted onto full-size electric transit buses</t>
         </is>
       </c>
-      <c r="F118" s="40" t="inlineStr">
+      <c r="F118" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -50632,7 +50632,7 @@
           <t>Assisted senior and accessible transportation platform serving agency paratransit overflow in 35+ metros</t>
         </is>
       </c>
-      <c r="F120" s="40" t="inlineStr">
+      <c r="F120" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -50692,7 +50692,7 @@
           <t>White-label multimodal TDM and commute platform for regional agencies, employers, and campuses</t>
         </is>
       </c>
-      <c r="F122" s="40" t="inlineStr">
+      <c r="F122" s="39" t="inlineStr">
         <is>
           <t>Unknown - HTTP 404 for https://www.rideshark.com/c</t>
         </is>
@@ -50744,7 +50744,7 @@
           <t>TripMaster paratransit scheduling and dispatch software for public transit providers</t>
         </is>
       </c>
-      <c r="F124" s="40" t="inlineStr">
+      <c r="F124" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -50802,7 +50802,7 @@
           <t>Demand-responsive transit dispatch and booking software for transit agencies - exhibited at CTAA EXPO 2026</t>
         </is>
       </c>
-      <c r="F126" s="40" t="inlineStr">
+      <c r="F126" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -50862,7 +50862,7 @@
           <t>Electric on-demand shuttle service contracted by cities and transit agencies - exhibited at WEFTEC 2026</t>
         </is>
       </c>
-      <c r="F128" s="40" t="inlineStr">
+      <c r="F128" s="39" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -50922,7 +50922,7 @@
           <t>On-demand ridepooling and mobility analytics software for public transit authorities</t>
         </is>
       </c>
-      <c r="F130" s="40" t="inlineStr">
+      <c r="F130" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -50982,7 +50982,7 @@
           <t>Ridepooling operations and autonomous shuttle services for public transport partners</t>
         </is>
       </c>
-      <c r="F132" s="40" t="inlineStr">
+      <c r="F132" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51034,7 +51034,7 @@
           <t>ADA paratransit eligibility, call center and mobility management technology for agencies</t>
         </is>
       </c>
-      <c r="F134" s="40" t="inlineStr">
+      <c r="F134" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51094,7 +51094,7 @@
           <t>Whoosh autonomous cable-driven transit pods for cities and campuses</t>
         </is>
       </c>
-      <c r="F136" s="40" t="inlineStr">
+      <c r="F136" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51154,7 +51154,7 @@
           <t>Autonomous shuttle vehicles for public transport and campus deployments</t>
         </is>
       </c>
-      <c r="F138" s="40" t="inlineStr">
+      <c r="F138" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51214,7 +51214,7 @@
           <t>Electric and autonomous buses sold to public transit operators worldwide</t>
         </is>
       </c>
-      <c r="F140" s="40" t="inlineStr">
+      <c r="F140" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51274,7 +51274,7 @@
           <t>Automated people mover and group rapid transit systems for public authorities</t>
         </is>
       </c>
-      <c r="F142" s="40" t="inlineStr">
+      <c r="F142" s="39" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -51334,7 +51334,7 @@
           <t>Autonomy software powering driverless shuttles for transit and airport operators</t>
         </is>
       </c>
-      <c r="F144" s="40" t="inlineStr">
+      <c r="F144" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -51394,7 +51394,7 @@
           <t>Autonomous shuttles for public transport agencies, airports and campuses</t>
         </is>
       </c>
-      <c r="F146" s="40" t="inlineStr">
+      <c r="F146" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51454,7 +51454,7 @@
           <t>Leading mobile parking payments app (EasyPark Group)</t>
         </is>
       </c>
-      <c r="F148" s="40" t="inlineStr">
+      <c r="F148" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -51484,9 +51484,9 @@
           <t>Smart single-space parking meters and enforcement systems</t>
         </is>
       </c>
-      <c r="F149" s="11" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Sr. Client Success Manager only</t>
+      <c r="F149" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -51514,7 +51514,7 @@
           <t>Computer vision curb management and automated loading-zone payments</t>
         </is>
       </c>
-      <c r="F150" s="40" t="inlineStr">
+      <c r="F150" s="39" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -51574,7 +51574,7 @@
           <t>Gateless LPR parking operations (GLIDEPARCS) for private lots, universities, and some municipalities</t>
         </is>
       </c>
-      <c r="F152" s="40" t="inlineStr">
+      <c r="F152" s="39" t="inlineStr">
         <is>
           <t>Unknown - page too small - likely JS-rendered</t>
         </is>
@@ -51634,7 +51634,7 @@
           <t>Towing lifecycle software for city towing programs and impound management (ex-AutoReturn + TSD)</t>
         </is>
       </c>
-      <c r="F154" s="40" t="inlineStr">
+      <c r="F154" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -51664,7 +51664,7 @@
           <t>Parking permits, enforcement, PARCS, and pay stations for universities and cities (Verra Mobility)</t>
         </is>
       </c>
-      <c r="F155" s="9" t="inlineStr">
+      <c r="F155" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -51694,7 +51694,7 @@
           <t>Sentry solar smart kiosks and vision-based automated parking enforcement</t>
         </is>
       </c>
-      <c r="F156" s="40" t="inlineStr">
+      <c r="F156" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51724,7 +51724,7 @@
           <t>Mobility and curb/parking technology platform - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F157" s="9" t="inlineStr">
+      <c r="F157" s="10" t="inlineStr">
         <is>
           <t>Yes - Junior B2B Account Executive (Prague)</t>
         </is>
@@ -51754,7 +51754,7 @@
           <t>Single-space smart parking meters and pay stations for municipalities</t>
         </is>
       </c>
-      <c r="F158" s="40" t="inlineStr">
+      <c r="F158" s="39" t="inlineStr">
         <is>
           <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
@@ -51814,7 +51814,7 @@
           <t>Wireless parking occupancy sensors for city and campus parking</t>
         </is>
       </c>
-      <c r="F160" s="40" t="inlineStr">
+      <c r="F160" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51874,7 +51874,7 @@
           <t>Smart parking sensors and LoRaWAN networks for cities</t>
         </is>
       </c>
-      <c r="F162" s="40" t="inlineStr">
+      <c r="F162" s="39" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -51934,7 +51934,7 @@
           <t>Parking payments, permits and enforcement software for municipalities</t>
         </is>
       </c>
-      <c r="F164" s="40" t="inlineStr">
+      <c r="F164" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51994,7 +51994,7 @@
           <t>Parking citation processing and permit services for California cities</t>
         </is>
       </c>
-      <c r="F166" s="40" t="inlineStr">
+      <c r="F166" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52054,7 +52054,7 @@
           <t>Parking citation, permit and enforcement management software for agencies</t>
         </is>
       </c>
-      <c r="F168" s="40" t="inlineStr">
+      <c r="F168" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52110,7 +52110,7 @@
           <t>Control room video wall visualization software - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F170" s="40" t="inlineStr">
+      <c r="F170" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -52162,7 +52162,7 @@
           <t>Transit fare collection and ticketing software - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F172" s="40" t="inlineStr">
+      <c r="F172" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52210,7 +52210,7 @@
           <t>Infrastructure engineering and asset software - exhibited at APTA 2026, AWWA ACE 2026</t>
         </is>
       </c>
-      <c r="F174" s="40" t="inlineStr">
+      <c r="F174" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52262,7 +52262,7 @@
           <t>Fuel and fleet management systems - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F176" s="40" t="inlineStr">
+      <c r="F176" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -52312,7 +52312,7 @@
           <t>Transit ITS, fare collection, scheduling software - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F178" s="40" t="inlineStr">
+      <c r="F178" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52368,7 +52368,7 @@
           <t>Ticketing, traffic and transit management systems - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F180" s="40" t="inlineStr">
+      <c r="F180" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52392,7 +52392,7 @@
           <t>Security and intelligence analytics software - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F181" s="9" t="inlineStr">
+      <c r="F181" s="10" t="inlineStr">
         <is>
           <t>Yes - Enterprise Sales Executive – New L (2 Locations)</t>
         </is>
@@ -52416,7 +52416,7 @@
           <t>LiDAR 3D digital twin capture for transit - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F182" s="40" t="inlineStr">
+      <c r="F182" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52464,7 +52464,7 @@
           <t>Medical transportation ride management software - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F184" s="40" t="inlineStr">
+      <c r="F184" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52514,7 +52514,7 @@
           <t>AI video analytics perimeter security software - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F186" s="40" t="inlineStr">
+      <c r="F186" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -52562,7 +52562,7 @@
           <t>Transit CAD/AVL, APC, passenger information systems - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F188" s="40" t="inlineStr">
+      <c r="F188" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52586,7 +52586,7 @@
           <t>GPS fleet tracking and telematics software - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F189" s="9" t="inlineStr">
+      <c r="F189" s="10" t="inlineStr">
         <is>
           <t>Yes - Sales Account Executive – Mid-Mark</t>
         </is>
@@ -52616,7 +52616,7 @@
           <t>EV fleet charge management software - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F190" s="40" t="inlineStr">
+      <c r="F190" s="39" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -52664,7 +52664,7 @@
           <t>Immersive VR training software platform - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F192" s="40" t="inlineStr">
+      <c r="F192" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52728,7 +52728,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/22/26)</t>
+          <t>Hiring AEs? (9/23/26)</t>
         </is>
       </c>
     </row>
@@ -52846,7 +52846,7 @@
           <t>Autonomous off-grid solar streetlights with remote monitoring; 1,000+ municipalities, 43 states (French parent)</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
+      <c r="F5" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -53386,7 +53386,7 @@
           <t>Aluminum and steel lighting poles for municipal and DOT projects</t>
         </is>
       </c>
-      <c r="F23" s="9" t="inlineStr">
+      <c r="F23" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -53446,7 +53446,7 @@
           <t>Adaptive smart street lighting sensors and CMS for municipalities</t>
         </is>
       </c>
-      <c r="F25" s="11" t="inlineStr">
+      <c r="F25" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -53506,7 +53506,7 @@
           <t>Street lighting luminaires and connected controls for public authorities</t>
         </is>
       </c>
-      <c r="F27" s="9" t="inlineStr">
+      <c r="F27" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -53986,7 +53986,7 @@
           <t>Exterior LED site and streetscape lighting for public projects</t>
         </is>
       </c>
-      <c r="F43" s="9" t="inlineStr">
+      <c r="F43" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -54046,7 +54046,7 @@
           <t>Pole-mounted sensors + AI (Gridscope) detecting grid faults, vegetation strikes, and wildfire-risk events</t>
         </is>
       </c>
-      <c r="F45" s="11" t="inlineStr">
+      <c r="F45" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Customer Success Manager only</t>
         </is>
@@ -54106,7 +54106,7 @@
           <t>Satellite + AI vegetation management (IVMS) and climate/asset risk SaaS for utilities</t>
         </is>
       </c>
-      <c r="F47" s="11" t="inlineStr">
+      <c r="F47" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Business Analyst - Customer Succes only</t>
         </is>
@@ -54166,7 +54166,7 @@
           <t>EV ARC transportable solar EV charging and storage for government fleets (Nasdaq: BEEM; ex-Envision Solar)</t>
         </is>
       </c>
-      <c r="F49" s="9" t="inlineStr">
+      <c r="F49" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -54286,7 +54286,7 @@
           <t>Metering, CIS, billing and grid analytics for public power utilities</t>
         </is>
       </c>
-      <c r="F53" s="11" t="inlineStr">
+      <c r="F53" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -54438,7 +54438,7 @@
       </c>
       <c r="F58" s="45" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -54466,7 +54466,7 @@
           <t>Smart grid AMI and grid analytics for public power utilities and co-ops</t>
         </is>
       </c>
-      <c r="F59" s="11" t="inlineStr">
+      <c r="F59" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Office &amp; Sales Support Coordinator only</t>
         </is>
@@ -54706,7 +54706,7 @@
           <t>DERMS and virtual power plant programs for utilities including public power</t>
         </is>
       </c>
-      <c r="F67" s="11" t="inlineStr">
+      <c r="F67" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Sales Engineer only</t>
         </is>
@@ -54946,7 +54946,7 @@
           <t>Utility bill management and energy analytics for cities, counties and schools</t>
         </is>
       </c>
-      <c r="F75" s="9" t="inlineStr">
+      <c r="F75" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Executive</t>
         </is>
@@ -55184,7 +55184,7 @@
           <t>Outage notification, billing, and omnichannel customer communication platform for investor-owned, municipal, and cooperative utilities - exhibited at APPA Public Power 2026</t>
         </is>
       </c>
-      <c r="F83" s="9" t="inlineStr">
+      <c r="F83" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Executive (US - Remote)</t>
         </is>
@@ -55598,7 +55598,7 @@
           <t>Geospatial network design and field software for telecom and public utilities</t>
         </is>
       </c>
-      <c r="F97" s="11" t="inlineStr">
+      <c r="F97" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Sales Engineer only</t>
         </is>
@@ -55718,7 +55718,7 @@
           <t>Broadband grant, challenge process and mapping software for state broadband offices</t>
         </is>
       </c>
-      <c r="F101" s="11" t="inlineStr">
+      <c r="F101" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Product Solutions Engineer only</t>
         </is>
@@ -56194,7 +56194,7 @@
       </c>
       <c r="F117" s="7" t="inlineStr">
         <is>
-          <t>None found</t>
+          <t>Unknown - HTTP 404 for https://sifinetworks.com/co</t>
         </is>
       </c>
     </row>
@@ -56286,7 +56286,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/22/26)</t>
+          <t>Hiring AEs? (9/23/26)</t>
         </is>
       </c>
     </row>
@@ -56756,7 +56756,7 @@
           <t>Aviation design and simulation software (AviPLAN, AeroTURN, GuideSIGN) used by airport planners for aircraft movement, apron layout and airside safety analysis.</t>
         </is>
       </c>
-      <c r="F17" s="9" t="inlineStr">
+      <c r="F17" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Manager (Sales)</t>
         </is>
@@ -57172,7 +57172,7 @@
           <t>Airport weather observation systems and runway condition sensors for airports - exhibited at NACE 2026</t>
         </is>
       </c>
-      <c r="F31" s="9" t="inlineStr">
+      <c r="F31" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -57232,7 +57232,7 @@
           <t>Bird-strike avoidance radar and wildlife management systems for airports</t>
         </is>
       </c>
-      <c r="F33" s="11" t="inlineStr">
+      <c r="F33" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -57352,7 +57352,7 @@
           <t>ARINC airport systems portfolio: vMUSE common-use passenger processing, SelfPass biometrics, self bag drop, AODB/resource management, FIDS and airport communications sold to airport authorities.</t>
         </is>
       </c>
-      <c r="F37" s="11" t="inlineStr">
+      <c r="F37" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -57590,7 +57590,7 @@
           <t>Passenger flow, queue measurement and airport revenue software for airport operators</t>
         </is>
       </c>
-      <c r="F45" s="9" t="inlineStr">
+      <c r="F45" s="10" t="inlineStr">
         <is>
           <t>Yes - Sales Director Americas (US-based within th)</t>
         </is>
@@ -57710,7 +57710,7 @@
           <t>Gate, docking guidance and apron systems for airport operators</t>
         </is>
       </c>
-      <c r="F49" s="9" t="inlineStr">
+      <c r="F49" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -57890,7 +57890,7 @@
           <t>Self-service kiosks, bag drop and passenger processing for airports</t>
         </is>
       </c>
-      <c r="F55" s="9" t="inlineStr">
+      <c r="F55" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -58070,7 +58070,7 @@
           <t>Airport IQ operations, property and lease management software for airports</t>
         </is>
       </c>
-      <c r="F61" s="9" t="inlineStr">
+      <c r="F61" s="10" t="inlineStr">
         <is>
           <t>Yes - Senior Account Executive</t>
         </is>
@@ -58610,7 +58610,7 @@
           <t>Biometric identity, TSA PreCheck enrollment and airport boarding systems</t>
         </is>
       </c>
-      <c r="F79" s="9" t="inlineStr">
+      <c r="F79" s="10" t="inlineStr">
         <is>
           <t>Yes - Key Account Manager - Smart Biomet</t>
         </is>
@@ -58670,7 +58670,7 @@
           <t>Biometric identity lanes operated under airport and TSA agreements</t>
         </is>
       </c>
-      <c r="F81" s="9" t="inlineStr">
+      <c r="F81" s="10" t="inlineStr">
         <is>
           <t>Yes - Enterprise Account Executive (C1 - (New York, New York)</t>
         </is>
@@ -58790,7 +58790,7 @@
           <t>Perimeter intrusion detection and fence sensors for airports and utilities</t>
         </is>
       </c>
-      <c r="F85" s="9" t="inlineStr">
+      <c r="F85" s="10" t="inlineStr">
         <is>
           <t>Yes - Business Development Manager (Ottawa, Ontario, C)</t>
         </is>
@@ -59028,7 +59028,7 @@
           <t>Automated vehicle inspection portals for airports, borders and government</t>
         </is>
       </c>
-      <c r="F93" s="9" t="inlineStr">
+      <c r="F93" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -59148,7 +59148,7 @@
           <t>Computer-vision checkout-free parking payment platform (drive-in/drive-out billing) plus parking operations and revenue management for airports; owner of SP+.</t>
         </is>
       </c>
-      <c r="F97" s="9" t="inlineStr">
+      <c r="F97" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Manager (Remote USA)</t>
         </is>
@@ -59326,7 +59326,7 @@
           <t>Airport parking reservations and demand channel for airport operators</t>
         </is>
       </c>
-      <c r="F103" s="9" t="inlineStr">
+      <c r="F103" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -59386,7 +59386,7 @@
           <t>Full-service automated parking operations for cities and airports</t>
         </is>
       </c>
-      <c r="F105" s="11" t="inlineStr">
+      <c r="F105" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Sales Development Representative only</t>
         </is>
@@ -59506,7 +59506,7 @@
           <t>AVI readers and ground transportation management systems for airports</t>
         </is>
       </c>
-      <c r="F109" s="9" t="inlineStr">
+      <c r="F109" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -59746,7 +59746,7 @@
           <t>Web-based capital program and construction project management software (cost, contracts, documents, scheduling) used by airport owner-operators and public agencies.</t>
         </is>
       </c>
-      <c r="F117" s="9" t="inlineStr">
+      <c r="F117" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -59810,7 +59810,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/22/26)</t>
+          <t>Hiring AEs? (9/23/26)</t>
         </is>
       </c>
     </row>
@@ -60146,7 +60146,7 @@
           <t>Digital courtroom recording and speech recognition systems for courts</t>
         </is>
       </c>
-      <c r="F13" s="9" t="inlineStr">
+      <c r="F13" s="10" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -60264,7 +60264,7 @@
           <t>Criminal justice data collection and public dashboards for counties and states</t>
         </is>
       </c>
-      <c r="F17" s="11" t="inlineStr">
+      <c r="F17" s="9" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -60324,7 +60324,7 @@
           <t>Cloud ediscovery and litigation platform for law firms, corporations, county DAs, and state AGs - exhibited at IMLA 2026, NASCIO 2026</t>
         </is>
       </c>
-      <c r="F19" s="9" t="inlineStr">
+      <c r="F19" s="10" t="inlineStr">
         <is>
           <t>Yes - Enterprise Account Executive (Stat (United States)</t>
         </is>
@@ -60384,7 +60384,7 @@
           <t>PROSECUTORbyKarpel case management software for prosecutor offices - exhibited at IMLA 2026</t>
         </is>
       </c>
-      <c r="F21" s="9" t="inlineStr">
+      <c r="F21" s="10" t="inlineStr">
         <is>
           <t>Yes - Account Manager (Remote Worker - N/)</t>
         </is>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-09-25)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -296,8 +296,8 @@
     <xf numFmtId="1" fontId="2" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/23/26)</t>
+          <t>Hiring AEs? (9/25/26)</t>
         </is>
       </c>
     </row>
@@ -2100,9 +2100,9 @@
           <t>Autonomous drones for police DFR programs and public-sector inspection - exhibited at NLC City Summit 2026, IAFC FRI 2026</t>
         </is>
       </c>
-      <c r="F40" s="8" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F40" s="11" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2522,7 @@
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.365labs.com/car</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -3182,7 +3182,7 @@
       </c>
       <c r="F76" s="8" t="inlineStr">
         <is>
-          <t>Yes - Account Executive, Corporate Secur (2 Locations)</t>
+          <t>Yes - Account Executive, Federal Civilia (US Remote)</t>
         </is>
       </c>
     </row>
@@ -3330,9 +3330,9 @@
           <t>Drone-as-first-responder software and hardware auto-launching to 911 calls</t>
         </is>
       </c>
-      <c r="F81" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Account Executive</t>
+      <c r="F81" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -3482,7 +3482,7 @@
       </c>
       <c r="F86" s="8" t="inlineStr">
         <is>
-          <t>Yes - Associate Sales Executive (Waltham, MA)</t>
+          <t>Yes - Senior Sales Executive (2 Locations)</t>
         </is>
       </c>
     </row>
@@ -5774,7 +5774,7 @@
       </c>
       <c r="F164" s="4" t="inlineStr">
         <is>
-          <t>None found</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -6282,9 +6282,9 @@
           <t>Pediatric emergency dosing system and app for EMS agencies</t>
         </is>
       </c>
-      <c r="F181" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Enterprise Account Executive</t>
+      <c r="F181" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -11136,7 +11136,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/23/26)</t>
+          <t>Hiring AEs? (9/25/26)</t>
         </is>
       </c>
     </row>
@@ -11518,7 +11518,7 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 500 for https://company.getinsured.</t>
         </is>
       </c>
     </row>
@@ -12904,9 +12904,9 @@
           <t>Crisis response, closed-loop referral, care management, and bed board software for behavioral health agencies - exhibited at NatCon 2026</t>
         </is>
       </c>
-      <c r="F64" s="63" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F64" s="65" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - VP of Customer Success only</t>
         </is>
       </c>
     </row>
@@ -14420,7 +14420,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/23/26)</t>
+          <t>Hiring AEs? (9/25/26)</t>
         </is>
       </c>
     </row>
@@ -16386,7 +16386,7 @@
       </c>
       <c r="F72" s="70" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Vice President, Sales only</t>
+          <t>Sales (non-AE) - Senior Solutions Engineer only</t>
         </is>
       </c>
     </row>
@@ -16760,9 +16760,9 @@
           <t>Student billing, payments, net price calculator, and pre-collections software for colleges and universities - exhibited at NACUBO 2026</t>
         </is>
       </c>
-      <c r="F86" s="69" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F86" s="70" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Customer Success Manager only</t>
         </is>
       </c>
     </row>
@@ -17026,7 +17026,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/23/26)</t>
+          <t>Hiring AEs? (9/25/26)</t>
         </is>
       </c>
     </row>
@@ -17494,7 +17494,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/23/26)</t>
+          <t>Hiring AEs? (9/25/26)</t>
         </is>
       </c>
     </row>
@@ -20198,7 +20198,7 @@
       </c>
       <c r="F92" s="15" t="inlineStr">
         <is>
-          <t>None found</t>
+          <t>Unknown - non-JSON response</t>
         </is>
       </c>
     </row>
@@ -22712,7 +22712,7 @@
       </c>
       <c r="F177" s="10" t="inlineStr">
         <is>
-          <t>Yes - Enterprise Account Executive (US | Illinois | Ch)</t>
+          <t>Yes - Enterprise Account Executive (US | Massachusetts)</t>
         </is>
       </c>
     </row>
@@ -24624,7 +24624,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/23/26)</t>
+          <t>Hiring AEs? (9/25/26)</t>
         </is>
       </c>
     </row>
@@ -24684,7 +24684,7 @@
       </c>
       <c r="F3" s="10" t="inlineStr">
         <is>
-          <t>Yes - Local Government Account Executive</t>
+          <t>Yes - Enterprise Account Executive - Col</t>
         </is>
       </c>
     </row>
@@ -26690,9 +26690,9 @@
           <t>Social media management, listening, archiving and community engagement platform built for government communications teams - exhibited at 3CMA 2026</t>
         </is>
       </c>
-      <c r="F71" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F71" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -26858,9 +26858,9 @@
           <t>Permitting, licensing, and code enforcement platform for state and local government - exhibited at NLC City Summit 2026</t>
         </is>
       </c>
-      <c r="F77" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Account Executive (Remote Based - US)</t>
+      <c r="F77" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Business Development Representativ only</t>
         </is>
       </c>
     </row>
@@ -26890,7 +26890,7 @@
       </c>
       <c r="F78" s="22" t="inlineStr">
         <is>
-          <t>Yes - Enterprise Account Executive (US | Illinois | Ch)</t>
+          <t>Yes - Enterprise Account Executive (US | Massachusetts)</t>
         </is>
       </c>
     </row>
@@ -30844,7 +30844,7 @@
       </c>
       <c r="F212" s="22" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (Singapore, Singapo)</t>
+          <t>Yes - Account Executive (London)</t>
         </is>
       </c>
     </row>
@@ -35212,7 +35212,7 @@
       </c>
       <c r="F361" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 404 for https://www.easyvotesolutio</t>
         </is>
       </c>
     </row>
@@ -36530,9 +36530,9 @@
           <t>Research databases, ebook collections and discovery software licensed to public libraries, academic libraries, schools and healthcare organizations - exhibited at PLA 2026</t>
         </is>
       </c>
-      <c r="F408" s="23" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Customer Account Specialist, FOLIO only</t>
+      <c r="F408" s="22" t="inlineStr">
+        <is>
+          <t>Yes - Regional Sales Manager, K12 &amp; Publ</t>
         </is>
       </c>
     </row>
@@ -38708,7 +38708,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/23/26)</t>
+          <t>Hiring AEs? (9/25/26)</t>
         </is>
       </c>
     </row>
@@ -42536,7 +42536,7 @@
       </c>
       <c r="F129" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Executive - Mid-Market and (London, United Kin)</t>
+          <t>Yes - Enterprise Account Executive - AME (Austin, Texas)</t>
         </is>
       </c>
     </row>
@@ -42990,7 +42990,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/23/26)</t>
+          <t>Hiring AEs? (9/25/26)</t>
         </is>
       </c>
     </row>
@@ -43880,9 +43880,9 @@
           <t>InformaCast mass notification and paging for school districts</t>
         </is>
       </c>
-      <c r="F31" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -47086,7 +47086,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/23/26)</t>
+          <t>Hiring AEs? (9/25/26)</t>
         </is>
       </c>
     </row>
@@ -47116,7 +47116,7 @@
       </c>
       <c r="F2" s="39" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 520 for https://cubic.wd1.myworkday</t>
+          <t>Yes - Account Manager - East Coast (2 Locations)</t>
         </is>
       </c>
     </row>
@@ -47174,7 +47174,7 @@
           <t>Mobile fare payment app covering 200+ North American agencies</t>
         </is>
       </c>
-      <c r="F4" s="39" t="inlineStr">
+      <c r="F4" s="40" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -47234,7 +47234,7 @@
           <t>Automated fare collection plus parking and rail signalling systems (US office Lowell, MA)</t>
         </is>
       </c>
-      <c r="F6" s="39" t="inlineStr">
+      <c r="F6" s="40" t="inlineStr">
         <is>
           <t>Unknown - HTTP 404 for https://www.scheidt-bachman</t>
         </is>
@@ -47294,7 +47294,7 @@
           <t>Account-based ticketing and open-loop EMV fare collection in 150+ cities (BPC Group)</t>
         </is>
       </c>
-      <c r="F8" s="39" t="inlineStr">
+      <c r="F8" s="40" t="inlineStr">
         <is>
           <t>Unknown - board is another company's - not read</t>
         </is>
@@ -47354,7 +47354,7 @@
           <t>KubaPay cloud fare collection and account-based ticketing in 500+ cities (ICM group, not Cubic)</t>
         </is>
       </c>
-      <c r="F10" s="39" t="inlineStr">
+      <c r="F10" s="40" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -47414,7 +47414,7 @@
           <t>Automated fare collection and tolling/ITS for US agencies (LA, Bay Area, DC); Samsung SDS lineage</t>
         </is>
       </c>
-      <c r="F12" s="39" t="inlineStr">
+      <c r="F12" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -47472,7 +47472,7 @@
           <t>Fareboxes, validators, and the Universal Platform for automated fare management</t>
         </is>
       </c>
-      <c r="F14" s="39" t="inlineStr">
+      <c r="F14" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -47502,7 +47502,7 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -47530,7 +47530,7 @@
           <t>Transit scheduling, fare and paratransit software for public operators</t>
         </is>
       </c>
-      <c r="F16" s="39" t="inlineStr">
+      <c r="F16" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -47590,7 +47590,7 @@
           <t>Tolling operations and back-office payment services for toll agencies</t>
         </is>
       </c>
-      <c r="F18" s="39" t="inlineStr">
+      <c r="F18" s="40" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -47650,7 +47650,7 @@
           <t>Account-based fare collection and validators for public transit operators</t>
         </is>
       </c>
-      <c r="F20" s="40" t="inlineStr">
+      <c r="F20" s="39" t="inlineStr">
         <is>
           <t>Yes - Senior Enterprise Account Executiv (Spain, Spain)</t>
         </is>
@@ -47710,7 +47710,7 @@
           <t>Bus ITS: CAD/AVL, real-time passenger info, and fleet health</t>
         </is>
       </c>
-      <c r="F22" s="39" t="inlineStr">
+      <c r="F22" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -47770,7 +47770,7 @@
           <t>Real-time transit data: arrival predictions and on-time performance</t>
         </is>
       </c>
-      <c r="F24" s="40" t="inlineStr">
+      <c r="F24" s="39" t="inlineStr">
         <is>
           <t>Yes - Senior Account Manager (United States)</t>
         </is>
@@ -47830,7 +47830,7 @@
           <t>myAvail enterprise transit management ITS and CAD/AVL for mid-size US agencies</t>
         </is>
       </c>
-      <c r="F26" s="39" t="inlineStr">
+      <c r="F26" s="40" t="inlineStr">
         <is>
           <t>Unknown - HTTP 404 for https://availtec.com/career</t>
         </is>
@@ -47890,7 +47890,7 @@
           <t>IVU.suite planning, scheduling, dispatch, and ticketing for transit and rail operators</t>
         </is>
       </c>
-      <c r="F28" s="39" t="inlineStr">
+      <c r="F28" s="40" t="inlineStr">
         <is>
           <t>Unknown - HTTP 404 for https://www.ivu.com/career</t>
         </is>
@@ -47950,7 +47950,7 @@
           <t>Transit dispatch, CAD/AVL, and communications software (Modaxo brand, ex-Trapeze ITS)</t>
         </is>
       </c>
-      <c r="F30" s="39" t="inlineStr">
+      <c r="F30" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -48010,7 +48010,7 @@
           <t>Consat Telematics real-time CAD/AVL, passenger info, and electromobility analytics (NA office Sudbury ON)</t>
         </is>
       </c>
-      <c r="F32" s="39" t="inlineStr">
+      <c r="F32" s="40" t="inlineStr">
         <is>
           <t>Unknown - HTTP 404 for https://www.consat.com/care</t>
         </is>
@@ -48070,7 +48070,7 @@
           <t>Transit performance data warehousing, BI, and automated NTD reporting (Modaxo brand) - exhibited at CTAA EXPO 2026</t>
         </is>
       </c>
-      <c r="F34" s="39" t="inlineStr">
+      <c r="F34" s="40" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -48124,7 +48124,7 @@
           <t>Cloud CAD/AVL and in-vehicle tech for transit agencies and campus systems (SDVOSB)</t>
         </is>
       </c>
-      <c r="F36" s="39" t="inlineStr">
+      <c r="F36" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -48184,7 +48184,7 @@
           <t>IBM Maximo consulting plus Mobile Informer EAM for transit agencies, airports, and utilities</t>
         </is>
       </c>
-      <c r="F38" s="39" t="inlineStr">
+      <c r="F38" s="40" t="inlineStr">
         <is>
           <t>Unknown - HTTP 404 for https://www.interlocsolutio</t>
         </is>
@@ -48244,7 +48244,7 @@
           <t>Trainwise onboard train control/monitoring and Fleetwise wayside fleet management for transit</t>
         </is>
       </c>
-      <c r="F40" s="39" t="inlineStr">
+      <c r="F40" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -48304,7 +48304,7 @@
           <t>Rail terminal management, track inspection, and crew compliance for short lines and commuter rail</t>
         </is>
       </c>
-      <c r="F42" s="39" t="inlineStr">
+      <c r="F42" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -48364,7 +48364,7 @@
           <t>Ultra-wideband train positioning, worker protection, and ATP for transit agencies (NYC MTA)</t>
         </is>
       </c>
-      <c r="F44" s="39" t="inlineStr">
+      <c r="F44" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -48424,7 +48424,7 @@
           <t>CylusOne rail OT cybersecurity: threat detection for signaling, trackside, and onboard networks</t>
         </is>
       </c>
-      <c r="F46" s="39" t="inlineStr">
+      <c r="F46" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -48482,7 +48482,7 @@
           <t>ConnX Maestro unified communications and contact center for transit agencies (SEPTA)</t>
         </is>
       </c>
-      <c r="F48" s="39" t="inlineStr">
+      <c r="F48" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -48540,7 +48540,7 @@
           <t>Non-invasive sensors and cloud analytics for elevator, escalator, and HVAC uptime in transit stations</t>
         </is>
       </c>
-      <c r="F50" s="39" t="inlineStr">
+      <c r="F50" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -48598,7 +48598,7 @@
           <t>Virtual Optical Fiber high-speed data offload between transit vehicles and depots</t>
         </is>
       </c>
-      <c r="F52" s="39" t="inlineStr">
+      <c r="F52" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -48658,7 +48658,7 @@
           <t>AI smart inspection for rail infrastructure: sensor robot plus defect detection and predictive maintenance</t>
         </is>
       </c>
-      <c r="F54" s="39" t="inlineStr">
+      <c r="F54" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -48714,7 +48714,7 @@
           <t>Mobile video surveillance, DVRs, and MotoTrax analytics for transit, school, and municipal fleets - exhibited at CTAA EXPO 2026, NAPT Summit 2026</t>
         </is>
       </c>
-      <c r="F56" s="40" t="inlineStr">
+      <c r="F56" s="39" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -48774,7 +48774,7 @@
           <t>Onboard transit systems: Horizon CCTV, NetSpire passenger info, iConnex real-time (US in Buffalo NY)</t>
         </is>
       </c>
-      <c r="F58" s="39" t="inlineStr">
+      <c r="F58" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -48834,7 +48834,7 @@
           <t>Intelligent video, AI stop-arm analytics, and cloud safety platforms for transit and school districts - exhibited at CTAA EXPO 2026, NAPT Summit 2026</t>
         </is>
       </c>
-      <c r="F60" s="39" t="inlineStr">
+      <c r="F60" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -48894,7 +48894,7 @@
           <t>AI dashcams, MDVRs, and fleet video telematics for transit, school bus, and commercial fleets (US: Houston)</t>
         </is>
       </c>
-      <c r="F62" s="39" t="inlineStr">
+      <c r="F62" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -48954,7 +48954,7 @@
           <t>3D AI people-flow sensors for passenger counting, queue, and dwell in transit hubs and airports</t>
         </is>
       </c>
-      <c r="F64" s="39" t="inlineStr">
+      <c r="F64" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -49014,7 +49014,7 @@
           <t>Automatic passenger counting hardware and analysis software for bus, rail, and paratransit</t>
         </is>
       </c>
-      <c r="F66" s="39" t="inlineStr">
+      <c r="F66" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -49074,7 +49074,7 @@
           <t>Video telematics and driver safety for municipal and transit fleets - exhibited at SWANA WASTECON 2025</t>
         </is>
       </c>
-      <c r="F68" s="39" t="inlineStr">
+      <c r="F68" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -49134,7 +49134,7 @@
           <t>Telematics devices and fleet tracking software for public fleets</t>
         </is>
       </c>
-      <c r="F70" s="39" t="inlineStr">
+      <c r="F70" s="40" t="inlineStr">
         <is>
           <t>Unknown - no jobs parsed from iCIMS portal</t>
         </is>
@@ -49194,7 +49194,7 @@
           <t>FleetWave fleet asset management for public sector fleets</t>
         </is>
       </c>
-      <c r="F72" s="39" t="inlineStr">
+      <c r="F72" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -49254,7 +49254,7 @@
           <t>FleetCommander motor pool and vehicle sharing for agencies</t>
         </is>
       </c>
-      <c r="F74" s="39" t="inlineStr">
+      <c r="F74" s="40" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -49314,7 +49314,7 @@
           <t>Fleet data analytics and benchmarking for public and utility fleets</t>
         </is>
       </c>
-      <c r="F76" s="39" t="inlineStr">
+      <c r="F76" s="40" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -49374,7 +49374,7 @@
           <t>Fleet automation and motor pool platform for public agencies</t>
         </is>
       </c>
-      <c r="F78" s="39" t="inlineStr">
+      <c r="F78" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -49434,7 +49434,7 @@
           <t>Onboard surveillance and video management for transit fleets</t>
         </is>
       </c>
-      <c r="F80" s="39" t="inlineStr">
+      <c r="F80" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -49554,7 +49554,7 @@
           <t>On-demand transit and shared mobility software for public agencies</t>
         </is>
       </c>
-      <c r="F84" s="39" t="inlineStr">
+      <c r="F84" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -49614,7 +49614,7 @@
           <t>Parking meters, kiosks and transit fare systems for cities</t>
         </is>
       </c>
-      <c r="F86" s="39" t="inlineStr">
+      <c r="F86" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -49674,7 +49674,7 @@
           <t>Mobile parking payments for city and municipal parking operators</t>
         </is>
       </c>
-      <c r="F88" s="40" t="inlineStr">
+      <c r="F88" s="39" t="inlineStr">
         <is>
           <t>Yes - Corporate Sales Executive</t>
         </is>
@@ -49734,7 +49734,7 @@
           <t>Parking access and revenue control systems for public garages</t>
         </is>
       </c>
-      <c r="F90" s="39" t="inlineStr">
+      <c r="F90" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -49794,7 +49794,7 @@
           <t>Automated enforcement: school-zone speed, red-light, and bus-lane cameras - exhibited at North Carolina Sheriffs' Association 2026</t>
         </is>
       </c>
-      <c r="F92" s="40" t="inlineStr">
+      <c r="F92" s="39" t="inlineStr">
         <is>
           <t>Yes - Mass Market Account Executive (Arizona_Remote)</t>
         </is>
@@ -49854,7 +49854,7 @@
           <t>Multimodal trip planning app plus a paid agency suite (white-label apps, sponsored Royale, rider data) - exhibited at CTAA EXPO 2026, NAPT Summit 2026</t>
         </is>
       </c>
-      <c r="F94" s="39" t="inlineStr">
+      <c r="F94" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -49914,7 +49914,7 @@
           <t>ePaper Digital Bus Stop, SmartStop kiosks, and CPAM content management for transit agencies</t>
         </is>
       </c>
-      <c r="F96" s="39" t="inlineStr">
+      <c r="F96" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -49976,7 +49976,7 @@
       </c>
       <c r="F98" s="41" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Sales Backoffice Specialist only</t>
+          <t>Sales (non-AE) - Sales Backoffice Specialist with G only</t>
         </is>
       </c>
     </row>
@@ -50034,7 +50034,7 @@
           <t>Bus destination displays, controllers, and next-stop passenger information systems</t>
         </is>
       </c>
-      <c r="F100" s="39" t="inlineStr">
+      <c r="F100" s="40" t="inlineStr">
         <is>
           <t>Unknown - HTTP 403 for https://www.hanoverdisplays</t>
         </is>
@@ -50092,7 +50092,7 @@
           <t>TRACC travel-time and accessibility analysis plus transport datasets for government transport agencies</t>
         </is>
       </c>
-      <c r="F102" s="39" t="inlineStr">
+      <c r="F102" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -50152,7 +50152,7 @@
           <t>Solar smart bus stops with edge AI plus the ORA platform: signage, lane enforcement, passenger counting</t>
         </is>
       </c>
-      <c r="F104" s="39" t="inlineStr">
+      <c r="F104" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -50212,7 +50212,7 @@
           <t>Real-time transit display screens and rider information for agencies and cities</t>
         </is>
       </c>
-      <c r="F106" s="39" t="inlineStr">
+      <c r="F106" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -50272,7 +50272,7 @@
           <t>Elevated automated transit pods on prefabricated guideways (ex-skyTran team) for cities and campuses</t>
         </is>
       </c>
-      <c r="F108" s="39" t="inlineStr">
+      <c r="F108" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -50332,7 +50332,7 @@
           <t>On-demand microtransit software with rider/driver apps and AI dispatch for large agencies - exhibited at CTAA EXPO 2026</t>
         </is>
       </c>
-      <c r="F110" s="40" t="inlineStr">
+      <c r="F110" s="39" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -50392,7 +50392,7 @@
           <t>Assisted-mobility platform and driver network delivering ADA paratransit and door-through-door trips - exhibited at CTAA EXPO 2026</t>
         </is>
       </c>
-      <c r="F112" s="39" t="inlineStr">
+      <c r="F112" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -50452,7 +50452,7 @@
           <t>Transit management software for paratransit, demand-response, microtransit, and taxi fleets - exhibited at CTAA EXPO 2026</t>
         </is>
       </c>
-      <c r="F114" s="39" t="inlineStr">
+      <c r="F114" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -50512,7 +50512,7 @@
           <t>Autonomous vehicle technology and driverless shuttle service for transit agencies and cities</t>
         </is>
       </c>
-      <c r="F116" s="39" t="inlineStr">
+      <c r="F116" s="40" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -50572,7 +50572,7 @@
           <t>flowride.ai SAE Level-4 automated driving software retrofitted onto full-size electric transit buses</t>
         </is>
       </c>
-      <c r="F118" s="39" t="inlineStr">
+      <c r="F118" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -50632,7 +50632,7 @@
           <t>Assisted senior and accessible transportation platform serving agency paratransit overflow in 35+ metros</t>
         </is>
       </c>
-      <c r="F120" s="39" t="inlineStr">
+      <c r="F120" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -50692,7 +50692,7 @@
           <t>White-label multimodal TDM and commute platform for regional agencies, employers, and campuses</t>
         </is>
       </c>
-      <c r="F122" s="39" t="inlineStr">
+      <c r="F122" s="40" t="inlineStr">
         <is>
           <t>Unknown - HTTP 404 for https://www.rideshark.com/c</t>
         </is>
@@ -50744,7 +50744,7 @@
           <t>TripMaster paratransit scheduling and dispatch software for public transit providers</t>
         </is>
       </c>
-      <c r="F124" s="39" t="inlineStr">
+      <c r="F124" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -50802,7 +50802,7 @@
           <t>Demand-responsive transit dispatch and booking software for transit agencies - exhibited at CTAA EXPO 2026</t>
         </is>
       </c>
-      <c r="F126" s="39" t="inlineStr">
+      <c r="F126" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -50862,7 +50862,7 @@
           <t>Electric on-demand shuttle service contracted by cities and transit agencies - exhibited at WEFTEC 2026</t>
         </is>
       </c>
-      <c r="F128" s="39" t="inlineStr">
+      <c r="F128" s="40" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -50922,7 +50922,7 @@
           <t>On-demand ridepooling and mobility analytics software for public transit authorities</t>
         </is>
       </c>
-      <c r="F130" s="39" t="inlineStr">
+      <c r="F130" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -50982,7 +50982,7 @@
           <t>Ridepooling operations and autonomous shuttle services for public transport partners</t>
         </is>
       </c>
-      <c r="F132" s="39" t="inlineStr">
+      <c r="F132" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51034,7 +51034,7 @@
           <t>ADA paratransit eligibility, call center and mobility management technology for agencies</t>
         </is>
       </c>
-      <c r="F134" s="39" t="inlineStr">
+      <c r="F134" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51094,7 +51094,7 @@
           <t>Whoosh autonomous cable-driven transit pods for cities and campuses</t>
         </is>
       </c>
-      <c r="F136" s="39" t="inlineStr">
+      <c r="F136" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51154,7 +51154,7 @@
           <t>Autonomous shuttle vehicles for public transport and campus deployments</t>
         </is>
       </c>
-      <c r="F138" s="39" t="inlineStr">
+      <c r="F138" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51214,7 +51214,7 @@
           <t>Electric and autonomous buses sold to public transit operators worldwide</t>
         </is>
       </c>
-      <c r="F140" s="39" t="inlineStr">
+      <c r="F140" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51274,7 +51274,7 @@
           <t>Automated people mover and group rapid transit systems for public authorities</t>
         </is>
       </c>
-      <c r="F142" s="39" t="inlineStr">
+      <c r="F142" s="40" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -51334,7 +51334,7 @@
           <t>Autonomy software powering driverless shuttles for transit and airport operators</t>
         </is>
       </c>
-      <c r="F144" s="39" t="inlineStr">
+      <c r="F144" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -51394,7 +51394,7 @@
           <t>Autonomous shuttles for public transport agencies, airports and campuses</t>
         </is>
       </c>
-      <c r="F146" s="39" t="inlineStr">
+      <c r="F146" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51454,7 +51454,7 @@
           <t>Leading mobile parking payments app (EasyPark Group)</t>
         </is>
       </c>
-      <c r="F148" s="39" t="inlineStr">
+      <c r="F148" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -51514,7 +51514,7 @@
           <t>Computer vision curb management and automated loading-zone payments</t>
         </is>
       </c>
-      <c r="F150" s="39" t="inlineStr">
+      <c r="F150" s="40" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -51574,7 +51574,7 @@
           <t>Gateless LPR parking operations (GLIDEPARCS) for private lots, universities, and some municipalities</t>
         </is>
       </c>
-      <c r="F152" s="39" t="inlineStr">
+      <c r="F152" s="40" t="inlineStr">
         <is>
           <t>Unknown - page too small - likely JS-rendered</t>
         </is>
@@ -51634,7 +51634,7 @@
           <t>Towing lifecycle software for city towing programs and impound management (ex-AutoReturn + TSD)</t>
         </is>
       </c>
-      <c r="F154" s="39" t="inlineStr">
+      <c r="F154" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -51694,7 +51694,7 @@
           <t>Sentry solar smart kiosks and vision-based automated parking enforcement</t>
         </is>
       </c>
-      <c r="F156" s="39" t="inlineStr">
+      <c r="F156" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51754,7 +51754,7 @@
           <t>Single-space smart parking meters and pay stations for municipalities</t>
         </is>
       </c>
-      <c r="F158" s="39" t="inlineStr">
+      <c r="F158" s="40" t="inlineStr">
         <is>
           <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
@@ -51814,7 +51814,7 @@
           <t>Wireless parking occupancy sensors for city and campus parking</t>
         </is>
       </c>
-      <c r="F160" s="39" t="inlineStr">
+      <c r="F160" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51874,7 +51874,7 @@
           <t>Smart parking sensors and LoRaWAN networks for cities</t>
         </is>
       </c>
-      <c r="F162" s="39" t="inlineStr">
+      <c r="F162" s="40" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -51934,7 +51934,7 @@
           <t>Parking payments, permits and enforcement software for municipalities</t>
         </is>
       </c>
-      <c r="F164" s="39" t="inlineStr">
+      <c r="F164" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51994,7 +51994,7 @@
           <t>Parking citation processing and permit services for California cities</t>
         </is>
       </c>
-      <c r="F166" s="39" t="inlineStr">
+      <c r="F166" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52054,7 +52054,7 @@
           <t>Parking citation, permit and enforcement management software for agencies</t>
         </is>
       </c>
-      <c r="F168" s="39" t="inlineStr">
+      <c r="F168" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52110,7 +52110,7 @@
           <t>Control room video wall visualization software - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F170" s="39" t="inlineStr">
+      <c r="F170" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -52162,7 +52162,7 @@
           <t>Transit fare collection and ticketing software - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F172" s="39" t="inlineStr">
+      <c r="F172" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52210,7 +52210,7 @@
           <t>Infrastructure engineering and asset software - exhibited at APTA 2026, AWWA ACE 2026</t>
         </is>
       </c>
-      <c r="F174" s="39" t="inlineStr">
+      <c r="F174" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52262,7 +52262,7 @@
           <t>Fuel and fleet management systems - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F176" s="39" t="inlineStr">
+      <c r="F176" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -52312,7 +52312,7 @@
           <t>Transit ITS, fare collection, scheduling software - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F178" s="39" t="inlineStr">
+      <c r="F178" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52340,7 +52340,7 @@
       </c>
       <c r="F179" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 403 for https://www.intangles.ai/ca</t>
         </is>
       </c>
     </row>
@@ -52368,7 +52368,7 @@
           <t>Ticketing, traffic and transit management systems - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F180" s="39" t="inlineStr">
+      <c r="F180" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52416,7 +52416,7 @@
           <t>LiDAR 3D digital twin capture for transit - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F182" s="39" t="inlineStr">
+      <c r="F182" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52464,7 +52464,7 @@
           <t>Medical transportation ride management software - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F184" s="39" t="inlineStr">
+      <c r="F184" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52514,7 +52514,7 @@
           <t>AI video analytics perimeter security software - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F186" s="39" t="inlineStr">
+      <c r="F186" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -52562,7 +52562,7 @@
           <t>Transit CAD/AVL, APC, passenger information systems - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F188" s="39" t="inlineStr">
+      <c r="F188" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52616,7 +52616,7 @@
           <t>EV fleet charge management software - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F190" s="39" t="inlineStr">
+      <c r="F190" s="40" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -52664,7 +52664,7 @@
           <t>Immersive VR training software platform - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F192" s="39" t="inlineStr">
+      <c r="F192" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52728,7 +52728,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/23/26)</t>
+          <t>Hiring AEs? (9/25/26)</t>
         </is>
       </c>
     </row>
@@ -54198,7 +54198,7 @@
       </c>
       <c r="F50" s="45" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: ('Connection aborted.', C</t>
         </is>
       </c>
     </row>
@@ -54438,7 +54438,7 @@
       </c>
       <c r="F58" s="45" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -54796,9 +54796,9 @@
           <t>Non-contact transmission line monitoring and dynamic line ratings for utilities</t>
         </is>
       </c>
-      <c r="F70" s="45" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F70" s="47" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -56286,7 +56286,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/23/26)</t>
+          <t>Hiring AEs? (9/25/26)</t>
         </is>
       </c>
     </row>
@@ -59810,7 +59810,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/23/26)</t>
+          <t>Hiring AEs? (9/25/26)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-09-26)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/25/26)</t>
+          <t>Hiring AEs? (9/26/26)</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2522,7 @@
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - HTTP 403 for https://www.365labs.com/car</t>
         </is>
       </c>
     </row>
@@ -5982,9 +5982,9 @@
           <t>Assistive AI for 911 centers: transcription, translation, text-to-911, and video</t>
         </is>
       </c>
-      <c r="F171" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F171" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -6282,9 +6282,9 @@
           <t>Pediatric emergency dosing system and app for EMS agencies</t>
         </is>
       </c>
-      <c r="F181" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F181" s="10" t="inlineStr">
+        <is>
+          <t>Yes - Mid-Market Account Executive</t>
         </is>
       </c>
     </row>
@@ -9658,7 +9658,7 @@
       </c>
       <c r="F297" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -11136,7 +11136,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/25/26)</t>
+          <t>Hiring AEs? (9/26/26)</t>
         </is>
       </c>
     </row>
@@ -11518,7 +11518,7 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 500 for https://company.getinsured.</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -12190,7 +12190,7 @@
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://tootris.com/careers</t>
+          <t>Unknown - page too small - likely JS-rendered</t>
         </is>
       </c>
     </row>
@@ -14420,7 +14420,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/25/26)</t>
+          <t>Hiring AEs? (9/26/26)</t>
         </is>
       </c>
     </row>
@@ -17026,7 +17026,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/25/26)</t>
+          <t>Hiring AEs? (9/26/26)</t>
         </is>
       </c>
     </row>
@@ -17494,7 +17494,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/25/26)</t>
+          <t>Hiring AEs? (9/26/26)</t>
         </is>
       </c>
     </row>
@@ -17642,9 +17642,9 @@
           <t>AI recycling-sorting robots and real-time bale/line data</t>
         </is>
       </c>
-      <c r="F6" s="15" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F6" s="16" t="inlineStr">
+        <is>
+          <t>Yes - Account Executive - Climate Tech ( (Remote East Coast )</t>
         </is>
       </c>
     </row>
@@ -22340,7 +22340,7 @@
       </c>
       <c r="F164" s="15" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -23462,7 +23462,7 @@
       </c>
       <c r="F202" s="15" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -24624,7 +24624,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/25/26)</t>
+          <t>Hiring AEs? (9/26/26)</t>
         </is>
       </c>
     </row>
@@ -38708,7 +38708,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/25/26)</t>
+          <t>Hiring AEs? (9/26/26)</t>
         </is>
       </c>
     </row>
@@ -39064,7 +39064,7 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -39362,7 +39362,7 @@
       </c>
       <c r="F23" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Manager, Large Market (Remote)</t>
+          <t>Yes - Account Manager (Remote)</t>
         </is>
       </c>
     </row>
@@ -40916,9 +40916,9 @@
           <t>WeatherTRAK smart irrigation and water management for public agencies</t>
         </is>
       </c>
-      <c r="F75" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F75" s="10" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -42990,7 +42990,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/25/26)</t>
+          <t>Hiring AEs? (9/26/26)</t>
         </is>
       </c>
     </row>
@@ -43050,7 +43050,7 @@
       </c>
       <c r="F3" s="10" t="inlineStr">
         <is>
-          <t>Yes - Sales Executive - Pacific Northwes (Remote Worker - N/)</t>
+          <t>Yes - Sales Executive, Cross-Sell (North (Remote Worker - N/)</t>
         </is>
       </c>
     </row>
@@ -44322,9 +44322,9 @@
           <t>Longtime standard for school bus routing and planning software</t>
         </is>
       </c>
-      <c r="F46" s="34" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F46" s="35" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -47086,7 +47086,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/25/26)</t>
+          <t>Hiring AEs? (9/26/26)</t>
         </is>
       </c>
     </row>
@@ -47502,7 +47502,7 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -52728,7 +52728,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/25/26)</t>
+          <t>Hiring AEs? (9/26/26)</t>
         </is>
       </c>
     </row>
@@ -54198,7 +54198,7 @@
       </c>
       <c r="F50" s="45" t="inlineStr">
         <is>
-          <t>Unknown - network error: ('Connection aborted.', C</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -54438,7 +54438,7 @@
       </c>
       <c r="F58" s="45" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -56286,7 +56286,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/25/26)</t>
+          <t>Hiring AEs? (9/26/26)</t>
         </is>
       </c>
     </row>
@@ -56758,7 +56758,7 @@
       </c>
       <c r="F17" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Manager (Sales)</t>
+          <t>Yes - Account Manager</t>
         </is>
       </c>
     </row>
@@ -58672,7 +58672,7 @@
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
-          <t>Yes - Enterprise Account Executive (C1 - (New York, New York)</t>
+          <t>Yes - Enterprise Account Executive (C1 - (Dallas, TX, United)</t>
         </is>
       </c>
     </row>
@@ -59150,7 +59150,7 @@
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Manager (Remote USA)</t>
+          <t>Yes - Associate Account Executive (Cleve (Cleveland, Ohio, U)</t>
         </is>
       </c>
     </row>
@@ -59810,7 +59810,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/25/26)</t>
+          <t>Hiring AEs? (9/26/26)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-09-27)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/26/26)</t>
+          <t>Hiring AEs? (9/27/26)</t>
         </is>
       </c>
     </row>
@@ -1802,7 +1802,7 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 500 for https://www.bullard.com/car</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2522,7 @@
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.365labs.com/car</t>
+          <t>Unknown - HTTP 202 for https://www.365labs.com/car</t>
         </is>
       </c>
     </row>
@@ -9658,7 +9658,7 @@
       </c>
       <c r="F297" s="7" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -11136,7 +11136,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/26/26)</t>
+          <t>Hiring AEs? (9/27/26)</t>
         </is>
       </c>
     </row>
@@ -12190,7 +12190,7 @@
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page too small - likely JS-rendered</t>
+          <t>Unknown - HTTP 403 for https://tootris.com/careers</t>
         </is>
       </c>
     </row>
@@ -14420,7 +14420,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/26/26)</t>
+          <t>Hiring AEs? (9/27/26)</t>
         </is>
       </c>
     </row>
@@ -15364,7 +15364,7 @@
       </c>
       <c r="F34" s="69" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -17026,7 +17026,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/26/26)</t>
+          <t>Hiring AEs? (9/27/26)</t>
         </is>
       </c>
     </row>
@@ -17494,7 +17494,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/26/26)</t>
+          <t>Hiring AEs? (9/27/26)</t>
         </is>
       </c>
     </row>
@@ -23696,9 +23696,9 @@
           <t>Enterprise asset and field service management for utilities and municipalities</t>
         </is>
       </c>
-      <c r="F210" s="15" t="inlineStr">
-        <is>
-          <t>Unknown - no ATS on file</t>
+      <c r="F210" s="16" t="inlineStr">
+        <is>
+          <t>Yes - Regional Account Executive, Energy (Ottawa, Ontario)</t>
         </is>
       </c>
     </row>
@@ -24624,7 +24624,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/26/26)</t>
+          <t>Hiring AEs? (9/27/26)</t>
         </is>
       </c>
     </row>
@@ -31856,7 +31856,7 @@
       </c>
       <c r="F246" s="21" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://passportworkforce.c</t>
+          <t>Unknown - HTTP 202 for https://passportworkforce.c</t>
         </is>
       </c>
     </row>
@@ -35596,7 +35596,7 @@
       </c>
       <c r="F374" s="21" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -38708,7 +38708,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/26/26)</t>
+          <t>Hiring AEs? (9/27/26)</t>
         </is>
       </c>
     </row>
@@ -39064,7 +39064,7 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -42990,7 +42990,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/26/26)</t>
+          <t>Hiring AEs? (9/27/26)</t>
         </is>
       </c>
     </row>
@@ -46338,9 +46338,9 @@
           <t>Classroom communication and engagement app connecting K-12 teachers, students, and families - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F114" s="34" t="inlineStr">
-        <is>
-          <t>Unknown - no ATS on file</t>
+      <c r="F114" s="33" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Revenue Product Lead only</t>
         </is>
       </c>
     </row>
@@ -47086,7 +47086,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/26/26)</t>
+          <t>Hiring AEs? (9/27/26)</t>
         </is>
       </c>
     </row>
@@ -47386,7 +47386,7 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.modeshift.com/c</t>
+          <t>Unknown - HTTP 202 for https://www.modeshift.com/c</t>
         </is>
       </c>
     </row>
@@ -47982,7 +47982,7 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.enghouse.com/ca</t>
+          <t>Unknown - HTTP 202 for https://www.enghouse.com/ca</t>
         </is>
       </c>
     </row>
@@ -49796,7 +49796,7 @@
       </c>
       <c r="F92" s="39" t="inlineStr">
         <is>
-          <t>Yes - Mass Market Account Executive (Arizona_Remote)</t>
+          <t>Yes - Mass Market Account Executive (California_Remote)</t>
         </is>
       </c>
     </row>
@@ -50036,7 +50036,7 @@
       </c>
       <c r="F100" s="40" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.hanoverdisplays</t>
+          <t>Unknown - HTTP 202 for https://www.hanoverdisplays</t>
         </is>
       </c>
     </row>
@@ -50424,7 +50424,7 @@
       </c>
       <c r="F113" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://qryde.com/employmen</t>
+          <t>Unknown - HTTP 202 for https://qryde.com/employmen</t>
         </is>
       </c>
     </row>
@@ -52728,7 +52728,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/26/26)</t>
+          <t>Hiring AEs? (9/27/26)</t>
         </is>
       </c>
     </row>
@@ -54438,7 +54438,7 @@
       </c>
       <c r="F58" s="45" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -56286,7 +56286,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/26/26)</t>
+          <t>Hiring AEs? (9/27/26)</t>
         </is>
       </c>
     </row>
@@ -58640,9 +58640,9 @@
           <t>Airport biometric border control, e-gates and identity systems for governments</t>
         </is>
       </c>
-      <c r="F80" s="51" t="inlineStr">
-        <is>
-          <t>Unknown - no ATS on file</t>
+      <c r="F80" s="52" t="inlineStr">
+        <is>
+          <t>Yes - Sales Account Manager (3 Locations)</t>
         </is>
       </c>
     </row>
@@ -59810,7 +59810,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/26/26)</t>
+          <t>Hiring AEs? (9/27/26)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-09-29)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -296,8 +296,8 @@
     <xf numFmtId="1" fontId="2" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/28/26)</t>
+          <t>Hiring AEs? (9/29/26)</t>
         </is>
       </c>
     </row>
@@ -5982,9 +5982,9 @@
           <t>Assistive AI for 911 centers: transcription, translation, text-to-911, and video</t>
         </is>
       </c>
-      <c r="F171" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+      <c r="F171" s="10" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -9458,9 +9458,9 @@
           <t>Digital forensics and investigation management software - exhibited at IACP 2026</t>
         </is>
       </c>
-      <c r="F289" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Sales Operations &amp; GTM Systems Man only</t>
+      <c r="F289" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -10292,9 +10292,9 @@
           <t>Endpoint management and IT automation software - exhibited at NSA 2026, GMIS International 2026, EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F323" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F323" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -11088,7 +11088,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/28/26)</t>
+          <t>Hiring AEs? (9/29/26)</t>
         </is>
       </c>
     </row>
@@ -14372,7 +14372,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/28/26)</t>
+          <t>Hiring AEs? (9/29/26)</t>
         </is>
       </c>
     </row>
@@ -15090,9 +15090,9 @@
           <t>Multi-model collaborative AI workspace for university and college faculty, staff, and students - exhibited at EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F26" s="70" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F26" s="71" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -16714,7 +16714,7 @@
       </c>
       <c r="F86" s="70" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Customer Success Manager only</t>
+          <t>Sales (non-AE) - Business Development Representativ only</t>
         </is>
       </c>
     </row>
@@ -16978,7 +16978,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/28/26)</t>
+          <t>Hiring AEs? (9/29/26)</t>
         </is>
       </c>
     </row>
@@ -17446,7 +17446,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/28/26)</t>
+          <t>Hiring AEs? (9/29/26)</t>
         </is>
       </c>
     </row>
@@ -22664,7 +22664,7 @@
       </c>
       <c r="F177" s="10" t="inlineStr">
         <is>
-          <t>Yes - Enterprise Account Executive (US | Massachusetts)</t>
+          <t>Yes - Account Executive I, SMG (US | Massachusetts)</t>
         </is>
       </c>
     </row>
@@ -23650,7 +23650,7 @@
       </c>
       <c r="F210" s="16" t="inlineStr">
         <is>
-          <t>Yes - Regional Account Executive, Energy (Ottawa, Ontario)</t>
+          <t>Yes - Account Executive Install Base (Ja (Tokyo, Tokyo)</t>
         </is>
       </c>
     </row>
@@ -24576,7 +24576,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/28/26)</t>
+          <t>Hiring AEs? (9/29/26)</t>
         </is>
       </c>
     </row>
@@ -26210,9 +26210,9 @@
           <t>CodeRED public alerting and critical event management for local jurisdictions</t>
         </is>
       </c>
-      <c r="F56" s="23" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F56" s="21" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -26754,7 +26754,7 @@
       </c>
       <c r="F75" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - board is another company's - not read</t>
         </is>
       </c>
     </row>
@@ -26812,7 +26812,7 @@
       </c>
       <c r="F77" s="9" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Business Development Representativ only</t>
+          <t>Sales (non-AE) - Commercial Counsel, Revenue only</t>
         </is>
       </c>
     </row>
@@ -26842,7 +26842,7 @@
       </c>
       <c r="F78" s="22" t="inlineStr">
         <is>
-          <t>Yes - Enterprise Account Executive (US | Massachusetts)</t>
+          <t>Yes - Account Executive I, SMG (US | Massachusetts)</t>
         </is>
       </c>
     </row>
@@ -30946,7 +30946,7 @@
       </c>
       <c r="F217" s="7" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -31868,7 +31868,7 @@
       </c>
       <c r="F248" s="23" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Associate Director, Client Success only</t>
+          <t>Sales (non-AE) - Director, Labor Sales only</t>
         </is>
       </c>
     </row>
@@ -34222,7 +34222,7 @@
       </c>
       <c r="F329" s="7" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -38634,7 +38634,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/28/26)</t>
+          <t>Hiring AEs? (9/29/26)</t>
         </is>
       </c>
     </row>
@@ -38844,7 +38844,7 @@
       </c>
       <c r="F8" s="27" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Sales Development Representative only</t>
+          <t>Sales (non-AE) - Salesforce &amp; RevOps Systems Admini only</t>
         </is>
       </c>
     </row>
@@ -42916,7 +42916,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/28/26)</t>
+          <t>Hiring AEs? (9/29/26)</t>
         </is>
       </c>
     </row>
@@ -43806,9 +43806,9 @@
           <t>InformaCast mass notification and paging for school districts</t>
         </is>
       </c>
-      <c r="F31" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -45298,9 +45298,9 @@
           <t>K-12 ERP, nutrition, payments and forms platform for districts</t>
         </is>
       </c>
-      <c r="F81" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F81" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Solutions Consultant only</t>
         </is>
       </c>
     </row>
@@ -47012,7 +47012,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/28/26)</t>
+          <t>Hiring AEs? (9/29/26)</t>
         </is>
       </c>
     </row>
@@ -47042,7 +47042,7 @@
       </c>
       <c r="F2" s="39" t="inlineStr">
         <is>
-          <t>Yes - Account Manager - East Coast (2 Locations)</t>
+          <t>Unknown - HTTP 502 for https://cubic.wd1.myworkday</t>
         </is>
       </c>
     </row>
@@ -47100,7 +47100,7 @@
           <t>Mobile fare payment app covering 200+ North American agencies</t>
         </is>
       </c>
-      <c r="F4" s="40" t="inlineStr">
+      <c r="F4" s="39" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -47160,7 +47160,7 @@
           <t>Automated fare collection plus parking and rail signalling systems (US office Lowell, MA)</t>
         </is>
       </c>
-      <c r="F6" s="40" t="inlineStr">
+      <c r="F6" s="39" t="inlineStr">
         <is>
           <t>Unknown - HTTP 404 for https://www.scheidt-bachman</t>
         </is>
@@ -47220,7 +47220,7 @@
           <t>Account-based ticketing and open-loop EMV fare collection in 150+ cities (BPC Group)</t>
         </is>
       </c>
-      <c r="F8" s="40" t="inlineStr">
+      <c r="F8" s="39" t="inlineStr">
         <is>
           <t>Unknown - board is another company's - not read</t>
         </is>
@@ -47280,7 +47280,7 @@
           <t>KubaPay cloud fare collection and account-based ticketing in 500+ cities (ICM group, not Cubic)</t>
         </is>
       </c>
-      <c r="F10" s="40" t="inlineStr">
+      <c r="F10" s="39" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -47340,7 +47340,7 @@
           <t>Automated fare collection and tolling/ITS for US agencies (LA, Bay Area, DC); Samsung SDS lineage</t>
         </is>
       </c>
-      <c r="F12" s="40" t="inlineStr">
+      <c r="F12" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -47398,7 +47398,7 @@
           <t>Fareboxes, validators, and the Universal Platform for automated fare management</t>
         </is>
       </c>
-      <c r="F14" s="40" t="inlineStr">
+      <c r="F14" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -47456,7 +47456,7 @@
           <t>Transit scheduling, fare and paratransit software for public operators</t>
         </is>
       </c>
-      <c r="F16" s="40" t="inlineStr">
+      <c r="F16" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -47516,7 +47516,7 @@
           <t>Tolling operations and back-office payment services for toll agencies</t>
         </is>
       </c>
-      <c r="F18" s="40" t="inlineStr">
+      <c r="F18" s="39" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -47576,7 +47576,7 @@
           <t>Account-based fare collection and validators for public transit operators</t>
         </is>
       </c>
-      <c r="F20" s="39" t="inlineStr">
+      <c r="F20" s="40" t="inlineStr">
         <is>
           <t>Yes - Senior Enterprise Account Executiv (Spain, Spain)</t>
         </is>
@@ -47636,7 +47636,7 @@
           <t>Bus ITS: CAD/AVL, real-time passenger info, and fleet health</t>
         </is>
       </c>
-      <c r="F22" s="40" t="inlineStr">
+      <c r="F22" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -47696,7 +47696,7 @@
           <t>Real-time transit data: arrival predictions and on-time performance</t>
         </is>
       </c>
-      <c r="F24" s="39" t="inlineStr">
+      <c r="F24" s="40" t="inlineStr">
         <is>
           <t>Yes - Senior Account Manager (United States)</t>
         </is>
@@ -47756,7 +47756,7 @@
           <t>myAvail enterprise transit management ITS and CAD/AVL for mid-size US agencies</t>
         </is>
       </c>
-      <c r="F26" s="40" t="inlineStr">
+      <c r="F26" s="39" t="inlineStr">
         <is>
           <t>Unknown - HTTP 404 for https://availtec.com/career</t>
         </is>
@@ -47816,7 +47816,7 @@
           <t>IVU.suite planning, scheduling, dispatch, and ticketing for transit and rail operators</t>
         </is>
       </c>
-      <c r="F28" s="40" t="inlineStr">
+      <c r="F28" s="39" t="inlineStr">
         <is>
           <t>Unknown - HTTP 404 for https://www.ivu.com/career</t>
         </is>
@@ -47876,7 +47876,7 @@
           <t>Transit dispatch, CAD/AVL, and communications software (Modaxo brand, ex-Trapeze ITS)</t>
         </is>
       </c>
-      <c r="F30" s="40" t="inlineStr">
+      <c r="F30" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -47936,7 +47936,7 @@
           <t>Consat Telematics real-time CAD/AVL, passenger info, and electromobility analytics (NA office Sudbury ON)</t>
         </is>
       </c>
-      <c r="F32" s="40" t="inlineStr">
+      <c r="F32" s="39" t="inlineStr">
         <is>
           <t>Unknown - HTTP 404 for https://www.consat.com/care</t>
         </is>
@@ -47996,7 +47996,7 @@
           <t>Transit performance data warehousing, BI, and automated NTD reporting (Modaxo brand) - exhibited at CTAA EXPO 2026</t>
         </is>
       </c>
-      <c r="F34" s="40" t="inlineStr">
+      <c r="F34" s="39" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -48050,7 +48050,7 @@
           <t>Cloud CAD/AVL and in-vehicle tech for transit agencies and campus systems (SDVOSB)</t>
         </is>
       </c>
-      <c r="F36" s="40" t="inlineStr">
+      <c r="F36" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -48110,7 +48110,7 @@
           <t>IBM Maximo consulting plus Mobile Informer EAM for transit agencies, airports, and utilities</t>
         </is>
       </c>
-      <c r="F38" s="40" t="inlineStr">
+      <c r="F38" s="39" t="inlineStr">
         <is>
           <t>Unknown - HTTP 404 for https://www.interlocsolutio</t>
         </is>
@@ -48142,7 +48142,7 @@
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -48170,7 +48170,7 @@
           <t>Trainwise onboard train control/monitoring and Fleetwise wayside fleet management for transit</t>
         </is>
       </c>
-      <c r="F40" s="40" t="inlineStr">
+      <c r="F40" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -48230,7 +48230,7 @@
           <t>Rail terminal management, track inspection, and crew compliance for short lines and commuter rail</t>
         </is>
       </c>
-      <c r="F42" s="40" t="inlineStr">
+      <c r="F42" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -48290,7 +48290,7 @@
           <t>Ultra-wideband train positioning, worker protection, and ATP for transit agencies (NYC MTA)</t>
         </is>
       </c>
-      <c r="F44" s="40" t="inlineStr">
+      <c r="F44" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -48350,7 +48350,7 @@
           <t>CylusOne rail OT cybersecurity: threat detection for signaling, trackside, and onboard networks</t>
         </is>
       </c>
-      <c r="F46" s="40" t="inlineStr">
+      <c r="F46" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -48408,7 +48408,7 @@
           <t>ConnX Maestro unified communications and contact center for transit agencies (SEPTA)</t>
         </is>
       </c>
-      <c r="F48" s="40" t="inlineStr">
+      <c r="F48" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -48466,7 +48466,7 @@
           <t>Non-invasive sensors and cloud analytics for elevator, escalator, and HVAC uptime in transit stations</t>
         </is>
       </c>
-      <c r="F50" s="40" t="inlineStr">
+      <c r="F50" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -48524,7 +48524,7 @@
           <t>Virtual Optical Fiber high-speed data offload between transit vehicles and depots</t>
         </is>
       </c>
-      <c r="F52" s="40" t="inlineStr">
+      <c r="F52" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -48584,7 +48584,7 @@
           <t>AI smart inspection for rail infrastructure: sensor robot plus defect detection and predictive maintenance</t>
         </is>
       </c>
-      <c r="F54" s="40" t="inlineStr">
+      <c r="F54" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -48640,7 +48640,7 @@
           <t>Mobile video surveillance, DVRs, and MotoTrax analytics for transit, school, and municipal fleets - exhibited at CTAA EXPO 2026, NAPT Summit 2026</t>
         </is>
       </c>
-      <c r="F56" s="39" t="inlineStr">
+      <c r="F56" s="40" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -48700,7 +48700,7 @@
           <t>Onboard transit systems: Horizon CCTV, NetSpire passenger info, iConnex real-time (US in Buffalo NY)</t>
         </is>
       </c>
-      <c r="F58" s="40" t="inlineStr">
+      <c r="F58" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -48760,7 +48760,7 @@
           <t>Intelligent video, AI stop-arm analytics, and cloud safety platforms for transit and school districts - exhibited at CTAA EXPO 2026, NAPT Summit 2026</t>
         </is>
       </c>
-      <c r="F60" s="40" t="inlineStr">
+      <c r="F60" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -48820,7 +48820,7 @@
           <t>AI dashcams, MDVRs, and fleet video telematics for transit, school bus, and commercial fleets (US: Houston)</t>
         </is>
       </c>
-      <c r="F62" s="40" t="inlineStr">
+      <c r="F62" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -48880,7 +48880,7 @@
           <t>3D AI people-flow sensors for passenger counting, queue, and dwell in transit hubs and airports</t>
         </is>
       </c>
-      <c r="F64" s="40" t="inlineStr">
+      <c r="F64" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -48940,7 +48940,7 @@
           <t>Automatic passenger counting hardware and analysis software for bus, rail, and paratransit</t>
         </is>
       </c>
-      <c r="F66" s="40" t="inlineStr">
+      <c r="F66" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -49000,7 +49000,7 @@
           <t>Video telematics and driver safety for municipal and transit fleets - exhibited at SWANA WASTECON 2025</t>
         </is>
       </c>
-      <c r="F68" s="40" t="inlineStr">
+      <c r="F68" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -49032,7 +49032,7 @@
       </c>
       <c r="F69" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Executive, Mid-Market (USA)</t>
+          <t>Yes - Enterprise Core Account Executive  (Remote)</t>
         </is>
       </c>
     </row>
@@ -49060,7 +49060,7 @@
           <t>Telematics devices and fleet tracking software for public fleets</t>
         </is>
       </c>
-      <c r="F70" s="40" t="inlineStr">
+      <c r="F70" s="39" t="inlineStr">
         <is>
           <t>Unknown - no jobs parsed from iCIMS portal</t>
         </is>
@@ -49120,7 +49120,7 @@
           <t>FleetWave fleet asset management for public sector fleets</t>
         </is>
       </c>
-      <c r="F72" s="40" t="inlineStr">
+      <c r="F72" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -49180,7 +49180,7 @@
           <t>FleetCommander motor pool and vehicle sharing for agencies</t>
         </is>
       </c>
-      <c r="F74" s="40" t="inlineStr">
+      <c r="F74" s="39" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -49240,7 +49240,7 @@
           <t>Fleet data analytics and benchmarking for public and utility fleets</t>
         </is>
       </c>
-      <c r="F76" s="40" t="inlineStr">
+      <c r="F76" s="39" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -49300,7 +49300,7 @@
           <t>Fleet automation and motor pool platform for public agencies</t>
         </is>
       </c>
-      <c r="F78" s="40" t="inlineStr">
+      <c r="F78" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -49360,7 +49360,7 @@
           <t>Onboard surveillance and video management for transit fleets</t>
         </is>
       </c>
-      <c r="F80" s="40" t="inlineStr">
+      <c r="F80" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -49480,7 +49480,7 @@
           <t>On-demand transit and shared mobility software for public agencies</t>
         </is>
       </c>
-      <c r="F84" s="40" t="inlineStr">
+      <c r="F84" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -49540,7 +49540,7 @@
           <t>Parking meters, kiosks and transit fare systems for cities</t>
         </is>
       </c>
-      <c r="F86" s="40" t="inlineStr">
+      <c r="F86" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -49600,7 +49600,7 @@
           <t>Mobile parking payments for city and municipal parking operators</t>
         </is>
       </c>
-      <c r="F88" s="39" t="inlineStr">
+      <c r="F88" s="40" t="inlineStr">
         <is>
           <t>Yes - Corporate Sales Executive</t>
         </is>
@@ -49660,7 +49660,7 @@
           <t>Parking access and revenue control systems for public garages</t>
         </is>
       </c>
-      <c r="F90" s="40" t="inlineStr">
+      <c r="F90" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -49720,7 +49720,7 @@
           <t>Automated enforcement: school-zone speed, red-light, and bus-lane cameras - exhibited at North Carolina Sheriffs' Association 2026</t>
         </is>
       </c>
-      <c r="F92" s="39" t="inlineStr">
+      <c r="F92" s="40" t="inlineStr">
         <is>
           <t>Yes - Mass Market Account Executive (California_Remote)</t>
         </is>
@@ -49780,7 +49780,7 @@
           <t>Multimodal trip planning app plus a paid agency suite (white-label apps, sponsored Royale, rider data) - exhibited at CTAA EXPO 2026, NAPT Summit 2026</t>
         </is>
       </c>
-      <c r="F94" s="40" t="inlineStr">
+      <c r="F94" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -49840,7 +49840,7 @@
           <t>ePaper Digital Bus Stop, SmartStop kiosks, and CPAM content management for transit agencies</t>
         </is>
       </c>
-      <c r="F96" s="40" t="inlineStr">
+      <c r="F96" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -49960,7 +49960,7 @@
           <t>Bus destination displays, controllers, and next-stop passenger information systems</t>
         </is>
       </c>
-      <c r="F100" s="40" t="inlineStr">
+      <c r="F100" s="39" t="inlineStr">
         <is>
           <t>Unknown - HTTP 202 for https://www.hanoverdisplays</t>
         </is>
@@ -50018,7 +50018,7 @@
           <t>TRACC travel-time and accessibility analysis plus transport datasets for government transport agencies</t>
         </is>
       </c>
-      <c r="F102" s="40" t="inlineStr">
+      <c r="F102" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -50078,7 +50078,7 @@
           <t>Solar smart bus stops with edge AI plus the ORA platform: signage, lane enforcement, passenger counting</t>
         </is>
       </c>
-      <c r="F104" s="40" t="inlineStr">
+      <c r="F104" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -50138,7 +50138,7 @@
           <t>Real-time transit display screens and rider information for agencies and cities</t>
         </is>
       </c>
-      <c r="F106" s="40" t="inlineStr">
+      <c r="F106" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -50198,7 +50198,7 @@
           <t>Elevated automated transit pods on prefabricated guideways (ex-skyTran team) for cities and campuses</t>
         </is>
       </c>
-      <c r="F108" s="40" t="inlineStr">
+      <c r="F108" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -50258,7 +50258,7 @@
           <t>On-demand microtransit software with rider/driver apps and AI dispatch for large agencies - exhibited at CTAA EXPO 2026</t>
         </is>
       </c>
-      <c r="F110" s="39" t="inlineStr">
+      <c r="F110" s="40" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -50318,7 +50318,7 @@
           <t>Assisted-mobility platform and driver network delivering ADA paratransit and door-through-door trips - exhibited at CTAA EXPO 2026</t>
         </is>
       </c>
-      <c r="F112" s="40" t="inlineStr">
+      <c r="F112" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -50378,7 +50378,7 @@
           <t>Transit management software for paratransit, demand-response, microtransit, and taxi fleets - exhibited at CTAA EXPO 2026</t>
         </is>
       </c>
-      <c r="F114" s="40" t="inlineStr">
+      <c r="F114" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -50438,7 +50438,7 @@
           <t>Autonomous vehicle technology and driverless shuttle service for transit agencies and cities</t>
         </is>
       </c>
-      <c r="F116" s="40" t="inlineStr">
+      <c r="F116" s="39" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -50498,7 +50498,7 @@
           <t>flowride.ai SAE Level-4 automated driving software retrofitted onto full-size electric transit buses</t>
         </is>
       </c>
-      <c r="F118" s="40" t="inlineStr">
+      <c r="F118" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -50558,7 +50558,7 @@
           <t>Assisted senior and accessible transportation platform serving agency paratransit overflow in 35+ metros</t>
         </is>
       </c>
-      <c r="F120" s="40" t="inlineStr">
+      <c r="F120" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -50618,7 +50618,7 @@
           <t>White-label multimodal TDM and commute platform for regional agencies, employers, and campuses</t>
         </is>
       </c>
-      <c r="F122" s="40" t="inlineStr">
+      <c r="F122" s="39" t="inlineStr">
         <is>
           <t>Unknown - HTTP 404 for https://www.rideshark.com/c</t>
         </is>
@@ -50670,7 +50670,7 @@
           <t>TripMaster paratransit scheduling and dispatch software for public transit providers</t>
         </is>
       </c>
-      <c r="F124" s="40" t="inlineStr">
+      <c r="F124" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -50728,7 +50728,7 @@
           <t>Demand-responsive transit dispatch and booking software for transit agencies - exhibited at CTAA EXPO 2026</t>
         </is>
       </c>
-      <c r="F126" s="40" t="inlineStr">
+      <c r="F126" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -50788,7 +50788,7 @@
           <t>Electric on-demand shuttle service contracted by cities and transit agencies - exhibited at WEFTEC 2026</t>
         </is>
       </c>
-      <c r="F128" s="40" t="inlineStr">
+      <c r="F128" s="39" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -50848,7 +50848,7 @@
           <t>On-demand ridepooling and mobility analytics software for public transit authorities</t>
         </is>
       </c>
-      <c r="F130" s="40" t="inlineStr">
+      <c r="F130" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -50908,7 +50908,7 @@
           <t>Ridepooling operations and autonomous shuttle services for public transport partners</t>
         </is>
       </c>
-      <c r="F132" s="40" t="inlineStr">
+      <c r="F132" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -50960,7 +50960,7 @@
           <t>ADA paratransit eligibility, call center and mobility management technology for agencies</t>
         </is>
       </c>
-      <c r="F134" s="40" t="inlineStr">
+      <c r="F134" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51020,7 +51020,7 @@
           <t>Whoosh autonomous cable-driven transit pods for cities and campuses</t>
         </is>
       </c>
-      <c r="F136" s="40" t="inlineStr">
+      <c r="F136" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51080,7 +51080,7 @@
           <t>Autonomous shuttle vehicles for public transport and campus deployments</t>
         </is>
       </c>
-      <c r="F138" s="40" t="inlineStr">
+      <c r="F138" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51140,7 +51140,7 @@
           <t>Electric and autonomous buses sold to public transit operators worldwide</t>
         </is>
       </c>
-      <c r="F140" s="40" t="inlineStr">
+      <c r="F140" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51200,7 +51200,7 @@
           <t>Automated people mover and group rapid transit systems for public authorities</t>
         </is>
       </c>
-      <c r="F142" s="40" t="inlineStr">
+      <c r="F142" s="39" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -51260,7 +51260,7 @@
           <t>Autonomy software powering driverless shuttles for transit and airport operators</t>
         </is>
       </c>
-      <c r="F144" s="40" t="inlineStr">
+      <c r="F144" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -51320,7 +51320,7 @@
           <t>Autonomous shuttles for public transport agencies, airports and campuses</t>
         </is>
       </c>
-      <c r="F146" s="40" t="inlineStr">
+      <c r="F146" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51380,7 +51380,7 @@
           <t>Leading mobile parking payments app (EasyPark Group)</t>
         </is>
       </c>
-      <c r="F148" s="40" t="inlineStr">
+      <c r="F148" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -51440,7 +51440,7 @@
           <t>Computer vision curb management and automated loading-zone payments</t>
         </is>
       </c>
-      <c r="F150" s="40" t="inlineStr">
+      <c r="F150" s="39" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -51500,7 +51500,7 @@
           <t>Gateless LPR parking operations (GLIDEPARCS) for private lots, universities, and some municipalities</t>
         </is>
       </c>
-      <c r="F152" s="40" t="inlineStr">
+      <c r="F152" s="39" t="inlineStr">
         <is>
           <t>Unknown - page too small - likely JS-rendered</t>
         </is>
@@ -51560,7 +51560,7 @@
           <t>Towing lifecycle software for city towing programs and impound management (ex-AutoReturn + TSD)</t>
         </is>
       </c>
-      <c r="F154" s="40" t="inlineStr">
+      <c r="F154" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -51620,7 +51620,7 @@
           <t>Sentry solar smart kiosks and vision-based automated parking enforcement</t>
         </is>
       </c>
-      <c r="F156" s="40" t="inlineStr">
+      <c r="F156" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51680,7 +51680,7 @@
           <t>Single-space smart parking meters and pay stations for municipalities</t>
         </is>
       </c>
-      <c r="F158" s="40" t="inlineStr">
+      <c r="F158" s="39" t="inlineStr">
         <is>
           <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
@@ -51740,7 +51740,7 @@
           <t>Wireless parking occupancy sensors for city and campus parking</t>
         </is>
       </c>
-      <c r="F160" s="40" t="inlineStr">
+      <c r="F160" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51800,7 +51800,7 @@
           <t>Smart parking sensors and LoRaWAN networks for cities</t>
         </is>
       </c>
-      <c r="F162" s="40" t="inlineStr">
+      <c r="F162" s="39" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -51860,7 +51860,7 @@
           <t>Parking payments, permits and enforcement software for municipalities</t>
         </is>
       </c>
-      <c r="F164" s="40" t="inlineStr">
+      <c r="F164" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51920,7 +51920,7 @@
           <t>Parking citation processing and permit services for California cities</t>
         </is>
       </c>
-      <c r="F166" s="40" t="inlineStr">
+      <c r="F166" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51980,7 +51980,7 @@
           <t>Parking citation, permit and enforcement management software for agencies</t>
         </is>
       </c>
-      <c r="F168" s="40" t="inlineStr">
+      <c r="F168" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52036,7 +52036,7 @@
           <t>Control room video wall visualization software - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F170" s="40" t="inlineStr">
+      <c r="F170" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -52088,7 +52088,7 @@
           <t>Transit fare collection and ticketing software - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F172" s="40" t="inlineStr">
+      <c r="F172" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52136,7 +52136,7 @@
           <t>Infrastructure engineering and asset software - exhibited at APTA 2026, AWWA ACE 2026</t>
         </is>
       </c>
-      <c r="F174" s="40" t="inlineStr">
+      <c r="F174" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52188,7 +52188,7 @@
           <t>Fuel and fleet management systems - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F176" s="40" t="inlineStr">
+      <c r="F176" s="39" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -52238,7 +52238,7 @@
           <t>AI predictive fleet analytics platform - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F178" s="40" t="inlineStr">
+      <c r="F178" s="39" t="inlineStr">
         <is>
           <t>Unknown - HTTP 403 for https://www.intangles.ai/ca</t>
         </is>
@@ -52292,7 +52292,7 @@
           <t>Security and intelligence analytics software - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F180" s="39" t="inlineStr">
+      <c r="F180" s="40" t="inlineStr">
         <is>
           <t>Yes - Enterprise Sales Executive – New L (2 Locations)</t>
         </is>
@@ -52340,7 +52340,7 @@
           <t>Smart EV charging management software - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F182" s="40" t="inlineStr">
+      <c r="F182" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52388,7 +52388,7 @@
           <t>Transit operations software - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F184" s="40" t="inlineStr">
+      <c r="F184" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52438,7 +52438,7 @@
           <t>Rail/transit software, AI and asset monitoring - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F186" s="40" t="inlineStr">
+      <c r="F186" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52486,7 +52486,7 @@
           <t>GPS fleet tracking and telematics software - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F188" s="39" t="inlineStr">
+      <c r="F188" s="40" t="inlineStr">
         <is>
           <t>Yes - Sales Account Executive – Mid-Mark</t>
         </is>
@@ -52540,7 +52540,7 @@
           <t>On-demand mobility platform for agency partnerships - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F190" s="40" t="inlineStr">
+      <c r="F190" s="39" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52628,7 +52628,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/28/26)</t>
+          <t>Hiring AEs? (9/29/26)</t>
         </is>
       </c>
     </row>
@@ -56186,7 +56186,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/28/26)</t>
+          <t>Hiring AEs? (9/29/26)</t>
         </is>
       </c>
     </row>
@@ -57822,7 +57822,7 @@
       </c>
       <c r="F56" s="51" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 403 for https://www.elenium.com/car</t>
         </is>
       </c>
     </row>
@@ -58602,7 +58602,7 @@
       </c>
       <c r="F82" s="53" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Senior Enterprise Solutions Archit only</t>
+          <t>Sales (non-AE) - USAF and USSF (US Space Force) Str only</t>
         </is>
       </c>
     </row>
@@ -59048,9 +59048,9 @@
           <t>Computer-vision checkout-free parking payment platform (drive-in/drive-out billing) plus parking operations and revenue management for airports; owner of SP+.</t>
         </is>
       </c>
-      <c r="F97" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Associate Account Executive (Cleve (Cleveland, Ohio, U)</t>
+      <c r="F97" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -59710,7 +59710,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/28/26)</t>
+          <t>Hiring AEs? (9/29/26)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-09-30)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -296,8 +296,8 @@
     <xf numFmtId="1" fontId="2" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/29/26)</t>
+          <t>Hiring AEs? (9/30/26)</t>
         </is>
       </c>
     </row>
@@ -5864,7 +5864,7 @@
       </c>
       <c r="F167" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Manager (Remote, US (TN/KY))</t>
+          <t>Yes - Account Manager (Remote, US (West))</t>
         </is>
       </c>
     </row>
@@ -6012,9 +6012,9 @@
           <t>Defibrillators, monitors, and EMS software (ePCR, dispatch, billing)</t>
         </is>
       </c>
-      <c r="F172" s="8" t="inlineStr">
-        <is>
-          <t>Yes - Account Executive - TherOx (SS02)  (6 Locations)</t>
+      <c r="F172" s="4" t="inlineStr">
+        <is>
+          <t>Unknown - HTTP 502 for https://zoll.wd5.myworkdayj</t>
         </is>
       </c>
     </row>
@@ -7120,7 +7120,7 @@
       </c>
       <c r="F209" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 404 for https://pratus.disastertech</t>
         </is>
       </c>
     </row>
@@ -11088,7 +11088,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/29/26)</t>
+          <t>Hiring AEs? (9/30/26)</t>
         </is>
       </c>
     </row>
@@ -14372,7 +14372,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/29/26)</t>
+          <t>Hiring AEs? (9/30/26)</t>
         </is>
       </c>
     </row>
@@ -14542,7 +14542,7 @@
       </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
-          <t>Yes - Junior Account Manager</t>
+          <t>Yes - Account Manager</t>
         </is>
       </c>
     </row>
@@ -14858,9 +14858,9 @@
           <t>VALT video observation and recording software for nursing simulation labs, clinical skills training, courtrooms, and child advocacy centers - exhibited at EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F18" s="69" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F18" s="70" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Regional Representative - Sales only</t>
         </is>
       </c>
     </row>
@@ -16978,7 +16978,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/29/26)</t>
+          <t>Hiring AEs? (9/30/26)</t>
         </is>
       </c>
     </row>
@@ -17446,7 +17446,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/29/26)</t>
+          <t>Hiring AEs? (9/30/26)</t>
         </is>
       </c>
     </row>
@@ -22664,7 +22664,7 @@
       </c>
       <c r="F177" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Executive I, SMG (US | Massachusetts)</t>
+          <t>Yes - Account Executive, SMG (US | Massachusetts)</t>
         </is>
       </c>
     </row>
@@ -24576,7 +24576,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/29/26)</t>
+          <t>Hiring AEs? (9/30/26)</t>
         </is>
       </c>
     </row>
@@ -25086,7 +25086,7 @@
       </c>
       <c r="F18" s="21" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 403 for https://www.revize.com/care</t>
         </is>
       </c>
     </row>
@@ -26842,7 +26842,7 @@
       </c>
       <c r="F78" s="22" t="inlineStr">
         <is>
-          <t>Yes - Account Executive I, SMG (US | Massachusetts)</t>
+          <t>Yes - Account Executive, SMG (US | Massachusetts)</t>
         </is>
       </c>
     </row>
@@ -28636,9 +28636,9 @@
           <t>Aerial imagery and property data analytics for county assessors, GIS, and insurers - exhibited at IAAO 2026</t>
         </is>
       </c>
-      <c r="F139" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F139" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -29584,7 +29584,7 @@
       </c>
       <c r="F171" s="10" t="inlineStr">
         <is>
-          <t>Yes - Mid Market Account Executive (Boston, MA)</t>
+          <t>Yes - Enterprise Account Executive - Pub (Georgia)</t>
         </is>
       </c>
     </row>
@@ -29734,7 +29734,7 @@
       </c>
       <c r="F176" s="22" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (United States)</t>
+          <t>Yes - Account Executive (Canada | Remote)</t>
         </is>
       </c>
     </row>
@@ -30532,7 +30532,7 @@
       </c>
       <c r="F203" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (United States)</t>
+          <t>Yes - Account Executive (Canada | Remote)</t>
         </is>
       </c>
     </row>
@@ -31808,7 +31808,7 @@
       </c>
       <c r="F246" s="21" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://passportworkforce.c</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -32428,9 +32428,9 @@
           <t>License verification and workforce compliance for agencies and regulators</t>
         </is>
       </c>
-      <c r="F267" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Sales Executive - Central Region ( (Remote - US)</t>
+      <c r="F267" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Sr. Customer Success Manager - Gov only</t>
         </is>
       </c>
     </row>
@@ -32816,7 +32816,7 @@
       </c>
       <c r="F280" s="21" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - page too small - likely JS-rendered</t>
         </is>
       </c>
     </row>
@@ -38634,7 +38634,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/29/26)</t>
+          <t>Hiring AEs? (9/30/26)</t>
         </is>
       </c>
     </row>
@@ -42916,7 +42916,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/29/26)</t>
+          <t>Hiring AEs? (9/30/26)</t>
         </is>
       </c>
     </row>
@@ -42976,7 +42976,7 @@
       </c>
       <c r="F3" s="10" t="inlineStr">
         <is>
-          <t>Yes - Sales Executive, Cross-Sell (North (Remote Worker - N/)</t>
+          <t>Yes - Sales Executive - Central Region</t>
         </is>
       </c>
     </row>
@@ -43480,7 +43480,7 @@
       </c>
       <c r="F20" s="35" t="inlineStr">
         <is>
-          <t>Yes - Commercial Account Executive - Cen (Dallas, Texas)</t>
+          <t>Yes - Commercial Account Executive - Cen (Denver, Colorado)</t>
         </is>
       </c>
     </row>
@@ -43806,9 +43806,9 @@
           <t>InformaCast mass notification and paging for school districts</t>
         </is>
       </c>
-      <c r="F31" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F31" s="10" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -44190,7 +44190,7 @@
       </c>
       <c r="F44" s="35" t="inlineStr">
         <is>
-          <t>Yes - Sr. Regional Account Manager (Remote USA)</t>
+          <t>Yes - Regional Account Manager- Future O (Remote USA)</t>
         </is>
       </c>
     </row>
@@ -45268,9 +45268,9 @@
           <t>Cloud SIS and LMS for K-12 districts and charter networks</t>
         </is>
       </c>
-      <c r="F80" s="35" t="inlineStr">
-        <is>
-          <t>Yes - Account Executive</t>
+      <c r="F80" s="34" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -47012,7 +47012,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/29/26)</t>
+          <t>Hiring AEs? (9/30/26)</t>
         </is>
       </c>
     </row>
@@ -47042,7 +47042,7 @@
       </c>
       <c r="F2" s="39" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 502 for https://cubic.wd1.myworkday</t>
+          <t>Yes - Account Manager - East Coast (2 Locations)</t>
         </is>
       </c>
     </row>
@@ -47100,7 +47100,7 @@
           <t>Mobile fare payment app covering 200+ North American agencies</t>
         </is>
       </c>
-      <c r="F4" s="39" t="inlineStr">
+      <c r="F4" s="40" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -47160,7 +47160,7 @@
           <t>Automated fare collection plus parking and rail signalling systems (US office Lowell, MA)</t>
         </is>
       </c>
-      <c r="F6" s="39" t="inlineStr">
+      <c r="F6" s="40" t="inlineStr">
         <is>
           <t>Unknown - HTTP 404 for https://www.scheidt-bachman</t>
         </is>
@@ -47220,7 +47220,7 @@
           <t>Account-based ticketing and open-loop EMV fare collection in 150+ cities (BPC Group)</t>
         </is>
       </c>
-      <c r="F8" s="39" t="inlineStr">
+      <c r="F8" s="40" t="inlineStr">
         <is>
           <t>Unknown - board is another company's - not read</t>
         </is>
@@ -47280,7 +47280,7 @@
           <t>KubaPay cloud fare collection and account-based ticketing in 500+ cities (ICM group, not Cubic)</t>
         </is>
       </c>
-      <c r="F10" s="39" t="inlineStr">
+      <c r="F10" s="40" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -47340,7 +47340,7 @@
           <t>Automated fare collection and tolling/ITS for US agencies (LA, Bay Area, DC); Samsung SDS lineage</t>
         </is>
       </c>
-      <c r="F12" s="39" t="inlineStr">
+      <c r="F12" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -47398,7 +47398,7 @@
           <t>Fareboxes, validators, and the Universal Platform for automated fare management</t>
         </is>
       </c>
-      <c r="F14" s="39" t="inlineStr">
+      <c r="F14" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -47456,7 +47456,7 @@
           <t>Transit scheduling, fare and paratransit software for public operators</t>
         </is>
       </c>
-      <c r="F16" s="39" t="inlineStr">
+      <c r="F16" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -47516,7 +47516,7 @@
           <t>Tolling operations and back-office payment services for toll agencies</t>
         </is>
       </c>
-      <c r="F18" s="39" t="inlineStr">
+      <c r="F18" s="40" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -47546,9 +47546,9 @@
           <t>Check-in/be-out mobile fare payment for public transport authorities</t>
         </is>
       </c>
-      <c r="F19" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Sales &amp; Business Development Manag</t>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Head of Strategic Accounts only</t>
         </is>
       </c>
     </row>
@@ -47576,7 +47576,7 @@
           <t>Account-based fare collection and validators for public transit operators</t>
         </is>
       </c>
-      <c r="F20" s="40" t="inlineStr">
+      <c r="F20" s="39" t="inlineStr">
         <is>
           <t>Yes - Senior Enterprise Account Executiv (Spain, Spain)</t>
         </is>
@@ -47636,7 +47636,7 @@
           <t>Bus ITS: CAD/AVL, real-time passenger info, and fleet health</t>
         </is>
       </c>
-      <c r="F22" s="39" t="inlineStr">
+      <c r="F22" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -47696,7 +47696,7 @@
           <t>Real-time transit data: arrival predictions and on-time performance</t>
         </is>
       </c>
-      <c r="F24" s="40" t="inlineStr">
+      <c r="F24" s="39" t="inlineStr">
         <is>
           <t>Yes - Senior Account Manager (United States)</t>
         </is>
@@ -47756,7 +47756,7 @@
           <t>myAvail enterprise transit management ITS and CAD/AVL for mid-size US agencies</t>
         </is>
       </c>
-      <c r="F26" s="39" t="inlineStr">
+      <c r="F26" s="40" t="inlineStr">
         <is>
           <t>Unknown - HTTP 404 for https://availtec.com/career</t>
         </is>
@@ -47816,7 +47816,7 @@
           <t>IVU.suite planning, scheduling, dispatch, and ticketing for transit and rail operators</t>
         </is>
       </c>
-      <c r="F28" s="39" t="inlineStr">
+      <c r="F28" s="40" t="inlineStr">
         <is>
           <t>Unknown - HTTP 404 for https://www.ivu.com/career</t>
         </is>
@@ -47876,7 +47876,7 @@
           <t>Transit dispatch, CAD/AVL, and communications software (Modaxo brand, ex-Trapeze ITS)</t>
         </is>
       </c>
-      <c r="F30" s="39" t="inlineStr">
+      <c r="F30" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -47936,7 +47936,7 @@
           <t>Consat Telematics real-time CAD/AVL, passenger info, and electromobility analytics (NA office Sudbury ON)</t>
         </is>
       </c>
-      <c r="F32" s="39" t="inlineStr">
+      <c r="F32" s="40" t="inlineStr">
         <is>
           <t>Unknown - HTTP 404 for https://www.consat.com/care</t>
         </is>
@@ -47996,7 +47996,7 @@
           <t>Transit performance data warehousing, BI, and automated NTD reporting (Modaxo brand) - exhibited at CTAA EXPO 2026</t>
         </is>
       </c>
-      <c r="F34" s="39" t="inlineStr">
+      <c r="F34" s="40" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -48050,7 +48050,7 @@
           <t>Cloud CAD/AVL and in-vehicle tech for transit agencies and campus systems (SDVOSB)</t>
         </is>
       </c>
-      <c r="F36" s="39" t="inlineStr">
+      <c r="F36" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -48110,7 +48110,7 @@
           <t>IBM Maximo consulting plus Mobile Informer EAM for transit agencies, airports, and utilities</t>
         </is>
       </c>
-      <c r="F38" s="39" t="inlineStr">
+      <c r="F38" s="40" t="inlineStr">
         <is>
           <t>Unknown - HTTP 404 for https://www.interlocsolutio</t>
         </is>
@@ -48142,7 +48142,7 @@
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -48170,7 +48170,7 @@
           <t>Trainwise onboard train control/monitoring and Fleetwise wayside fleet management for transit</t>
         </is>
       </c>
-      <c r="F40" s="39" t="inlineStr">
+      <c r="F40" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -48230,7 +48230,7 @@
           <t>Rail terminal management, track inspection, and crew compliance for short lines and commuter rail</t>
         </is>
       </c>
-      <c r="F42" s="39" t="inlineStr">
+      <c r="F42" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -48290,7 +48290,7 @@
           <t>Ultra-wideband train positioning, worker protection, and ATP for transit agencies (NYC MTA)</t>
         </is>
       </c>
-      <c r="F44" s="39" t="inlineStr">
+      <c r="F44" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -48350,7 +48350,7 @@
           <t>CylusOne rail OT cybersecurity: threat detection for signaling, trackside, and onboard networks</t>
         </is>
       </c>
-      <c r="F46" s="39" t="inlineStr">
+      <c r="F46" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -48408,7 +48408,7 @@
           <t>ConnX Maestro unified communications and contact center for transit agencies (SEPTA)</t>
         </is>
       </c>
-      <c r="F48" s="39" t="inlineStr">
+      <c r="F48" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -48466,7 +48466,7 @@
           <t>Non-invasive sensors and cloud analytics for elevator, escalator, and HVAC uptime in transit stations</t>
         </is>
       </c>
-      <c r="F50" s="39" t="inlineStr">
+      <c r="F50" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -48524,7 +48524,7 @@
           <t>Virtual Optical Fiber high-speed data offload between transit vehicles and depots</t>
         </is>
       </c>
-      <c r="F52" s="39" t="inlineStr">
+      <c r="F52" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -48584,7 +48584,7 @@
           <t>AI smart inspection for rail infrastructure: sensor robot plus defect detection and predictive maintenance</t>
         </is>
       </c>
-      <c r="F54" s="39" t="inlineStr">
+      <c r="F54" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -48640,7 +48640,7 @@
           <t>Mobile video surveillance, DVRs, and MotoTrax analytics for transit, school, and municipal fleets - exhibited at CTAA EXPO 2026, NAPT Summit 2026</t>
         </is>
       </c>
-      <c r="F56" s="40" t="inlineStr">
+      <c r="F56" s="39" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -48700,7 +48700,7 @@
           <t>Onboard transit systems: Horizon CCTV, NetSpire passenger info, iConnex real-time (US in Buffalo NY)</t>
         </is>
       </c>
-      <c r="F58" s="39" t="inlineStr">
+      <c r="F58" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -48760,7 +48760,7 @@
           <t>Intelligent video, AI stop-arm analytics, and cloud safety platforms for transit and school districts - exhibited at CTAA EXPO 2026, NAPT Summit 2026</t>
         </is>
       </c>
-      <c r="F60" s="39" t="inlineStr">
+      <c r="F60" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -48820,7 +48820,7 @@
           <t>AI dashcams, MDVRs, and fleet video telematics for transit, school bus, and commercial fleets (US: Houston)</t>
         </is>
       </c>
-      <c r="F62" s="39" t="inlineStr">
+      <c r="F62" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -48880,7 +48880,7 @@
           <t>3D AI people-flow sensors for passenger counting, queue, and dwell in transit hubs and airports</t>
         </is>
       </c>
-      <c r="F64" s="39" t="inlineStr">
+      <c r="F64" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -48940,7 +48940,7 @@
           <t>Automatic passenger counting hardware and analysis software for bus, rail, and paratransit</t>
         </is>
       </c>
-      <c r="F66" s="39" t="inlineStr">
+      <c r="F66" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -49000,7 +49000,7 @@
           <t>Video telematics and driver safety for municipal and transit fleets - exhibited at SWANA WASTECON 2025</t>
         </is>
       </c>
-      <c r="F68" s="39" t="inlineStr">
+      <c r="F68" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -49060,7 +49060,7 @@
           <t>Telematics devices and fleet tracking software for public fleets</t>
         </is>
       </c>
-      <c r="F70" s="39" t="inlineStr">
+      <c r="F70" s="40" t="inlineStr">
         <is>
           <t>Unknown - no jobs parsed from iCIMS portal</t>
         </is>
@@ -49120,7 +49120,7 @@
           <t>FleetWave fleet asset management for public sector fleets</t>
         </is>
       </c>
-      <c r="F72" s="39" t="inlineStr">
+      <c r="F72" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -49180,7 +49180,7 @@
           <t>FleetCommander motor pool and vehicle sharing for agencies</t>
         </is>
       </c>
-      <c r="F74" s="39" t="inlineStr">
+      <c r="F74" s="40" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -49240,7 +49240,7 @@
           <t>Fleet data analytics and benchmarking for public and utility fleets</t>
         </is>
       </c>
-      <c r="F76" s="39" t="inlineStr">
+      <c r="F76" s="40" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -49300,7 +49300,7 @@
           <t>Fleet automation and motor pool platform for public agencies</t>
         </is>
       </c>
-      <c r="F78" s="39" t="inlineStr">
+      <c r="F78" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -49360,7 +49360,7 @@
           <t>Onboard surveillance and video management for transit fleets</t>
         </is>
       </c>
-      <c r="F80" s="39" t="inlineStr">
+      <c r="F80" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -49480,7 +49480,7 @@
           <t>On-demand transit and shared mobility software for public agencies</t>
         </is>
       </c>
-      <c r="F84" s="39" t="inlineStr">
+      <c r="F84" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -49540,7 +49540,7 @@
           <t>Parking meters, kiosks and transit fare systems for cities</t>
         </is>
       </c>
-      <c r="F86" s="39" t="inlineStr">
+      <c r="F86" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -49600,7 +49600,7 @@
           <t>Mobile parking payments for city and municipal parking operators</t>
         </is>
       </c>
-      <c r="F88" s="40" t="inlineStr">
+      <c r="F88" s="39" t="inlineStr">
         <is>
           <t>Yes - Corporate Sales Executive</t>
         </is>
@@ -49660,7 +49660,7 @@
           <t>Parking access and revenue control systems for public garages</t>
         </is>
       </c>
-      <c r="F90" s="39" t="inlineStr">
+      <c r="F90" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -49720,7 +49720,7 @@
           <t>Automated enforcement: school-zone speed, red-light, and bus-lane cameras - exhibited at North Carolina Sheriffs' Association 2026</t>
         </is>
       </c>
-      <c r="F92" s="40" t="inlineStr">
+      <c r="F92" s="39" t="inlineStr">
         <is>
           <t>Yes - Mass Market Account Executive (California_Remote)</t>
         </is>
@@ -49780,7 +49780,7 @@
           <t>Multimodal trip planning app plus a paid agency suite (white-label apps, sponsored Royale, rider data) - exhibited at CTAA EXPO 2026, NAPT Summit 2026</t>
         </is>
       </c>
-      <c r="F94" s="39" t="inlineStr">
+      <c r="F94" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -49840,7 +49840,7 @@
           <t>ePaper Digital Bus Stop, SmartStop kiosks, and CPAM content management for transit agencies</t>
         </is>
       </c>
-      <c r="F96" s="39" t="inlineStr">
+      <c r="F96" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -49960,7 +49960,7 @@
           <t>Bus destination displays, controllers, and next-stop passenger information systems</t>
         </is>
       </c>
-      <c r="F100" s="39" t="inlineStr">
+      <c r="F100" s="40" t="inlineStr">
         <is>
           <t>Unknown - HTTP 202 for https://www.hanoverdisplays</t>
         </is>
@@ -50018,7 +50018,7 @@
           <t>TRACC travel-time and accessibility analysis plus transport datasets for government transport agencies</t>
         </is>
       </c>
-      <c r="F102" s="39" t="inlineStr">
+      <c r="F102" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -50078,7 +50078,7 @@
           <t>Solar smart bus stops with edge AI plus the ORA platform: signage, lane enforcement, passenger counting</t>
         </is>
       </c>
-      <c r="F104" s="39" t="inlineStr">
+      <c r="F104" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -50138,7 +50138,7 @@
           <t>Real-time transit display screens and rider information for agencies and cities</t>
         </is>
       </c>
-      <c r="F106" s="39" t="inlineStr">
+      <c r="F106" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -50198,7 +50198,7 @@
           <t>Elevated automated transit pods on prefabricated guideways (ex-skyTran team) for cities and campuses</t>
         </is>
       </c>
-      <c r="F108" s="39" t="inlineStr">
+      <c r="F108" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -50258,7 +50258,7 @@
           <t>On-demand microtransit software with rider/driver apps and AI dispatch for large agencies - exhibited at CTAA EXPO 2026</t>
         </is>
       </c>
-      <c r="F110" s="40" t="inlineStr">
+      <c r="F110" s="39" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -50318,7 +50318,7 @@
           <t>Assisted-mobility platform and driver network delivering ADA paratransit and door-through-door trips - exhibited at CTAA EXPO 2026</t>
         </is>
       </c>
-      <c r="F112" s="39" t="inlineStr">
+      <c r="F112" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -50378,7 +50378,7 @@
           <t>Transit management software for paratransit, demand-response, microtransit, and taxi fleets - exhibited at CTAA EXPO 2026</t>
         </is>
       </c>
-      <c r="F114" s="39" t="inlineStr">
+      <c r="F114" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -50438,7 +50438,7 @@
           <t>Autonomous vehicle technology and driverless shuttle service for transit agencies and cities</t>
         </is>
       </c>
-      <c r="F116" s="39" t="inlineStr">
+      <c r="F116" s="40" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -50498,7 +50498,7 @@
           <t>flowride.ai SAE Level-4 automated driving software retrofitted onto full-size electric transit buses</t>
         </is>
       </c>
-      <c r="F118" s="39" t="inlineStr">
+      <c r="F118" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -50558,7 +50558,7 @@
           <t>Assisted senior and accessible transportation platform serving agency paratransit overflow in 35+ metros</t>
         </is>
       </c>
-      <c r="F120" s="39" t="inlineStr">
+      <c r="F120" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -50618,7 +50618,7 @@
           <t>White-label multimodal TDM and commute platform for regional agencies, employers, and campuses</t>
         </is>
       </c>
-      <c r="F122" s="39" t="inlineStr">
+      <c r="F122" s="40" t="inlineStr">
         <is>
           <t>Unknown - HTTP 404 for https://www.rideshark.com/c</t>
         </is>
@@ -50670,7 +50670,7 @@
           <t>TripMaster paratransit scheduling and dispatch software for public transit providers</t>
         </is>
       </c>
-      <c r="F124" s="39" t="inlineStr">
+      <c r="F124" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -50728,7 +50728,7 @@
           <t>Demand-responsive transit dispatch and booking software for transit agencies - exhibited at CTAA EXPO 2026</t>
         </is>
       </c>
-      <c r="F126" s="39" t="inlineStr">
+      <c r="F126" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -50788,7 +50788,7 @@
           <t>Electric on-demand shuttle service contracted by cities and transit agencies - exhibited at WEFTEC 2026</t>
         </is>
       </c>
-      <c r="F128" s="39" t="inlineStr">
+      <c r="F128" s="40" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -50848,7 +50848,7 @@
           <t>On-demand ridepooling and mobility analytics software for public transit authorities</t>
         </is>
       </c>
-      <c r="F130" s="39" t="inlineStr">
+      <c r="F130" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -50908,7 +50908,7 @@
           <t>Ridepooling operations and autonomous shuttle services for public transport partners</t>
         </is>
       </c>
-      <c r="F132" s="39" t="inlineStr">
+      <c r="F132" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -50960,7 +50960,7 @@
           <t>ADA paratransit eligibility, call center and mobility management technology for agencies</t>
         </is>
       </c>
-      <c r="F134" s="39" t="inlineStr">
+      <c r="F134" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51020,7 +51020,7 @@
           <t>Whoosh autonomous cable-driven transit pods for cities and campuses</t>
         </is>
       </c>
-      <c r="F136" s="39" t="inlineStr">
+      <c r="F136" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51080,7 +51080,7 @@
           <t>Autonomous shuttle vehicles for public transport and campus deployments</t>
         </is>
       </c>
-      <c r="F138" s="39" t="inlineStr">
+      <c r="F138" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51140,7 +51140,7 @@
           <t>Electric and autonomous buses sold to public transit operators worldwide</t>
         </is>
       </c>
-      <c r="F140" s="39" t="inlineStr">
+      <c r="F140" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51200,7 +51200,7 @@
           <t>Automated people mover and group rapid transit systems for public authorities</t>
         </is>
       </c>
-      <c r="F142" s="39" t="inlineStr">
+      <c r="F142" s="40" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -51260,7 +51260,7 @@
           <t>Autonomy software powering driverless shuttles for transit and airport operators</t>
         </is>
       </c>
-      <c r="F144" s="39" t="inlineStr">
+      <c r="F144" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -51320,7 +51320,7 @@
           <t>Autonomous shuttles for public transport agencies, airports and campuses</t>
         </is>
       </c>
-      <c r="F146" s="39" t="inlineStr">
+      <c r="F146" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51380,7 +51380,7 @@
           <t>Leading mobile parking payments app (EasyPark Group)</t>
         </is>
       </c>
-      <c r="F148" s="39" t="inlineStr">
+      <c r="F148" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -51440,7 +51440,7 @@
           <t>Computer vision curb management and automated loading-zone payments</t>
         </is>
       </c>
-      <c r="F150" s="39" t="inlineStr">
+      <c r="F150" s="40" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -51500,7 +51500,7 @@
           <t>Gateless LPR parking operations (GLIDEPARCS) for private lots, universities, and some municipalities</t>
         </is>
       </c>
-      <c r="F152" s="39" t="inlineStr">
+      <c r="F152" s="40" t="inlineStr">
         <is>
           <t>Unknown - page too small - likely JS-rendered</t>
         </is>
@@ -51560,7 +51560,7 @@
           <t>Towing lifecycle software for city towing programs and impound management (ex-AutoReturn + TSD)</t>
         </is>
       </c>
-      <c r="F154" s="39" t="inlineStr">
+      <c r="F154" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -51620,7 +51620,7 @@
           <t>Sentry solar smart kiosks and vision-based automated parking enforcement</t>
         </is>
       </c>
-      <c r="F156" s="39" t="inlineStr">
+      <c r="F156" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51680,7 +51680,7 @@
           <t>Single-space smart parking meters and pay stations for municipalities</t>
         </is>
       </c>
-      <c r="F158" s="39" t="inlineStr">
+      <c r="F158" s="40" t="inlineStr">
         <is>
           <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
@@ -51740,7 +51740,7 @@
           <t>Wireless parking occupancy sensors for city and campus parking</t>
         </is>
       </c>
-      <c r="F160" s="39" t="inlineStr">
+      <c r="F160" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51800,7 +51800,7 @@
           <t>Smart parking sensors and LoRaWAN networks for cities</t>
         </is>
       </c>
-      <c r="F162" s="39" t="inlineStr">
+      <c r="F162" s="40" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -51860,7 +51860,7 @@
           <t>Parking payments, permits and enforcement software for municipalities</t>
         </is>
       </c>
-      <c r="F164" s="39" t="inlineStr">
+      <c r="F164" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51920,7 +51920,7 @@
           <t>Parking citation processing and permit services for California cities</t>
         </is>
       </c>
-      <c r="F166" s="39" t="inlineStr">
+      <c r="F166" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -51980,7 +51980,7 @@
           <t>Parking citation, permit and enforcement management software for agencies</t>
         </is>
       </c>
-      <c r="F168" s="39" t="inlineStr">
+      <c r="F168" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52036,7 +52036,7 @@
           <t>Control room video wall visualization software - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F170" s="39" t="inlineStr">
+      <c r="F170" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -52088,7 +52088,7 @@
           <t>Transit fare collection and ticketing software - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F172" s="39" t="inlineStr">
+      <c r="F172" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52136,7 +52136,7 @@
           <t>Infrastructure engineering and asset software - exhibited at APTA 2026, AWWA ACE 2026</t>
         </is>
       </c>
-      <c r="F174" s="39" t="inlineStr">
+      <c r="F174" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52188,7 +52188,7 @@
           <t>Fuel and fleet management systems - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F176" s="39" t="inlineStr">
+      <c r="F176" s="40" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -52238,7 +52238,7 @@
           <t>AI predictive fleet analytics platform - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F178" s="39" t="inlineStr">
+      <c r="F178" s="40" t="inlineStr">
         <is>
           <t>Unknown - HTTP 403 for https://www.intangles.ai/ca</t>
         </is>
@@ -52292,7 +52292,7 @@
           <t>Security and intelligence analytics software - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F180" s="40" t="inlineStr">
+      <c r="F180" s="39" t="inlineStr">
         <is>
           <t>Yes - Enterprise Sales Executive – New L (2 Locations)</t>
         </is>
@@ -52340,7 +52340,7 @@
           <t>Smart EV charging management software - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F182" s="39" t="inlineStr">
+      <c r="F182" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52388,7 +52388,7 @@
           <t>Transit operations software - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F184" s="39" t="inlineStr">
+      <c r="F184" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52438,7 +52438,7 @@
           <t>Rail/transit software, AI and asset monitoring - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F186" s="39" t="inlineStr">
+      <c r="F186" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52486,7 +52486,7 @@
           <t>GPS fleet tracking and telematics software - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F188" s="40" t="inlineStr">
+      <c r="F188" s="39" t="inlineStr">
         <is>
           <t>Yes - Sales Account Executive – Mid-Mark</t>
         </is>
@@ -52540,7 +52540,7 @@
           <t>On-demand mobility platform for agency partnerships - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F190" s="39" t="inlineStr">
+      <c r="F190" s="40" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -52628,7 +52628,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/29/26)</t>
+          <t>Hiring AEs? (9/30/26)</t>
         </is>
       </c>
     </row>
@@ -54126,9 +54126,9 @@
           <t>Grid software, ADMS and transmission equipment for public and investor utilities</t>
         </is>
       </c>
-      <c r="F51" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F51" s="10" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -56186,7 +56186,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/29/26)</t>
+          <t>Hiring AEs? (9/30/26)</t>
         </is>
       </c>
     </row>
@@ -56598,7 +56598,7 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>None found</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -57822,7 +57822,7 @@
       </c>
       <c r="F56" s="51" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.elenium.com/car</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -58572,7 +58572,7 @@
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
-          <t>Yes - Enterprise Account Executive (C1 - (New York, New York)</t>
+          <t>Yes - Enterprise Account Executive (C1 - (Austin, TX, United)</t>
         </is>
       </c>
     </row>
@@ -59048,9 +59048,9 @@
           <t>Computer-vision checkout-free parking payment platform (drive-in/drive-out billing) plus parking operations and revenue management for airports; owner of SP+.</t>
         </is>
       </c>
-      <c r="F97" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+      <c r="F97" s="10" t="inlineStr">
+        <is>
+          <t>Yes - Associate Account Executive (Cleve (Cleveland, Ohio, U)</t>
         </is>
       </c>
     </row>
@@ -59710,7 +59710,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/29/26)</t>
+          <t>Hiring AEs? (9/30/26)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-10-01)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -286,9 +286,9 @@
     <xf numFmtId="1" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/30/26)</t>
+          <t>Hiring AEs? (10/1/26)</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2522,7 @@
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://www.365labs.com/car</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -5864,7 +5864,7 @@
       </c>
       <c r="F167" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Manager (Remote, US (West))</t>
+          <t>Yes - Account Manager (Remote, US (TN/KY))</t>
         </is>
       </c>
     </row>
@@ -5924,7 +5924,7 @@
       </c>
       <c r="F169" s="9" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Director, Customer Solutions Engin only</t>
+          <t>Sales (non-AE) - Join our Go-To-Market Talent Commu only</t>
         </is>
       </c>
     </row>
@@ -5982,9 +5982,9 @@
           <t>Assistive AI for 911 centers: transcription, translation, text-to-911, and video</t>
         </is>
       </c>
-      <c r="F171" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F171" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -6012,9 +6012,9 @@
           <t>Defibrillators, monitors, and EMS software (ePCR, dispatch, billing)</t>
         </is>
       </c>
-      <c r="F172" s="4" t="inlineStr">
-        <is>
-          <t>Unknown - HTTP 502 for https://zoll.wd5.myworkdayj</t>
+      <c r="F172" s="8" t="inlineStr">
+        <is>
+          <t>Yes - Account Executive - TherOx (SS02)  (6 Locations)</t>
         </is>
       </c>
     </row>
@@ -8786,9 +8786,9 @@
           <t>Community corrections supervision and electronic monitoring for courts</t>
         </is>
       </c>
-      <c r="F265" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F265" s="10" t="inlineStr">
+        <is>
+          <t>Yes - Regional Sales Manager - Southwest (remote, remote, US)</t>
         </is>
       </c>
     </row>
@@ -11088,7 +11088,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/30/26)</t>
+          <t>Hiring AEs? (10/1/26)</t>
         </is>
       </c>
     </row>
@@ -11440,7 +11440,7 @@
       </c>
       <c r="F14" s="64" t="inlineStr">
         <is>
-          <t>Yes - Strategic Account Executive, Marke (Remote – United St)</t>
+          <t>Yes - Commercial Account Executive, Truv (Remote – United St)</t>
         </is>
       </c>
     </row>
@@ -12718,9 +12718,9 @@
           <t>Digital substance use disorder prevention, intervention, and recovery support platform for treatment providers, state and county health agencies, drug courts, and Medicaid plans - exhibited at NatCon 2026, NACCHO 360 2026</t>
         </is>
       </c>
-      <c r="F59" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Senior Customer Success Consultant only</t>
+      <c r="F59" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -12856,9 +12856,9 @@
           <t>Crisis response, closed-loop referral, care management, and bed board software for behavioral health agencies - exhibited at NatCon 2026</t>
         </is>
       </c>
-      <c r="F64" s="65" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - VP of Customer Success only</t>
+      <c r="F64" s="64" t="inlineStr">
+        <is>
+          <t>Yes - Senior Sales Account Executive (Long Beach (Hybrid)</t>
         </is>
       </c>
     </row>
@@ -12934,9 +12934,9 @@
           <t>Human services EHR and care coordination software for behavioral health, residential, vocational rehab, and food assistance providers - exhibited at NatCon 2026</t>
         </is>
       </c>
-      <c r="F67" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Customer Success Manager only</t>
+      <c r="F67" s="10" t="inlineStr">
+        <is>
+          <t>Yes - Senior Account Executive (Remote)</t>
         </is>
       </c>
     </row>
@@ -13654,7 +13654,7 @@
       </c>
       <c r="F94" s="63" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 504 for https://eccovia.com/careers</t>
         </is>
       </c>
     </row>
@@ -14372,7 +14372,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/30/26)</t>
+          <t>Hiring AEs? (10/1/26)</t>
         </is>
       </c>
     </row>
@@ -14828,9 +14828,9 @@
           <t>Peer review, group work, and AI feedback tools that plug into university learning management systems - exhibited at EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>Yes - Account Executive (Texas) (US Remote)</t>
         </is>
       </c>
     </row>
@@ -16978,7 +16978,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/30/26)</t>
+          <t>Hiring AEs? (10/1/26)</t>
         </is>
       </c>
     </row>
@@ -17446,7 +17446,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/30/26)</t>
+          <t>Hiring AEs? (10/1/26)</t>
         </is>
       </c>
     </row>
@@ -19342,7 +19342,7 @@
       </c>
       <c r="F65" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - page too small - likely JS-rendered</t>
         </is>
       </c>
     </row>
@@ -24576,7 +24576,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/30/26)</t>
+          <t>Hiring AEs? (10/1/26)</t>
         </is>
       </c>
     </row>
@@ -24846,7 +24846,7 @@
       </c>
       <c r="F10" s="21" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://zencity.io/careers</t>
+          <t>Unknown - HTTP 403 for https://zencity.io/careers</t>
         </is>
       </c>
     </row>
@@ -26332,7 +26332,7 @@
       </c>
       <c r="F60" s="22" t="inlineStr">
         <is>
-          <t>Yes - Outbound Sales Representative-iWor</t>
+          <t>Yes - Account Executive - GovTech Softwa</t>
         </is>
       </c>
     </row>
@@ -28636,9 +28636,9 @@
           <t>Aerial imagery and property data analytics for county assessors, GIS, and insurers - exhibited at IAAO 2026</t>
         </is>
       </c>
-      <c r="F139" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F139" s="10" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -32428,9 +32428,9 @@
           <t>License verification and workforce compliance for agencies and regulators</t>
         </is>
       </c>
-      <c r="F267" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Sr. Customer Success Manager - Gov only</t>
+      <c r="F267" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -32816,7 +32816,7 @@
       </c>
       <c r="F280" s="21" t="inlineStr">
         <is>
-          <t>Unknown - page too small - likely JS-rendered</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -33814,9 +33814,9 @@
           <t>Policy and rulemaking workflow: draft, route, approve, and track regulations for agencies</t>
         </is>
       </c>
-      <c r="F315" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Strategic Account Executive - West (Remote)</t>
+      <c r="F315" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Customer Success Lead only</t>
         </is>
       </c>
     </row>
@@ -38634,7 +38634,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/30/26)</t>
+          <t>Hiring AEs? (10/1/26)</t>
         </is>
       </c>
     </row>
@@ -42916,7 +42916,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/30/26)</t>
+          <t>Hiring AEs? (10/1/26)</t>
         </is>
       </c>
     </row>
@@ -42946,7 +42946,7 @@
       </c>
       <c r="F2" s="33" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Director, GTM Finance only</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -42976,7 +42976,7 @@
       </c>
       <c r="F3" s="10" t="inlineStr">
         <is>
-          <t>Yes - Sales Executive - Central Region</t>
+          <t>Yes - Sales Executive - Pacific Northwes (Remote Worker - N/)</t>
         </is>
       </c>
     </row>
@@ -43004,7 +43004,7 @@
           <t>AI gun detection layered onto existing school security cameras</t>
         </is>
       </c>
-      <c r="F4" s="34" t="inlineStr">
+      <c r="F4" s="33" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -43064,7 +43064,7 @@
           <t>Monitors school email/docs for self-harm and threat signals - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F6" s="34" t="inlineStr">
+      <c r="F6" s="33" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -43096,7 +43096,7 @@
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - New Business Executive - Strategic only</t>
+          <t>Sales (non-AE) - Customer Success Manager - Mid Mar only</t>
         </is>
       </c>
     </row>
@@ -43124,7 +43124,7 @@
           <t>Cloud web filtering and student safety monitoring - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F8" s="35" t="inlineStr">
+      <c r="F8" s="34" t="inlineStr">
         <is>
           <t>Yes - Account Executive, Large/Enterpris (United States of A)</t>
         </is>
@@ -43184,7 +43184,7 @@
           <t>Web filtering and student safety monitoring for school districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F10" s="35" t="inlineStr">
+      <c r="F10" s="34" t="inlineStr">
         <is>
           <t>Yes - Account Executive (Austin, Texas, Uni)</t>
         </is>
@@ -43244,7 +43244,7 @@
           <t>Student wellbeing, filtering and safety monitoring for school districts</t>
         </is>
       </c>
-      <c r="F12" s="34" t="inlineStr">
+      <c r="F12" s="33" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -43304,7 +43304,7 @@
           <t>AI web filtering and student threat detection for K-12 districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F14" s="33" t="inlineStr">
+      <c r="F14" s="35" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -43362,7 +43362,7 @@
           <t>Real-time AI content filtering and self-harm detection for schools - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F16" s="34" t="inlineStr">
+      <c r="F16" s="33" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -43420,7 +43420,7 @@
           <t>Mass notification and emergency response app for schools and campuses</t>
         </is>
       </c>
-      <c r="F18" s="34" t="inlineStr">
+      <c r="F18" s="33" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -43478,7 +43478,7 @@
           <t>Cloud video security and sensors for schools and public agencies</t>
         </is>
       </c>
-      <c r="F20" s="35" t="inlineStr">
+      <c r="F20" s="34" t="inlineStr">
         <is>
           <t>Yes - Commercial Account Executive - Cen (Denver, Colorado)</t>
         </is>
@@ -43538,7 +43538,7 @@
           <t>AI gun detection and emergency notification for schools and campuses</t>
         </is>
       </c>
-      <c r="F22" s="34" t="inlineStr">
+      <c r="F22" s="33" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -43598,7 +43598,7 @@
           <t>Computer vision threat and weapon detection for schools and public facilities</t>
         </is>
       </c>
-      <c r="F24" s="34" t="inlineStr">
+      <c r="F24" s="33" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -43658,7 +43658,7 @@
           <t>AI-based weapons screening gateways for schools, venues and public buildings</t>
         </is>
       </c>
-      <c r="F26" s="35" t="inlineStr">
+      <c r="F26" s="34" t="inlineStr">
         <is>
           <t>Yes - Regional Sales Manager (Boston, Massachuse)</t>
         </is>
@@ -43718,7 +43718,7 @@
           <t>Anonymous reporting and crisis support platform for K-12 schools</t>
         </is>
       </c>
-      <c r="F28" s="34" t="inlineStr">
+      <c r="F28" s="33" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -43776,7 +43776,7 @@
           <t>Visitor screening and sex-offender check kiosks for schools</t>
         </is>
       </c>
-      <c r="F30" s="34" t="inlineStr">
+      <c r="F30" s="33" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -43836,7 +43836,7 @@
           <t>Emergency mass notification hardware and software for schools and agencies - exhibited at EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F32" s="35" t="inlineStr">
+      <c r="F32" s="34" t="inlineStr">
         <is>
           <t>Yes - Regional Account Manager - Educati (Baltimore, MD)</t>
         </is>
@@ -43894,7 +43894,7 @@
           <t>FlySense vape and bullying sensors for school bathrooms and hallways</t>
         </is>
       </c>
-      <c r="F34" s="34" t="inlineStr">
+      <c r="F34" s="33" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -43952,7 +43952,7 @@
           <t>Multi-sensor vape, gunshot and aggression detection for schools</t>
         </is>
       </c>
-      <c r="F36" s="34" t="inlineStr">
+      <c r="F36" s="33" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -44012,7 +44012,7 @@
           <t>Cloud security, content filtering, and student safety monitoring for Google Workspace and Microsoft 365 in K-12 districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F38" s="34" t="inlineStr">
+      <c r="F38" s="33" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -44072,7 +44072,7 @@
           <t>Gamified phishing simulation and security awareness training built only for K-12 districts, staff and students - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F40" s="34" t="inlineStr">
+      <c r="F40" s="33" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -44128,7 +44128,7 @@
           <t>Web filtering, classroom management, self-harm and threat detection and parent engagement software for K-12 school districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F42" s="34" t="inlineStr">
+      <c r="F42" s="33" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -44188,7 +44188,7 @@
           <t>Vetted small-vehicle student rides supplementing district bus fleets - exhibited at NAPT Summit 2026</t>
         </is>
       </c>
-      <c r="F44" s="35" t="inlineStr">
+      <c r="F44" s="34" t="inlineStr">
         <is>
           <t>Yes - Regional Account Manager- Future O (Remote USA)</t>
         </is>
@@ -44248,7 +44248,7 @@
           <t>Longtime standard for school bus routing and planning software</t>
         </is>
       </c>
-      <c r="F46" s="35" t="inlineStr">
+      <c r="F46" s="34" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -44308,7 +44308,7 @@
           <t>Student transportation routing and fleet software for districts - exhibited at CTAA EXPO 2026</t>
         </is>
       </c>
-      <c r="F48" s="34" t="inlineStr">
+      <c r="F48" s="33" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -44368,7 +44368,7 @@
           <t>School bus operations, driver pay and dispatch software for districts</t>
         </is>
       </c>
-      <c r="F50" s="34" t="inlineStr">
+      <c r="F50" s="33" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -44428,7 +44428,7 @@
           <t>School bus tracking and communication app sold to districts</t>
         </is>
       </c>
-      <c r="F52" s="34" t="inlineStr">
+      <c r="F52" s="33" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -44488,7 +44488,7 @@
           <t>Contracted school bus transportation services for K-12 districts - exhibited at NAPT Summit 2026</t>
         </is>
       </c>
-      <c r="F54" s="34" t="inlineStr">
+      <c r="F54" s="33" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -44548,7 +44548,7 @@
           <t>Contracted school bus transportation for K-12 districts nationwide</t>
         </is>
       </c>
-      <c r="F56" s="34" t="inlineStr">
+      <c r="F56" s="33" t="inlineStr">
         <is>
           <t>Unknown - network error: Exceeded 30 redirects.</t>
         </is>
@@ -44608,7 +44608,7 @@
           <t>Bus video, audio and fleet electronics for school districts</t>
         </is>
       </c>
-      <c r="F58" s="34" t="inlineStr">
+      <c r="F58" s="33" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -44668,7 +44668,7 @@
           <t>School buses and electric Jouley buses for K-12 districts - exhibited at NAPT Summit 2026</t>
         </is>
       </c>
-      <c r="F60" s="34" t="inlineStr">
+      <c r="F60" s="33" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -44728,7 +44728,7 @@
           <t>All-electric school buses and trucks for school districts</t>
         </is>
       </c>
-      <c r="F62" s="34" t="inlineStr">
+      <c r="F62" s="33" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -44788,7 +44788,7 @@
           <t>Electric school bus fleet-as-a-service subscriptions for districts</t>
         </is>
       </c>
-      <c r="F64" s="34" t="inlineStr">
+      <c r="F64" s="33" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -44848,7 +44848,7 @@
           <t>Student information system giant plus enrollment, comms, and analytics - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F66" s="34" t="inlineStr">
+      <c r="F66" s="33" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -44908,7 +44908,7 @@
           <t>K-12 HR, absence and substitute management, and operations software</t>
         </is>
       </c>
-      <c r="F68" s="34" t="inlineStr">
+      <c r="F68" s="33" t="inlineStr">
         <is>
           <t>Unknown - HTTP 403 for https://careers.frontlineed</t>
         </is>
@@ -44968,7 +44968,7 @@
           <t>Thrillshare K-12 communications: district websites, apps, notifications, branding - exhibited at NLC City Summit 2026, CoSN 2026</t>
         </is>
       </c>
-      <c r="F70" s="34" t="inlineStr">
+      <c r="F70" s="33" t="inlineStr">
         <is>
           <t>Unknown - HTTP 404 for https://api.lever.co/v0/pos</t>
         </is>
@@ -45028,7 +45028,7 @@
           <t>Digital flyer distribution and parent communication for K-12 districts</t>
         </is>
       </c>
-      <c r="F72" s="34" t="inlineStr">
+      <c r="F72" s="33" t="inlineStr">
         <is>
           <t>Unknown - HTTP 404 for https://app.trinethire.com/</t>
         </is>
@@ -45088,7 +45088,7 @@
           <t>Student information system and school business/ERP suite for K-12 districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F74" s="33" t="inlineStr">
+      <c r="F74" s="35" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Customer Success Technical Special only</t>
         </is>
@@ -45148,7 +45148,7 @@
           <t>SIS, ERP and gradebook for K-12 districts and state agencies</t>
         </is>
       </c>
-      <c r="F76" s="34" t="inlineStr">
+      <c r="F76" s="33" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -45208,7 +45208,7 @@
           <t>Genesis SIS and parent portal for New Jersey-area public districts</t>
         </is>
       </c>
-      <c r="F78" s="34" t="inlineStr">
+      <c r="F78" s="33" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -45268,7 +45268,7 @@
           <t>Cloud SIS and LMS for K-12 districts and charter networks</t>
         </is>
       </c>
-      <c r="F80" s="34" t="inlineStr">
+      <c r="F80" s="33" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -45298,9 +45298,9 @@
           <t>K-12 ERP, nutrition, payments and forms platform for districts</t>
         </is>
       </c>
-      <c r="F81" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Solutions Consultant only</t>
+      <c r="F81" s="10" t="inlineStr">
+        <is>
+          <t>Yes - Account Executive (Austin, Texas)</t>
         </is>
       </c>
     </row>
@@ -45328,7 +45328,7 @@
           <t>K-12 finance, HR and payroll ERP for California school agencies</t>
         </is>
       </c>
-      <c r="F82" s="34" t="inlineStr">
+      <c r="F82" s="33" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -45388,7 +45388,7 @@
           <t>School nutrition, inventory and POS software for districts and states</t>
         </is>
       </c>
-      <c r="F84" s="34" t="inlineStr">
+      <c r="F84" s="33" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -45446,7 +45446,7 @@
           <t>School bus routing, fleet and student transportation software for districts</t>
         </is>
       </c>
-      <c r="F86" s="35" t="inlineStr">
+      <c r="F86" s="34" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -45506,7 +45506,7 @@
           <t>Enrollment, school choice and behavior management for public districts</t>
         </is>
       </c>
-      <c r="F88" s="34" t="inlineStr">
+      <c r="F88" s="33" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -45566,7 +45566,7 @@
           <t>Website, CMS and mass communications platform for school districts</t>
         </is>
       </c>
-      <c r="F90" s="33" t="inlineStr">
+      <c r="F90" s="35" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -45626,7 +45626,7 @@
           <t>Family engagement, attendance and communications platform for districts</t>
         </is>
       </c>
-      <c r="F92" s="35" t="inlineStr">
+      <c r="F92" s="34" t="inlineStr">
         <is>
           <t>Yes - Account Executive (Future Opportun (Remote)</t>
         </is>
@@ -45686,7 +45686,7 @@
           <t>Absence, substitute placement and time tracking for school districts</t>
         </is>
       </c>
-      <c r="F94" s="35" t="inlineStr">
+      <c r="F94" s="34" t="inlineStr">
         <is>
           <t>Yes - Account Executive (Remote Worker - N/)</t>
         </is>
@@ -45746,7 +45746,7 @@
           <t>K-12 hiring, applicant tracking and talent matching for districts</t>
         </is>
       </c>
-      <c r="F96" s="33" t="inlineStr">
+      <c r="F96" s="35" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -45806,7 +45806,7 @@
           <t>Facility use request and scheduling software for K-12 districts</t>
         </is>
       </c>
-      <c r="F98" s="34" t="inlineStr">
+      <c r="F98" s="33" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -45866,7 +45866,7 @@
           <t>School safety, threat assessment and preparedness software for districts</t>
         </is>
       </c>
-      <c r="F100" s="34" t="inlineStr">
+      <c r="F100" s="33" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -45926,7 +45926,7 @@
           <t>District identity, rostering and application access platform for K-12 - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F102" s="34" t="inlineStr">
+      <c r="F102" s="33" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -45984,7 +45984,7 @@
           <t>Cafeteria point-of-sale, free and reduced meal eligibility, and claims reporting software for K-12 school nutrition programs - exhibited at SNA ANC 2027</t>
         </is>
       </c>
-      <c r="F104" s="34" t="inlineStr">
+      <c r="F104" s="33" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -46036,7 +46036,7 @@
           <t>Chromebook checkout, device inventory, and student login security for K-12 districts running Google Workspace - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F106" s="34" t="inlineStr">
+      <c r="F106" s="33" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -46092,7 +46092,7 @@
           <t>AI point-of-sale and dining operations software for K-12 school nutrition programs and campus dining - exhibited at SNA ANC 2027</t>
         </is>
       </c>
-      <c r="F108" s="34" t="inlineStr">
+      <c r="F108" s="33" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -46150,7 +46150,7 @@
           <t>Data warehouse and analytics platform that unifies SIS, LMS, assessment, and attendance data for K-12 schools and districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F110" s="34" t="inlineStr">
+      <c r="F110" s="33" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -46206,9 +46206,9 @@
           <t>Library, technology asset, and facilities management software for K-12 school districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F112" s="34" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F112" s="35" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Inside Sales Account Executive only</t>
         </is>
       </c>
     </row>
@@ -46264,7 +46264,7 @@
           <t>Classroom communication and engagement app connecting K-12 teachers, students, and families - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F114" s="33" t="inlineStr">
+      <c r="F114" s="35" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Revenue Product Lead only</t>
         </is>
@@ -46314,7 +46314,7 @@
           <t>AI browser extension that generates lesson plans, quizzes, and student feedback inside Google Workspace and LMS tools for teachers and school districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F116" s="35" t="inlineStr">
+      <c r="F116" s="34" t="inlineStr">
         <is>
           <t>Yes - Mid-Market Account Executive (Remote)</t>
         </is>
@@ -46372,7 +46372,7 @@
           <t>Behavior referral and discipline management software plus a student dismissal board for K-12 school districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F118" s="34" t="inlineStr">
+      <c r="F118" s="33" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -46426,7 +46426,7 @@
           <t>IT help desk ticketing, device asset management and facilities service software built for K-12 school districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F120" s="34" t="inlineStr">
+      <c r="F120" s="33" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -46480,7 +46480,7 @@
           <t>Free keyboarding, digital citizenship and AI literacy curriculum for K-12 schools, with a paid ad-free district edition - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F122" s="34" t="inlineStr">
+      <c r="F122" s="33" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -46538,7 +46538,7 @@
           <t>AI platform for K-12 districts giving teachers lesson and assessment generation tools and students guided AI, with district-level policy and privacy controls - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F124" s="33" t="inlineStr">
+      <c r="F124" s="35" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Senior Customer Success Manager -  only</t>
         </is>
@@ -46596,7 +46596,7 @@
           <t>Handwriting and annotation app that lets students write on assignments inside Google Classroom or Canvas and submit back to the LMS, sold to schools - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F126" s="34" t="inlineStr">
+      <c r="F126" s="33" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -46648,7 +46648,7 @@
           <t>Free and reduced meal application processing, cafeteria point-of-sale and school fee payment software for K-12 districts and state education agencies - exhibited at SNA ANC 2027</t>
         </is>
       </c>
-      <c r="F128" s="34" t="inlineStr">
+      <c r="F128" s="33" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -46704,7 +46704,7 @@
           <t>Browser-delivered virtual computer labs, classroom AI safety controls and work-based learning software for school districts and colleges - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F130" s="35" t="inlineStr">
+      <c r="F130" s="34" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -46760,7 +46760,7 @@
           <t>School district financial management, school nutrition and student data software for K-12 districts - exhibited at SNA ANC 2027</t>
         </is>
       </c>
-      <c r="F132" s="34" t="inlineStr">
+      <c r="F132" s="33" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -46818,7 +46818,7 @@
           <t>Identity and access management, rostering and access governance for K-12 school districts and universities - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F134" s="34" t="inlineStr">
+      <c r="F134" s="33" t="inlineStr">
         <is>
           <t>Unknown - board is another company's - not read</t>
         </is>
@@ -46870,7 +46870,7 @@
           <t>AI math tutoring platform with a teacher dashboard for K-12 schools and districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F136" s="34" t="inlineStr">
+      <c r="F136" s="33" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -46922,7 +46922,7 @@
           <t>Web research, annotation and writing platform licensed by schools and districts for students and teachers - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F138" s="34" t="inlineStr">
+      <c r="F138" s="33" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -47012,7 +47012,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/30/26)</t>
+          <t>Hiring AEs? (10/1/26)</t>
         </is>
       </c>
     </row>
@@ -47312,7 +47312,7 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://www.modeshift.com/c</t>
+          <t>Unknown - HTTP 403 for https://www.modeshift.com/c</t>
         </is>
       </c>
     </row>
@@ -47696,9 +47696,9 @@
           <t>Real-time transit data: arrival predictions and on-time performance</t>
         </is>
       </c>
-      <c r="F24" s="39" t="inlineStr">
-        <is>
-          <t>Yes - Senior Account Manager (United States)</t>
+      <c r="F24" s="40" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -47908,7 +47908,7 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://www.enghouse.com/ca</t>
+          <t>Unknown - HTTP 403 for https://www.enghouse.com/ca</t>
         </is>
       </c>
     </row>
@@ -49902,7 +49902,7 @@
       </c>
       <c r="F98" s="41" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Sales Backoffice Specialist with G only</t>
+          <t>Sales (non-AE) - Sales Backoffice Specialist only</t>
         </is>
       </c>
     </row>
@@ -49962,7 +49962,7 @@
       </c>
       <c r="F100" s="40" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://www.hanoverdisplays</t>
+          <t>Unknown - HTTP 403 for https://www.hanoverdisplays</t>
         </is>
       </c>
     </row>
@@ -50350,7 +50350,7 @@
       </c>
       <c r="F113" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://qryde.com/employmen</t>
+          <t>Unknown - HTTP 403 for https://qryde.com/employmen</t>
         </is>
       </c>
     </row>
@@ -52628,7 +52628,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/30/26)</t>
+          <t>Hiring AEs? (10/1/26)</t>
         </is>
       </c>
     </row>
@@ -54126,9 +54126,9 @@
           <t>Grid software, ADMS and transmission equipment for public and investor utilities</t>
         </is>
       </c>
-      <c r="F51" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -56186,7 +56186,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/30/26)</t>
+          <t>Hiring AEs? (10/1/26)</t>
         </is>
       </c>
     </row>
@@ -56598,7 +56598,7 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -59646,9 +59646,9 @@
           <t>Web-based capital program and construction project management software (cost, contracts, documents, scheduling) used by airport owner-operators and public agencies.</t>
         </is>
       </c>
-      <c r="F117" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F117" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -59710,7 +59710,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/30/26)</t>
+          <t>Hiring AEs? (10/1/26)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-10-02)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -286,9 +286,9 @@
     <xf numFmtId="1" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/1/26)</t>
+          <t>Hiring AEs? (10/2/26)</t>
         </is>
       </c>
     </row>
@@ -2012,7 +2012,7 @@
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 403 for https://www.axon.com/career</t>
         </is>
       </c>
     </row>
@@ -2070,9 +2070,9 @@
           <t>License plate readers, gunshot detection, and drone-as-first-responder (Aerodome)</t>
         </is>
       </c>
-      <c r="F39" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Senior Deal Desk Analyst only</t>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2522,7 @@
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - HTTP 403 for https://www.365labs.com/car</t>
         </is>
       </c>
     </row>
@@ -5954,7 +5954,7 @@
       </c>
       <c r="F170" s="4" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 403 for https://www.carbyne.com/car</t>
         </is>
       </c>
     </row>
@@ -11088,7 +11088,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/1/26)</t>
+          <t>Hiring AEs? (10/2/26)</t>
         </is>
       </c>
     </row>
@@ -13654,7 +13654,7 @@
       </c>
       <c r="F94" s="63" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 504 for https://eccovia.com/careers</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -14372,7 +14372,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/1/26)</t>
+          <t>Hiring AEs? (10/2/26)</t>
         </is>
       </c>
     </row>
@@ -16978,7 +16978,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/1/26)</t>
+          <t>Hiring AEs? (10/2/26)</t>
         </is>
       </c>
     </row>
@@ -17446,7 +17446,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/1/26)</t>
+          <t>Hiring AEs? (10/2/26)</t>
         </is>
       </c>
     </row>
@@ -17594,9 +17594,9 @@
           <t>AI recycling-sorting robots and real-time bale/line data</t>
         </is>
       </c>
-      <c r="F6" s="16" t="inlineStr">
-        <is>
-          <t>Yes - Account Executive - Climate Tech ( (Remote East Coast )</t>
+      <c r="F6" s="15" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -20984,7 +20984,7 @@
       </c>
       <c r="F120" s="16" t="inlineStr">
         <is>
-          <t>Yes - Account Executive - Government (Ca (Remote)</t>
+          <t>Yes - Account Executive - Government (Te (Remote)</t>
         </is>
       </c>
     </row>
@@ -24576,7 +24576,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/1/26)</t>
+          <t>Hiring AEs? (10/2/26)</t>
         </is>
       </c>
     </row>
@@ -25504,9 +25504,9 @@
           <t>Citizen identity and digital service portals (CitizenOne) plus digital trust/signatures (Notarius)</t>
         </is>
       </c>
-      <c r="F32" s="23" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Représentant du développement des  only</t>
+      <c r="F32" s="21" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -31808,7 +31808,7 @@
       </c>
       <c r="F246" s="21" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - HTTP 403 for https://passportworkforce.c</t>
         </is>
       </c>
     </row>
@@ -38634,7 +38634,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/1/26)</t>
+          <t>Hiring AEs? (10/2/26)</t>
         </is>
       </c>
     </row>
@@ -42916,7 +42916,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/1/26)</t>
+          <t>Hiring AEs? (10/2/26)</t>
         </is>
       </c>
     </row>
@@ -42946,7 +42946,7 @@
       </c>
       <c r="F2" s="33" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Sales (non-AE) - Director, GTM Finance only</t>
         </is>
       </c>
     </row>
@@ -42976,7 +42976,7 @@
       </c>
       <c r="F3" s="10" t="inlineStr">
         <is>
-          <t>Yes - Sales Executive - Pacific Northwes (Remote Worker - N/)</t>
+          <t>Yes - Sales Executive - Central Region</t>
         </is>
       </c>
     </row>
@@ -43004,7 +43004,7 @@
           <t>AI gun detection layered onto existing school security cameras</t>
         </is>
       </c>
-      <c r="F4" s="33" t="inlineStr">
+      <c r="F4" s="34" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -43064,7 +43064,7 @@
           <t>Monitors school email/docs for self-harm and threat signals - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F6" s="33" t="inlineStr">
+      <c r="F6" s="34" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -43124,7 +43124,7 @@
           <t>Cloud web filtering and student safety monitoring - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F8" s="34" t="inlineStr">
+      <c r="F8" s="35" t="inlineStr">
         <is>
           <t>Yes - Account Executive, Large/Enterpris (United States of A)</t>
         </is>
@@ -43184,7 +43184,7 @@
           <t>Web filtering and student safety monitoring for school districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F10" s="34" t="inlineStr">
+      <c r="F10" s="35" t="inlineStr">
         <is>
           <t>Yes - Account Executive (Austin, Texas, Uni)</t>
         </is>
@@ -43244,7 +43244,7 @@
           <t>Student wellbeing, filtering and safety monitoring for school districts</t>
         </is>
       </c>
-      <c r="F12" s="33" t="inlineStr">
+      <c r="F12" s="34" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -43304,7 +43304,7 @@
           <t>AI web filtering and student threat detection for K-12 districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F14" s="35" t="inlineStr">
+      <c r="F14" s="33" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -43362,7 +43362,7 @@
           <t>Real-time AI content filtering and self-harm detection for schools - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F16" s="33" t="inlineStr">
+      <c r="F16" s="34" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -43420,7 +43420,7 @@
           <t>Mass notification and emergency response app for schools and campuses</t>
         </is>
       </c>
-      <c r="F18" s="33" t="inlineStr">
+      <c r="F18" s="34" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -43478,7 +43478,7 @@
           <t>Cloud video security and sensors for schools and public agencies</t>
         </is>
       </c>
-      <c r="F20" s="34" t="inlineStr">
+      <c r="F20" s="35" t="inlineStr">
         <is>
           <t>Yes - Commercial Account Executive - Cen (Denver, Colorado)</t>
         </is>
@@ -43538,7 +43538,7 @@
           <t>AI gun detection and emergency notification for schools and campuses</t>
         </is>
       </c>
-      <c r="F22" s="33" t="inlineStr">
+      <c r="F22" s="34" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -43598,7 +43598,7 @@
           <t>Computer vision threat and weapon detection for schools and public facilities</t>
         </is>
       </c>
-      <c r="F24" s="33" t="inlineStr">
+      <c r="F24" s="34" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -43658,7 +43658,7 @@
           <t>AI-based weapons screening gateways for schools, venues and public buildings</t>
         </is>
       </c>
-      <c r="F26" s="34" t="inlineStr">
+      <c r="F26" s="35" t="inlineStr">
         <is>
           <t>Yes - Regional Sales Manager (Boston, Massachuse)</t>
         </is>
@@ -43718,7 +43718,7 @@
           <t>Anonymous reporting and crisis support platform for K-12 schools</t>
         </is>
       </c>
-      <c r="F28" s="33" t="inlineStr">
+      <c r="F28" s="34" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -43776,7 +43776,7 @@
           <t>Visitor screening and sex-offender check kiosks for schools</t>
         </is>
       </c>
-      <c r="F30" s="33" t="inlineStr">
+      <c r="F30" s="34" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -43836,7 +43836,7 @@
           <t>Emergency mass notification hardware and software for schools and agencies - exhibited at EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F32" s="34" t="inlineStr">
+      <c r="F32" s="35" t="inlineStr">
         <is>
           <t>Yes - Regional Account Manager - Educati (Baltimore, MD)</t>
         </is>
@@ -43894,7 +43894,7 @@
           <t>FlySense vape and bullying sensors for school bathrooms and hallways</t>
         </is>
       </c>
-      <c r="F34" s="33" t="inlineStr">
+      <c r="F34" s="34" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -43952,7 +43952,7 @@
           <t>Multi-sensor vape, gunshot and aggression detection for schools</t>
         </is>
       </c>
-      <c r="F36" s="33" t="inlineStr">
+      <c r="F36" s="34" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -44012,7 +44012,7 @@
           <t>Cloud security, content filtering, and student safety monitoring for Google Workspace and Microsoft 365 in K-12 districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F38" s="33" t="inlineStr">
+      <c r="F38" s="34" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -44072,7 +44072,7 @@
           <t>Gamified phishing simulation and security awareness training built only for K-12 districts, staff and students - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F40" s="33" t="inlineStr">
+      <c r="F40" s="34" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -44128,7 +44128,7 @@
           <t>Web filtering, classroom management, self-harm and threat detection and parent engagement software for K-12 school districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F42" s="33" t="inlineStr">
+      <c r="F42" s="34" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -44188,7 +44188,7 @@
           <t>Vetted small-vehicle student rides supplementing district bus fleets - exhibited at NAPT Summit 2026</t>
         </is>
       </c>
-      <c r="F44" s="34" t="inlineStr">
+      <c r="F44" s="35" t="inlineStr">
         <is>
           <t>Yes - Regional Account Manager- Future O (Remote USA)</t>
         </is>
@@ -44248,7 +44248,7 @@
           <t>Longtime standard for school bus routing and planning software</t>
         </is>
       </c>
-      <c r="F46" s="34" t="inlineStr">
+      <c r="F46" s="35" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -44308,7 +44308,7 @@
           <t>Student transportation routing and fleet software for districts - exhibited at CTAA EXPO 2026</t>
         </is>
       </c>
-      <c r="F48" s="33" t="inlineStr">
+      <c r="F48" s="34" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -44368,7 +44368,7 @@
           <t>School bus operations, driver pay and dispatch software for districts</t>
         </is>
       </c>
-      <c r="F50" s="33" t="inlineStr">
+      <c r="F50" s="34" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -44428,7 +44428,7 @@
           <t>School bus tracking and communication app sold to districts</t>
         </is>
       </c>
-      <c r="F52" s="33" t="inlineStr">
+      <c r="F52" s="34" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -44488,7 +44488,7 @@
           <t>Contracted school bus transportation services for K-12 districts - exhibited at NAPT Summit 2026</t>
         </is>
       </c>
-      <c r="F54" s="33" t="inlineStr">
+      <c r="F54" s="34" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -44548,7 +44548,7 @@
           <t>Contracted school bus transportation for K-12 districts nationwide</t>
         </is>
       </c>
-      <c r="F56" s="33" t="inlineStr">
+      <c r="F56" s="34" t="inlineStr">
         <is>
           <t>Unknown - network error: Exceeded 30 redirects.</t>
         </is>
@@ -44608,7 +44608,7 @@
           <t>Bus video, audio and fleet electronics for school districts</t>
         </is>
       </c>
-      <c r="F58" s="33" t="inlineStr">
+      <c r="F58" s="34" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -44668,7 +44668,7 @@
           <t>School buses and electric Jouley buses for K-12 districts - exhibited at NAPT Summit 2026</t>
         </is>
       </c>
-      <c r="F60" s="33" t="inlineStr">
+      <c r="F60" s="34" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -44728,7 +44728,7 @@
           <t>All-electric school buses and trucks for school districts</t>
         </is>
       </c>
-      <c r="F62" s="33" t="inlineStr">
+      <c r="F62" s="34" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -44788,7 +44788,7 @@
           <t>Electric school bus fleet-as-a-service subscriptions for districts</t>
         </is>
       </c>
-      <c r="F64" s="33" t="inlineStr">
+      <c r="F64" s="34" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -44848,7 +44848,7 @@
           <t>Student information system giant plus enrollment, comms, and analytics - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F66" s="33" t="inlineStr">
+      <c r="F66" s="34" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -44908,7 +44908,7 @@
           <t>K-12 HR, absence and substitute management, and operations software</t>
         </is>
       </c>
-      <c r="F68" s="33" t="inlineStr">
+      <c r="F68" s="34" t="inlineStr">
         <is>
           <t>Unknown - HTTP 403 for https://careers.frontlineed</t>
         </is>
@@ -44968,7 +44968,7 @@
           <t>Thrillshare K-12 communications: district websites, apps, notifications, branding - exhibited at NLC City Summit 2026, CoSN 2026</t>
         </is>
       </c>
-      <c r="F70" s="33" t="inlineStr">
+      <c r="F70" s="34" t="inlineStr">
         <is>
           <t>Unknown - HTTP 404 for https://api.lever.co/v0/pos</t>
         </is>
@@ -45028,7 +45028,7 @@
           <t>Digital flyer distribution and parent communication for K-12 districts</t>
         </is>
       </c>
-      <c r="F72" s="33" t="inlineStr">
+      <c r="F72" s="34" t="inlineStr">
         <is>
           <t>Unknown - HTTP 404 for https://app.trinethire.com/</t>
         </is>
@@ -45088,7 +45088,7 @@
           <t>Student information system and school business/ERP suite for K-12 districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F74" s="35" t="inlineStr">
+      <c r="F74" s="33" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Customer Success Technical Special only</t>
         </is>
@@ -45148,7 +45148,7 @@
           <t>SIS, ERP and gradebook for K-12 districts and state agencies</t>
         </is>
       </c>
-      <c r="F76" s="33" t="inlineStr">
+      <c r="F76" s="34" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -45208,7 +45208,7 @@
           <t>Genesis SIS and parent portal for New Jersey-area public districts</t>
         </is>
       </c>
-      <c r="F78" s="33" t="inlineStr">
+      <c r="F78" s="34" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -45268,7 +45268,7 @@
           <t>Cloud SIS and LMS for K-12 districts and charter networks</t>
         </is>
       </c>
-      <c r="F80" s="33" t="inlineStr">
+      <c r="F80" s="34" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -45328,7 +45328,7 @@
           <t>K-12 finance, HR and payroll ERP for California school agencies</t>
         </is>
       </c>
-      <c r="F82" s="33" t="inlineStr">
+      <c r="F82" s="34" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -45388,7 +45388,7 @@
           <t>School nutrition, inventory and POS software for districts and states</t>
         </is>
       </c>
-      <c r="F84" s="33" t="inlineStr">
+      <c r="F84" s="34" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -45446,7 +45446,7 @@
           <t>School bus routing, fleet and student transportation software for districts</t>
         </is>
       </c>
-      <c r="F86" s="34" t="inlineStr">
+      <c r="F86" s="35" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -45506,7 +45506,7 @@
           <t>Enrollment, school choice and behavior management for public districts</t>
         </is>
       </c>
-      <c r="F88" s="33" t="inlineStr">
+      <c r="F88" s="34" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -45566,7 +45566,7 @@
           <t>Website, CMS and mass communications platform for school districts</t>
         </is>
       </c>
-      <c r="F90" s="35" t="inlineStr">
+      <c r="F90" s="33" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -45626,7 +45626,7 @@
           <t>Family engagement, attendance and communications platform for districts</t>
         </is>
       </c>
-      <c r="F92" s="34" t="inlineStr">
+      <c r="F92" s="35" t="inlineStr">
         <is>
           <t>Yes - Account Executive (Future Opportun (Remote)</t>
         </is>
@@ -45686,7 +45686,7 @@
           <t>Absence, substitute placement and time tracking for school districts</t>
         </is>
       </c>
-      <c r="F94" s="34" t="inlineStr">
+      <c r="F94" s="35" t="inlineStr">
         <is>
           <t>Yes - Account Executive (Remote Worker - N/)</t>
         </is>
@@ -45746,7 +45746,7 @@
           <t>K-12 hiring, applicant tracking and talent matching for districts</t>
         </is>
       </c>
-      <c r="F96" s="35" t="inlineStr">
+      <c r="F96" s="33" t="inlineStr">
         <is>
           <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
@@ -45806,7 +45806,7 @@
           <t>Facility use request and scheduling software for K-12 districts</t>
         </is>
       </c>
-      <c r="F98" s="33" t="inlineStr">
+      <c r="F98" s="34" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -45866,7 +45866,7 @@
           <t>School safety, threat assessment and preparedness software for districts</t>
         </is>
       </c>
-      <c r="F100" s="33" t="inlineStr">
+      <c r="F100" s="34" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -45926,7 +45926,7 @@
           <t>District identity, rostering and application access platform for K-12 - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F102" s="33" t="inlineStr">
+      <c r="F102" s="34" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -45984,7 +45984,7 @@
           <t>Cafeteria point-of-sale, free and reduced meal eligibility, and claims reporting software for K-12 school nutrition programs - exhibited at SNA ANC 2027</t>
         </is>
       </c>
-      <c r="F104" s="33" t="inlineStr">
+      <c r="F104" s="34" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -46036,7 +46036,7 @@
           <t>Chromebook checkout, device inventory, and student login security for K-12 districts running Google Workspace - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F106" s="33" t="inlineStr">
+      <c r="F106" s="34" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -46092,7 +46092,7 @@
           <t>AI point-of-sale and dining operations software for K-12 school nutrition programs and campus dining - exhibited at SNA ANC 2027</t>
         </is>
       </c>
-      <c r="F108" s="33" t="inlineStr">
+      <c r="F108" s="34" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -46150,7 +46150,7 @@
           <t>Data warehouse and analytics platform that unifies SIS, LMS, assessment, and attendance data for K-12 schools and districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F110" s="33" t="inlineStr">
+      <c r="F110" s="34" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -46208,7 +46208,7 @@
       </c>
       <c r="F112" s="35" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Inside Sales Account Executive only</t>
+          <t>Yes - Expression of Interest: Outside Sa (Remote - USA)</t>
         </is>
       </c>
     </row>
@@ -46264,7 +46264,7 @@
           <t>Classroom communication and engagement app connecting K-12 teachers, students, and families - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F114" s="35" t="inlineStr">
+      <c r="F114" s="33" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Revenue Product Lead only</t>
         </is>
@@ -46314,7 +46314,7 @@
           <t>AI browser extension that generates lesson plans, quizzes, and student feedback inside Google Workspace and LMS tools for teachers and school districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F116" s="34" t="inlineStr">
+      <c r="F116" s="35" t="inlineStr">
         <is>
           <t>Yes - Mid-Market Account Executive (Remote)</t>
         </is>
@@ -46372,7 +46372,7 @@
           <t>Behavior referral and discipline management software plus a student dismissal board for K-12 school districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F118" s="33" t="inlineStr">
+      <c r="F118" s="34" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -46426,7 +46426,7 @@
           <t>IT help desk ticketing, device asset management and facilities service software built for K-12 school districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F120" s="33" t="inlineStr">
+      <c r="F120" s="34" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -46480,7 +46480,7 @@
           <t>Free keyboarding, digital citizenship and AI literacy curriculum for K-12 schools, with a paid ad-free district edition - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F122" s="33" t="inlineStr">
+      <c r="F122" s="34" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -46538,7 +46538,7 @@
           <t>AI platform for K-12 districts giving teachers lesson and assessment generation tools and students guided AI, with district-level policy and privacy controls - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F124" s="35" t="inlineStr">
+      <c r="F124" s="33" t="inlineStr">
         <is>
           <t>Sales (non-AE) - Senior Customer Success Manager -  only</t>
         </is>
@@ -46596,7 +46596,7 @@
           <t>Handwriting and annotation app that lets students write on assignments inside Google Classroom or Canvas and submit back to the LMS, sold to schools - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F126" s="33" t="inlineStr">
+      <c r="F126" s="34" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -46648,7 +46648,7 @@
           <t>Free and reduced meal application processing, cafeteria point-of-sale and school fee payment software for K-12 districts and state education agencies - exhibited at SNA ANC 2027</t>
         </is>
       </c>
-      <c r="F128" s="33" t="inlineStr">
+      <c r="F128" s="34" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -46704,7 +46704,7 @@
           <t>Browser-delivered virtual computer labs, classroom AI safety controls and work-based learning software for school districts and colleges - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F130" s="34" t="inlineStr">
+      <c r="F130" s="35" t="inlineStr">
         <is>
           <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
@@ -46760,7 +46760,7 @@
           <t>School district financial management, school nutrition and student data software for K-12 districts - exhibited at SNA ANC 2027</t>
         </is>
       </c>
-      <c r="F132" s="33" t="inlineStr">
+      <c r="F132" s="34" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -46818,7 +46818,7 @@
           <t>Identity and access management, rostering and access governance for K-12 school districts and universities - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F134" s="33" t="inlineStr">
+      <c r="F134" s="34" t="inlineStr">
         <is>
           <t>Unknown - board is another company's - not read</t>
         </is>
@@ -46870,7 +46870,7 @@
           <t>AI math tutoring platform with a teacher dashboard for K-12 schools and districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F136" s="33" t="inlineStr">
+      <c r="F136" s="34" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -46922,7 +46922,7 @@
           <t>Web research, annotation and writing platform licensed by schools and districts for students and teachers - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F138" s="33" t="inlineStr">
+      <c r="F138" s="34" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -47012,7 +47012,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/1/26)</t>
+          <t>Hiring AEs? (10/2/26)</t>
         </is>
       </c>
     </row>
@@ -52628,7 +52628,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/1/26)</t>
+          <t>Hiring AEs? (10/2/26)</t>
         </is>
       </c>
     </row>
@@ -54126,9 +54126,9 @@
           <t>Grid software, ADMS and transmission equipment for public and investor utilities</t>
         </is>
       </c>
-      <c r="F51" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F51" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -54186,9 +54186,9 @@
           <t>Metering, CIS, billing and grid analytics for public power utilities</t>
         </is>
       </c>
-      <c r="F53" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F53" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - HTTP 301 for https://www.oracle.com/corp</t>
         </is>
       </c>
     </row>
@@ -56186,7 +56186,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/1/26)</t>
+          <t>Hiring AEs? (10/2/26)</t>
         </is>
       </c>
     </row>
@@ -57670,9 +57670,9 @@
           <t>Baggage handling systems and terminal logistics for airports</t>
         </is>
       </c>
-      <c r="F51" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F51" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -58572,7 +58572,7 @@
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
-          <t>Yes - Enterprise Account Executive (C1 - (Austin, TX, United)</t>
+          <t>Yes - Enterprise Account Executive (C1 - (Chicago, IL, Unite)</t>
         </is>
       </c>
     </row>
@@ -58722,7 +58722,7 @@
       </c>
       <c r="F86" s="51" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 403 for https://www.axon.com/career</t>
         </is>
       </c>
     </row>
@@ -59710,7 +59710,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/1/26)</t>
+          <t>Hiring AEs? (10/2/26)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-10-03)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/2/26)</t>
+          <t>Hiring AEs? (10/3/26)</t>
         </is>
       </c>
     </row>
@@ -3182,7 +3182,7 @@
       </c>
       <c r="F76" s="8" t="inlineStr">
         <is>
-          <t>Yes - Account Executive, Federal Civilia (US Remote)</t>
+          <t>Yes - Senior Account Executive, Corporat (2 Locations)</t>
         </is>
       </c>
     </row>
@@ -11088,7 +11088,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/2/26)</t>
+          <t>Hiring AEs? (10/3/26)</t>
         </is>
       </c>
     </row>
@@ -14372,7 +14372,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/2/26)</t>
+          <t>Hiring AEs? (10/3/26)</t>
         </is>
       </c>
     </row>
@@ -16978,7 +16978,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/2/26)</t>
+          <t>Hiring AEs? (10/3/26)</t>
         </is>
       </c>
     </row>
@@ -17446,7 +17446,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/2/26)</t>
+          <t>Hiring AEs? (10/3/26)</t>
         </is>
       </c>
     </row>
@@ -24576,7 +24576,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/2/26)</t>
+          <t>Hiring AEs? (10/3/26)</t>
         </is>
       </c>
     </row>
@@ -26210,9 +26210,9 @@
           <t>CodeRED public alerting and critical event management for local jurisdictions</t>
         </is>
       </c>
-      <c r="F56" s="21" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F56" s="23" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -32428,9 +32428,9 @@
           <t>License verification and workforce compliance for agencies and regulators</t>
         </is>
       </c>
-      <c r="F267" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F267" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Sr. Customer Success Manager - Gov only</t>
         </is>
       </c>
     </row>
@@ -33078,7 +33078,7 @@
       </c>
       <c r="F289" s="7" t="inlineStr">
         <is>
-          <t>Unknown - board is another company's - not read</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -33104,9 +33104,9 @@
           <t>Deathcare technology suite including cemetery and memorial management software</t>
         </is>
       </c>
-      <c r="F290" s="23" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F290" s="21" t="inlineStr">
+        <is>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -38634,7 +38634,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/2/26)</t>
+          <t>Hiring AEs? (10/3/26)</t>
         </is>
       </c>
     </row>
@@ -39766,9 +39766,9 @@
           <t>Club and league management platform for youth soccer organizations</t>
         </is>
       </c>
-      <c r="F39" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -42916,7 +42916,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/2/26)</t>
+          <t>Hiring AEs? (10/3/26)</t>
         </is>
       </c>
     </row>
@@ -47012,7 +47012,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/2/26)</t>
+          <t>Hiring AEs? (10/3/26)</t>
         </is>
       </c>
     </row>
@@ -52628,7 +52628,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/2/26)</t>
+          <t>Hiring AEs? (10/3/26)</t>
         </is>
       </c>
     </row>
@@ -54126,9 +54126,9 @@
           <t>Grid software, ADMS and transmission equipment for public and investor utilities</t>
         </is>
       </c>
-      <c r="F51" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -54186,9 +54186,9 @@
           <t>Metering, CIS, billing and grid analytics for public power utilities</t>
         </is>
       </c>
-      <c r="F53" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - HTTP 301 for https://www.oracle.com/corp</t>
+      <c r="F53" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -56186,7 +56186,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/2/26)</t>
+          <t>Hiring AEs? (10/3/26)</t>
         </is>
       </c>
     </row>
@@ -57822,7 +57822,7 @@
       </c>
       <c r="F56" s="51" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -58510,9 +58510,9 @@
           <t>Biometric identity, TSA PreCheck enrollment and airport boarding systems</t>
         </is>
       </c>
-      <c r="F79" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Key Account Manager - Smart Biomet</t>
+      <c r="F79" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Sales Manager - Smart Biometrics only</t>
         </is>
       </c>
     </row>
@@ -58572,7 +58572,7 @@
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
-          <t>Yes - Enterprise Account Executive (C1 - (Chicago, IL, Unite)</t>
+          <t>Yes - Enterprise Account Executive (C1 - (Dallas, TX, United)</t>
         </is>
       </c>
     </row>
@@ -59710,7 +59710,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/2/26)</t>
+          <t>Hiring AEs? (10/3/26)</t>
         </is>
       </c>
     </row>
@@ -60226,7 +60226,7 @@
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>Yes - Enterprise Account Executive (Stat (United States)</t>
+          <t>Yes - Enterprise Account Executive (Stat (New York, New York)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-10-04)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/3/26)</t>
+          <t>Hiring AEs? (10/4/26)</t>
         </is>
       </c>
     </row>
@@ -5894,7 +5894,7 @@
       </c>
       <c r="F168" s="4" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 404 for https://careers.jobscore.co</t>
         </is>
       </c>
     </row>
@@ -7870,7 +7870,7 @@
       </c>
       <c r="F234" s="4" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -8368,7 +8368,7 @@
       </c>
       <c r="F251" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -11088,7 +11088,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/3/26)</t>
+          <t>Hiring AEs? (10/4/26)</t>
         </is>
       </c>
     </row>
@@ -14372,7 +14372,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/3/26)</t>
+          <t>Hiring AEs? (10/4/26)</t>
         </is>
       </c>
     </row>
@@ -16978,7 +16978,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/3/26)</t>
+          <t>Hiring AEs? (10/4/26)</t>
         </is>
       </c>
     </row>
@@ -17446,7 +17446,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/3/26)</t>
+          <t>Hiring AEs? (10/4/26)</t>
         </is>
       </c>
     </row>
@@ -18542,7 +18542,7 @@
       </c>
       <c r="F38" s="15" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -24576,7 +24576,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/3/26)</t>
+          <t>Hiring AEs? (10/4/26)</t>
         </is>
       </c>
     </row>
@@ -26210,9 +26210,9 @@
           <t>CodeRED public alerting and critical event management for local jurisdictions</t>
         </is>
       </c>
-      <c r="F56" s="23" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F56" s="21" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -26242,7 +26242,7 @@
       </c>
       <c r="F57" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -30184,7 +30184,7 @@
       </c>
       <c r="F191" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -30736,7 +30736,7 @@
       </c>
       <c r="F210" s="21" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - board is another company's - not read</t>
         </is>
       </c>
     </row>
@@ -33078,7 +33078,7 @@
       </c>
       <c r="F289" s="7" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - board is another company's - not read</t>
         </is>
       </c>
     </row>
@@ -33104,9 +33104,9 @@
           <t>Deathcare technology suite including cemetery and memorial management software</t>
         </is>
       </c>
-      <c r="F290" s="21" t="inlineStr">
-        <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+      <c r="F290" s="23" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -37266,7 +37266,7 @@
       </c>
       <c r="F436" s="21" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -37510,9 +37510,9 @@
           <t>Government contract and procurement software - exhibited at NIGP 2026</t>
         </is>
       </c>
-      <c r="F445" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - no ATS on file</t>
+      <c r="F445" s="10" t="inlineStr">
+        <is>
+          <t>Yes - Founding Account Executive (New York City)</t>
         </is>
       </c>
     </row>
@@ -37932,7 +37932,7 @@
       </c>
       <c r="F462" s="21" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -37954,9 +37954,9 @@
           <t>Business phone and unified communications systems - exhibited at NIGP 2026</t>
         </is>
       </c>
-      <c r="F463" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - no ATS on file</t>
+      <c r="F463" s="10" t="inlineStr">
+        <is>
+          <t>Yes - Hunter / Account Executive (2 Locations)</t>
         </is>
       </c>
     </row>
@@ -38634,7 +38634,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/3/26)</t>
+          <t>Hiring AEs? (10/4/26)</t>
         </is>
       </c>
     </row>
@@ -39526,9 +39526,9 @@
           <t>Club and league operations platform for youth sports organizations</t>
         </is>
       </c>
-      <c r="F31" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - no ATS on file</t>
+      <c r="F31" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -39766,9 +39766,9 @@
           <t>Club and league management platform for youth soccer organizations</t>
         </is>
       </c>
-      <c r="F39" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+      <c r="F39" s="10" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -42916,7 +42916,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/3/26)</t>
+          <t>Hiring AEs? (10/4/26)</t>
         </is>
       </c>
     </row>
@@ -47012,7 +47012,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/3/26)</t>
+          <t>Hiring AEs? (10/4/26)</t>
         </is>
       </c>
     </row>
@@ -49932,7 +49932,7 @@
       </c>
       <c r="F99" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -52628,7 +52628,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/3/26)</t>
+          <t>Hiring AEs? (10/4/26)</t>
         </is>
       </c>
     </row>
@@ -53918,7 +53918,7 @@
       </c>
       <c r="F44" s="45" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 404 for https://www.itron.com/compa</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -53978,7 +53978,7 @@
       </c>
       <c r="F46" s="45" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -54338,7 +54338,7 @@
       </c>
       <c r="F58" s="45" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -54788,7 +54788,7 @@
       </c>
       <c r="F73" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 404 for https://www.anterix.com/car</t>
         </is>
       </c>
     </row>
@@ -56186,7 +56186,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/3/26)</t>
+          <t>Hiring AEs? (10/4/26)</t>
         </is>
       </c>
     </row>
@@ -58572,7 +58572,7 @@
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
-          <t>Yes - Enterprise Account Executive (C1 - (Dallas, TX, United)</t>
+          <t>Yes - Enterprise Account Executive (C1 - (Chicago, IL, Unite)</t>
         </is>
       </c>
     </row>
@@ -59710,7 +59710,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/3/26)</t>
+          <t>Hiring AEs? (10/4/26)</t>
         </is>
       </c>
     </row>
@@ -60226,7 +60226,7 @@
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>Yes - Enterprise Account Executive (Stat (New York, New York)</t>
+          <t>Yes - Enterprise Account Executive (Stat (United States)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-10-05)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/4/26)</t>
+          <t>Hiring AEs? (10/5/26)</t>
         </is>
       </c>
     </row>
@@ -5894,7 +5894,7 @@
       </c>
       <c r="F168" s="4" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 404 for https://careers.jobscore.co</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -11088,7 +11088,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/4/26)</t>
+          <t>Hiring AEs? (10/5/26)</t>
         </is>
       </c>
     </row>
@@ -14372,7 +14372,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/4/26)</t>
+          <t>Hiring AEs? (10/5/26)</t>
         </is>
       </c>
     </row>
@@ -16978,7 +16978,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/4/26)</t>
+          <t>Hiring AEs? (10/5/26)</t>
         </is>
       </c>
     </row>
@@ -17446,7 +17446,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/4/26)</t>
+          <t>Hiring AEs? (10/5/26)</t>
         </is>
       </c>
     </row>
@@ -23650,7 +23650,7 @@
       </c>
       <c r="F210" s="16" t="inlineStr">
         <is>
-          <t>Yes - Account Executive Install Base (Ja (Tokyo, Tokyo)</t>
+          <t>Yes - Account Executive - New Business ( (Paris, Île-de-Fran)</t>
         </is>
       </c>
     </row>
@@ -24576,7 +24576,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/4/26)</t>
+          <t>Hiring AEs? (10/5/26)</t>
         </is>
       </c>
     </row>
@@ -25594,9 +25594,9 @@
           <t>Interpretation management and delivery platform (video/phone) used by courts and agencies</t>
         </is>
       </c>
-      <c r="F35" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F35" s="10" t="inlineStr">
+        <is>
+          <t>Yes - Account Executive, SMB (United States (Rem)</t>
         </is>
       </c>
     </row>
@@ -29346,7 +29346,7 @@
       </c>
       <c r="F163" s="10" t="inlineStr">
         <is>
-          <t>Yes - (Remote) Sr Account Executive (26 Locations)</t>
+          <t>Yes - Account Executive (5 Locations)</t>
         </is>
       </c>
     </row>
@@ -30796,7 +30796,7 @@
       </c>
       <c r="F212" s="22" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (London)</t>
+          <t>Yes - Account Executive (Singapore, Singapo)</t>
         </is>
       </c>
     </row>
@@ -38634,7 +38634,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/4/26)</t>
+          <t>Hiring AEs? (10/5/26)</t>
         </is>
       </c>
     </row>
@@ -42916,7 +42916,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/4/26)</t>
+          <t>Hiring AEs? (10/5/26)</t>
         </is>
       </c>
     </row>
@@ -42976,7 +42976,7 @@
       </c>
       <c r="F3" s="10" t="inlineStr">
         <is>
-          <t>Yes - Sales Executive - Central Region</t>
+          <t>Yes - Sales Executive, Cross-Sell (Utah  (Remote Worker - N/)</t>
         </is>
       </c>
     </row>
@@ -45686,9 +45686,9 @@
           <t>Absence, substitute placement and time tracking for school districts</t>
         </is>
       </c>
-      <c r="F94" s="35" t="inlineStr">
-        <is>
-          <t>Yes - Account Executive (Remote Worker - N/)</t>
+      <c r="F94" s="34" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -47012,7 +47012,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/4/26)</t>
+          <t>Hiring AEs? (10/5/26)</t>
         </is>
       </c>
     </row>
@@ -49932,7 +49932,7 @@
       </c>
       <c r="F99" s="7" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -52628,7 +52628,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/4/26)</t>
+          <t>Hiring AEs? (10/5/26)</t>
         </is>
       </c>
     </row>
@@ -53918,7 +53918,7 @@
       </c>
       <c r="F44" s="45" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - HTTP 404 for https://www.itron.com/compa</t>
         </is>
       </c>
     </row>
@@ -53978,7 +53978,7 @@
       </c>
       <c r="F46" s="45" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -54608,7 +54608,7 @@
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Sales Engineer only</t>
+          <t>Sales (non-AE) - Senior Client Success Manager only</t>
         </is>
       </c>
     </row>
@@ -56186,7 +56186,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/4/26)</t>
+          <t>Hiring AEs? (10/5/26)</t>
         </is>
       </c>
     </row>
@@ -57670,9 +57670,9 @@
           <t>Baggage handling systems and terminal logistics for airports</t>
         </is>
       </c>
-      <c r="F51" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -57702,7 +57702,7 @@
       </c>
       <c r="F52" s="51" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -57822,7 +57822,7 @@
       </c>
       <c r="F56" s="51" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -58572,7 +58572,7 @@
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
-          <t>Yes - Enterprise Account Executive (C1 - (Chicago, IL, Unite)</t>
+          <t>Yes - Enterprise Account Executive (C1 - (Austin, TX, United)</t>
         </is>
       </c>
     </row>
@@ -59050,7 +59050,7 @@
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
-          <t>Yes - Associate Account Executive (Cleve (Cleveland, Ohio, U)</t>
+          <t>Yes - Associate Account Executive (Atlan (Atlanta, Georgia, )</t>
         </is>
       </c>
     </row>
@@ -59710,7 +59710,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/4/26)</t>
+          <t>Hiring AEs? (10/5/26)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-10-06)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/5/26)</t>
+          <t>Hiring AEs? (10/6/26)</t>
         </is>
       </c>
     </row>
@@ -1122,7 +1122,7 @@
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Sr. Manager, FP&amp;A &amp; Sales Operatio only</t>
+          <t>Sales (non-AE) - Senior Customer Success Manager -  only</t>
         </is>
       </c>
     </row>
@@ -1362,7 +1362,7 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -3330,9 +3330,9 @@
           <t>Drone-as-first-responder software and hardware auto-launching to 911 calls</t>
         </is>
       </c>
-      <c r="F81" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F81" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Sales Development Representative ( only</t>
         </is>
       </c>
     </row>
@@ -5892,9 +5892,9 @@
           <t>Incident records and ePCR data platform for EMS and fire agencies - exhibited at IAFC FRI 2026</t>
         </is>
       </c>
-      <c r="F168" s="4" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F168" s="8" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -11088,7 +11088,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/5/26)</t>
+          <t>Hiring AEs? (10/6/26)</t>
         </is>
       </c>
     </row>
@@ -11800,7 +11800,7 @@
       </c>
       <c r="F26" s="65" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - GTM Strategy &amp; Operations Lead only</t>
+          <t>Sales (non-AE) - Customer Success Manager only</t>
         </is>
       </c>
     </row>
@@ -14372,7 +14372,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/5/26)</t>
+          <t>Hiring AEs? (10/6/26)</t>
         </is>
       </c>
     </row>
@@ -15036,9 +15036,9 @@
           <t>Academic scheduling, course demand analytics, and room and event management software for colleges and universities - exhibited at EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F24" s="71" t="inlineStr">
-        <is>
-          <t>Yes - Account Executive (Expansion) (Overland Park, KS,)</t>
+      <c r="F24" s="70" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Director of Client Success only</t>
         </is>
       </c>
     </row>
@@ -16978,7 +16978,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/5/26)</t>
+          <t>Hiring AEs? (10/6/26)</t>
         </is>
       </c>
     </row>
@@ -17446,7 +17446,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/5/26)</t>
+          <t>Hiring AEs? (10/6/26)</t>
         </is>
       </c>
     </row>
@@ -21314,7 +21314,7 @@
       </c>
       <c r="F131" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - no ATS on file</t>
         </is>
       </c>
     </row>
@@ -23830,7 +23830,7 @@
       </c>
       <c r="F216" s="15" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -24576,7 +24576,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/5/26)</t>
+          <t>Hiring AEs? (10/6/26)</t>
         </is>
       </c>
     </row>
@@ -24636,7 +24636,7 @@
       </c>
       <c r="F3" s="10" t="inlineStr">
         <is>
-          <t>Yes - Enterprise Account Executive - Col</t>
+          <t>Yes - Account Executive - New Logo - Nor</t>
         </is>
       </c>
     </row>
@@ -27230,9 +27230,9 @@
           <t>AI permitting and plan review: automated GIS/code compliance checks (Hernando County cut reviews 30 days to 2)</t>
         </is>
       </c>
-      <c r="F91" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F91" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -28104,7 +28104,7 @@
       </c>
       <c r="F121" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Executive - CES (London)</t>
+          <t>Yes - Business Development Manager (Brisbane)</t>
         </is>
       </c>
     </row>
@@ -29522,9 +29522,9 @@
           <t>Digital services and payments platform for state and local government - exhibited at GFOA 2026</t>
         </is>
       </c>
-      <c r="F169" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F169" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Client Success Manager (Northeast  only</t>
         </is>
       </c>
     </row>
@@ -30796,7 +30796,7 @@
       </c>
       <c r="F212" s="22" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (Singapore, Singapo)</t>
+          <t>Yes - Account Executive (London)</t>
         </is>
       </c>
     </row>
@@ -33506,9 +33506,9 @@
           <t>ChatGPT and the API, sold to public sector including named state and local government roles</t>
         </is>
       </c>
-      <c r="F304" s="23" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Account Director, Large Enterprise only</t>
+      <c r="F304" s="22" t="inlineStr">
+        <is>
+          <t>Yes - Business Development Manager, Prod (Munich, Germany)</t>
         </is>
       </c>
     </row>
@@ -36186,9 +36186,9 @@
           <t>Web-based mapping, demographic, and consumer data visualization application for university and public library patrons - exhibited at PLA 2026</t>
         </is>
       </c>
-      <c r="F397" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Senior Account Executive - B2B Saa</t>
+      <c r="F397" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -38634,7 +38634,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/5/26)</t>
+          <t>Hiring AEs? (10/6/26)</t>
         </is>
       </c>
     </row>
@@ -41472,9 +41472,9 @@
           <t>Weather data, alerting and decision tools for government agencies</t>
         </is>
       </c>
-      <c r="F96" s="27" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F96" s="28" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -42916,7 +42916,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/5/26)</t>
+          <t>Hiring AEs? (10/6/26)</t>
         </is>
       </c>
     </row>
@@ -42976,7 +42976,7 @@
       </c>
       <c r="F3" s="10" t="inlineStr">
         <is>
-          <t>Yes - Sales Executive, Cross-Sell (Utah  (Remote Worker - N/)</t>
+          <t>Yes - Sales Executive - Central Region (Remote Worker - N/)</t>
         </is>
       </c>
     </row>
@@ -47012,7 +47012,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/5/26)</t>
+          <t>Hiring AEs? (10/6/26)</t>
         </is>
       </c>
     </row>
@@ -50170,7 +50170,7 @@
       </c>
       <c r="F107" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Executive, Western Europe (Paris)</t>
+          <t>Yes - Principal Account Manager (Berlin)</t>
         </is>
       </c>
     </row>
@@ -52628,7 +52628,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/5/26)</t>
+          <t>Hiring AEs? (10/6/26)</t>
         </is>
       </c>
     </row>
@@ -54338,7 +54338,7 @@
       </c>
       <c r="F58" s="45" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -56186,7 +56186,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/5/26)</t>
+          <t>Hiring AEs? (10/6/26)</t>
         </is>
       </c>
     </row>
@@ -57702,7 +57702,7 @@
       </c>
       <c r="F52" s="51" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -58572,7 +58572,7 @@
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
-          <t>Yes - Enterprise Account Executive (C1 - (Austin, TX, United)</t>
+          <t>Yes - Enterprise Account Executive (C1 - (Dallas, TX, United)</t>
         </is>
       </c>
     </row>
@@ -59710,7 +59710,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/5/26)</t>
+          <t>Hiring AEs? (10/6/26)</t>
         </is>
       </c>
     </row>
@@ -60226,7 +60226,7 @@
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>Yes - Enterprise Account Executive (Stat (United States)</t>
+          <t>Yes - Enterprise Account Executive (Stat (New York, New York)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-10-07)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/6/26)</t>
+          <t>Hiring AEs? (10/7/26)</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2522,7 @@
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.365labs.com/car</t>
+          <t>Unknown - HTTP 202 for https://www.365labs.com/car</t>
         </is>
       </c>
     </row>
@@ -3092,7 +3092,7 @@
       </c>
       <c r="F73" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Executive, France (London)</t>
+          <t>Yes - Account Executive, Benelux (London)</t>
         </is>
       </c>
     </row>
@@ -3960,9 +3960,9 @@
           <t>Data platform unifying CAD/RMS/community data for officer context at dispatch</t>
         </is>
       </c>
-      <c r="F102" s="8" t="inlineStr">
-        <is>
-          <t>Yes - Regional Sales Manager FL area for</t>
+      <c r="F102" s="4" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -6284,7 +6284,7 @@
       </c>
       <c r="F181" s="10" t="inlineStr">
         <is>
-          <t>Yes - Mid-Market Account Executive</t>
+          <t>Yes - Enterprise Account Executive</t>
         </is>
       </c>
     </row>
@@ -7900,7 +7900,7 @@
       </c>
       <c r="F235" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 403 for https://www.keefegroup.com/</t>
         </is>
       </c>
     </row>
@@ -7930,7 +7930,7 @@
       </c>
       <c r="F236" s="4" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -11088,7 +11088,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/6/26)</t>
+          <t>Hiring AEs? (10/7/26)</t>
         </is>
       </c>
     </row>
@@ -13684,7 +13684,7 @@
       </c>
       <c r="F95" s="9" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Solutions Consultant only</t>
+          <t>Sales (non-AE) - Customer Success Manager only</t>
         </is>
       </c>
     </row>
@@ -14372,7 +14372,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/6/26)</t>
+          <t>Hiring AEs? (10/7/26)</t>
         </is>
       </c>
     </row>
@@ -14916,9 +14916,9 @@
           <t>No-code IT service management, asset management, project portfolio, and integration platform for universities, school districts, and government agencies - exhibited at EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F20" s="69" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F20" s="71" t="inlineStr">
+        <is>
+          <t>Yes - Enterprise Sales Executive, NY/PA (New York)</t>
         </is>
       </c>
     </row>
@@ -16978,7 +16978,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/6/26)</t>
+          <t>Hiring AEs? (10/7/26)</t>
         </is>
       </c>
     </row>
@@ -17446,7 +17446,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/6/26)</t>
+          <t>Hiring AEs? (10/7/26)</t>
         </is>
       </c>
     </row>
@@ -18922,7 +18922,7 @@
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Lead Salesforce Developer only</t>
+          <t>Sales (non-AE) - Vice President, Revenue Operations only</t>
         </is>
       </c>
     </row>
@@ -21282,9 +21282,9 @@
           <t>Water quality and level monitoring instruments for agencies and utilities - exhibited at AWWA ACE 2026, WEFTEC 2026, StormCon 2026</t>
         </is>
       </c>
-      <c r="F130" s="16" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F130" s="15" t="inlineStr">
+        <is>
+          <t>Unknown - HTTP 403 for https://in-situ.com/careers</t>
         </is>
       </c>
     </row>
@@ -23650,7 +23650,7 @@
       </c>
       <c r="F210" s="16" t="inlineStr">
         <is>
-          <t>Yes - Account Executive - New Business ( (Paris, Île-de-Fran)</t>
+          <t>Yes - Account Executive (new business de (Paris, Île-de-Fran)</t>
         </is>
       </c>
     </row>
@@ -23830,7 +23830,7 @@
       </c>
       <c r="F216" s="15" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -24576,7 +24576,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/6/26)</t>
+          <t>Hiring AEs? (10/7/26)</t>
         </is>
       </c>
     </row>
@@ -24846,7 +24846,7 @@
       </c>
       <c r="F10" s="21" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://zencity.io/careers</t>
+          <t>Unknown - HTTP 202 for https://zencity.io/careers</t>
         </is>
       </c>
     </row>
@@ -30796,7 +30796,7 @@
       </c>
       <c r="F212" s="22" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (London)</t>
+          <t>Yes - Account Executive (Singapore, Singapo)</t>
         </is>
       </c>
     </row>
@@ -30944,9 +30944,9 @@
           <t>Grantmaking and grants management platform for public funders</t>
         </is>
       </c>
-      <c r="F217" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F217" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Sr. Customer Success Manager only</t>
         </is>
       </c>
     </row>
@@ -31808,7 +31808,7 @@
       </c>
       <c r="F246" s="21" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://passportworkforce.c</t>
+          <t>Unknown - HTTP 202 for https://passportworkforce.c</t>
         </is>
       </c>
     </row>
@@ -34746,9 +34746,9 @@
           <t>Digital ballot scanning, tabulation and audit systems for election offices</t>
         </is>
       </c>
-      <c r="F347" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F347" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -35138,7 +35138,7 @@
       </c>
       <c r="F360" s="21" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 404 for https://www.easyvotesolutio</t>
+          <t>Unknown - HTTP 401 for https://www.easyvotesolutio</t>
         </is>
       </c>
     </row>
@@ -38634,7 +38634,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/6/26)</t>
+          <t>Hiring AEs? (10/7/26)</t>
         </is>
       </c>
     </row>
@@ -39048,7 +39048,7 @@
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (Shreveport, LA)</t>
+          <t>Yes - Account Executive (Memphis, TN)</t>
         </is>
       </c>
     </row>
@@ -39586,9 +39586,9 @@
           <t>Youth sports program, camp and league management software</t>
         </is>
       </c>
-      <c r="F33" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F33" s="10" t="inlineStr">
+        <is>
+          <t>Yes - Account Executive (INDIANAPOLIS, IN)</t>
         </is>
       </c>
     </row>
@@ -40186,9 +40186,9 @@
           <t>Campground reservation and management software for public and private campgrounds</t>
         </is>
       </c>
-      <c r="F53" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Manager, Account Management only</t>
+      <c r="F53" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -42916,7 +42916,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/6/26)</t>
+          <t>Hiring AEs? (10/7/26)</t>
         </is>
       </c>
     </row>
@@ -47012,7 +47012,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/6/26)</t>
+          <t>Hiring AEs? (10/7/26)</t>
         </is>
       </c>
     </row>
@@ -47312,7 +47312,7 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.modeshift.com/c</t>
+          <t>Unknown - HTTP 202 for https://www.modeshift.com/c</t>
         </is>
       </c>
     </row>
@@ -47578,7 +47578,7 @@
       </c>
       <c r="F20" s="39" t="inlineStr">
         <is>
-          <t>Yes - Senior Enterprise Account Executiv (Spain, Spain)</t>
+          <t>Yes - Technical Account Manager (Abu Dhabi, United )</t>
         </is>
       </c>
     </row>
@@ -47908,7 +47908,7 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.enghouse.com/ca</t>
+          <t>Unknown - HTTP 202 for https://www.enghouse.com/ca</t>
         </is>
       </c>
     </row>
@@ -49962,7 +49962,7 @@
       </c>
       <c r="F100" s="40" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.hanoverdisplays</t>
+          <t>Unknown - HTTP 202 for https://www.hanoverdisplays</t>
         </is>
       </c>
     </row>
@@ -50228,9 +50228,9 @@
           <t>AI microtransit and ADA paratransit operations: scheduling, dispatch, rider app, analytics - exhibited at CTAA EXPO 2026</t>
         </is>
       </c>
-      <c r="F109" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F109" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Senior Customer Success Manager only</t>
         </is>
       </c>
     </row>
@@ -50350,7 +50350,7 @@
       </c>
       <c r="F113" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://qryde.com/employmen</t>
+          <t>Unknown - HTTP 202 for https://qryde.com/employmen</t>
         </is>
       </c>
     </row>
@@ -52240,7 +52240,7 @@
       </c>
       <c r="F178" s="40" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.intangles.ai/ca</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -52628,7 +52628,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/6/26)</t>
+          <t>Hiring AEs? (10/7/26)</t>
         </is>
       </c>
     </row>
@@ -53138,7 +53138,7 @@
       </c>
       <c r="F18" s="45" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -54338,7 +54338,7 @@
       </c>
       <c r="F58" s="45" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 504 for https://www.sedata.com/care</t>
         </is>
       </c>
     </row>
@@ -56186,7 +56186,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/6/26)</t>
+          <t>Hiring AEs? (10/7/26)</t>
         </is>
       </c>
     </row>
@@ -59710,7 +59710,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/6/26)</t>
+          <t>Hiring AEs? (10/7/26)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-10-08)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/7/26)</t>
+          <t>Hiring AEs? (10/8/26)</t>
         </is>
       </c>
     </row>
@@ -2042,7 +2042,7 @@
       </c>
       <c r="F38" s="8" t="inlineStr">
         <is>
-          <t>Yes - Account Executive with German (Poland Offsite (ZP)</t>
+          <t>Yes - Senior Account Executive - Cyberse (Texas, US Offsite,)</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2522,7 @@
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://www.365labs.com/car</t>
+          <t>Unknown - HTTP 403 for https://www.365labs.com/car</t>
         </is>
       </c>
     </row>
@@ -3062,7 +3062,7 @@
       </c>
       <c r="F72" s="4" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 403 for https://www.milestonesys.co</t>
         </is>
       </c>
     </row>
@@ -5234,7 +5234,7 @@
       </c>
       <c r="F146" s="4" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 403 for https://www.briefcam.com/ca</t>
         </is>
       </c>
     </row>
@@ -6582,9 +6582,9 @@
           <t>911 call routing, Viper call handling and NG911 for PSAPs</t>
         </is>
       </c>
-      <c r="F191" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F191" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -7930,7 +7930,7 @@
       </c>
       <c r="F236" s="4" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - HTTP 504 for https://leotechnologies.com</t>
         </is>
       </c>
     </row>
@@ -11088,7 +11088,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/7/26)</t>
+          <t>Hiring AEs? (10/8/26)</t>
         </is>
       </c>
     </row>
@@ -13772,9 +13772,9 @@
           <t>Case management, intake, referral, and grant tracking software for public and nonprofit human services programs - exhibited at NatCon 2026, NACCHO 360 2026</t>
         </is>
       </c>
-      <c r="F98" s="64" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F98" s="63" t="inlineStr">
+        <is>
+          <t>Unknown - HTTP 403 for https://www.planstreet.com/</t>
         </is>
       </c>
     </row>
@@ -14372,7 +14372,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/7/26)</t>
+          <t>Hiring AEs? (10/8/26)</t>
         </is>
       </c>
     </row>
@@ -16978,7 +16978,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/7/26)</t>
+          <t>Hiring AEs? (10/8/26)</t>
         </is>
       </c>
     </row>
@@ -17220,7 +17220,7 @@
       </c>
       <c r="F10" s="75" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 403 for https://www.affordablehousi</t>
         </is>
       </c>
     </row>
@@ -17446,7 +17446,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/7/26)</t>
+          <t>Hiring AEs? (10/8/26)</t>
         </is>
       </c>
     </row>
@@ -23650,7 +23650,7 @@
       </c>
       <c r="F210" s="16" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (new business de (Paris, Île-de-Fran)</t>
+          <t>Yes - Senior Account Executive Net New - (Düsseldorf, North )</t>
         </is>
       </c>
     </row>
@@ -24576,7 +24576,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/7/26)</t>
+          <t>Hiring AEs? (10/8/26)</t>
         </is>
       </c>
     </row>
@@ -24846,7 +24846,7 @@
       </c>
       <c r="F10" s="21" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://zencity.io/careers</t>
+          <t>Unknown - HTTP 403 for https://zencity.io/careers</t>
         </is>
       </c>
     </row>
@@ -24936,7 +24936,7 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 403 for https://publicinput.com/car</t>
         </is>
       </c>
     </row>
@@ -28014,7 +28014,7 @@
       </c>
       <c r="F118" s="23" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Account Director only</t>
+          <t>Sales (non-AE) - Customer Success Manager only</t>
         </is>
       </c>
     </row>
@@ -28306,9 +28306,9 @@
           <t>Local government ERP: financials, property tax, assessing, utility billing - Michigan standard going national - exhibited at GFOA 2026</t>
         </is>
       </c>
-      <c r="F128" s="22" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F128" s="23" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -29524,7 +29524,7 @@
       </c>
       <c r="F169" s="9" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Client Success Manager (Northeast  only</t>
+          <t>Sales (non-AE) - Client Success Manager (Northeast) only</t>
         </is>
       </c>
     </row>
@@ -30004,7 +30004,7 @@
       </c>
       <c r="F185" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Executive/Enterprise Accou</t>
+          <t>Yes - Support Account Manager</t>
         </is>
       </c>
     </row>
@@ -30886,7 +30886,7 @@
       </c>
       <c r="F215" s="10" t="inlineStr">
         <is>
-          <t>Yes - Enterprise Account Executive (United States)</t>
+          <t>Yes - Enterprise Account Executive – Hea (United States)</t>
         </is>
       </c>
     </row>
@@ -31306,7 +31306,7 @@
       </c>
       <c r="F229" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (Credit Unions/B (Remote)</t>
+          <t>Yes - Sr. Account Executive (AI Solution (Remote)</t>
         </is>
       </c>
     </row>
@@ -31808,7 +31808,7 @@
       </c>
       <c r="F246" s="21" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://passportworkforce.c</t>
+          <t>Unknown - HTTP 403 for https://passportworkforce.c</t>
         </is>
       </c>
     </row>
@@ -35138,7 +35138,7 @@
       </c>
       <c r="F360" s="21" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 401 for https://www.easyvotesolutio</t>
+          <t>Unknown - HTTP 404 for https://www.easyvotesolutio</t>
         </is>
       </c>
     </row>
@@ -37510,9 +37510,9 @@
           <t>Government contract and procurement software - exhibited at NIGP 2026</t>
         </is>
       </c>
-      <c r="F445" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Founding Account Executive (New York City)</t>
+      <c r="F445" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - ruled out of scope by owner on 2026-08-24</t>
         </is>
       </c>
     </row>
@@ -38634,7 +38634,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/7/26)</t>
+          <t>Hiring AEs? (10/8/26)</t>
         </is>
       </c>
     </row>
@@ -40694,7 +40694,7 @@
       </c>
       <c r="F70" s="28" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 504 for https://www.weathermatic.co</t>
         </is>
       </c>
     </row>
@@ -42916,7 +42916,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/7/26)</t>
+          <t>Hiring AEs? (10/8/26)</t>
         </is>
       </c>
     </row>
@@ -42976,7 +42976,7 @@
       </c>
       <c r="F3" s="10" t="inlineStr">
         <is>
-          <t>Yes - Sales Executive - Central Region (Remote Worker - N/)</t>
+          <t>Yes - Sales Executive, Cross-Sell (Utah  (Remote Worker - N/)</t>
         </is>
       </c>
     </row>
@@ -43806,9 +43806,9 @@
           <t>InformaCast mass notification and paging for school districts</t>
         </is>
       </c>
-      <c r="F31" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -47012,7 +47012,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/7/26)</t>
+          <t>Hiring AEs? (10/8/26)</t>
         </is>
       </c>
     </row>
@@ -47312,7 +47312,7 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://www.modeshift.com/c</t>
+          <t>Unknown - HTTP 403 for https://www.modeshift.com/c</t>
         </is>
       </c>
     </row>
@@ -47908,7 +47908,7 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://www.enghouse.com/ca</t>
+          <t>Unknown - HTTP 403 for https://www.enghouse.com/ca</t>
         </is>
       </c>
     </row>
@@ -49032,7 +49032,7 @@
       </c>
       <c r="F69" s="10" t="inlineStr">
         <is>
-          <t>Yes - Enterprise Core Account Executive  (Remote)</t>
+          <t>Yes - Account Executive, Mid-Market (USA)</t>
         </is>
       </c>
     </row>
@@ -49962,7 +49962,7 @@
       </c>
       <c r="F100" s="40" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://www.hanoverdisplays</t>
+          <t>Unknown - HTTP 403 for https://www.hanoverdisplays</t>
         </is>
       </c>
     </row>
@@ -50350,7 +50350,7 @@
       </c>
       <c r="F113" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://qryde.com/employmen</t>
+          <t>Unknown - HTTP 403 for https://qryde.com/employmen</t>
         </is>
       </c>
     </row>
@@ -52628,7 +52628,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/7/26)</t>
+          <t>Hiring AEs? (10/8/26)</t>
         </is>
       </c>
     </row>
@@ -53798,7 +53798,7 @@
       </c>
       <c r="F40" s="45" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 403 for https://www.ledvance.com/en</t>
         </is>
       </c>
     </row>
@@ -54338,7 +54338,7 @@
       </c>
       <c r="F58" s="45" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 504 for https://www.sedata.com/care</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -54994,9 +54994,9 @@
           <t>Utility billing and customer information software for small and mid-size municipal water, sewer, and multi-service utilities - exhibited at AWWA ACE 2026, GFOA 2026</t>
         </is>
       </c>
-      <c r="F80" s="46" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F80" s="45" t="inlineStr">
+        <is>
+          <t>Unknown - HTTP 403 for https://cusi.com/careers/</t>
         </is>
       </c>
     </row>
@@ -56186,7 +56186,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/7/26)</t>
+          <t>Hiring AEs? (10/8/26)</t>
         </is>
       </c>
     </row>
@@ -57822,7 +57822,7 @@
       </c>
       <c r="F56" s="51" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -57970,9 +57970,9 @@
           <t>Airport IQ operations, property and lease management software for airports</t>
         </is>
       </c>
-      <c r="F61" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Senior Account Executive</t>
+      <c r="F61" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -58032,7 +58032,7 @@
       </c>
       <c r="F63" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 403 for https://www.grab.careers/en</t>
         </is>
       </c>
     </row>
@@ -58572,7 +58572,7 @@
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
-          <t>Yes - Enterprise Account Executive (C1 - (Dallas, TX, United)</t>
+          <t>Yes - Enterprise Account Executive (C1 - (Austin, TX, United)</t>
         </is>
       </c>
     </row>
@@ -59710,7 +59710,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/7/26)</t>
+          <t>Hiring AEs? (10/8/26)</t>
         </is>
       </c>
     </row>
@@ -60226,7 +60226,7 @@
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>Yes - Enterprise Account Executive (Stat (New York, New York)</t>
+          <t>Yes - Enterprise Account Executive (Stat (United States)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-10-10)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/9/26)</t>
+          <t>Hiring AEs? (10/10/26)</t>
         </is>
       </c>
     </row>
@@ -2732,7 +2732,7 @@
       </c>
       <c r="F61" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Executive - Public Sector  (Las Vegas, Nevada)</t>
+          <t>Yes - Account Executive (Sweden)</t>
         </is>
       </c>
     </row>
@@ -4788,9 +4788,9 @@
           <t>Software for first responder agencies - exhibited at IACP 2026, APCO 2026</t>
         </is>
       </c>
-      <c r="F131" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Account Executive (United States)</t>
+      <c r="F131" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -5774,7 +5774,7 @@
       </c>
       <c r="F164" s="4" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - robots.txt asks crawlers not to read www</t>
         </is>
       </c>
     </row>
@@ -5954,7 +5954,7 @@
       </c>
       <c r="F170" s="4" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.carbyne.com/car</t>
+          <t>Unknown - HTTP 403 for https://www.axon.com/career</t>
         </is>
       </c>
     </row>
@@ -7600,7 +7600,7 @@
       </c>
       <c r="F225" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 404 for https://www.cpcjail.com/car</t>
+          <t>Unknown - HTTP 404 for https://cpcjail.com/careers</t>
         </is>
       </c>
     </row>
@@ -7750,7 +7750,7 @@
       </c>
       <c r="F230" s="4" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://scramsystems.dejobs</t>
+          <t>Unknown - robots.txt on scramsystems.dejobs.org an</t>
         </is>
       </c>
     </row>
@@ -7900,7 +7900,7 @@
       </c>
       <c r="F235" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.keefegroup.com/</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -11088,7 +11088,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/9/26)</t>
+          <t>Hiring AEs? (10/10/26)</t>
         </is>
       </c>
     </row>
@@ -12498,7 +12498,7 @@
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: robots.txt on streamlineh</t>
         </is>
       </c>
     </row>
@@ -14372,7 +14372,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/9/26)</t>
+          <t>Hiring AEs? (10/10/26)</t>
         </is>
       </c>
     </row>
@@ -16978,7 +16978,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/9/26)</t>
+          <t>Hiring AEs? (10/10/26)</t>
         </is>
       </c>
     </row>
@@ -17446,7 +17446,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/9/26)</t>
+          <t>Hiring AEs? (10/10/26)</t>
         </is>
       </c>
     </row>
@@ -17476,7 +17476,7 @@
       </c>
       <c r="F2" s="15" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: robots.txt on www.rubicon</t>
         </is>
       </c>
     </row>
@@ -18042,9 +18042,9 @@
           <t>AI robotics and recovery analytics for material recovery facilities</t>
         </is>
       </c>
-      <c r="F21" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -19252,7 +19252,7 @@
       </c>
       <c r="F62" s="15" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://one.network/careers</t>
+          <t>Unknown - robots.txt asks crawlers not to read one</t>
         </is>
       </c>
     </row>
@@ -21282,9 +21282,9 @@
           <t>Water quality and level monitoring instruments for agencies and utilities - exhibited at AWWA ACE 2026, WEFTEC 2026, StormCon 2026</t>
         </is>
       </c>
-      <c r="F130" s="15" t="inlineStr">
-        <is>
-          <t>Unknown - HTTP 403 for https://in-situ.com/careers</t>
+      <c r="F130" s="16" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -21494,7 +21494,7 @@
       </c>
       <c r="F137" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.syrinix.com/car</t>
+          <t>Unknown - HTTP 403 for https://www.badgermeter.com</t>
         </is>
       </c>
     </row>
@@ -23414,7 +23414,7 @@
       </c>
       <c r="F202" s="15" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - robots.txt asks crawlers not to read www</t>
         </is>
       </c>
     </row>
@@ -23560,7 +23560,7 @@
       </c>
       <c r="F207" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://careers.jacobs.com</t>
+          <t>Unknown - robots.txt on careers.jacobs.com answere</t>
         </is>
       </c>
     </row>
@@ -23650,7 +23650,7 @@
       </c>
       <c r="F210" s="16" t="inlineStr">
         <is>
-          <t>Yes - Senior Account Executive Net New - (Düsseldorf, North )</t>
+          <t>Yes - Strategic Account Executive – Aero (Warsaw, Mazovia)</t>
         </is>
       </c>
     </row>
@@ -23830,7 +23830,7 @@
       </c>
       <c r="F216" s="15" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 504 for https://eptura.com/careers</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -24576,7 +24576,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/9/26)</t>
+          <t>Hiring AEs? (10/10/26)</t>
         </is>
       </c>
     </row>
@@ -25056,7 +25056,7 @@
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.revize.com/care</t>
+          <t>Unknown - robots.txt asks crawlers not to read www</t>
         </is>
       </c>
     </row>
@@ -29524,9 +29524,9 @@
           <t>Bill presentment and payments for governments and utilities (public co) - exhibited at GFOA 2026, NAHRO 2026, EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F169" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F169" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - network error: robots.txt on www.payment</t>
         </is>
       </c>
     </row>
@@ -29646,7 +29646,7 @@
       </c>
       <c r="F173" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 405 for https://planetbids.com/care</t>
+          <t>Unknown - HTTP 405 for https://files-prod01.planet</t>
         </is>
       </c>
     </row>
@@ -30768,7 +30768,7 @@
       </c>
       <c r="F211" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (London)</t>
+          <t>Yes - Account Executive (Denmark)</t>
         </is>
       </c>
     </row>
@@ -31218,7 +31218,7 @@
       </c>
       <c r="F226" s="21" t="inlineStr">
         <is>
-          <t>Unknown - board is another company's - not read</t>
+          <t>Unknown - robots.txt asks crawlers not to read www</t>
         </is>
       </c>
     </row>
@@ -32522,7 +32522,7 @@
       </c>
       <c r="F270" s="21" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 404 for https://harrislocalgov.com/</t>
+          <t>Unknown - HTTP 404 for https://www.harrislocalgov.</t>
         </is>
       </c>
     </row>
@@ -32788,7 +32788,7 @@
       </c>
       <c r="F279" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - robots.txt asks crawlers not to read rec</t>
         </is>
       </c>
     </row>
@@ -34222,7 +34222,7 @@
       </c>
       <c r="F329" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: robots.txt on www.maxar.c</t>
         </is>
       </c>
     </row>
@@ -35750,7 +35750,7 @@
       </c>
       <c r="F381" s="9" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Strategic Account Director only</t>
+          <t>Sales (non-AE) - Strategic Account Director -Wester only</t>
         </is>
       </c>
     </row>
@@ -37212,7 +37212,7 @@
       </c>
       <c r="F434" s="21" t="inlineStr">
         <is>
-          <t>Unknown - board is another company's - not read</t>
+          <t>Unknown - network error: robots.txt on careers.act</t>
         </is>
       </c>
     </row>
@@ -38606,7 +38606,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/9/26)</t>
+          <t>Hiring AEs? (10/10/26)</t>
         </is>
       </c>
     </row>
@@ -42888,7 +42888,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/9/26)</t>
+          <t>Hiring AEs? (10/10/26)</t>
         </is>
       </c>
     </row>
@@ -43008,7 +43008,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.evolvtechnology</t>
+          <t>Unknown - HTTP 403 for https://evolv.com/careers</t>
         </is>
       </c>
     </row>
@@ -44522,7 +44522,7 @@
       </c>
       <c r="F56" s="34" t="inlineStr">
         <is>
-          <t>Unknown - network error: Exceeded 30 redirects.</t>
+          <t>Unknown - more than 10 redirects from https://www.</t>
         </is>
       </c>
     </row>
@@ -45570,7 +45570,7 @@
       </c>
       <c r="F91" s="10" t="inlineStr">
         <is>
-          <t>Yes - Sales Executive (Remote Worker - N/)</t>
+          <t>Yes - Senior Account Executive — Payment</t>
         </is>
       </c>
     </row>
@@ -46984,7 +46984,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/9/26)</t>
+          <t>Hiring AEs? (10/10/26)</t>
         </is>
       </c>
     </row>
@@ -48114,7 +48114,7 @@
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - more than 10 redirects from https://wi-t</t>
         </is>
       </c>
     </row>
@@ -48734,7 +48734,7 @@
       </c>
       <c r="F60" s="40" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: robots.txt on www.gatekee</t>
         </is>
       </c>
     </row>
@@ -49062,9 +49062,9 @@
           <t>Fleet maintenance software for cities, counties and transit agencies</t>
         </is>
       </c>
-      <c r="F71" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Account Executive (Remote Worker)</t>
+      <c r="F71" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -51624,7 +51624,7 @@
       </c>
       <c r="F157" s="10" t="inlineStr">
         <is>
-          <t>Yes - Junior B2B Account Executive (Prague)</t>
+          <t>Yes - B2B Account Manager (Oslo)</t>
         </is>
       </c>
     </row>
@@ -51654,7 +51654,7 @@
       </c>
       <c r="F158" s="40" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - network error: robots.txt on www.pom.com</t>
         </is>
       </c>
     </row>
@@ -52600,7 +52600,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/9/26)</t>
+          <t>Hiring AEs? (10/10/26)</t>
         </is>
       </c>
     </row>
@@ -54578,9 +54578,9 @@
           <t>DERMS and virtual power plant programs for utilities including public power</t>
         </is>
       </c>
-      <c r="F67" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Senior Client Success Manager only</t>
+      <c r="F67" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -55262,7 +55262,7 @@
       </c>
       <c r="F90" s="47" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Head of Sales only</t>
+          <t>Sales (non-AE) - Intern, Business Development Assoc only</t>
         </is>
       </c>
     </row>
@@ -56066,7 +56066,7 @@
       </c>
       <c r="F117" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 404 for https://sifinetworks.com/co</t>
+          <t>Unknown - HTTP 404 for http://www.arclinkfiber.com</t>
         </is>
       </c>
     </row>
@@ -56158,7 +56158,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/9/26)</t>
+          <t>Hiring AEs? (10/10/26)</t>
         </is>
       </c>
     </row>
@@ -57642,9 +57642,9 @@
           <t>Baggage handling systems and terminal logistics for airports</t>
         </is>
       </c>
-      <c r="F51" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F51" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -57824,7 +57824,7 @@
       </c>
       <c r="F57" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page too small - likely JS-rendered</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -58452,9 +58452,9 @@
           <t>Explosive and chemical trace detection instruments for aviation security</t>
         </is>
       </c>
-      <c r="F78" s="52" t="inlineStr">
-        <is>
-          <t>Yes - Sales Account Manager</t>
+      <c r="F78" s="51" t="inlineStr">
+        <is>
+          <t>Unknown - robots.txt asks crawlers not to read wor</t>
         </is>
       </c>
     </row>
@@ -58484,7 +58484,7 @@
       </c>
       <c r="F79" s="9" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Sales Manager - Smart Biometrics only</t>
+          <t>Sales (non-AE) - Business Operations and Leadership only</t>
         </is>
       </c>
     </row>
@@ -58572,9 +58572,9 @@
           <t>Airport threat detection AI and biometric travel systems for government</t>
         </is>
       </c>
-      <c r="F82" s="53" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - USAF and USSF (US Space Force) Str only</t>
+      <c r="F82" s="51" t="inlineStr">
+        <is>
+          <t>Unknown - robots.txt asks crawlers not to read int</t>
         </is>
       </c>
     </row>
@@ -58962,7 +58962,7 @@
       </c>
       <c r="F95" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - robots.txt asks crawlers not to read www</t>
         </is>
       </c>
     </row>
@@ -59682,7 +59682,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/9/26)</t>
+          <t>Hiring AEs? (10/10/26)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-10-13)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/10/26)</t>
+          <t>Hiring AEs? (10/13/26)</t>
         </is>
       </c>
     </row>
@@ -4790,7 +4790,7 @@
       </c>
       <c r="F131" s="7" t="inlineStr">
         <is>
-          <t>None found</t>
+          <t>Unknown - HTTP 404 for https://api.ashbyhq.com/pos</t>
         </is>
       </c>
     </row>
@@ -7930,7 +7930,7 @@
       </c>
       <c r="F236" s="4" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -11088,7 +11088,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/10/26)</t>
+          <t>Hiring AEs? (10/13/26)</t>
         </is>
       </c>
     </row>
@@ -12498,7 +12498,7 @@
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>Unknown - network error: robots.txt on streamlineh</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -12936,7 +12936,7 @@
       </c>
       <c r="F67" s="10" t="inlineStr">
         <is>
-          <t>Yes - Senior Account Executive (Remote)</t>
+          <t>Yes - Account Executive (Remote)</t>
         </is>
       </c>
     </row>
@@ -14372,7 +14372,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/10/26)</t>
+          <t>Hiring AEs? (10/13/26)</t>
         </is>
       </c>
     </row>
@@ -16600,9 +16600,9 @@
           <t>Argos reporting, FormFusion document automation and IntelleCheck payment software built for higher education administrative systems - exhibited at EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F82" s="69" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F82" s="71" t="inlineStr">
+        <is>
+          <t>Yes - Account Executive (Houston, Texas, Un)</t>
         </is>
       </c>
     </row>
@@ -16978,7 +16978,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/10/26)</t>
+          <t>Hiring AEs? (10/13/26)</t>
         </is>
       </c>
     </row>
@@ -17446,7 +17446,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/10/26)</t>
+          <t>Hiring AEs? (10/13/26)</t>
         </is>
       </c>
     </row>
@@ -20984,7 +20984,7 @@
       </c>
       <c r="F120" s="16" t="inlineStr">
         <is>
-          <t>Yes - Account Executive - Government Wes (Remote)</t>
+          <t>Yes - Account Executive - Government (We (Remote)</t>
         </is>
       </c>
     </row>
@@ -21282,9 +21282,9 @@
           <t>Water quality and level monitoring instruments for agencies and utilities - exhibited at AWWA ACE 2026, WEFTEC 2026, StormCon 2026</t>
         </is>
       </c>
-      <c r="F130" s="16" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F130" s="15" t="inlineStr">
+        <is>
+          <t>Unknown - HTTP 403 for https://in-situ.com/careers</t>
         </is>
       </c>
     </row>
@@ -22464,7 +22464,7 @@
       </c>
       <c r="F170" s="15" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 404 for https://baseform.com/np4/ca</t>
         </is>
       </c>
     </row>
@@ -23650,7 +23650,7 @@
       </c>
       <c r="F210" s="16" t="inlineStr">
         <is>
-          <t>Yes - Strategic Account Executive – Aero (Warsaw, Mazovia)</t>
+          <t>Yes - Senior Account Executive, Aerospac (Itasca, Illinois)</t>
         </is>
       </c>
     </row>
@@ -23830,7 +23830,7 @@
       </c>
       <c r="F216" s="15" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 504 for https://eptura.com/careers/</t>
         </is>
       </c>
     </row>
@@ -24576,7 +24576,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/10/26)</t>
+          <t>Hiring AEs? (10/13/26)</t>
         </is>
       </c>
     </row>
@@ -26180,9 +26180,9 @@
           <t>CodeRED public alerting and critical event management for local jurisdictions</t>
         </is>
       </c>
-      <c r="F55" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F55" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -27986,7 +27986,7 @@
       </c>
       <c r="F117" s="9" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Customer Success Manager only</t>
+          <t>Sales (non-AE) - Account Director only</t>
         </is>
       </c>
     </row>
@@ -28076,7 +28076,7 @@
       </c>
       <c r="F120" s="22" t="inlineStr">
         <is>
-          <t>Yes - Business Development Manager (Brisbane)</t>
+          <t>Yes - Account Manager - Medical Billing (Amersham)</t>
         </is>
       </c>
     </row>
@@ -28188,9 +28188,9 @@
           <t>Procurement, budgeting, and grants suite - Bonfire, Questica, eCivis (formerly GTY) - exhibited at NACUBO 2026, GFOA 2026</t>
         </is>
       </c>
-      <c r="F124" s="23" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Solutions Consultant only</t>
+      <c r="F124" s="22" t="inlineStr">
+        <is>
+          <t>Yes - Account Executive - Payments (United States)</t>
         </is>
       </c>
     </row>
@@ -28368,9 +28368,9 @@
           <t>Cloud treasury: debt management, GASB 87/96 lease accounting, and cash management for gov finance - exhibited at NACUBO 2026, GFOA 2026</t>
         </is>
       </c>
-      <c r="F130" s="22" t="inlineStr">
-        <is>
-          <t>Yes - Enterprise Account Executive (Charlotte, NC)</t>
+      <c r="F130" s="21" t="inlineStr">
+        <is>
+          <t>Unknown - HTTP 404 for https://boards-api.greenhou</t>
         </is>
       </c>
     </row>
@@ -29524,9 +29524,9 @@
           <t>Bill presentment and payments for governments and utilities (public co) - exhibited at GFOA 2026, NAHRO 2026, EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F169" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - network error: robots.txt on www.payment</t>
+      <c r="F169" s="10" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -30768,7 +30768,7 @@
       </c>
       <c r="F211" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (Denmark)</t>
+          <t>Yes - Account Executive (London)</t>
         </is>
       </c>
     </row>
@@ -38606,7 +38606,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/10/26)</t>
+          <t>Hiring AEs? (10/13/26)</t>
         </is>
       </c>
     </row>
@@ -39020,7 +39020,7 @@
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (Memphis, TN)</t>
+          <t>Yes - Account Executive (Wildomar, CA)</t>
         </is>
       </c>
     </row>
@@ -42888,7 +42888,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/10/26)</t>
+          <t>Hiring AEs? (10/13/26)</t>
         </is>
       </c>
     </row>
@@ -45418,9 +45418,9 @@
           <t>School bus routing, fleet and student transportation software for districts</t>
         </is>
       </c>
-      <c r="F86" s="35" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F86" s="34" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -46984,7 +46984,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/10/26)</t>
+          <t>Hiring AEs? (10/13/26)</t>
         </is>
       </c>
     </row>
@@ -47162,9 +47162,9 @@
           <t>Contactless open-loop transit payment infrastructure for 400+ providers in 30+ countries</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>Yes - Senior Business Development Manage (London)</t>
         </is>
       </c>
     </row>
@@ -47400,7 +47400,7 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: robots.txt on www.pptexce</t>
         </is>
       </c>
     </row>
@@ -47548,9 +47548,9 @@
           <t>Account-based fare collection and validators for public transit operators</t>
         </is>
       </c>
-      <c r="F20" s="39" t="inlineStr">
-        <is>
-          <t>Yes - Technical Account Manager (Abu Dhabi, United )</t>
+      <c r="F20" s="40" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -51174,7 +51174,7 @@
       </c>
       <c r="F142" s="40" t="inlineStr">
         <is>
-          <t>None found</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -52600,7 +52600,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/10/26)</t>
+          <t>Hiring AEs? (10/13/26)</t>
         </is>
       </c>
     </row>
@@ -54310,7 +54310,7 @@
       </c>
       <c r="F58" s="45" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -54938,7 +54938,7 @@
       </c>
       <c r="F79" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: robots.txt on www.advance</t>
         </is>
       </c>
     </row>
@@ -56158,7 +56158,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/10/26)</t>
+          <t>Hiring AEs? (10/13/26)</t>
         </is>
       </c>
     </row>
@@ -57642,9 +57642,9 @@
           <t>Baggage handling systems and terminal logistics for airports</t>
         </is>
       </c>
-      <c r="F51" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -58242,9 +58242,9 @@
           <t>Ascento Guard autonomous outdoor security robot sold as robot-as-a-service: wheeled-legged patrol unit with thermal/RGB cameras plus AI software for perimeter patrol, intruder detection and site inspection.</t>
         </is>
       </c>
-      <c r="F71" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F71" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Business Development: French-Speak only</t>
         </is>
       </c>
     </row>
@@ -58544,7 +58544,7 @@
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
-          <t>Yes - Enterprise Account Executive (C1 - (Austin, TX, United)</t>
+          <t>Yes - Enterprise Account Executive (C1 - (New York, New York)</t>
         </is>
       </c>
     </row>
@@ -59682,7 +59682,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/10/26)</t>
+          <t>Hiring AEs? (10/13/26)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-10-14)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/13/26)</t>
+          <t>Hiring AEs? (10/14/26)</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2522,7 @@
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.365labs.com/car</t>
+          <t>Unknown - robots.txt on www.365labs.com answered H</t>
         </is>
       </c>
     </row>
@@ -2912,7 +2912,7 @@
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Account Director, Public Sector (D only</t>
+          <t>Sales (non-AE) - Customer Success Manager only</t>
         </is>
       </c>
     </row>
@@ -5382,9 +5382,9 @@
           <t>FBI-certified mobile fingerprint scanners for police and government</t>
         </is>
       </c>
-      <c r="F151" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F151" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -7930,7 +7930,7 @@
       </c>
       <c r="F236" s="4" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -8758,7 +8758,7 @@
       </c>
       <c r="F264" s="4" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -10612,9 +10612,9 @@
           <t>DigiTICKET electronic citation software - exhibited at IACP 2026</t>
         </is>
       </c>
-      <c r="F336" s="11" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F336" s="4" t="inlineStr">
+        <is>
+          <t>Unknown - network error: robots.txt on saltustechn</t>
         </is>
       </c>
     </row>
@@ -11088,7 +11088,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/13/26)</t>
+          <t>Hiring AEs? (10/14/26)</t>
         </is>
       </c>
     </row>
@@ -14372,7 +14372,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/13/26)</t>
+          <t>Hiring AEs? (10/14/26)</t>
         </is>
       </c>
     </row>
@@ -16916,7 +16916,7 @@
       </c>
       <c r="F93" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 504 for https://www.graydi.us/caree</t>
         </is>
       </c>
     </row>
@@ -16978,7 +16978,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/13/26)</t>
+          <t>Hiring AEs? (10/14/26)</t>
         </is>
       </c>
     </row>
@@ -17446,7 +17446,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/13/26)</t>
+          <t>Hiring AEs? (10/14/26)</t>
         </is>
       </c>
     </row>
@@ -20742,9 +20742,9 @@
           <t>AI pipe-failure prediction for main replacement planning - exhibited at AWWA ACE 2026</t>
         </is>
       </c>
-      <c r="F112" s="16" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F112" s="15" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -23830,7 +23830,7 @@
       </c>
       <c r="F216" s="15" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 504 for https://eptura.com/careers/</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -24576,7 +24576,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/13/26)</t>
+          <t>Hiring AEs? (10/14/26)</t>
         </is>
       </c>
     </row>
@@ -24846,7 +24846,7 @@
       </c>
       <c r="F10" s="21" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://zencity.io/careers</t>
+          <t>Unknown - robots.txt on zencity.io answered HTTP 2</t>
         </is>
       </c>
     </row>
@@ -26180,9 +26180,9 @@
           <t>CodeRED public alerting and critical event management for local jurisdictions</t>
         </is>
       </c>
-      <c r="F55" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F55" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -31780,7 +31780,7 @@
       </c>
       <c r="F245" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://passportworkforce.c</t>
+          <t>Unknown - robots.txt on passportworkforce.com answ</t>
         </is>
       </c>
     </row>
@@ -38606,7 +38606,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/13/26)</t>
+          <t>Hiring AEs? (10/14/26)</t>
         </is>
       </c>
     </row>
@@ -39020,7 +39020,7 @@
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (Wildomar, CA)</t>
+          <t>Yes - Account Executive (Fresno, CA)</t>
         </is>
       </c>
     </row>
@@ -41386,7 +41386,7 @@
       </c>
       <c r="F94" s="29" t="inlineStr">
         <is>
-          <t>Yes - Sales Executive (2 Locations)</t>
+          <t>Yes - Account Executive - Agriculture (4 Locations)</t>
         </is>
       </c>
     </row>
@@ -42192,9 +42192,9 @@
           <t>Event management SaaS: vendor applications, ticketing, maps, and sponsors for festivals and city events</t>
         </is>
       </c>
-      <c r="F121" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Enterprise Account Executive</t>
+      <c r="F121" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Account Strategist only</t>
         </is>
       </c>
     </row>
@@ -42888,7 +42888,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/13/26)</t>
+          <t>Hiring AEs? (10/14/26)</t>
         </is>
       </c>
     </row>
@@ -43452,7 +43452,7 @@
       </c>
       <c r="F20" s="35" t="inlineStr">
         <is>
-          <t>Yes - Commercial Account Executive - Cen (Denver, Colorado)</t>
+          <t>Yes - Commercial Account Executive - Cen (Denver, CO)</t>
         </is>
       </c>
     </row>
@@ -46984,7 +46984,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/13/26)</t>
+          <t>Hiring AEs? (10/14/26)</t>
         </is>
       </c>
     </row>
@@ -47284,7 +47284,7 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.modeshift.com/c</t>
+          <t>Unknown - robots.txt on www.modeshift.com answered</t>
         </is>
       </c>
     </row>
@@ -47400,7 +47400,7 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Unknown - network error: robots.txt on www.pptexce</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -47880,7 +47880,7 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.enghouse.com/ca</t>
+          <t xml:space="preserve">Unknown - robots.txt on www.enghouse.com answered </t>
         </is>
       </c>
     </row>
@@ -49872,9 +49872,9 @@
           <t>Destination signs, LED/LCD passenger displays, onboard infotainment, and CCTV for bus and rail</t>
         </is>
       </c>
-      <c r="F98" s="41" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Sales Backoffice Specialist only</t>
+      <c r="F98" s="39" t="inlineStr">
+        <is>
+          <t>Yes - Area Sales Manager - Middle German</t>
         </is>
       </c>
     </row>
@@ -49934,7 +49934,7 @@
       </c>
       <c r="F100" s="40" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.hanoverdisplays</t>
+          <t>Unknown - robots.txt on www.hanoverdisplays.com an</t>
         </is>
       </c>
     </row>
@@ -50322,7 +50322,7 @@
       </c>
       <c r="F113" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://qryde.com/employmen</t>
+          <t>Unknown - robots.txt on qryde.com answered HTTP 20</t>
         </is>
       </c>
     </row>
@@ -51382,9 +51382,9 @@
           <t>Smart single-space parking meters and enforcement systems</t>
         </is>
       </c>
-      <c r="F149" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F149" s="10" t="inlineStr">
+        <is>
+          <t>Yes - Regional Account Executive (San Diego, Califor)</t>
         </is>
       </c>
     </row>
@@ -52600,7 +52600,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/13/26)</t>
+          <t>Hiring AEs? (10/14/26)</t>
         </is>
       </c>
     </row>
@@ -54218,9 +54218,9 @@
           <t>SCADA, ADMS and outage management for municipal utilities and co-ops</t>
         </is>
       </c>
-      <c r="F55" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F55" s="10" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -54938,7 +54938,7 @@
       </c>
       <c r="F79" s="7" t="inlineStr">
         <is>
-          <t>Unknown - network error: robots.txt on www.advance</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -56158,7 +56158,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/13/26)</t>
+          <t>Hiring AEs? (10/14/26)</t>
         </is>
       </c>
     </row>
@@ -57794,7 +57794,7 @@
       </c>
       <c r="F56" s="51" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: robots.txt on www.elenium</t>
         </is>
       </c>
     </row>
@@ -58544,7 +58544,7 @@
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
-          <t>Yes - Enterprise Account Executive (C1 - (New York, New York)</t>
+          <t>Yes - Enterprise Account Executive (C1 - (Dallas, TX, United)</t>
         </is>
       </c>
     </row>
@@ -59682,7 +59682,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/13/26)</t>
+          <t>Hiring AEs? (10/14/26)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-10-15)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/14/26)</t>
+          <t>Hiring AEs? (10/15/26)</t>
         </is>
       </c>
     </row>
@@ -2912,7 +2912,7 @@
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Customer Success Manager only</t>
+          <t>Sales (non-AE) - Account Director, Financial Instit only</t>
         </is>
       </c>
     </row>
@@ -4112,7 +4112,7 @@
       </c>
       <c r="F107" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 500 for https://safience.io/careers</t>
         </is>
       </c>
     </row>
@@ -4740,7 +4740,7 @@
       </c>
       <c r="F129" s="10" t="inlineStr">
         <is>
-          <t>Yes - Enterprise Account Manager (Auror London Offic)</t>
+          <t>Yes - Enterprise Account Manager (12-mon (Auror London Offic)</t>
         </is>
       </c>
     </row>
@@ -10612,9 +10612,9 @@
           <t>DigiTICKET electronic citation software - exhibited at IACP 2026</t>
         </is>
       </c>
-      <c r="F336" s="4" t="inlineStr">
-        <is>
-          <t>Unknown - network error: robots.txt on saltustechn</t>
+      <c r="F336" s="11" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -11088,7 +11088,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/14/26)</t>
+          <t>Hiring AEs? (10/15/26)</t>
         </is>
       </c>
     </row>
@@ -14372,7 +14372,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/14/26)</t>
+          <t>Hiring AEs? (10/15/26)</t>
         </is>
       </c>
     </row>
@@ -14978,7 +14978,7 @@
       </c>
       <c r="F22" s="70" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Sales Support - Keyholder only</t>
+          <t>Sales (non-AE) - Sales Support only</t>
         </is>
       </c>
     </row>
@@ -16338,7 +16338,7 @@
       </c>
       <c r="F72" s="70" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Senior Solutions Engineer only</t>
+          <t>Sales (non-AE) - Vice President, Sales only</t>
         </is>
       </c>
     </row>
@@ -16916,7 +16916,7 @@
       </c>
       <c r="F93" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 504 for https://www.graydi.us/caree</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -16978,7 +16978,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/14/26)</t>
+          <t>Hiring AEs? (10/15/26)</t>
         </is>
       </c>
     </row>
@@ -17446,7 +17446,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/14/26)</t>
+          <t>Hiring AEs? (10/15/26)</t>
         </is>
       </c>
     </row>
@@ -19732,7 +19732,7 @@
       </c>
       <c r="F78" s="15" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 403 for https://www.q-free.com/care</t>
         </is>
       </c>
     </row>
@@ -20832,9 +20832,9 @@
           <t>AI defect detection and coding for sewer inspection video - exhibited at AWWA ACE 2026, WEFTEC 2026</t>
         </is>
       </c>
-      <c r="F115" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Account Executive, Enterprise (Remote)</t>
+      <c r="F115" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Revenue Operations Analyst only</t>
         </is>
       </c>
     </row>
@@ -20984,7 +20984,7 @@
       </c>
       <c r="F120" s="16" t="inlineStr">
         <is>
-          <t>Yes - Account Executive - Government (We (Remote)</t>
+          <t>Yes - Account Executive - Engineering Fi (Remote)</t>
         </is>
       </c>
     </row>
@@ -23022,9 +23022,9 @@
           <t>Unity AIoT fleet intelligence (incl. MiX Telematics, Fleet Complete) for enterprise and gov fleets</t>
         </is>
       </c>
-      <c r="F189" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F189" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -23650,7 +23650,7 @@
       </c>
       <c r="F210" s="16" t="inlineStr">
         <is>
-          <t>Yes - Senior Account Executive, Aerospac (Itasca, Illinois)</t>
+          <t>Yes - Sales Executive - Industrial Intel (Düsseldorf, North )</t>
         </is>
       </c>
     </row>
@@ -24576,7 +24576,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/14/26)</t>
+          <t>Hiring AEs? (10/15/26)</t>
         </is>
       </c>
     </row>
@@ -26062,7 +26062,7 @@
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 403 for https://www.civicplus.com/c</t>
         </is>
       </c>
     </row>
@@ -26150,9 +26150,9 @@
           <t>Emergency and routine mass notification for cities, counties and schools</t>
         </is>
       </c>
-      <c r="F54" s="23" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Customer Success Manager only</t>
+      <c r="F54" s="22" t="inlineStr">
+        <is>
+          <t>Yes - Saas Account Executive</t>
         </is>
       </c>
     </row>
@@ -30768,7 +30768,7 @@
       </c>
       <c r="F211" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (London)</t>
+          <t>Yes - Account Executive (Singapore, Singapo)</t>
         </is>
       </c>
     </row>
@@ -34194,7 +34194,7 @@
       </c>
       <c r="F328" s="21" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: robots.txt on www.planet.</t>
         </is>
       </c>
     </row>
@@ -34720,7 +34720,7 @@
       </c>
       <c r="F346" s="21" t="inlineStr">
         <is>
-          <t>None found</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -38606,7 +38606,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/14/26)</t>
+          <t>Hiring AEs? (10/15/26)</t>
         </is>
       </c>
     </row>
@@ -39020,7 +39020,7 @@
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (Fresno, CA)</t>
+          <t>Yes - Account Executive (Marble Falls, TX)</t>
         </is>
       </c>
     </row>
@@ -42888,7 +42888,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/14/26)</t>
+          <t>Hiring AEs? (10/15/26)</t>
         </is>
       </c>
     </row>
@@ -44044,9 +44044,9 @@
           <t>Gamified phishing simulation and security awareness training built only for K-12 districts, staff and students - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F40" s="34" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F40" s="35" t="inlineStr">
+        <is>
+          <t>Yes - Account Executive - West (United States (Rem)</t>
         </is>
       </c>
     </row>
@@ -46984,7 +46984,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/14/26)</t>
+          <t>Hiring AEs? (10/15/26)</t>
         </is>
       </c>
     </row>
@@ -47880,7 +47880,7 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unknown - robots.txt on www.enghouse.com answered </t>
+          <t>Unknown - HTTP 202 for https://www.enghouse.com/ca</t>
         </is>
       </c>
     </row>
@@ -50200,9 +50200,9 @@
           <t>AI microtransit and ADA paratransit operations: scheduling, dispatch, rider app, analytics - exhibited at CTAA EXPO 2026</t>
         </is>
       </c>
-      <c r="F109" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Senior Customer Success Manager only</t>
+      <c r="F109" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -52162,7 +52162,7 @@
       </c>
       <c r="F176" s="40" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -52600,7 +52600,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/14/26)</t>
+          <t>Hiring AEs? (10/15/26)</t>
         </is>
       </c>
     </row>
@@ -56158,7 +56158,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/14/26)</t>
+          <t>Hiring AEs? (10/15/26)</t>
         </is>
       </c>
     </row>
@@ -58544,7 +58544,7 @@
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
-          <t>Yes - Enterprise Account Executive (C1 - (Dallas, TX, United)</t>
+          <t>Yes - Enterprise Account Executive (C1 - (Chicago, IL, Unite)</t>
         </is>
       </c>
     </row>
@@ -59168,9 +59168,9 @@
           <t>Cloud parking OS and reservations for airports, cities and venues</t>
         </is>
       </c>
-      <c r="F102" s="53" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Estimator, Inside Sales only</t>
+      <c r="F102" s="51" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -59682,7 +59682,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/14/26)</t>
+          <t>Hiring AEs? (10/15/26)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-10-16)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/15/26)</t>
+          <t>Hiring AEs? (10/16/26)</t>
         </is>
       </c>
     </row>
@@ -1650,9 +1650,9 @@
           <t>Satellite vegetation intelligence for wildfire risk at utilities and agencies</t>
         </is>
       </c>
-      <c r="F25" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Enterprise Account Executive, Cana (Remote, Canada)</t>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -2162,7 +2162,7 @@
       </c>
       <c r="F42" s="8" t="inlineStr">
         <is>
-          <t>Yes - Strategic Account Executive (CO, N (CO, NM, UT)</t>
+          <t>Yes - Strategic Account Executive - NJ/N (New Jersey, New Yo)</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2522,7 @@
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>Unknown - robots.txt on www.365labs.com answered H</t>
+          <t>Unknown - HTTP 403 for https://www.365labs.com/car</t>
         </is>
       </c>
     </row>
@@ -3870,9 +3870,9 @@
           <t>OfficerTRAK off-duty detail management: scheduling, billing, insurance - exhibited at NLC City Summit 2026</t>
         </is>
       </c>
-      <c r="F99" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Business Development Manager - Mid (Charlotte, North C)</t>
+      <c r="F99" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -4112,7 +4112,7 @@
       </c>
       <c r="F107" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 500 for https://safience.io/careers</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -4350,9 +4350,9 @@
           <t>Cyber-over-RF counter-drone detect, track, and mitigate systems for LE, prisons, and infrastructure</t>
         </is>
       </c>
-      <c r="F115" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F115" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -4470,9 +4470,9 @@
           <t>AI ALPR mobile patrol units, speed enforcement, and officer safety systems for LE and municipalities</t>
         </is>
       </c>
-      <c r="F119" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F119" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - HTTP 404 for https://www.ekin.com/about/</t>
         </is>
       </c>
     </row>
@@ -11088,7 +11088,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/15/26)</t>
+          <t>Hiring AEs? (10/16/26)</t>
         </is>
       </c>
     </row>
@@ -11470,7 +11470,7 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - page too small - likely JS-rendered</t>
         </is>
       </c>
     </row>
@@ -14372,7 +14372,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/15/26)</t>
+          <t>Hiring AEs? (10/16/26)</t>
         </is>
       </c>
     </row>
@@ -16978,7 +16978,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/15/26)</t>
+          <t>Hiring AEs? (10/16/26)</t>
         </is>
       </c>
     </row>
@@ -17446,7 +17446,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/15/26)</t>
+          <t>Hiring AEs? (10/16/26)</t>
         </is>
       </c>
     </row>
@@ -18920,9 +18920,9 @@
           <t>School bus stop-arm cameras with violator-funded safety programs</t>
         </is>
       </c>
-      <c r="F51" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F51" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Vice President, Revenue Operations only</t>
         </is>
       </c>
     </row>
@@ -23920,7 +23920,7 @@
       </c>
       <c r="F219" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: robots.txt on www.ejward.</t>
         </is>
       </c>
     </row>
@@ -24576,7 +24576,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/15/26)</t>
+          <t>Hiring AEs? (10/16/26)</t>
         </is>
       </c>
     </row>
@@ -24846,7 +24846,7 @@
       </c>
       <c r="F10" s="21" t="inlineStr">
         <is>
-          <t>Unknown - robots.txt on zencity.io answered HTTP 2</t>
+          <t>Unknown - HTTP 403 for https://zencity.io/careers</t>
         </is>
       </c>
     </row>
@@ -30768,7 +30768,7 @@
       </c>
       <c r="F211" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (Singapore, Singapo)</t>
+          <t>Yes - Account Executive (Denmark)</t>
         </is>
       </c>
     </row>
@@ -31780,7 +31780,7 @@
       </c>
       <c r="F245" s="7" t="inlineStr">
         <is>
-          <t>Unknown - robots.txt on passportworkforce.com answ</t>
+          <t>Unknown - HTTP 403 for https://passportworkforce.c</t>
         </is>
       </c>
     </row>
@@ -34194,7 +34194,7 @@
       </c>
       <c r="F328" s="21" t="inlineStr">
         <is>
-          <t>Unknown - network error: robots.txt on www.planet.</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -38606,7 +38606,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/15/26)</t>
+          <t>Hiring AEs? (10/16/26)</t>
         </is>
       </c>
     </row>
@@ -39020,7 +39020,7 @@
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (Marble Falls, TX)</t>
+          <t>Yes - Account Executive (West Hollywood, CA)</t>
         </is>
       </c>
     </row>
@@ -42192,9 +42192,9 @@
           <t>Event management SaaS: vendor applications, ticketing, maps, and sponsors for festivals and city events</t>
         </is>
       </c>
-      <c r="F121" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Account Strategist only</t>
+      <c r="F121" s="10" t="inlineStr">
+        <is>
+          <t>Yes - Sales &amp; Business Development Manag</t>
         </is>
       </c>
     </row>
@@ -42888,7 +42888,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/15/26)</t>
+          <t>Hiring AEs? (10/16/26)</t>
         </is>
       </c>
     </row>
@@ -43778,9 +43778,9 @@
           <t>InformaCast mass notification and paging for school districts</t>
         </is>
       </c>
-      <c r="F31" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -46984,7 +46984,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/15/26)</t>
+          <t>Hiring AEs? (10/16/26)</t>
         </is>
       </c>
     </row>
@@ -47284,7 +47284,7 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Unknown - robots.txt on www.modeshift.com answered</t>
+          <t>Unknown - HTTP 403 for https://www.modeshift.com/c</t>
         </is>
       </c>
     </row>
@@ -47880,7 +47880,7 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://www.enghouse.com/ca</t>
+          <t>Unknown - HTTP 403 for https://www.enghouse.com/ca</t>
         </is>
       </c>
     </row>
@@ -49934,7 +49934,7 @@
       </c>
       <c r="F100" s="40" t="inlineStr">
         <is>
-          <t>Unknown - robots.txt on www.hanoverdisplays.com an</t>
+          <t>Unknown - HTTP 403 for https://www.hanoverdisplays</t>
         </is>
       </c>
     </row>
@@ -50142,7 +50142,7 @@
       </c>
       <c r="F107" s="10" t="inlineStr">
         <is>
-          <t>Yes - Principal Account Manager (Berlin)</t>
+          <t>Yes - Account Executive (Remix) (New York City)</t>
         </is>
       </c>
     </row>
@@ -50322,7 +50322,7 @@
       </c>
       <c r="F113" s="7" t="inlineStr">
         <is>
-          <t>Unknown - robots.txt on qryde.com answered HTTP 20</t>
+          <t>Unknown - HTTP 403 for https://qryde.com/employmen</t>
         </is>
       </c>
     </row>
@@ -52600,7 +52600,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/15/26)</t>
+          <t>Hiring AEs? (10/16/26)</t>
         </is>
       </c>
     </row>
@@ -53258,9 +53258,9 @@
           <t>Aluminum and steel lighting poles for municipal and DOT projects</t>
         </is>
       </c>
-      <c r="F23" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -55260,9 +55260,9 @@
           <t>Solid-state transformers and grid power electronics, sold to data centre and solar-plus-storage developers</t>
         </is>
       </c>
-      <c r="F90" s="47" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Intern, Business Development Assoc only</t>
+      <c r="F90" s="46" t="inlineStr">
+        <is>
+          <t>Yes - Senior Technical Account Manager (Scotts Valley)</t>
         </is>
       </c>
     </row>
@@ -56158,7 +56158,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/15/26)</t>
+          <t>Hiring AEs? (10/16/26)</t>
         </is>
       </c>
     </row>
@@ -57794,7 +57794,7 @@
       </c>
       <c r="F56" s="51" t="inlineStr">
         <is>
-          <t>Unknown - network error: robots.txt on www.elenium</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -58544,7 +58544,7 @@
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
-          <t>Yes - Enterprise Account Executive (C1 - (Chicago, IL, Unite)</t>
+          <t>Yes - Enterprise Account Executive (C1 - (Dallas, TX, United)</t>
         </is>
       </c>
     </row>
@@ -59682,7 +59682,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/15/26)</t>
+          <t>Hiring AEs? (10/16/26)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-10-17)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/16/26)</t>
+          <t>Hiring AEs? (10/17/26)</t>
         </is>
       </c>
     </row>
@@ -3182,7 +3182,7 @@
       </c>
       <c r="F76" s="8" t="inlineStr">
         <is>
-          <t>Yes - Senior Account Executive, Corporat (2 Locations)</t>
+          <t>Yes - Account Executive, Federal Civilia (VA - Hybrid)</t>
         </is>
       </c>
     </row>
@@ -3720,9 +3720,9 @@
           <t>Training LMS, scheduling, and readiness software (TargetSolutions, Guardian Tracking) - exhibited at IAFC FRI 2026, APCO 2026</t>
         </is>
       </c>
-      <c r="F94" s="11" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F94" s="4" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -11088,7 +11088,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/16/26)</t>
+          <t>Hiring AEs? (10/17/26)</t>
         </is>
       </c>
     </row>
@@ -13562,9 +13562,9 @@
           <t>Social care coordination network connecting health and social service referrals for govs and payers - exhibited at MESC 2026</t>
         </is>
       </c>
-      <c r="F91" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Strategic Sales Director (United States)</t>
+      <c r="F91" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Customer Success Executive - Flori only</t>
         </is>
       </c>
     </row>
@@ -14372,7 +14372,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/16/26)</t>
+          <t>Hiring AEs? (10/17/26)</t>
         </is>
       </c>
     </row>
@@ -16978,7 +16978,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/16/26)</t>
+          <t>Hiring AEs? (10/17/26)</t>
         </is>
       </c>
     </row>
@@ -17446,7 +17446,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/16/26)</t>
+          <t>Hiring AEs? (10/17/26)</t>
         </is>
       </c>
     </row>
@@ -23650,7 +23650,7 @@
       </c>
       <c r="F210" s="16" t="inlineStr">
         <is>
-          <t>Yes - Sales Executive - Industrial Intel (Düsseldorf, North )</t>
+          <t>Yes - Senior Account Executive – Enterpr (London, England)</t>
         </is>
       </c>
     </row>
@@ -23920,7 +23920,7 @@
       </c>
       <c r="F219" s="7" t="inlineStr">
         <is>
-          <t>Unknown - network error: robots.txt on www.ejward.</t>
+          <t>Unknown - HTTP 404 for https://www.wardfuel.com/as</t>
         </is>
       </c>
     </row>
@@ -24576,7 +24576,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/16/26)</t>
+          <t>Hiring AEs? (10/17/26)</t>
         </is>
       </c>
     </row>
@@ -26784,7 +26784,7 @@
       </c>
       <c r="F76" s="23" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Commercial Counsel, Revenue only</t>
+          <t>Sales (non-AE) - Account Director only</t>
         </is>
       </c>
     </row>
@@ -28608,9 +28608,9 @@
           <t>Aerial imagery and property data analytics for county assessors, GIS, and insurers - exhibited at IAAO 2026</t>
         </is>
       </c>
-      <c r="F138" s="22" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F138" s="21" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -29524,9 +29524,9 @@
           <t>Bill presentment and payments for governments and utilities (public co) - exhibited at GFOA 2026, NAHRO 2026, EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F169" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F169" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - network error: robots.txt on www.payment</t>
         </is>
       </c>
     </row>
@@ -31278,7 +31278,7 @@
       </c>
       <c r="F228" s="22" t="inlineStr">
         <is>
-          <t>Yes - Sr. Account Executive (AI Solution (Remote)</t>
+          <t>Yes - Sr. Account Executive (Tolling) (Remote)</t>
         </is>
       </c>
     </row>
@@ -31892,9 +31892,9 @@
           <t>Payroll and HR software - exhibited at AB Show 2026</t>
         </is>
       </c>
-      <c r="F249" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F249" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -38606,7 +38606,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/16/26)</t>
+          <t>Hiring AEs? (10/17/26)</t>
         </is>
       </c>
     </row>
@@ -39020,7 +39020,7 @@
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (West Hollywood, CA)</t>
+          <t>Yes - Account Executive (Glendale, AZ)</t>
         </is>
       </c>
     </row>
@@ -42252,9 +42252,9 @@
           <t>Venue and event management for convention centers and public authorities</t>
         </is>
       </c>
-      <c r="F123" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Director of Solutions Engineering only</t>
+      <c r="F123" s="10" t="inlineStr">
+        <is>
+          <t>Yes - Senior Account Manager (Germany)</t>
         </is>
       </c>
     </row>
@@ -42888,7 +42888,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/16/26)</t>
+          <t>Hiring AEs? (10/17/26)</t>
         </is>
       </c>
     </row>
@@ -43778,9 +43778,9 @@
           <t>InformaCast mass notification and paging for school districts</t>
         </is>
       </c>
-      <c r="F31" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F31" s="10" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -43810,7 +43810,7 @@
       </c>
       <c r="F32" s="35" t="inlineStr">
         <is>
-          <t>Yes - Regional Account Manager - Educati (Baltimore, MD)</t>
+          <t>Yes - Account Manager (Baltimore, MD)</t>
         </is>
       </c>
     </row>
@@ -46510,9 +46510,9 @@
           <t>AI platform for K-12 districts giving teachers lesson and assessment generation tools and students guided AI, with district-level policy and privacy controls - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F124" s="33" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Senior Customer Success Manager -  only</t>
+      <c r="F124" s="34" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -46984,7 +46984,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/16/26)</t>
+          <t>Hiring AEs? (10/17/26)</t>
         </is>
       </c>
     </row>
@@ -52600,7 +52600,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/16/26)</t>
+          <t>Hiring AEs? (10/17/26)</t>
         </is>
       </c>
     </row>
@@ -56158,7 +56158,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/16/26)</t>
+          <t>Hiring AEs? (10/17/26)</t>
         </is>
       </c>
     </row>
@@ -58544,7 +58544,7 @@
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
-          <t>Yes - Enterprise Account Executive (C1 - (Dallas, TX, United)</t>
+          <t>Yes - Senior Enterprise Account Executiv (Dallas, TX, United)</t>
         </is>
       </c>
     </row>
@@ -59682,7 +59682,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/16/26)</t>
+          <t>Hiring AEs? (10/17/26)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-10-18)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/17/26)</t>
+          <t>Hiring AEs? (10/18/26)</t>
         </is>
       </c>
     </row>
@@ -11088,7 +11088,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/17/26)</t>
+          <t>Hiring AEs? (10/18/26)</t>
         </is>
       </c>
     </row>
@@ -11260,7 +11260,7 @@
       </c>
       <c r="F8" s="63" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - page too small - likely JS-rendered</t>
         </is>
       </c>
     </row>
@@ -11680,7 +11680,7 @@
       </c>
       <c r="F22" s="63" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -11940,7 +11940,7 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -13802,9 +13802,9 @@
           <t>HCBS, Medicaid waiver and homelessness systems for public agencies - exhibited at USAging 2026</t>
         </is>
       </c>
-      <c r="F99" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - no ATS on file</t>
+      <c r="F99" s="10" t="inlineStr">
+        <is>
+          <t>Yes - Account Executive I - Personal Car (Overland Park, KS)</t>
         </is>
       </c>
     </row>
@@ -14372,7 +14372,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/17/26)</t>
+          <t>Hiring AEs? (10/18/26)</t>
         </is>
       </c>
     </row>
@@ -14512,7 +14512,7 @@
       </c>
       <c r="F6" s="69" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -16630,7 +16630,7 @@
       </c>
       <c r="F83" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -16978,7 +16978,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/17/26)</t>
+          <t>Hiring AEs? (10/18/26)</t>
         </is>
       </c>
     </row>
@@ -17446,7 +17446,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/17/26)</t>
+          <t>Hiring AEs? (10/18/26)</t>
         </is>
       </c>
     </row>
@@ -22320,7 +22320,7 @@
       </c>
       <c r="F165" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - HTTP 504 for https://streametric.io/care</t>
         </is>
       </c>
     </row>
@@ -22376,7 +22376,7 @@
       </c>
       <c r="F167" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -24576,7 +24576,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/17/26)</t>
+          <t>Hiring AEs? (10/18/26)</t>
         </is>
       </c>
     </row>
@@ -29524,9 +29524,9 @@
           <t>Bill presentment and payments for governments and utilities (public co) - exhibited at GFOA 2026, NAHRO 2026, EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F169" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - network error: robots.txt on www.payment</t>
+      <c r="F169" s="10" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -30768,7 +30768,7 @@
       </c>
       <c r="F211" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (Denmark)</t>
+          <t>Yes - Account Executive (United States)</t>
         </is>
       </c>
     </row>
@@ -37152,7 +37152,7 @@
       </c>
       <c r="F432" s="21" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -37320,7 +37320,7 @@
       </c>
       <c r="F438" s="21" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -37582,7 +37582,7 @@
       </c>
       <c r="F448" s="21" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -38606,7 +38606,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/17/26)</t>
+          <t>Hiring AEs? (10/18/26)</t>
         </is>
       </c>
     </row>
@@ -42888,7 +42888,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/17/26)</t>
+          <t>Hiring AEs? (10/18/26)</t>
         </is>
       </c>
     </row>
@@ -43336,7 +43336,7 @@
       </c>
       <c r="F16" s="34" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - page too small - likely JS-rendered</t>
         </is>
       </c>
     </row>
@@ -43542,7 +43542,7 @@
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - HTTP 410 for https://actuate.ai/careers</t>
         </is>
       </c>
     </row>
@@ -43750,7 +43750,7 @@
       </c>
       <c r="F30" s="34" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -44702,7 +44702,7 @@
       </c>
       <c r="F62" s="34" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - network error: robots.txt on lionlion.ca</t>
         </is>
       </c>
     </row>
@@ -46984,7 +46984,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/17/26)</t>
+          <t>Hiring AEs? (10/18/26)</t>
         </is>
       </c>
     </row>
@@ -48944,7 +48944,7 @@
       </c>
       <c r="F67" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -50620,7 +50620,7 @@
       </c>
       <c r="F123" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -50908,7 +50908,7 @@
       </c>
       <c r="F133" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -51980,7 +51980,7 @@
       </c>
       <c r="F169" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -52600,7 +52600,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/17/26)</t>
+          <t>Hiring AEs? (10/18/26)</t>
         </is>
       </c>
     </row>
@@ -52750,7 +52750,7 @@
       </c>
       <c r="F6" s="45" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -53110,7 +53110,7 @@
       </c>
       <c r="F18" s="45" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -56158,7 +56158,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/17/26)</t>
+          <t>Hiring AEs? (10/18/26)</t>
         </is>
       </c>
     </row>
@@ -57794,7 +57794,7 @@
       </c>
       <c r="F56" s="51" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: robots.txt on www.elenium</t>
         </is>
       </c>
     </row>
@@ -57854,7 +57854,7 @@
       </c>
       <c r="F58" s="51" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -58544,7 +58544,7 @@
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
-          <t>Yes - Senior Enterprise Account Executiv (Dallas, TX, United)</t>
+          <t>Yes - Senior Enterprise Account Executiv (Chicago, IL, Unite)</t>
         </is>
       </c>
     </row>
@@ -59682,7 +59682,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/17/26)</t>
+          <t>Hiring AEs? (10/18/26)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-10-23)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -943,7 +943,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/22/26)</t>
+          <t>Hiring AEs? (10/23/26)</t>
         </is>
       </c>
     </row>
@@ -2901,7 +2901,7 @@
       </c>
       <c r="F68" s="8" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (Sweden)</t>
+          <t>Yes - Account Executive - Public Sector  (Las Vegas, Nevada)</t>
         </is>
       </c>
     </row>
@@ -3081,7 +3081,7 @@
       </c>
       <c r="F74" s="10" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Sales Recruiter (Contract) only</t>
+          <t>Sales (non-AE) - Account Director, Pathfinder (Nati only</t>
         </is>
       </c>
     </row>
@@ -7925,7 +7925,7 @@
       </c>
       <c r="F241" s="9" t="inlineStr">
         <is>
-          <t>Yes - Sales Director (Hong Kong)</t>
+          <t>Yes - Sr Account Executive (United States (Rem)</t>
         </is>
       </c>
     </row>
@@ -8477,7 +8477,7 @@
       </c>
       <c r="F261" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: robots.txt on www.guard1.</t>
         </is>
       </c>
     </row>
@@ -11029,7 +11029,7 @@
       </c>
       <c r="F354" s="4" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: robots.txt on www.guard1.</t>
         </is>
       </c>
     </row>
@@ -12145,7 +12145,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/22/26)</t>
+          <t>Hiring AEs? (10/23/26)</t>
         </is>
       </c>
     </row>
@@ -16149,7 +16149,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/22/26)</t>
+          <t>Hiring AEs? (10/23/26)</t>
         </is>
       </c>
     </row>
@@ -17201,7 +17201,7 @@
       </c>
       <c r="F38" s="69" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 404 for https://writesea.com/career</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -18627,9 +18627,9 @@
           <t>Conversational AI agent platform sold to universities for admissions, financial aid and student support, and to banks, insurers, retailers and healthcare organizations - exhibited at NACUBO 2026</t>
         </is>
       </c>
-      <c r="F92" s="70" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F92" s="69" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -19451,7 +19451,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/22/26)</t>
+          <t>Hiring AEs? (10/23/26)</t>
         </is>
       </c>
     </row>
@@ -20663,7 +20663,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/22/26)</t>
+          <t>Hiring AEs? (10/23/26)</t>
         </is>
       </c>
     </row>
@@ -25999,9 +25999,9 @@
           <t>Sells satellite IoT connectivity and sensor devices, such as water tank monitors, to government agencies and local councils - exhibited at WEFTEC 2026</t>
         </is>
       </c>
-      <c r="F183" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F183" s="9" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -27107,7 +27107,7 @@
       </c>
       <c r="F220" s="16" t="inlineStr">
         <is>
-          <t>Yes - Account Executive – Strategic Acco (Itasca, Illinois)</t>
+          <t>Yes - Sales Director - Net New - Europe  (Staines-upon-Thame)</t>
         </is>
       </c>
     </row>
@@ -28057,7 +28057,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/22/26)</t>
+          <t>Hiring AEs? (10/23/26)</t>
         </is>
       </c>
     </row>
@@ -29661,9 +29661,9 @@
           <t>CodeRED public alerting and critical event management for local jurisdictions</t>
         </is>
       </c>
-      <c r="F55" s="11" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F55" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -33249,7 +33249,7 @@
       </c>
       <c r="F181" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: robots.txt on www.mtwsolu</t>
         </is>
       </c>
     </row>
@@ -35383,7 +35383,7 @@
       </c>
       <c r="F255" s="7" t="inlineStr">
         <is>
-          <t>Unknown - robots.txt on xpressbillpay.com answered</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -36155,7 +36155,7 @@
       </c>
       <c r="F282" s="22" t="inlineStr">
         <is>
-          <t>Yes - Business Development Manager (NYC Headquarters)</t>
+          <t>Yes - Enterprise Account Executive (US-Remote)</t>
         </is>
       </c>
     </row>
@@ -36419,7 +36419,7 @@
       </c>
       <c r="F291" s="9" t="inlineStr">
         <is>
-          <t>Yes - Account Manager (Denver, Colorado)</t>
+          <t>Yes - Account Manager (3 Locations)</t>
         </is>
       </c>
     </row>
@@ -38611,9 +38611,9 @@
           <t>Sells privileged access management, password management, DNS filtering and SASE software to local government, K-12 and higher education IT teams and to MSPs - exhibited at GMIS International 2026</t>
         </is>
       </c>
-      <c r="F371" s="9" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F371" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - HTTP 504 for https://www.cyberfox.com/ca</t>
         </is>
       </c>
     </row>
@@ -38827,9 +38827,9 @@
           <t>Managed endpoint detection and response, identity protection and 24/7 security monitoring for K-12 districts, colleges and state and local governments - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F380" s="22" t="inlineStr">
-        <is>
-          <t>Yes - Account Executive II, Mid-Market (United States of A)</t>
+      <c r="F380" s="23" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Director, Revenue Readiness only</t>
         </is>
       </c>
     </row>
@@ -44551,7 +44551,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/22/26)</t>
+          <t>Hiring AEs? (10/23/26)</t>
         </is>
       </c>
     </row>
@@ -44761,7 +44761,7 @@
       </c>
       <c r="F8" s="27" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Salesforce &amp; RevOps Systems Admini only</t>
+          <t>Sales (non-AE) - Sales Development Representative only</t>
         </is>
       </c>
     </row>
@@ -47403,7 +47403,7 @@
       </c>
       <c r="F97" s="9" t="inlineStr">
         <is>
-          <t>Yes - Account Executive - Agriculture (4 Locations)</t>
+          <t>Yes - SaaS Account Executive - Weather (5 Locations)</t>
         </is>
       </c>
     </row>
@@ -48929,7 +48929,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/22/26)</t>
+          <t>Hiring AEs? (10/23/26)</t>
         </is>
       </c>
     </row>
@@ -53175,7 +53175,7 @@
       </c>
       <c r="F148" s="35" t="inlineStr">
         <is>
-          <t>Yes - Account Executive | SMB | New Logo (Minneapolis, MN)</t>
+          <t>Yes - Account Executive, Commercial, ANZ (Sydney, Australia)</t>
         </is>
       </c>
     </row>
@@ -53765,7 +53765,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/22/26)</t>
+          <t>Hiring AEs? (10/23/26)</t>
         </is>
       </c>
     </row>
@@ -53915,7 +53915,7 @@
       </c>
       <c r="F6" s="40" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 401 for https://www.scheidt-bachman</t>
+          <t>Unknown - HTTP 404 for https://www.scheidt-bachman</t>
         </is>
       </c>
     </row>
@@ -55557,7 +55557,7 @@
       </c>
       <c r="F62" s="40" t="inlineStr">
         <is>
-          <t>Unknown - network error: robots.txt on www.gatekee</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -58921,7 +58921,7 @@
       </c>
       <c r="F176" s="39" t="inlineStr">
         <is>
-          <t>Yes - Account Manager, Enterprise (2 Locations)</t>
+          <t>Yes - Support Account Manager, Enterpris (Ireland Dublin Off)</t>
         </is>
       </c>
     </row>
@@ -59411,7 +59411,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/22/26)</t>
+          <t>Hiring AEs? (10/23/26)</t>
         </is>
       </c>
     </row>
@@ -62993,7 +62993,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/22/26)</t>
+          <t>Hiring AEs? (10/23/26)</t>
         </is>
       </c>
     </row>
@@ -64477,9 +64477,9 @@
           <t>Baggage handling systems and terminal logistics for airports</t>
         </is>
       </c>
-      <c r="F51" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F51" s="11" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -65349,7 +65349,7 @@
       </c>
       <c r="F80" s="52" t="inlineStr">
         <is>
-          <t>Yes - Senior Enterprise Account Executiv (New York, New York)</t>
+          <t>Yes - Senior Enterprise Account Executiv (Austin, TX, United)</t>
         </is>
       </c>
     </row>
@@ -66305,7 +66305,7 @@
       </c>
       <c r="F112" s="51" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -66487,7 +66487,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/22/26)</t>
+          <t>Hiring AEs? (10/23/26)</t>
         </is>
       </c>
     </row>
@@ -66633,7 +66633,7 @@
       </c>
       <c r="F6" s="58" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 403 for https://www.tybera.com/care</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-10-24)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -943,7 +943,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/23/26)</t>
+          <t>Hiring AEs? (10/24/26)</t>
         </is>
       </c>
     </row>
@@ -1803,7 +1803,7 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 502 for https://www.bullard.com/car</t>
         </is>
       </c>
     </row>
@@ -3049,9 +3049,9 @@
           <t>Threat intelligence and OSINT platform for enterprises and public safety</t>
         </is>
       </c>
-      <c r="F73" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F73" s="9" t="inlineStr">
+        <is>
+          <t>Yes - Sales Director - New England (Remote in the Unit)</t>
         </is>
       </c>
     </row>
@@ -3499,9 +3499,9 @@
           <t>Drone-as-first-responder software and hardware auto-launching to 911 calls</t>
         </is>
       </c>
-      <c r="F88" s="10" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Sales Development Representative ( only</t>
+      <c r="F88" s="4" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="F193" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - board is another company's - not read</t>
         </is>
       </c>
     </row>
@@ -8477,7 +8477,7 @@
       </c>
       <c r="F261" s="7" t="inlineStr">
         <is>
-          <t>Unknown - network error: robots.txt on www.guard1.</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -10665,9 +10665,9 @@
           <t>Public safety CAD, RMS, jail software - exhibited at IACP 2026, APCO 2026</t>
         </is>
       </c>
-      <c r="F339" s="9" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F339" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - HTTP 503 for https://www.cis.com/careers</t>
         </is>
       </c>
     </row>
@@ -11029,7 +11029,7 @@
       </c>
       <c r="F354" s="4" t="inlineStr">
         <is>
-          <t>Unknown - network error: robots.txt on www.guard1.</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -11669,9 +11669,9 @@
           <t>DigiTICKET electronic citation software - exhibited at IACP 2026</t>
         </is>
       </c>
-      <c r="F380" s="10" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F380" s="4" t="inlineStr">
+        <is>
+          <t>Unknown - network error: robots.txt on saltustechn</t>
         </is>
       </c>
     </row>
@@ -12145,7 +12145,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/23/26)</t>
+          <t>Hiring AEs? (10/24/26)</t>
         </is>
       </c>
     </row>
@@ -13649,7 +13649,7 @@
       </c>
       <c r="F58" s="64" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Senior Solutions Consultant - Risk only</t>
+          <t>Sales (non-AE) - Revenue Integrity Analyst only</t>
         </is>
       </c>
     </row>
@@ -14131,7 +14131,7 @@
       </c>
       <c r="F75" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -16149,7 +16149,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/23/26)</t>
+          <t>Hiring AEs? (10/24/26)</t>
         </is>
       </c>
     </row>
@@ -16343,9 +16343,9 @@
           <t>AI enrollment engagement platform that personalizes web, email, SMS, and voice outreach to prospective students for colleges and independent schools - exhibited at EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F8" s="69" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F8" s="70" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -18115,7 +18115,7 @@
       </c>
       <c r="F72" s="70" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Vice President, Sales only</t>
+          <t>Sales (non-AE) - Sales Development Representative only</t>
         </is>
       </c>
     </row>
@@ -19451,7 +19451,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/23/26)</t>
+          <t>Hiring AEs? (10/24/26)</t>
         </is>
       </c>
     </row>
@@ -20663,7 +20663,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/23/26)</t>
+          <t>Hiring AEs? (10/24/26)</t>
         </is>
       </c>
     </row>
@@ -27107,7 +27107,7 @@
       </c>
       <c r="F220" s="16" t="inlineStr">
         <is>
-          <t>Yes - Sales Director - Net New - Europe  (Staines-upon-Thame)</t>
+          <t>Yes - Senior Account Executive – Strateg (Itasca, Illinois)</t>
         </is>
       </c>
     </row>
@@ -27287,7 +27287,7 @@
       </c>
       <c r="F226" s="15" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 504 for https://eptura.com/careers</t>
         </is>
       </c>
     </row>
@@ -28057,7 +28057,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/23/26)</t>
+          <t>Hiring AEs? (10/24/26)</t>
         </is>
       </c>
     </row>
@@ -30207,7 +30207,7 @@
       </c>
       <c r="F74" s="21" t="inlineStr">
         <is>
-          <t>Unknown - board is another company's - not read</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -33749,9 +33749,9 @@
           <t>Bill presentment and payments for governments and utilities (public co) - exhibited at GFOA 2026, NAHRO 2026, EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F200" s="22" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F200" s="21" t="inlineStr">
+        <is>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -34993,7 +34993,7 @@
       </c>
       <c r="F242" s="22" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (United States)</t>
+          <t>Yes - Account Executive (Singapore, Singapo)</t>
         </is>
       </c>
     </row>
@@ -35501,9 +35501,9 @@
           <t>Cash and digital payments for child support, tolls and government billers</t>
         </is>
       </c>
-      <c r="F259" s="9" t="inlineStr">
-        <is>
-          <t>Yes - Sr. Account Executive (Tolling) (Remote)</t>
+      <c r="F259" s="11" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Vice President, Accounting only</t>
         </is>
       </c>
     </row>
@@ -36003,9 +36003,9 @@
           <t>Benefits administration and enrollment built exclusively for public-sector employers - exhibited at SALGBA 2026, ASBO School Business 2026</t>
         </is>
       </c>
-      <c r="F277" s="11" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F277" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown - robots.txt on www.mybentek.com answered </t>
         </is>
       </c>
     </row>
@@ -36747,7 +36747,7 @@
       </c>
       <c r="F302" s="23" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Sr. Customer Success Manager - Gov only</t>
+          <t>Sales (non-AE) - Manager of Customer Success (Remot only</t>
         </is>
       </c>
     </row>
@@ -38087,9 +38087,9 @@
           <t>ChatGPT and the API, sold to public sector including named state and local government roles - exhibited at NLC City Summit 2026</t>
         </is>
       </c>
-      <c r="F350" s="22" t="inlineStr">
-        <is>
-          <t>Yes - Business Development Manager, Prod (Munich, Germany)</t>
+      <c r="F350" s="23" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Backend Software Engineer, GTM Inn only</t>
         </is>
       </c>
     </row>
@@ -38611,9 +38611,9 @@
           <t>Sells privileged access management, password management, DNS filtering and SASE software to local government, K-12 and higher education IT teams and to MSPs - exhibited at GMIS International 2026</t>
         </is>
       </c>
-      <c r="F371" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - HTTP 504 for https://www.cyberfox.com/ca</t>
+      <c r="F371" s="9" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -40487,7 +40487,7 @@
       </c>
       <c r="F442" s="21" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 404 for https://contentactive.com/c</t>
+          <t>Unknown - network error: robots.txt on contentacti</t>
         </is>
       </c>
     </row>
@@ -42305,7 +42305,7 @@
       </c>
       <c r="F506" s="22" t="inlineStr">
         <is>
-          <t>Yes - Regional Sales Manager, K12 &amp; Publ</t>
+          <t>Yes - Sr Account Executive, AMC</t>
         </is>
       </c>
     </row>
@@ -44551,7 +44551,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/23/26)</t>
+          <t>Hiring AEs? (10/24/26)</t>
         </is>
       </c>
     </row>
@@ -44759,9 +44759,9 @@
           <t>SmartRec activity registration and facility management platform - exhibited at NRPA 2026, Washington Recreation and Park Association 2026</t>
         </is>
       </c>
-      <c r="F8" s="27" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Sales Development Representative only</t>
+      <c r="F8" s="29" t="inlineStr">
+        <is>
+          <t>Yes - Account Executive (Montreal, Quebec, )</t>
         </is>
       </c>
     </row>
@@ -48929,7 +48929,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/23/26)</t>
+          <t>Hiring AEs? (10/24/26)</t>
         </is>
       </c>
     </row>
@@ -48989,7 +48989,7 @@
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>Yes - Sales Executive - Central Region (Remote Worker - N/)</t>
+          <t>Yes - Sales Executive - Pacific Northwes (Remote Worker - N/)</t>
         </is>
       </c>
     </row>
@@ -50277,7 +50277,7 @@
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>Yes - Sales Account Executive – Mid-Mark</t>
+          <t>Yes - Strategic Sales Director - Enterpr</t>
         </is>
       </c>
     </row>
@@ -52191,9 +52191,9 @@
           <t>Digital hall pass, tardy tracking, behavior management, and campus engagement platform for K-12 schools and districts - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F112" s="35" t="inlineStr">
-        <is>
-          <t>Yes - Account Manager (INTERNAL APPLICAN</t>
+      <c r="F112" s="33" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Entry Level Sales Opportunity - SD only</t>
         </is>
       </c>
     </row>
@@ -53765,7 +53765,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/23/26)</t>
+          <t>Hiring AEs? (10/24/26)</t>
         </is>
       </c>
     </row>
@@ -55557,7 +55557,7 @@
       </c>
       <c r="F62" s="40" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: robots.txt on www.gatekee</t>
         </is>
       </c>
     </row>
@@ -56785,7 +56785,7 @@
       </c>
       <c r="F103" s="7" t="inlineStr">
         <is>
-          <t>Unknown - robots.txt on basemap.co.uk answered HTT</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -59271,7 +59271,7 @@
       </c>
       <c r="F190" s="39" t="inlineStr">
         <is>
-          <t>Yes - Sales Account Executive – Mid-Mark</t>
+          <t>Yes - Strategic Sales Director - Enterpr</t>
         </is>
       </c>
     </row>
@@ -59411,7 +59411,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/23/26)</t>
+          <t>Hiring AEs? (10/24/26)</t>
         </is>
       </c>
     </row>
@@ -61749,7 +61749,7 @@
       </c>
       <c r="F79" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -62993,7 +62993,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/23/26)</t>
+          <t>Hiring AEs? (10/24/26)</t>
         </is>
       </c>
     </row>
@@ -64477,9 +64477,9 @@
           <t>Baggage handling systems and terminal logistics for airports</t>
         </is>
       </c>
-      <c r="F51" s="11" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -65349,7 +65349,7 @@
       </c>
       <c r="F80" s="52" t="inlineStr">
         <is>
-          <t>Yes - Senior Enterprise Account Executiv (Austin, TX, United)</t>
+          <t>Yes - Senior Enterprise Account Executiv (New York, New York)</t>
         </is>
       </c>
     </row>
@@ -65527,9 +65527,9 @@
           <t>Passive airspace monitoring sensors for airports and government agencies</t>
         </is>
       </c>
-      <c r="F86" s="51" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F86" s="53" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Director of Business Development - only</t>
         </is>
       </c>
     </row>
@@ -66487,7 +66487,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/23/26)</t>
+          <t>Hiring AEs? (10/24/26)</t>
         </is>
       </c>
     </row>
@@ -66633,7 +66633,7 @@
       </c>
       <c r="F6" s="58" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.tybera.com/care</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-10-25)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -230,7 +230,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -358,6 +358,7 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="25" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="25" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="25" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -943,7 +944,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/24/26)</t>
+          <t>Hiring AEs? (10/25/26)</t>
         </is>
       </c>
     </row>
@@ -1803,7 +1804,7 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 502 for https://www.bullard.com/car</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -6711,7 +6712,7 @@
       </c>
       <c r="F198" s="4" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -6951,7 +6952,7 @@
       </c>
       <c r="F206" s="4" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -7973,7 +7974,7 @@
       </c>
       <c r="F243" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -10047,7 +10048,7 @@
       </c>
       <c r="F314" s="4" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -10143,7 +10144,7 @@
       </c>
       <c r="F318" s="4" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -10213,9 +10214,9 @@
           <t>Mobile core and radio network products, including the iNAC managed access system that blocks contraband cellphones in correctional facilities - exhibited at ACA Congress 2026</t>
         </is>
       </c>
-      <c r="F321" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - no ATS on file</t>
+      <c r="F321" s="11" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -10263,7 +10264,7 @@
       </c>
       <c r="F323" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -10665,9 +10666,9 @@
           <t>Public safety CAD, RMS, jail software - exhibited at IACP 2026, APCO 2026</t>
         </is>
       </c>
-      <c r="F339" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - HTTP 503 for https://www.cis.com/careers</t>
+      <c r="F339" s="9" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -11469,9 +11470,9 @@
           <t>Enterprise database, cloud and ERP software - exhibited at IACP 2026, NSA 2026, GFOA 2026, PSHRA 2026, NatCon 2026, APTA 2026, ICC 2026, ASBO School Business 2026</t>
         </is>
       </c>
-      <c r="F372" s="4" t="inlineStr">
-        <is>
-          <t>Unknown - no ATS on file</t>
+      <c r="F372" s="10" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -11669,9 +11670,9 @@
           <t>DigiTICKET electronic citation software - exhibited at IACP 2026</t>
         </is>
       </c>
-      <c r="F380" s="4" t="inlineStr">
-        <is>
-          <t>Unknown - network error: robots.txt on saltustechn</t>
+      <c r="F380" s="10" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -12145,7 +12146,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/24/26)</t>
+          <t>Hiring AEs? (10/25/26)</t>
         </is>
       </c>
     </row>
@@ -12605,7 +12606,7 @@
       </c>
       <c r="F20" s="63" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -12627,9 +12628,9 @@
           <t>Roving and stationary air pollution and greenhouse gas sensor network with Aclima Pro analytics software for governments, companies and communities</t>
         </is>
       </c>
-      <c r="F21" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - no ATS on file</t>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Vice President, Business Developme only</t>
         </is>
       </c>
     </row>
@@ -12777,9 +12778,9 @@
           <t>AI decision and case platforms for state health and human services</t>
         </is>
       </c>
-      <c r="F26" s="63" t="inlineStr">
-        <is>
-          <t>Unknown - no ATS on file</t>
+      <c r="F26" s="64" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -13409,7 +13410,7 @@
       </c>
       <c r="F48" s="63" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -13803,9 +13804,9 @@
           <t>MCase case management for child welfare and human services agencies - exhibited at APHSA 2026</t>
         </is>
       </c>
-      <c r="F64" s="63" t="inlineStr">
-        <is>
-          <t>Unknown - no ATS on file</t>
+      <c r="F64" s="64" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -14131,7 +14132,7 @@
       </c>
       <c r="F75" s="7" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -15479,7 +15480,7 @@
       </c>
       <c r="F125" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -16149,7 +16150,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/24/26)</t>
+          <t>Hiring AEs? (10/25/26)</t>
         </is>
       </c>
     </row>
@@ -19199,7 +19200,7 @@
       </c>
       <c r="F115" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -19225,9 +19226,9 @@
           <t>Tuition payment plans, billing, cashiering, and payment processing software for colleges and universities - exhibited at NACUBO 2026</t>
         </is>
       </c>
-      <c r="F116" s="69" t="inlineStr">
-        <is>
-          <t>Unknown - no ATS on file</t>
+      <c r="F116" s="70" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - CRM Solutions Architect only</t>
         </is>
       </c>
     </row>
@@ -19451,7 +19452,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/24/26)</t>
+          <t>Hiring AEs? (10/25/26)</t>
         </is>
       </c>
     </row>
@@ -19899,7 +19900,7 @@
       </c>
       <c r="F18" s="75" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -19971,7 +19972,7 @@
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -20019,7 +20020,7 @@
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -20043,7 +20044,7 @@
       </c>
       <c r="F24" s="75" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -20091,7 +20092,7 @@
       </c>
       <c r="F26" s="75" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -20115,7 +20116,7 @@
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -20139,7 +20140,7 @@
       </c>
       <c r="F28" s="75" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -20161,9 +20162,9 @@
           <t>MRI Software sells public housing software for HUD compliance reporting, voucher management, waitlists and resident portals to public housing agencies - exhibited at NAHRO 2026</t>
         </is>
       </c>
-      <c r="F29" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - no ATS on file</t>
+      <c r="F29" s="9" t="inlineStr">
+        <is>
+          <t>Yes - Account Executive (Cleveland, Ohio Of)</t>
         </is>
       </c>
     </row>
@@ -20361,7 +20362,7 @@
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -20505,7 +20506,7 @@
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -20527,9 +20528,9 @@
           <t>JobsEQ labor market data and analytics platform, including a Housing Demand tool, for economic development, workforce development, education and corporate users</t>
         </is>
       </c>
-      <c r="F44" s="75" t="inlineStr">
-        <is>
-          <t>Unknown - no ATS on file</t>
+      <c r="F44" s="77" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Sales Development Representative only</t>
         </is>
       </c>
     </row>
@@ -20575,9 +20576,9 @@
           <t>Economic impact modeling software and data used by governments, economic development organizations and other industries</t>
         </is>
       </c>
-      <c r="F46" s="75" t="inlineStr">
-        <is>
-          <t>Unknown - no ATS on file</t>
+      <c r="F46" s="76" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -20663,7 +20664,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/24/26)</t>
+          <t>Hiring AEs? (10/25/26)</t>
         </is>
       </c>
     </row>
@@ -27287,7 +27288,7 @@
       </c>
       <c r="F226" s="15" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 504 for https://eptura.com/careers</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -28057,7 +28058,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/24/26)</t>
+          <t>Hiring AEs? (10/25/26)</t>
         </is>
       </c>
     </row>
@@ -32065,9 +32066,9 @@
           <t>License portability platform that helps state licensing boards process out-of-state credentials for military families and veterans</t>
         </is>
       </c>
-      <c r="F141" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - no ATS on file</t>
+      <c r="F141" s="9" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -33581,9 +33582,9 @@
           <t>AI workflow software for county assessor offices: homestead exemption monitoring, application vetting and property transfer automation</t>
         </is>
       </c>
-      <c r="F194" s="21" t="inlineStr">
-        <is>
-          <t>Unknown - no ATS on file</t>
+      <c r="F194" s="22" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -33749,9 +33750,9 @@
           <t>Bill presentment and payments for governments and utilities (public co) - exhibited at GFOA 2026, NAHRO 2026, EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F200" s="21" t="inlineStr">
-        <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+      <c r="F200" s="22" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -34669,7 +34670,7 @@
       </c>
       <c r="F231" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - board is another company's - not read</t>
         </is>
       </c>
     </row>
@@ -34993,7 +34994,7 @@
       </c>
       <c r="F242" s="22" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (Singapore, Singapo)</t>
+          <t>Yes - Account Executive (United States)</t>
         </is>
       </c>
     </row>
@@ -35023,7 +35024,7 @@
       </c>
       <c r="F243" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -35855,7 +35856,7 @@
       </c>
       <c r="F272" s="21" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -36003,9 +36004,9 @@
           <t>Benefits administration and enrollment built exclusively for public-sector employers - exhibited at SALGBA 2026, ASBO School Business 2026</t>
         </is>
       </c>
-      <c r="F277" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Unknown - robots.txt on www.mybentek.com answered </t>
+      <c r="F277" s="11" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -37247,7 +37248,7 @@
       </c>
       <c r="F321" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -39427,9 +39428,9 @@
           <t>AI agents for state government staff and public-facing AI concierges that help residents complete permits and licenses - exhibited at NCSL Legislative Summit 2026</t>
         </is>
       </c>
-      <c r="F405" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - no ATS on file</t>
+      <c r="F405" s="11" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -39453,7 +39454,7 @@
       </c>
       <c r="F406" s="21" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -39475,9 +39476,9 @@
           <t>AI governance platform that discovers AI tool use, enforces AI policy and runs governed AI workflows for state and local agencies</t>
         </is>
       </c>
-      <c r="F407" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - no ATS on file</t>
+      <c r="F407" s="9" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -40487,7 +40488,7 @@
       </c>
       <c r="F442" s="21" t="inlineStr">
         <is>
-          <t>Unknown - network error: robots.txt on contentacti</t>
+          <t>Unknown - HTTP 404 for https://contentactive.com/c</t>
         </is>
       </c>
     </row>
@@ -40757,7 +40758,7 @@
       </c>
       <c r="F451" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -43649,9 +43650,9 @@
           <t>Content management and workflow automation software - exhibited at ICMA 2025</t>
         </is>
       </c>
-      <c r="F556" s="21" t="inlineStr">
-        <is>
-          <t>Unknown - no ATS on file</t>
+      <c r="F556" s="22" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -44551,7 +44552,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/24/26)</t>
+          <t>Hiring AEs? (10/25/26)</t>
         </is>
       </c>
     </row>
@@ -46183,7 +46184,7 @@
       </c>
       <c r="F56" s="28" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -47253,7 +47254,7 @@
       </c>
       <c r="F92" s="28" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -48929,7 +48930,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/24/26)</t>
+          <t>Hiring AEs? (10/25/26)</t>
         </is>
       </c>
     </row>
@@ -49289,7 +49290,7 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -50185,9 +50186,9 @@
           <t>Enterprise browser with built-in security, data protection and CIPA content filtering, sold to K-12 districts among other industries - exhibited at NASCIO 2026</t>
         </is>
       </c>
-      <c r="F44" s="34" t="inlineStr">
-        <is>
-          <t>Unknown - no ATS on file</t>
+      <c r="F44" s="35" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -53557,9 +53558,9 @@
           <t>Fixed asset tracking software for K-12 school districts, plus physical inventory audits, barcode asset tags and consulting - exhibited at ASBO School Business 2026</t>
         </is>
       </c>
-      <c r="F164" s="34" t="inlineStr">
-        <is>
-          <t>Unknown - no ATS on file</t>
+      <c r="F164" s="35" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -53607,7 +53608,7 @@
       </c>
       <c r="F166" s="34" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -53677,9 +53678,9 @@
           <t>Online diagnostic assessments and personalized math and reading instruction for K-12 special education and intervention, sold to schools and districts - exhibited at CEC Convention 2027</t>
         </is>
       </c>
-      <c r="F169" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - no ATS on file</t>
+      <c r="F169" s="9" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -53765,7 +53766,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/24/26)</t>
+          <t>Hiring AEs? (10/25/26)</t>
         </is>
       </c>
     </row>
@@ -55407,7 +55408,7 @@
       </c>
       <c r="F57" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -58945,9 +58946,9 @@
           <t>Transit CAD/AVL and asset management software - exhibited at APTA 2026</t>
         </is>
       </c>
-      <c r="F177" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - no ATS on file</t>
+      <c r="F177" s="9" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -59411,7 +59412,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/24/26)</t>
+          <t>Hiring AEs? (10/25/26)</t>
         </is>
       </c>
     </row>
@@ -61451,7 +61452,7 @@
       </c>
       <c r="F69" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -61749,7 +61750,7 @@
       </c>
       <c r="F79" s="7" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -62097,7 +62098,7 @@
       </c>
       <c r="F91" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -62993,7 +62994,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/24/26)</t>
+          <t>Hiring AEs? (10/25/26)</t>
         </is>
       </c>
     </row>
@@ -65349,7 +65350,7 @@
       </c>
       <c r="F80" s="52" t="inlineStr">
         <is>
-          <t>Yes - Senior Enterprise Account Executiv (New York, New York)</t>
+          <t>Yes - Senior Enterprise Account Executiv (Austin, TX, United)</t>
         </is>
       </c>
     </row>
@@ -66213,9 +66214,9 @@
           <t>Parking access and revenue control systems for airports and cities</t>
         </is>
       </c>
-      <c r="F109" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - no ATS on file</t>
+      <c r="F109" s="9" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -66487,7 +66488,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/24/26)</t>
+          <t>Hiring AEs? (10/25/26)</t>
         </is>
       </c>
     </row>
@@ -66997,7 +66998,7 @@
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-10-28)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -944,7 +944,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/27/26)</t>
+          <t>Hiring AEs? (10/28/26)</t>
         </is>
       </c>
     </row>
@@ -3166,7 +3166,7 @@
       </c>
       <c r="F79" s="9" t="inlineStr">
         <is>
-          <t>Yes - Account Executive - Public Sector  (Las Vegas, Nevada)</t>
+          <t>Yes - Enterprise Account Executive - Cor (California)</t>
         </is>
       </c>
     </row>
@@ -6290,9 +6290,9 @@
           <t>Sells Pro ATE automated speed-camera enforcement systems, with AI violation processing and ticketing back-office services, to police departments, cities and counties - exhibited at Maryland Municipal League 2026, North Carolina Sheriffs' Association 2026</t>
         </is>
       </c>
-      <c r="F185" s="9" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F185" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - HTTP 404 for https://altumint.com/career</t>
         </is>
       </c>
     </row>
@@ -9106,9 +9106,9 @@
           <t>Verus AI platform transcribing and analyzing inmate calls for threat and contraband investigations - exhibited at ACA Congress 2026</t>
         </is>
       </c>
-      <c r="F285" s="9" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F285" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -12506,7 +12506,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/27/26)</t>
+          <t>Hiring AEs? (10/28/26)</t>
         </is>
       </c>
     </row>
@@ -16510,7 +16510,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/27/26)</t>
+          <t>Hiring AEs? (10/28/26)</t>
         </is>
       </c>
     </row>
@@ -19812,7 +19812,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/27/26)</t>
+          <t>Hiring AEs? (10/28/26)</t>
         </is>
       </c>
     </row>
@@ -20524,7 +20524,7 @@
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (Cleveland, Ohio Of)</t>
+          <t>Yes - Account Executive I (Cleveland, Ohio Of)</t>
         </is>
       </c>
     </row>
@@ -21048,7 +21048,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/27/26)</t>
+          <t>Hiring AEs? (10/28/26)</t>
         </is>
       </c>
     </row>
@@ -21166,9 +21166,9 @@
           <t>AI robotic sorting systems for recycling facilities (MRFs) - exhibited at SWANA WASTECON 2025, WasteExpo 2027</t>
         </is>
       </c>
-      <c r="F5" s="11" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Director, Commercial Origination &amp; only</t>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -22200,9 +22200,9 @@
           <t>Carts, containers and compactors supplied to municipal waste programs</t>
         </is>
       </c>
-      <c r="F40" s="15" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F40" s="16" t="inlineStr">
+        <is>
+          <t>Yes - Outside Sales Representative (4 Locations)</t>
         </is>
       </c>
     </row>
@@ -24506,9 +24506,9 @@
           <t>Permitting, compliance, and workflow software for water utilities - exhibited at AWWA ACE 2026, WEFTEC 2026</t>
         </is>
       </c>
-      <c r="F119" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F119" s="11" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Senior Customer Success Manager only</t>
         </is>
       </c>
     </row>
@@ -26114,7 +26114,7 @@
       </c>
       <c r="F173" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 404 for https://streametric.io/care</t>
+          <t>Unknown - HTTP 504 for https://streametric.io/care</t>
         </is>
       </c>
     </row>
@@ -26596,7 +26596,7 @@
       </c>
       <c r="F191" s="9" t="inlineStr">
         <is>
-          <t>Yes - Key Account Executive (Remote) (Remote - Australia)</t>
+          <t>Yes - Business Development Manager - Mon (Monterrey, Nuevo L)</t>
         </is>
       </c>
     </row>
@@ -27792,7 +27792,7 @@
       </c>
       <c r="F231" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 403 for https://eptura.com/careers</t>
         </is>
       </c>
     </row>
@@ -28610,7 +28610,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/27/26)</t>
+          <t>Hiring AEs? (10/28/26)</t>
         </is>
       </c>
     </row>
@@ -28670,7 +28670,7 @@
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>Yes - Account Executive - New Logo - Nor</t>
+          <t>Yes - Associate Account Executive</t>
         </is>
       </c>
     </row>
@@ -28758,9 +28758,9 @@
           <t>Community surveys, benchmarking, and budget simulation (owns National Research Center)</t>
         </is>
       </c>
-      <c r="F6" s="22" t="inlineStr">
-        <is>
-          <t>Yes - Account Executive (Madison, WI)</t>
+      <c r="F6" s="21" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -30836,7 +30836,7 @@
       </c>
       <c r="F77" s="9" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (London)</t>
+          <t>Yes - Account Executive (San Francisco)</t>
         </is>
       </c>
     </row>
@@ -35246,7 +35246,7 @@
       </c>
       <c r="F232" s="21" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - board is another company's - not read</t>
         </is>
       </c>
     </row>
@@ -35570,7 +35570,7 @@
       </c>
       <c r="F243" s="9" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (Denmark)</t>
+          <t>Yes - Account Executive (United States)</t>
         </is>
       </c>
     </row>
@@ -38260,7 +38260,7 @@
       </c>
       <c r="F337" s="7" t="inlineStr">
         <is>
-          <t>Unknown - network error: robots.txt on www.tribute</t>
+          <t>Unknown - board is another company's - not read</t>
         </is>
       </c>
     </row>
@@ -38286,9 +38286,9 @@
           <t>Deathcare technology suite including cemetery and memorial management software</t>
         </is>
       </c>
-      <c r="F338" s="21" t="inlineStr">
-        <is>
-          <t>Unknown - network error: robots.txt on www.tribute</t>
+      <c r="F338" s="23" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -40268,9 +40268,9 @@
           <t>Policy and rulemaking workflow: draft, route, approve, and track regulations for agencies</t>
         </is>
       </c>
-      <c r="F416" s="23" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Customer Success Lead only</t>
+      <c r="F416" s="22" t="inlineStr">
+        <is>
+          <t>Yes - Enterprise Sales Lead, Southeast (Southeast)</t>
         </is>
       </c>
     </row>
@@ -41638,9 +41638,9 @@
           <t>Ballot tracking, electronic ballot delivery and election tools for jurisdictions</t>
         </is>
       </c>
-      <c r="F463" s="11" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F463" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - HTTP 404 for https://www.enhancedvoting.</t>
         </is>
       </c>
     </row>
@@ -45248,7 +45248,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/27/26)</t>
+          <t>Hiring AEs? (10/28/26)</t>
         </is>
       </c>
     </row>
@@ -46190,9 +46190,9 @@
           <t>Club and league operations platform for youth sports organizations</t>
         </is>
       </c>
-      <c r="F33" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - network error: robots.txt on home.playme</t>
+      <c r="F33" s="11" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -46430,9 +46430,9 @@
           <t>Club and league management platform for youth soccer organizations</t>
         </is>
       </c>
-      <c r="F41" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - network error: robots.txt on byga.net di</t>
+      <c r="F41" s="9" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -48126,7 +48126,7 @@
       </c>
       <c r="F98" s="29" t="inlineStr">
         <is>
-          <t>Yes - SaaS Account Executive - Weather (5 Locations)</t>
+          <t>Yes - Account Manager - Agriculture (4 Locations)</t>
         </is>
       </c>
     </row>
@@ -49626,7 +49626,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/27/26)</t>
+          <t>Hiring AEs? (10/28/26)</t>
         </is>
       </c>
     </row>
@@ -50488,9 +50488,9 @@
           <t>InformaCast mass notification and paging for school districts</t>
         </is>
       </c>
-      <c r="F30" s="34" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F30" s="35" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -51484,7 +51484,7 @@
       </c>
       <c r="F64" s="34" t="inlineStr">
         <is>
-          <t>Unknown - network error: robots.txt on lionlion.ca</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -54462,7 +54462,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/27/26)</t>
+          <t>Hiring AEs? (10/28/26)</t>
         </is>
       </c>
     </row>
@@ -56584,7 +56584,7 @@
       </c>
       <c r="F73" s="11" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Customer Success Manager only</t>
+          <t>Sales (non-AE) - Customer Success Manager (Client S only</t>
         </is>
       </c>
     </row>
@@ -56912,9 +56912,9 @@
           <t>Fare collection and transit operations systems for agencies</t>
         </is>
       </c>
-      <c r="F84" s="41" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Solution Architect only</t>
+      <c r="F84" s="40" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -60108,7 +60108,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/27/26)</t>
+          <t>Hiring AEs? (10/28/26)</t>
         </is>
       </c>
     </row>
@@ -61452,7 +61452,7 @@
       </c>
       <c r="F46" s="46" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Customer Success Manager only</t>
+          <t>Sales (non-AE) - Customer Success Manager (CA or TX only</t>
         </is>
       </c>
     </row>
@@ -62350,9 +62350,9 @@
           <t>Utility bill management and energy analytics for cities, counties and schools</t>
         </is>
       </c>
-      <c r="F76" s="47" t="inlineStr">
-        <is>
-          <t>Yes - Account Executive</t>
+      <c r="F76" s="45" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -64338,7 +64338,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/27/26)</t>
+          <t>Hiring AEs? (10/28/26)</t>
         </is>
       </c>
     </row>
@@ -66694,7 +66694,7 @@
       </c>
       <c r="F80" s="52" t="inlineStr">
         <is>
-          <t>Yes - Senior Enterprise Account Executiv (Dallas, TX, United)</t>
+          <t>Yes - Senior Enterprise Account Executiv (New York, New York)</t>
         </is>
       </c>
     </row>
@@ -67832,7 +67832,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/27/26)</t>
+          <t>Hiring AEs? (10/28/26)</t>
         </is>
       </c>
     </row>
@@ -68572,9 +68572,9 @@
           <t>Legal case management software sold to law firms and to state and municipal legal departments, prosecutors and public defenders - exhibited at IMLA 2026</t>
         </is>
       </c>
-      <c r="F27" s="9" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-10-29)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -944,7 +944,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/28/26)</t>
+          <t>Hiring AEs? (10/29/26)</t>
         </is>
       </c>
     </row>
@@ -2504,9 +2504,9 @@
           <t>License plate readers, gunshot detection, and drone-as-first-responder (Aerodome) - exhibited at ITS America 2026, FDIC International 2026, TRB 2027</t>
         </is>
       </c>
-      <c r="F57" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F57" s="11" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Principal Sales Operations Busines only</t>
         </is>
       </c>
     </row>
@@ -6616,7 +6616,7 @@
       </c>
       <c r="F197" s="9" t="inlineStr">
         <is>
-          <t>Yes - Sales Executive, Strategic Account (Seattle, WA)</t>
+          <t>Yes - Strategic Account Manager, Hospita (2 Locations)</t>
         </is>
       </c>
     </row>
@@ -6826,7 +6826,7 @@
       </c>
       <c r="F204" s="4" t="inlineStr">
         <is>
-          <t>Unknown - board is another company's - not read</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -11827,7 +11827,7 @@
       </c>
       <c r="E387" s="5" t="inlineStr">
         <is>
-          <t>Enterprise database, cloud and ERP software - exhibited at IACP 2026, NSA 2026, GFOA 2026, PSHRA 2026, NatCon 2026, APTA 2026, ICC 2026, ASBO School Business 2026, DISTRIBUTECH 2026</t>
+          <t>Enterprise database, cloud and ERP software - exhibited at IACP 2026, NSA 2026, GFOA 2026, PSHRA 2026, NatCon 2026, APTA 2026, ICC 2026, ASBO School Business 2026, DISTRIBUTECH 2026, APA California Chapter 2026</t>
         </is>
       </c>
       <c r="F387" s="11" t="inlineStr">
@@ -12506,7 +12506,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/28/26)</t>
+          <t>Hiring AEs? (10/29/26)</t>
         </is>
       </c>
     </row>
@@ -12577,7 +12577,7 @@
       </c>
       <c r="E4" s="61" t="inlineStr">
         <is>
-          <t>Casetivity-based public health software - immunization information systems, electronic disease surveillance, early intervention, lead poisoning prevention and vital records - for state and local public health agencies - exhibited at AIRA 2026</t>
+          <t>Casetivity-based public health software - immunization information systems, electronic disease surveillance, early intervention, lead poisoning prevention and vital records - for state and local public health agencies - exhibited at AIRA 2026, Pennsylvania Chapter of the APA 2026</t>
         </is>
       </c>
       <c r="F4" s="63" t="inlineStr">
@@ -13170,7 +13170,7 @@
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>Yes - Commercial Account Executive, Truv (Remote – United St)</t>
+          <t>Yes - Account Executive, Springbuk (Remote – United St)</t>
         </is>
       </c>
     </row>
@@ -16510,7 +16510,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/28/26)</t>
+          <t>Hiring AEs? (10/29/26)</t>
         </is>
       </c>
     </row>
@@ -16966,9 +16966,9 @@
           <t>Peer review, group work, and AI feedback tools that plug into university learning management systems - exhibited at EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F17" s="9" t="inlineStr">
-        <is>
-          <t>Yes - Account Executive (Texas) (US Remote)</t>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -17726,9 +17726,9 @@
           <t>Scaffold platform for LMS migration, course archiving, and data warehousing across LMS, SIS, and CRM systems at colleges and universities - exhibited at EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F44" s="71" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F44" s="70" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -19586,9 +19586,9 @@
           <t>Tuition payment plans, billing, cashiering, and payment processing software for colleges and universities - exhibited at NACUBO 2026</t>
         </is>
       </c>
-      <c r="F116" s="70" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - CRM Solutions Architect only</t>
+      <c r="F116" s="71" t="inlineStr">
+        <is>
+          <t>Yes - Senior Account Manager- G&amp;A/SGO -  (Remote)</t>
         </is>
       </c>
     </row>
@@ -19750,7 +19750,7 @@
       </c>
       <c r="F122" s="71" t="inlineStr">
         <is>
-          <t>Yes - Senior Account Executive (London)</t>
+          <t>Yes - Account Executive - Denmark (2 Locations)</t>
         </is>
       </c>
     </row>
@@ -19812,7 +19812,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/28/26)</t>
+          <t>Hiring AEs? (10/29/26)</t>
         </is>
       </c>
     </row>
@@ -21048,7 +21048,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/28/26)</t>
+          <t>Hiring AEs? (10/29/26)</t>
         </is>
       </c>
     </row>
@@ -22998,7 +22998,7 @@
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>Yes - (Mid-Level) Account Manager Nether (Zaltbommel, Gelder)</t>
+          <t>Yes - Account Manager Netherlands (Zaltbommel, Gelder)</t>
         </is>
       </c>
     </row>
@@ -24776,9 +24776,9 @@
           <t>Underground utility, geotech, and environmental records aggregated into one map for capital projects</t>
         </is>
       </c>
-      <c r="F128" s="17" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Strategic Customer Success Manager only</t>
+      <c r="F128" s="16" t="inlineStr">
+        <is>
+          <t>Yes - Account Executive - Engineering Fi (Remote)</t>
         </is>
       </c>
     </row>
@@ -26114,7 +26114,7 @@
       </c>
       <c r="F173" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 504 for https://streametric.io/care</t>
+          <t>Unknown - HTTP 404 for https://streametric.io/care</t>
         </is>
       </c>
     </row>
@@ -26531,7 +26531,7 @@
       </c>
       <c r="E189" s="5" t="inlineStr">
         <is>
-          <t>ArcGIS - the mapping and asset data backbone of most public works departments - exhibited at NLC City Summit 2026, AWWA ACE 2026, IAAO 2026, NASCIO 2026, WEFTEC 2026, IAFC FRI 2026, APCO 2026, APTA 2026, NRPA 2026, IAEM 2026, NCSL Legislative Summit 2026, URISA GIS-Pro 2026, NSGIC 2026, DISTRIBUTECH 2026, FDIC International 2026, FDIC International 2027, TRB 2027, DISTRIBUTECH 2027</t>
+          <t>ArcGIS - the mapping and asset data backbone of most public works departments - exhibited at NLC City Summit 2026, AWWA ACE 2026, IAAO 2026, NASCIO 2026, WEFTEC 2026, IAFC FRI 2026, APCO 2026, APTA 2026, NRPA 2026, IAEM 2026, NCSL Legislative Summit 2026, URISA GIS-Pro 2026, NSGIC 2026, DISTRIBUTECH 2026, FDIC International 2026, FDIC International 2027, TRB 2027, DISTRIBUTECH 2027, APA Texas Chapter 2026</t>
         </is>
       </c>
       <c r="F189" s="7" t="inlineStr">
@@ -26956,7 +26956,7 @@
       </c>
       <c r="F203" s="9" t="inlineStr">
         <is>
-          <t>Yes - Account Executive, CMRL - MX (Mexico City - Hybr)</t>
+          <t>Yes - Account Executive, Enterprise - Mo (United States - Re)</t>
         </is>
       </c>
     </row>
@@ -27612,7 +27612,7 @@
       </c>
       <c r="F225" s="9" t="inlineStr">
         <is>
-          <t>Yes - Senior Account Executive – Strateg (Itasca, Illinois)</t>
+          <t>Yes - Customer Account Manager, Manufact (Itasca, Illinois)</t>
         </is>
       </c>
     </row>
@@ -27792,7 +27792,7 @@
       </c>
       <c r="F231" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://eptura.com/careers</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -28610,7 +28610,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/28/26)</t>
+          <t>Hiring AEs? (10/29/26)</t>
         </is>
       </c>
     </row>
@@ -29265,7 +29265,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>AI assistant trained on a government's institutional knowledge; $3.5M seed backed by Granicus founders - exhibited at GFOA 2026, AWWA ACE 2026, GMIS International 2026</t>
+          <t>AI assistant trained on a government's institutional knowledge; $3.5M seed backed by Granicus founders - exhibited at GFOA 2026, AWWA ACE 2026, GMIS International 2026, APA California Chapter 2026</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
@@ -30031,7 +30031,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>Interactive document feedback and public comment tool for agencies</t>
+          <t>Interactive document feedback and public comment tool for agencies - exhibited at APA California Chapter 2026, APA Colorado Chapter 2026</t>
         </is>
       </c>
       <c r="F49" s="7" t="inlineStr">
@@ -30531,7 +30531,7 @@
       </c>
       <c r="E66" s="19" t="inlineStr">
         <is>
-          <t>Community engagement and stakeholder relationship management platform for councils, transportation agencies, and infrastructure project owners - exhibited at 3CMA 2026</t>
+          <t>Community engagement and stakeholder relationship management platform for councils, transportation agencies, and infrastructure project owners - exhibited at 3CMA 2026, APA California Chapter 2026</t>
         </is>
       </c>
       <c r="F66" s="21" t="inlineStr">
@@ -31125,7 +31125,7 @@
       </c>
       <c r="E89" s="5" t="inlineStr">
         <is>
-          <t>Permitting, licensing, and code enforcement platform for state and local government - exhibited at NLC City Summit 2026, ICMA 2026, NRPA 2026, ICC 2026</t>
+          <t>Permitting, licensing, and code enforcement platform for state and local government - exhibited at NLC City Summit 2026, ICMA 2026, NRPA 2026, ICC 2026, APA California Chapter 2026, APA - Illinois Chapter 2026, APA Virginia Chapter 2026</t>
         </is>
       </c>
       <c r="F89" s="11" t="inlineStr">
@@ -31155,7 +31155,7 @@
       </c>
       <c r="E90" s="19" t="inlineStr">
         <is>
-          <t>Permitting, budgeting, procurement, and asset management cloud suite (Cox-owned) - exhibited at GFOA 2026, NLC City Summit 2026, NACE 2026, AWWA ACE 2026, GMIS International 2026, Maryland Municipal League 2026, WEFTEC 2026, NRPA 2026, ICC 2026, ASBO School Business 2026</t>
+          <t>Permitting, budgeting, procurement, and asset management cloud suite (Cox-owned) - exhibited at GFOA 2026, NLC City Summit 2026, NACE 2026, AWWA ACE 2026, GMIS International 2026, Maryland Municipal League 2026, WEFTEC 2026, NRPA 2026, ICC 2026, ASBO School Business 2026, APA Texas Chapter 2026</t>
         </is>
       </c>
       <c r="F90" s="22" t="inlineStr">
@@ -31215,7 +31215,7 @@
       </c>
       <c r="E92" s="19" t="inlineStr">
         <is>
-          <t>AI permitting and licensing platform: 24/7 resident assistant, AI code-compliance review - exhibited at NLC City Summit 2026, Maryland Municipal League 2026, ICC 2026</t>
+          <t>AI permitting and licensing platform: 24/7 resident assistant, AI code-compliance review - exhibited at NLC City Summit 2026, Maryland Municipal League 2026, ICC 2026, APA Colorado Chapter 2026, APA Minnesota Chapter 2026, APA Texas Chapter 2026, APA Virginia Chapter 2026, APA Washington Chapter 2026, APA Wisconsin Chapter 2026, American Planning Association Ohio Chapter 2026, Georgia Planning Association 2026, Joint Montana &amp; Idaho Chapter Conference 2026, NY Upstate Chapter of the APA 2026, Pennsylvania Chapter of the APA 2026</t>
         </is>
       </c>
       <c r="F92" s="22" t="inlineStr">
@@ -31545,7 +31545,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t>AI permitting and plan review: automated GIS/code compliance checks (Hernando County cut reviews 30 days to 2)</t>
+          <t>AI permitting and plan review: automated GIS/code compliance checks (Hernando County cut reviews 30 days to 2) - exhibited at APA Maryland 2026, APA Washington Chapter 2026</t>
         </is>
       </c>
       <c r="F103" s="7" t="inlineStr">
@@ -31575,7 +31575,7 @@
       </c>
       <c r="E104" s="19" t="inlineStr">
         <is>
-          <t>AI-native land-use permit management: reads applications, flags issues, drafts review reports (YC S26) - exhibited at NLC City Summit 2026</t>
+          <t>AI-native land-use permit management: reads applications, flags issues, drafts review reports (YC S26) - exhibited at NLC City Summit 2026, APA California Chapter 2026, APA Oklahoma Chapter 2026</t>
         </is>
       </c>
       <c r="F104" s="21" t="inlineStr">
@@ -31668,9 +31668,9 @@
           <t>Agent-native AI 'GovOS' for local gov permitting, licensing, and procurement (~$55M Series A, ex-DeepMind) - exhibited at ICMA 2026, NIGP 2026, ICC 2026, NLC City Summit 2026</t>
         </is>
       </c>
-      <c r="F107" s="11" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Sales Engineer only</t>
+      <c r="F107" s="9" t="inlineStr">
+        <is>
+          <t>Yes - Account Executive, State (Remote)</t>
         </is>
       </c>
     </row>
@@ -32357,7 +32357,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t>AI planning and building code assessment tools sold to councils and cities - exhibited at ICMA 2026, Smart Cities Connect 2026, ICC 2026</t>
+          <t>AI planning and building code assessment tools sold to councils and cities - exhibited at ICMA 2026, Smart Cities Connect 2026, ICC 2026, APA California Chapter 2026</t>
         </is>
       </c>
       <c r="F131" s="7" t="inlineStr">
@@ -32519,7 +32519,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t>Sells AI site-feasibility software to home builders and AI permit intake and plan review software to local government planning and permitting departments - exhibited at ICMA 2026</t>
+          <t>Sells AI site-feasibility software to home builders and AI permit intake and plan review software to local government planning and permitting departments - exhibited at ICMA 2026, APA California Chapter 2026</t>
         </is>
       </c>
       <c r="F137" s="7" t="inlineStr">
@@ -32639,7 +32639,7 @@
       </c>
       <c r="E142" s="19" t="inlineStr">
         <is>
-          <t>Permitting and entitlements software for city, county and state planning departments: guided applicant intake, auto-drafted review checklists, jurisdiction fee calculators and a searchable staff answer base</t>
+          <t>Permitting and entitlements software for city, county and state planning departments: guided applicant intake, auto-drafted review checklists, jurisdiction fee calculators and a searchable staff answer base - exhibited at APA California Chapter 2026</t>
         </is>
       </c>
       <c r="F142" s="22" t="inlineStr">
@@ -32669,7 +32669,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t>The govtech giant: ERP, courts, public safety, permitting, and payments - exhibited at GFOA 2026, NLC City Summit 2026, PSHRA 2026, AWWA ACE 2026, IAAO 2026, NASCIO 2026, GMIS International 2026, NACM 2026, APPA Probation 2026, Iowa State Association of Counties 2026, Maryland Municipal League 2026, IAFC FRI 2026, APCO 2026, NAPT Summit 2026, Connecticut Conference of Municipalities 2026, Illinois Chapter of APCO 2026, ICC 2026, ASBO School Business 2026, NACVSO 2026, ACA Congress 2026, FDIC International 2026</t>
+          <t>The govtech giant: ERP, courts, public safety, permitting, and payments - exhibited at GFOA 2026, NLC City Summit 2026, PSHRA 2026, AWWA ACE 2026, IAAO 2026, NASCIO 2026, GMIS International 2026, NACM 2026, APPA Probation 2026, Iowa State Association of Counties 2026, Maryland Municipal League 2026, IAFC FRI 2026, APCO 2026, NAPT Summit 2026, Connecticut Conference of Municipalities 2026, Illinois Chapter of APCO 2026, ICC 2026, ASBO School Business 2026, NACVSO 2026, ACA Congress 2026, FDIC International 2026, APA Colorado Chapter 2026, APA - Illinois Chapter 2026, APA Minnesota Chapter 2026, APA Texas Chapter 2026, APA Virginia Chapter 2026, APA Wisconsin Chapter 2026, American Planning Association Ohio Chapter 2026, Georgia Planning Association 2026, Michigan Association of Planning 2026</t>
         </is>
       </c>
       <c r="F143" s="9" t="inlineStr">
@@ -35570,7 +35570,7 @@
       </c>
       <c r="F243" s="9" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (United States)</t>
+          <t>Yes - Account Executive (Denmark)</t>
         </is>
       </c>
     </row>
@@ -37322,9 +37322,9 @@
           <t>License verification and workforce compliance for agencies and regulators</t>
         </is>
       </c>
-      <c r="F303" s="11" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Manager of Customer Success (Remot only</t>
+      <c r="F303" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -37444,7 +37444,7 @@
       </c>
       <c r="F307" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 404 for https://www.harrislocalgov.</t>
+          <t>Unknown - HTTP 503 for https://www.harrislocalgov.</t>
         </is>
       </c>
     </row>
@@ -39404,9 +39404,9 @@
           <t>Sells a vulnerability discovery, bug bounty and pentesting platform to state and local government agencies, schools and universities - exhibited at EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F381" s="11" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Applications Engineer, GTM Systems only</t>
+      <c r="F381" s="9" t="inlineStr">
+        <is>
+          <t>Yes - Account Executive – Commercial, En (San Francisco)</t>
         </is>
       </c>
     </row>
@@ -40270,7 +40270,7 @@
       </c>
       <c r="F416" s="22" t="inlineStr">
         <is>
-          <t>Yes - Enterprise Sales Lead, Southeast (Southeast)</t>
+          <t>Yes - Enterprise Sales Lead, Northeast (Northeast)</t>
         </is>
       </c>
     </row>
@@ -40355,7 +40355,7 @@
       </c>
       <c r="E419" s="5" t="inlineStr">
         <is>
-          <t>Demographic data, mapping, and visualization with 500K+ variables for gov, academia, and planning</t>
+          <t>Demographic data, mapping, and visualization with 500K+ variables for gov, academia, and planning - exhibited at NY Upstate Chapter of the APA 2026</t>
         </is>
       </c>
       <c r="F419" s="7" t="inlineStr">
@@ -40704,7 +40704,7 @@
       </c>
       <c r="F431" s="7" t="inlineStr">
         <is>
-          <t>Unknown - network error: robots.txt on www.maxar.c</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -44319,7 +44319,7 @@
       </c>
       <c r="E561" s="5" t="inlineStr">
         <is>
-          <t>Code Council digital permitting/code solutions - exhibited at ICMA 2025, IMLA 2026, Maryland Municipal League 2026</t>
+          <t>Code Council digital permitting/code solutions - exhibited at ICMA 2025, IMLA 2026, Maryland Municipal League 2026, APA California Chapter 2026, APA Texas Chapter 2026</t>
         </is>
       </c>
       <c r="F561" s="7" t="inlineStr">
@@ -45248,7 +45248,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/28/26)</t>
+          <t>Hiring AEs? (10/29/26)</t>
         </is>
       </c>
     </row>
@@ -48126,7 +48126,7 @@
       </c>
       <c r="F98" s="29" t="inlineStr">
         <is>
-          <t>Yes - Account Manager - Agriculture (4 Locations)</t>
+          <t>Yes - SaaS Account Executive - Weather (United Kingdom - R)</t>
         </is>
       </c>
     </row>
@@ -48932,9 +48932,9 @@
           <t>Event management SaaS: vendor applications, ticketing, maps, and sponsors for festivals and city events - exhibited at NRPA 2026</t>
         </is>
       </c>
-      <c r="F125" s="11" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Account Strategist only</t>
+      <c r="F125" s="9" t="inlineStr">
+        <is>
+          <t>Yes - Sales &amp; Business Development Manag</t>
         </is>
       </c>
     </row>
@@ -49626,7 +49626,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/28/26)</t>
+          <t>Hiring AEs? (10/29/26)</t>
         </is>
       </c>
     </row>
@@ -50488,9 +50488,9 @@
           <t>InformaCast mass notification and paging for school districts</t>
         </is>
       </c>
-      <c r="F30" s="35" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F30" s="34" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -51484,7 +51484,7 @@
       </c>
       <c r="F64" s="34" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: robots.txt on lionlion.ca</t>
         </is>
       </c>
     </row>
@@ -52186,7 +52186,7 @@
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
-          <t>None found</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -52890,7 +52890,7 @@
       </c>
       <c r="F112" s="33" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Entry Level Sales Opportunity - SD only</t>
+          <t>Sales (non-AE) - Sales Development Representative - only</t>
         </is>
       </c>
     </row>
@@ -53364,9 +53364,9 @@
           <t>AI platform for K-12 districts giving teachers lesson and assessment generation tools and students guided AI, with district-level policy and privacy controls - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F129" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F129" s="9" t="inlineStr">
+        <is>
+          <t>Yes - Account Executive (K12 Education)  (Alabama)</t>
         </is>
       </c>
     </row>
@@ -54462,7 +54462,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/28/26)</t>
+          <t>Hiring AEs? (10/29/26)</t>
         </is>
       </c>
     </row>
@@ -54966,9 +54966,9 @@
           <t>Check-in/be-out mobile fare payment for public transport authorities</t>
         </is>
       </c>
-      <c r="F18" s="41" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Head of Strategic Accounts only</t>
+      <c r="F18" s="40" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -56254,7 +56254,7 @@
       </c>
       <c r="F62" s="40" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: robots.txt on www.gatekee</t>
         </is>
       </c>
     </row>
@@ -57627,7 +57627,7 @@
       </c>
       <c r="E108" s="37" t="inlineStr">
         <is>
-          <t>On-demand transit, paratransit, and network planning software for agencies - exhibited at CTAA EXPO 2026, APTA 2026</t>
+          <t>On-demand transit, paratransit, and network planning software for agencies - exhibited at CTAA EXPO 2026, APTA 2026, APA Texas Chapter 2026</t>
         </is>
       </c>
       <c r="F108" s="39" t="inlineStr">
@@ -60108,7 +60108,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/28/26)</t>
+          <t>Hiring AEs? (10/29/26)</t>
         </is>
       </c>
     </row>
@@ -61452,7 +61452,7 @@
       </c>
       <c r="F46" s="46" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Customer Success Manager (CA or TX only</t>
+          <t>Sales (non-AE) - Customer Success Manager only</t>
         </is>
       </c>
     </row>
@@ -64338,7 +64338,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/28/26)</t>
+          <t>Hiring AEs? (10/29/26)</t>
         </is>
       </c>
     </row>
@@ -65822,9 +65822,9 @@
           <t>Baggage handling systems and terminal logistics for airports</t>
         </is>
       </c>
-      <c r="F51" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F51" s="9" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -66694,7 +66694,7 @@
       </c>
       <c r="F80" s="52" t="inlineStr">
         <is>
-          <t>Yes - Senior Enterprise Account Executiv (New York, New York)</t>
+          <t>Yes - Senior Enterprise Account Executiv (Chicago, IL, Unite)</t>
         </is>
       </c>
     </row>
@@ -67832,7 +67832,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/28/26)</t>
+          <t>Hiring AEs? (10/29/26)</t>
         </is>
       </c>
     </row>
@@ -68572,9 +68572,9 @@
           <t>Legal case management software sold to law firms and to state and municipal legal departments, prosecutors and public defenders - exhibited at IMLA 2026</t>
         </is>
       </c>
-      <c r="F27" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+      <c r="F27" s="9" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-10-30)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -230,7 +230,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -358,7 +358,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="25" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="25" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="25" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -944,7 +943,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/29/26)</t>
+          <t>Hiring AEs? (10/30/26)</t>
         </is>
       </c>
     </row>
@@ -2956,7 +2955,7 @@
       </c>
       <c r="F72" s="4" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - robots.txt on www.365labs.com answered H</t>
         </is>
       </c>
     </row>
@@ -12506,7 +12505,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/29/26)</t>
+          <t>Hiring AEs? (10/30/26)</t>
         </is>
       </c>
     </row>
@@ -16510,7 +16509,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/29/26)</t>
+          <t>Hiring AEs? (10/30/26)</t>
         </is>
       </c>
     </row>
@@ -16966,9 +16965,9 @@
           <t>Peer review, group work, and AI feedback tools that plug into university learning management systems - exhibited at EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F17" s="11" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Customer Success Manager North Ame only</t>
         </is>
       </c>
     </row>
@@ -19812,7 +19811,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/29/26)</t>
+          <t>Hiring AEs? (10/30/26)</t>
         </is>
       </c>
     </row>
@@ -20888,9 +20887,9 @@
           <t>JobsEQ labor market data and analytics platform, including a Housing Demand tool, for economic development, workforce development, education and corporate users</t>
         </is>
       </c>
-      <c r="F44" s="77" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Sales Development Representative only</t>
+      <c r="F44" s="76" t="inlineStr">
+        <is>
+          <t>Yes - Account Executive (Richmond, VA)</t>
         </is>
       </c>
     </row>
@@ -21048,7 +21047,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/29/26)</t>
+          <t>Hiring AEs? (10/30/26)</t>
         </is>
       </c>
     </row>
@@ -26866,7 +26865,7 @@
       </c>
       <c r="F200" s="15" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.aurigo.com/care</t>
+          <t>Unknown - HTTP 404 for https://www.aurigo.com/care</t>
         </is>
       </c>
     </row>
@@ -26956,7 +26955,7 @@
       </c>
       <c r="F203" s="9" t="inlineStr">
         <is>
-          <t>Yes - Account Executive, Enterprise - Mo (United States - Re)</t>
+          <t>Yes - Account Executive, Mid-Market - MX (Mexico City - Hybr)</t>
         </is>
       </c>
     </row>
@@ -27346,7 +27345,7 @@
       </c>
       <c r="F216" s="15" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - robots.txt on www.projectmates.com answe</t>
         </is>
       </c>
     </row>
@@ -27792,7 +27791,7 @@
       </c>
       <c r="F231" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 403 for https://eptura.com/careers</t>
         </is>
       </c>
     </row>
@@ -28610,7 +28609,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/29/26)</t>
+          <t>Hiring AEs? (10/30/26)</t>
         </is>
       </c>
     </row>
@@ -28878,9 +28877,9 @@
           <t>AI resident feedback: surveys, sentiment analytics, and engagement for cities and police - exhibited at 3CMA 2026</t>
         </is>
       </c>
-      <c r="F10" s="22" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F10" s="21" t="inlineStr">
+        <is>
+          <t>Unknown - robots.txt on zencity.io answered HTTP 2</t>
         </is>
       </c>
     </row>
@@ -32332,7 +32331,7 @@
       </c>
       <c r="F130" s="22" t="inlineStr">
         <is>
-          <t>Yes - Strategic Account Executive (New Zealand)</t>
+          <t>Yes - Business Development Manager (Reading)</t>
         </is>
       </c>
     </row>
@@ -35222,7 +35221,7 @@
       </c>
       <c r="F231" s="9" t="inlineStr">
         <is>
-          <t>Yes - Account Executive - Midmarket (rem (United States (Wes)</t>
+          <t>Yes - Account Executive - Midmarket (Dal (Dallas, TX)</t>
         </is>
       </c>
     </row>
@@ -35246,7 +35245,7 @@
       </c>
       <c r="F232" s="21" t="inlineStr">
         <is>
-          <t>Unknown - board is another company's - not read</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -36108,7 +36107,7 @@
       </c>
       <c r="F261" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -36702,7 +36701,7 @@
       </c>
       <c r="F282" s="21" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 404 for https://passportworkforce.c</t>
+          <t>Unknown - robots.txt on passportworkforce.com answ</t>
         </is>
       </c>
     </row>
@@ -37656,7 +37655,7 @@
       </c>
       <c r="F315" s="9" t="inlineStr">
         <is>
-          <t>Yes - Enterprise Account Executive (2 Locations)</t>
+          <t>Yes - Regional Sales Director - APAC (Remote - Australia)</t>
         </is>
       </c>
     </row>
@@ -39046,7 +39045,7 @@
       </c>
       <c r="F366" s="22" t="inlineStr">
         <is>
-          <t>Yes - Enterprise Account Executive (Canada &gt; Ontario &gt;)</t>
+          <t>Yes - Account Executive - SLED (6 Locations)</t>
         </is>
       </c>
     </row>
@@ -44796,7 +44795,7 @@
       </c>
       <c r="F580" s="21" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - robots.txt on www.proofpoint.com answere</t>
         </is>
       </c>
     </row>
@@ -45248,7 +45247,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/29/26)</t>
+          <t>Hiring AEs? (10/30/26)</t>
         </is>
       </c>
     </row>
@@ -49626,7 +49625,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/29/26)</t>
+          <t>Hiring AEs? (10/30/26)</t>
         </is>
       </c>
     </row>
@@ -50342,7 +50341,7 @@
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>Yes - Regional Sales Manager (Boston, Massachuse)</t>
+          <t>Yes - Regional Sales Manager (District of Columb)</t>
         </is>
       </c>
     </row>
@@ -50488,9 +50487,9 @@
           <t>InformaCast mass notification and paging for school districts</t>
         </is>
       </c>
-      <c r="F30" s="34" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F30" s="35" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -50518,9 +50517,9 @@
           <t>Emergency mass notification hardware and software for schools and agencies - exhibited at EDUCAUSE 2026, IAEM 2026</t>
         </is>
       </c>
-      <c r="F31" s="9" t="inlineStr">
-        <is>
-          <t>Yes - Account Manager (Baltimore, MD)</t>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -52186,7 +52185,7 @@
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -54086,9 +54085,9 @@
           <t>Digital ticketing, live streaming, athletic websites and stats tools for high school athletic programs, under the GoFan, NFHS Network and MaxPreps brands - exhibited at ASBO School Business 2026</t>
         </is>
       </c>
-      <c r="F157" s="9" t="inlineStr">
-        <is>
-          <t>Yes - Account Executive (New York, NY)</t>
+      <c r="F157" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -54462,7 +54461,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/29/26)</t>
+          <t>Hiring AEs? (10/30/26)</t>
         </is>
       </c>
     </row>
@@ -54762,7 +54761,7 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - robots.txt on www.modeshift.com answered</t>
         </is>
       </c>
     </row>
@@ -55400,7 +55399,7 @@
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 202 for https://www.enghouse.com/ca</t>
         </is>
       </c>
     </row>
@@ -57424,7 +57423,7 @@
       </c>
       <c r="F101" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - robots.txt on www.hanoverdisplays.com an</t>
         </is>
       </c>
     </row>
@@ -57812,7 +57811,7 @@
       </c>
       <c r="F114" s="40" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - robots.txt on qryde.com answered HTTP 20</t>
         </is>
       </c>
     </row>
@@ -60108,7 +60107,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/29/26)</t>
+          <t>Hiring AEs? (10/30/26)</t>
         </is>
       </c>
     </row>
@@ -64338,7 +64337,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/29/26)</t>
+          <t>Hiring AEs? (10/30/26)</t>
         </is>
       </c>
     </row>
@@ -64750,7 +64749,7 @@
       </c>
       <c r="F15" s="11" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Senior Sales Operations Analyst only</t>
+          <t>Sales (non-AE) - Lead Sales Engineer only</t>
         </is>
       </c>
     </row>
@@ -65822,9 +65821,9 @@
           <t>Baggage handling systems and terminal logistics for airports</t>
         </is>
       </c>
-      <c r="F51" s="9" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F51" s="11" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -66694,7 +66693,7 @@
       </c>
       <c r="F80" s="52" t="inlineStr">
         <is>
-          <t>Yes - Senior Enterprise Account Executiv (Chicago, IL, Unite)</t>
+          <t>Yes - Senior Enterprise Account Executiv (Dallas, TX, United)</t>
         </is>
       </c>
     </row>
@@ -67832,7 +67831,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/29/26)</t>
+          <t>Hiring AEs? (10/30/26)</t>
         </is>
       </c>
     </row>
@@ -68622,7 +68621,7 @@
       </c>
       <c r="F29" s="11" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Customer Success Manager - LegalFi only</t>
+          <t>Sales (non-AE) - Mid-Market Customer Success Manage only</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-10-31)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -943,7 +943,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/30/26)</t>
+          <t>Hiring AEs? (10/31/26)</t>
         </is>
       </c>
     </row>
@@ -2475,7 +2475,7 @@
       </c>
       <c r="F56" s="8" t="inlineStr">
         <is>
-          <t>Yes - Senior Account Executive - Cyberse (Texas, US Offsite,)</t>
+          <t>Yes - Senior Account Executive (Arizona) (Phoenix, AZ, More.)</t>
         </is>
       </c>
     </row>
@@ -2595,7 +2595,7 @@
       </c>
       <c r="F60" s="8" t="inlineStr">
         <is>
-          <t>Yes - Strategic Account Executive - NJ/N (New Jersey, New Yo)</t>
+          <t>Yes - Regional Account Executive - NJ/NY (New Jersey, New Yo)</t>
         </is>
       </c>
     </row>
@@ -6465,7 +6465,7 @@
       </c>
       <c r="F192" s="8" t="inlineStr">
         <is>
-          <t>Yes - Account Manager (Remote, US (TN/KY))</t>
+          <t>Yes - Account Manager (Remote, US (West))</t>
         </is>
       </c>
     </row>
@@ -12505,7 +12505,7 @@
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/30/26)</t>
+          <t>Hiring AEs? (10/31/26)</t>
         </is>
       </c>
     </row>
@@ -14223,9 +14223,9 @@
           <t>Foster care, adoption and child welfare software for county/state agencies - exhibited at APHSA 2026</t>
         </is>
       </c>
-      <c r="F66" s="64" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F66" s="63" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -14491,7 +14491,7 @@
       </c>
       <c r="F75" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: robots.txt on streamlineh</t>
         </is>
       </c>
     </row>
@@ -16509,7 +16509,7 @@
       </c>
       <c r="F1" s="66" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/30/26)</t>
+          <t>Hiring AEs? (10/31/26)</t>
         </is>
       </c>
     </row>
@@ -17863,9 +17863,9 @@
           <t>Wi-Fi-based space occupancy analytics and planning software for colleges and universities - exhibited at NACUBO 2026</t>
         </is>
       </c>
-      <c r="F49" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F49" s="9" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -19811,7 +19811,7 @@
       </c>
       <c r="F1" s="72" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/30/26)</t>
+          <t>Hiring AEs? (10/31/26)</t>
         </is>
       </c>
     </row>
@@ -21047,7 +21047,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/30/26)</t>
+          <t>Hiring AEs? (10/31/26)</t>
         </is>
       </c>
     </row>
@@ -21255,9 +21255,9 @@
           <t>Smart bin fill-level sensors and collection route optimization</t>
         </is>
       </c>
-      <c r="F8" s="17" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F8" s="15" t="inlineStr">
+        <is>
+          <t>Unknown - HTTP 404 for https://www.sensoneo.com/ca</t>
         </is>
       </c>
     </row>
@@ -24627,7 +24627,7 @@
       </c>
       <c r="F123" s="11" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Revenue Operations Analyst only</t>
+          <t>Sales (non-AE) - Sales Development Representative only</t>
         </is>
       </c>
     </row>
@@ -27345,7 +27345,7 @@
       </c>
       <c r="F216" s="15" t="inlineStr">
         <is>
-          <t>Unknown - robots.txt on www.projectmates.com answe</t>
+          <t>Unknown - HTTP 502 for https://www.projectmates.co</t>
         </is>
       </c>
     </row>
@@ -27611,7 +27611,7 @@
       </c>
       <c r="F225" s="9" t="inlineStr">
         <is>
-          <t>Yes - Customer Account Manager, Manufact (Itasca, Illinois)</t>
+          <t>Yes - Strategic Account Manager, Manufac (Itasca, Illinois)</t>
         </is>
       </c>
     </row>
@@ -28371,7 +28371,7 @@
       </c>
       <c r="F253" s="7" t="inlineStr">
         <is>
-          <t>None found</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -28609,7 +28609,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/30/26)</t>
+          <t>Hiring AEs? (10/31/26)</t>
         </is>
       </c>
     </row>
@@ -28879,7 +28879,7 @@
       </c>
       <c r="F10" s="21" t="inlineStr">
         <is>
-          <t>Unknown - robots.txt on zencity.io answered HTTP 2</t>
+          <t xml:space="preserve">Unknown - network error: robots.txt on zencity.io </t>
         </is>
       </c>
     </row>
@@ -30955,7 +30955,7 @@
       </c>
       <c r="F82" s="22" t="inlineStr">
         <is>
-          <t>Yes - Enterprise Account Executive, Fina (Richmond)</t>
+          <t>Yes - Enterprise Account Executive, Fina (Boston)</t>
         </is>
       </c>
     </row>
@@ -31669,7 +31669,7 @@
       </c>
       <c r="F107" s="9" t="inlineStr">
         <is>
-          <t>Yes - Account Executive, State (Remote)</t>
+          <t>Yes - Account Executive, Gov (Remote)</t>
         </is>
       </c>
     </row>
@@ -33801,7 +33801,7 @@
       </c>
       <c r="F181" s="7" t="inlineStr">
         <is>
-          <t>Unknown - network error: robots.txt on www.mtwsolu</t>
+          <t>Unknown - page too small - likely JS-rendered</t>
         </is>
       </c>
     </row>
@@ -35569,7 +35569,7 @@
       </c>
       <c r="F243" s="9" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (Denmark)</t>
+          <t>Yes - Account Executive (Singapore, Singapo)</t>
         </is>
       </c>
     </row>
@@ -36107,7 +36107,7 @@
       </c>
       <c r="F261" s="7" t="inlineStr">
         <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -36579,9 +36579,9 @@
           <t>Benefits administration and enrollment built exclusively for public-sector employers - exhibited at SALGBA 2026, ASBO School Business 2026</t>
         </is>
       </c>
-      <c r="F278" s="23" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F278" s="21" t="inlineStr">
+        <is>
+          <t>Unknown - network error: robots.txt on www.mybente</t>
         </is>
       </c>
     </row>
@@ -39427,9 +39427,9 @@
           <t>Managed endpoint detection and response, identity protection and 24/7 security monitoring for K-12 districts, colleges and state and local governments - exhibited at CoSN 2026</t>
         </is>
       </c>
-      <c r="F382" s="23" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Director, Revenue Readiness only</t>
+      <c r="F382" s="22" t="inlineStr">
+        <is>
+          <t>Yes - Technical Account Manager II (United States of A)</t>
         </is>
       </c>
     </row>
@@ -40237,9 +40237,9 @@
           <t>Strategic plan and KPI reporting (balanced scorecard) for local governments and enterprises</t>
         </is>
       </c>
-      <c r="F415" s="9" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F415" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -41099,7 +41099,7 @@
       </c>
       <c r="F445" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 404 for https://runbeck.net/careers</t>
+          <t xml:space="preserve">Unknown - robots.txt on runbeck.net answered HTTP </t>
         </is>
       </c>
     </row>
@@ -44795,7 +44795,7 @@
       </c>
       <c r="F580" s="21" t="inlineStr">
         <is>
-          <t>Unknown - robots.txt on www.proofpoint.com answere</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -45247,7 +45247,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/30/26)</t>
+          <t>Hiring AEs? (10/31/26)</t>
         </is>
       </c>
     </row>
@@ -47529,9 +47529,9 @@
           <t>WeatherTRAK smart irrigation and water management for public agencies</t>
         </is>
       </c>
-      <c r="F78" s="28" t="inlineStr">
-        <is>
-          <t>Unknown - HTTP 404 for https://www.hydropoint.com/</t>
+      <c r="F78" s="29" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -49625,7 +49625,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/30/26)</t>
+          <t>Hiring AEs? (10/31/26)</t>
         </is>
       </c>
     </row>
@@ -50487,9 +50487,9 @@
           <t>InformaCast mass notification and paging for school districts</t>
         </is>
       </c>
-      <c r="F30" s="35" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F30" s="34" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -50517,9 +50517,9 @@
           <t>Emergency mass notification hardware and software for schools and agencies - exhibited at EDUCAUSE 2026, IAEM 2026</t>
         </is>
       </c>
-      <c r="F31" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
+      <c r="F31" s="9" t="inlineStr">
+        <is>
+          <t>Yes - Account Manager (Baltimore, MD)</t>
         </is>
       </c>
     </row>
@@ -54037,9 +54037,9 @@
           <t>School payment and fundraising platform for K-12 districts, schools, PTOs and booster clubs, covering student fees, ticketing and stores - exhibited at ASBO School Business 2026</t>
         </is>
       </c>
-      <c r="F155" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F155" s="9" t="inlineStr">
+        <is>
+          <t>Yes - District Account Executive</t>
         </is>
       </c>
     </row>
@@ -54461,7 +54461,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/30/26)</t>
+          <t>Hiring AEs? (10/31/26)</t>
         </is>
       </c>
     </row>
@@ -54761,7 +54761,7 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Unknown - robots.txt on www.modeshift.com answered</t>
+          <t>Unknown - network error: robots.txt on www.modeshi</t>
         </is>
       </c>
     </row>
@@ -54877,7 +54877,7 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: robots.txt on www.pptexce</t>
         </is>
       </c>
     </row>
@@ -55399,7 +55399,7 @@
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 202 for https://www.enghouse.com/ca</t>
+          <t>Unknown - network error: robots.txt on www.enghous</t>
         </is>
       </c>
     </row>
@@ -57423,7 +57423,7 @@
       </c>
       <c r="F101" s="7" t="inlineStr">
         <is>
-          <t>Unknown - robots.txt on www.hanoverdisplays.com an</t>
+          <t>Unknown - network error: robots.txt on www.hanover</t>
         </is>
       </c>
     </row>
@@ -57631,7 +57631,7 @@
       </c>
       <c r="F108" s="39" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (Remix) (New York City)</t>
+          <t>Yes - Account Executive (Remix) (San Francisco)</t>
         </is>
       </c>
     </row>
@@ -57811,7 +57811,7 @@
       </c>
       <c r="F114" s="40" t="inlineStr">
         <is>
-          <t>Unknown - robots.txt on qryde.com answered HTTP 20</t>
+          <t>Unknown - network error: robots.txt on qryde.com d</t>
         </is>
       </c>
     </row>
@@ -60107,7 +60107,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/30/26)</t>
+          <t>Hiring AEs? (10/31/26)</t>
         </is>
       </c>
     </row>
@@ -64337,7 +64337,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/30/26)</t>
+          <t>Hiring AEs? (10/31/26)</t>
         </is>
       </c>
     </row>
@@ -65821,9 +65821,9 @@
           <t>Baggage handling systems and terminal logistics for airports</t>
         </is>
       </c>
-      <c r="F51" s="11" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -66693,7 +66693,7 @@
       </c>
       <c r="F80" s="52" t="inlineStr">
         <is>
-          <t>Yes - Senior Enterprise Account Executiv (Dallas, TX, United)</t>
+          <t>Yes - Senior Enterprise Account Executiv (Chicago, IL, Unite)</t>
         </is>
       </c>
     </row>
@@ -67831,7 +67831,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (10/30/26)</t>
+          <t>Hiring AEs? (10/31/26)</t>
         </is>
       </c>
     </row>

</xml_diff>